<commit_message>
Ongoing progress on the revision of all fields of LL reporting form
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572FFABB-AE42-4937-BE52-0B59947384C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A18521BD-DF0E-4F27-9D3E-9002B9472DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="MYxIjE9TGmSeigdKyCHOw3lH9f8J4EUilH0KgCjagDp50KBSM76xHJC56lRzGivfQGZgzVWvoHo9ImRSo1hl1A==" workbookSaltValue="vppty2a252bIjxbLncHPYg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" activeTab="4" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" activeTab="7" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -264,21 +264,6 @@
     <t>ADDITIONAL_BRANCHLINE_DETAILS</t>
   </si>
   <si>
-    <t>DEVICE_1_CODE</t>
-  </si>
-  <si>
-    <t>DEVICE_2_CODE</t>
-  </si>
-  <si>
-    <t>DEVICE_3_CODE</t>
-  </si>
-  <si>
-    <t>DEVICE_4_CODE</t>
-  </si>
-  <si>
-    <t>DEVICE_5_CODE</t>
-  </si>
-  <si>
     <t>STREAMER</t>
   </si>
   <si>
@@ -289,9 +274,6 @@
   </si>
   <si>
     <t>TOWED_OBJECTS</t>
-  </si>
-  <si>
-    <t>TORI_LINE_DETAILS</t>
   </si>
   <si>
     <t>CONFIGURATION_NUMBER</t>
@@ -696,9 +678,6 @@
     <t>GEAR</t>
   </si>
   <si>
-    <t>LINE_SETTER/SHOOTER</t>
-  </si>
-  <si>
     <t>Longline general gear specifications &gt; Mitigation devices</t>
   </si>
   <si>
@@ -766,18 +745,6 @@
   </si>
   <si>
     <t>IOTC_ID</t>
-  </si>
-  <si>
-    <t>LINE_LENGTH_MAX (M)</t>
-  </si>
-  <si>
-    <t>LINE_LENGTH_MIN (M)</t>
-  </si>
-  <si>
-    <t>DISTANCE_BETWEEN_STREAMERS (M)</t>
-  </si>
-  <si>
-    <t>TORI_LINE_ATTACHED_HEIGHT (M)</t>
   </si>
   <si>
     <t>PERSONNEL</t>
@@ -915,7 +882,7 @@
     <t>DIAMETER_CM</t>
   </si>
   <si>
-    <t>TORR_LINE_LENGTH</t>
+    <t>TORI_LINE_LENGTH</t>
   </si>
   <si>
     <t>FISH_STORAGE_CAPACITY_M3</t>
@@ -931,6 +898,39 @@
   </si>
   <si>
     <t>REGISTRATION_NUMBER</t>
+  </si>
+  <si>
+    <t>TORI LINE DETAILS</t>
+  </si>
+  <si>
+    <t>LINE_LENGTH_MAX_M</t>
+  </si>
+  <si>
+    <t>LINE_LENGTH_MIN_M</t>
+  </si>
+  <si>
+    <t>DISTANCE_BETWEEN_STREAMERS_M</t>
+  </si>
+  <si>
+    <t>TORI_LINE_ATTACHED_HEIGHT_M</t>
+  </si>
+  <si>
+    <t>DEVICE_1</t>
+  </si>
+  <si>
+    <t>LINE_SETTER_SHOOTER</t>
+  </si>
+  <si>
+    <t>DEVICE_2</t>
+  </si>
+  <si>
+    <t>DEVICE_3</t>
+  </si>
+  <si>
+    <t>DEVICE_4</t>
+  </si>
+  <si>
+    <t>DEVICE_5</t>
   </si>
 </sst>
 </file>
@@ -997,14 +997,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="10"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -1040,6 +1032,15 @@
       <b/>
       <u/>
       <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10"/>
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1364,7 +1365,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="196">
+  <cellXfs count="201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
@@ -1432,9 +1433,6 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1468,7 +1466,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1489,7 +1487,7 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1509,17 +1507,10 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1541,25 +1532,25 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1853,39 +1844,39 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1895,11 +1886,11 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1917,6 +1908,33 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -2260,282 +2278,282 @@
   <sheetData>
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="79" t="s">
-        <v>244</v>
+      <c r="B2" s="76" t="s">
+        <v>233</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="81"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="78"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="82"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="84"/>
+      <c r="B3" s="79"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="81"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="42"/>
-      <c r="C4" s="43" t="s">
+      <c r="B4" s="41"/>
+      <c r="C4" s="42" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>227</v>
+      </c>
+      <c r="E4" s="44"/>
+      <c r="F4" s="42" t="s">
+        <v>218</v>
+      </c>
+      <c r="G4" s="45">
+        <v>1</v>
+      </c>
+      <c r="H4" s="46"/>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="47"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="49"/>
+    </row>
+    <row r="6" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B6" s="47"/>
+      <c r="C6" s="50" t="s">
+        <v>219</v>
+      </c>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="49"/>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="47"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="49"/>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="47"/>
+      <c r="C8" s="82" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" s="82"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="82" t="s">
+        <v>234</v>
+      </c>
+      <c r="G8" s="82"/>
+      <c r="H8" s="49"/>
+    </row>
+    <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="47"/>
+      <c r="C9" s="51" t="s">
+        <v>220</v>
+      </c>
+      <c r="D9" s="52"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="G9" s="52"/>
+      <c r="H9" s="49"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="47"/>
+      <c r="C10" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="D10" s="52"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48" t="s">
+        <v>222</v>
+      </c>
+      <c r="G10" s="52"/>
+      <c r="H10" s="49"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="47"/>
+      <c r="C11" s="53"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="53"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="49"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="47"/>
+      <c r="C12" s="53" t="s">
+        <v>223</v>
+      </c>
+      <c r="D12" s="55"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
+      <c r="H12" s="49"/>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="47"/>
+      <c r="C13" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="D13" s="55"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="48"/>
+      <c r="G13" s="48"/>
+      <c r="H13" s="49"/>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="47"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="49"/>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="47"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
+      <c r="G15" s="56"/>
+      <c r="H15" s="49"/>
+    </row>
+    <row r="16" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B16" s="47"/>
+      <c r="C16" s="50" t="s">
         <v>224</v>
       </c>
-      <c r="D4" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="E4" s="45"/>
-      <c r="F4" s="43" t="s">
+      <c r="D16" s="48"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="48"/>
+      <c r="H16" s="49"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="47"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
+      <c r="H17" s="49"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="47"/>
+      <c r="C18" s="53" t="s">
         <v>225</v>
       </c>
-      <c r="G4" s="46">
-        <v>1</v>
-      </c>
-      <c r="H4" s="47"/>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="48"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="50"/>
-    </row>
-    <row r="6" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B6" s="48"/>
-      <c r="C6" s="51" t="s">
+      <c r="D18" s="57"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="53"/>
+      <c r="G18" s="53"/>
+      <c r="H18" s="49"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="47"/>
+      <c r="C19" s="58" t="s">
         <v>226</v>
       </c>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="50"/>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="48"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="48"/>
-      <c r="C8" s="85" t="s">
-        <v>246</v>
+      <c r="D19" s="57"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
+      <c r="H19" s="49"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="47"/>
+      <c r="C20" s="75" t="s">
+        <v>191</v>
       </c>
-      <c r="D8" s="85"/>
-      <c r="E8" s="49"/>
-      <c r="F8" s="85" t="s">
-        <v>245</v>
-      </c>
-      <c r="G8" s="85"/>
-      <c r="H8" s="50"/>
-    </row>
-    <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="48"/>
-      <c r="C9" s="52" t="s">
-        <v>227</v>
-      </c>
-      <c r="D9" s="53"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="52" t="s">
+      <c r="D20" s="57"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="49"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="47"/>
+      <c r="C21" s="53" t="s">
         <v>228</v>
       </c>
-      <c r="G9" s="53"/>
-      <c r="H9" s="50"/>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="48"/>
-      <c r="C10" s="54" t="s">
-        <v>229</v>
+      <c r="D21" s="57"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
+      <c r="H21" s="49"/>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="47"/>
+      <c r="C22" s="53"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="H22" s="49"/>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="47"/>
+      <c r="C23" s="59"/>
+      <c r="D23" s="60"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="49"/>
+    </row>
+    <row r="24" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B24" s="47"/>
+      <c r="C24" s="50" t="s">
+        <v>193</v>
       </c>
-      <c r="D10" s="53"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49" t="s">
-        <v>229</v>
-      </c>
-      <c r="G10" s="53"/>
-      <c r="H10" s="50"/>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="48"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="55"/>
-      <c r="E11" s="49"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="50"/>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="48"/>
-      <c r="C12" s="54" t="s">
-        <v>230</v>
-      </c>
-      <c r="D12" s="56"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="49"/>
-      <c r="H12" s="50"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="48"/>
-      <c r="C13" s="54" t="s">
-        <v>198</v>
-      </c>
-      <c r="D13" s="56"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="49"/>
-      <c r="H13" s="50"/>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="48"/>
-      <c r="C14" s="49"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="49"/>
-      <c r="H14" s="50"/>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="48"/>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="57"/>
-      <c r="G15" s="57"/>
-      <c r="H15" s="50"/>
-    </row>
-    <row r="16" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B16" s="48"/>
-      <c r="C16" s="51" t="s">
-        <v>231</v>
-      </c>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="50"/>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="48"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="49"/>
-      <c r="H17" s="50"/>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="48"/>
-      <c r="C18" s="54" t="s">
-        <v>232</v>
-      </c>
-      <c r="D18" s="58"/>
-      <c r="E18" s="49"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="50"/>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="48"/>
-      <c r="C19" s="59" t="s">
-        <v>233</v>
-      </c>
-      <c r="D19" s="58"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="50"/>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="48"/>
-      <c r="C20" s="78" t="s">
-        <v>197</v>
-      </c>
-      <c r="D20" s="58"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="49"/>
-      <c r="H20" s="50"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B21" s="48"/>
-      <c r="C21" s="54" t="s">
-        <v>235</v>
-      </c>
-      <c r="D21" s="58"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="50"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="48"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="55"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="49"/>
-      <c r="H22" s="50"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B23" s="48"/>
-      <c r="C23" s="60"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="50"/>
-    </row>
-    <row r="24" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B24" s="48"/>
-      <c r="C24" s="51" t="s">
-        <v>199</v>
-      </c>
-      <c r="D24" s="55"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="49"/>
-      <c r="H24" s="50"/>
+      <c r="D24" s="54"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="49"/>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="48"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="50"/>
+      <c r="B25" s="47"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="49"/>
     </row>
     <row r="26" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="48"/>
-      <c r="C26" s="86"/>
-      <c r="D26" s="87"/>
-      <c r="E26" s="87"/>
-      <c r="F26" s="87"/>
-      <c r="G26" s="88"/>
-      <c r="H26" s="50"/>
+      <c r="B26" s="47"/>
+      <c r="C26" s="83"/>
+      <c r="D26" s="84"/>
+      <c r="E26" s="84"/>
+      <c r="F26" s="84"/>
+      <c r="G26" s="85"/>
+      <c r="H26" s="49"/>
     </row>
     <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="62"/>
-      <c r="C27" s="63"/>
-      <c r="D27" s="63"/>
-      <c r="E27" s="63"/>
-      <c r="F27" s="63"/>
-      <c r="G27" s="63"/>
-      <c r="H27" s="64"/>
+      <c r="B27" s="61"/>
+      <c r="C27" s="62"/>
+      <c r="D27" s="62"/>
+      <c r="E27" s="62"/>
+      <c r="F27" s="62"/>
+      <c r="G27" s="62"/>
+      <c r="H27" s="63"/>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C28" s="1"/>
-      <c r="D28" s="65"/>
+      <c r="D28" s="64"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
@@ -2576,7 +2594,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -2584,45 +2602,45 @@
       <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
-        <v>211</v>
+      <c r="A2" s="89" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="92" t="s">
-        <v>216</v>
+      <c r="B2" s="89" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="120" t="s">
-        <v>81</v>
+      <c r="C2" s="117" t="s">
+        <v>75</v>
       </c>
-      <c r="D2" s="120"/>
-      <c r="E2" s="120"/>
+      <c r="D2" s="117"/>
+      <c r="E2" s="117"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
-      <c r="B3" s="92"/>
-      <c r="C3" s="94" t="s">
-        <v>90</v>
+      <c r="A3" s="89"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="91" t="s">
+        <v>84</v>
       </c>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="92"/>
-      <c r="C4" s="94"/>
-      <c r="D4" s="94"/>
-      <c r="E4" s="94"/>
+      <c r="A4" s="89"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="91"/>
+      <c r="D4" s="91"/>
+      <c r="E4" s="91"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="92"/>
+      <c r="A5" s="89"/>
+      <c r="B5" s="89"/>
       <c r="C5" s="23" t="s">
         <v>32</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
-      <c r="E5" s="72" t="s">
-        <v>193</v>
+      <c r="E5" s="69" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -4070,7 +4088,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -4089,115 +4107,115 @@
       <c r="P1" s="16"/>
     </row>
     <row r="2" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
-        <v>211</v>
+      <c r="A2" s="89" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="142" t="s">
-        <v>216</v>
+      <c r="B2" s="139" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="128" t="s">
-        <v>81</v>
+      <c r="C2" s="125" t="s">
+        <v>75</v>
       </c>
-      <c r="D2" s="129"/>
-      <c r="E2" s="129"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="129"/>
-      <c r="H2" s="129"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="129"/>
-      <c r="K2" s="129"/>
-      <c r="L2" s="129"/>
-      <c r="M2" s="129"/>
-      <c r="N2" s="129"/>
-      <c r="O2" s="129"/>
-      <c r="P2" s="130"/>
+      <c r="D2" s="126"/>
+      <c r="E2" s="126"/>
+      <c r="F2" s="126"/>
+      <c r="G2" s="126"/>
+      <c r="H2" s="126"/>
+      <c r="I2" s="126"/>
+      <c r="J2" s="126"/>
+      <c r="K2" s="126"/>
+      <c r="L2" s="126"/>
+      <c r="M2" s="126"/>
+      <c r="N2" s="126"/>
+      <c r="O2" s="126"/>
+      <c r="P2" s="127"/>
     </row>
     <row r="3" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
-      <c r="B3" s="143"/>
-      <c r="C3" s="128" t="s">
-        <v>105</v>
-      </c>
-      <c r="D3" s="129"/>
-      <c r="E3" s="129"/>
-      <c r="F3" s="129"/>
-      <c r="G3" s="129"/>
-      <c r="H3" s="129"/>
-      <c r="I3" s="129"/>
-      <c r="J3" s="129"/>
-      <c r="K3" s="129"/>
-      <c r="L3" s="129"/>
-      <c r="M3" s="129"/>
-      <c r="N3" s="129"/>
-      <c r="O3" s="129"/>
-      <c r="P3" s="130"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="143"/>
-      <c r="C4" s="135" t="s">
-        <v>187</v>
-      </c>
-      <c r="D4" s="135" t="s">
-        <v>106</v>
-      </c>
-      <c r="E4" s="135" t="s">
-        <v>107</v>
-      </c>
-      <c r="F4" s="113" t="s">
-        <v>98</v>
-      </c>
-      <c r="G4" s="135" t="s">
-        <v>109</v>
-      </c>
-      <c r="H4" s="135" t="s">
+      <c r="A3" s="89"/>
+      <c r="B3" s="140"/>
+      <c r="C3" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="I4" s="135" t="s">
+      <c r="D3" s="126"/>
+      <c r="E3" s="126"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="126"/>
+      <c r="H3" s="126"/>
+      <c r="I3" s="126"/>
+      <c r="J3" s="126"/>
+      <c r="K3" s="126"/>
+      <c r="L3" s="126"/>
+      <c r="M3" s="126"/>
+      <c r="N3" s="126"/>
+      <c r="O3" s="126"/>
+      <c r="P3" s="127"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="89"/>
+      <c r="B4" s="140"/>
+      <c r="C4" s="132" t="s">
+        <v>181</v>
+      </c>
+      <c r="D4" s="132" t="s">
         <v>100</v>
       </c>
-      <c r="J4" s="121" t="s">
-        <v>219</v>
+      <c r="E4" s="132" t="s">
+        <v>101</v>
       </c>
-      <c r="K4" s="99" t="s">
-        <v>110</v>
+      <c r="F4" s="110" t="s">
+        <v>92</v>
       </c>
-      <c r="L4" s="103"/>
-      <c r="M4" s="145" t="s">
-        <v>108</v>
+      <c r="G4" s="132" t="s">
+        <v>103</v>
       </c>
-      <c r="N4" s="146"/>
-      <c r="O4" s="146"/>
-      <c r="P4" s="147"/>
+      <c r="H4" s="132" t="s">
+        <v>93</v>
+      </c>
+      <c r="I4" s="132" t="s">
+        <v>94</v>
+      </c>
+      <c r="J4" s="118" t="s">
+        <v>212</v>
+      </c>
+      <c r="K4" s="96" t="s">
+        <v>104</v>
+      </c>
+      <c r="L4" s="100"/>
+      <c r="M4" s="142" t="s">
+        <v>102</v>
+      </c>
+      <c r="N4" s="143"/>
+      <c r="O4" s="143"/>
+      <c r="P4" s="144"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="144"/>
-      <c r="C5" s="136"/>
-      <c r="D5" s="136"/>
-      <c r="E5" s="136"/>
-      <c r="F5" s="114"/>
-      <c r="G5" s="136"/>
-      <c r="H5" s="136"/>
-      <c r="I5" s="136"/>
-      <c r="J5" s="123"/>
+      <c r="A5" s="89"/>
+      <c r="B5" s="141"/>
+      <c r="C5" s="133"/>
+      <c r="D5" s="133"/>
+      <c r="E5" s="133"/>
+      <c r="F5" s="111"/>
+      <c r="G5" s="133"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="120"/>
       <c r="K5" s="6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="M5" s="23" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="N5" s="23" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="O5" s="23" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="P5" s="23" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -7849,7 +7867,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -7857,47 +7875,47 @@
       <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
-        <v>211</v>
+      <c r="A2" s="89" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="92" t="s">
-        <v>216</v>
+      <c r="B2" s="89" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="120" t="s">
-        <v>81</v>
+      <c r="C2" s="117" t="s">
+        <v>75</v>
       </c>
-      <c r="D2" s="120"/>
-      <c r="E2" s="120"/>
+      <c r="D2" s="117"/>
+      <c r="E2" s="117"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
-      <c r="B3" s="92"/>
-      <c r="C3" s="145" t="s">
-        <v>154</v>
+      <c r="A3" s="89"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="142" t="s">
+        <v>148</v>
       </c>
-      <c r="D3" s="146"/>
-      <c r="E3" s="147"/>
+      <c r="D3" s="143"/>
+      <c r="E3" s="144"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="92"/>
-      <c r="C4" s="145" t="s">
-        <v>153</v>
+      <c r="A4" s="89"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="142" t="s">
+        <v>147</v>
       </c>
-      <c r="D4" s="146"/>
-      <c r="E4" s="147"/>
+      <c r="D4" s="143"/>
+      <c r="E4" s="144"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="92"/>
+      <c r="A5" s="89"/>
+      <c r="B5" s="89"/>
       <c r="C5" s="23" t="s">
         <v>32</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -9339,7 +9357,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -9348,53 +9366,53 @@
       <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
-        <v>211</v>
+      <c r="A2" s="89" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="92" t="s">
-        <v>216</v>
+      <c r="B2" s="89" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="120" t="s">
-        <v>81</v>
+      <c r="C2" s="117" t="s">
+        <v>75</v>
       </c>
-      <c r="D2" s="120"/>
-      <c r="E2" s="120"/>
-      <c r="F2" s="120"/>
+      <c r="D2" s="117"/>
+      <c r="E2" s="117"/>
+      <c r="F2" s="117"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
-      <c r="B3" s="92"/>
-      <c r="C3" s="145" t="s">
-        <v>155</v>
+      <c r="A3" s="89"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="142" t="s">
+        <v>149</v>
       </c>
-      <c r="D3" s="146"/>
-      <c r="E3" s="146"/>
-      <c r="F3" s="147"/>
+      <c r="D3" s="143"/>
+      <c r="E3" s="143"/>
+      <c r="F3" s="144"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="92"/>
-      <c r="C4" s="145" t="s">
-        <v>151</v>
+      <c r="A4" s="89"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="142" t="s">
+        <v>145</v>
       </c>
-      <c r="D4" s="146"/>
-      <c r="E4" s="146"/>
-      <c r="F4" s="147"/>
+      <c r="D4" s="143"/>
+      <c r="E4" s="143"/>
+      <c r="F4" s="144"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="92"/>
+      <c r="A5" s="89"/>
+      <c r="B5" s="89"/>
       <c r="C5" s="23" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -11045,7 +11063,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -11065,126 +11083,126 @@
       <c r="Q1" s="16"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
-        <v>211</v>
+      <c r="A2" s="89" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="92" t="s">
-        <v>216</v>
+      <c r="B2" s="89" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="75" t="s">
-        <v>119</v>
+      <c r="C2" s="72" t="s">
+        <v>113</v>
       </c>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="76"/>
-      <c r="P2" s="76"/>
-      <c r="Q2" s="77"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
+      <c r="P2" s="73"/>
+      <c r="Q2" s="74"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
-      <c r="B3" s="92"/>
-      <c r="C3" s="133" t="s">
-        <v>184</v>
+      <c r="A3" s="89"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="130" t="s">
+        <v>178</v>
       </c>
-      <c r="D3" s="137"/>
-      <c r="E3" s="134"/>
-      <c r="F3" s="133" t="s">
-        <v>185</v>
+      <c r="D3" s="134"/>
+      <c r="E3" s="131"/>
+      <c r="F3" s="130" t="s">
+        <v>179</v>
       </c>
-      <c r="G3" s="137"/>
-      <c r="H3" s="134"/>
-      <c r="I3" s="124" t="s">
+      <c r="G3" s="134"/>
+      <c r="H3" s="131"/>
+      <c r="I3" s="121" t="s">
+        <v>105</v>
+      </c>
+      <c r="J3" s="116" t="s">
+        <v>110</v>
+      </c>
+      <c r="K3" s="116"/>
+      <c r="L3" s="116"/>
+      <c r="M3" s="116"/>
+      <c r="N3" s="117" t="s">
         <v>111</v>
       </c>
-      <c r="J3" s="119" t="s">
-        <v>116</v>
+      <c r="O3" s="117" t="s">
+        <v>213</v>
       </c>
-      <c r="K3" s="119"/>
-      <c r="L3" s="119"/>
-      <c r="M3" s="119"/>
-      <c r="N3" s="120" t="s">
-        <v>117</v>
+      <c r="P3" s="117" t="s">
+        <v>180</v>
       </c>
-      <c r="O3" s="120" t="s">
-        <v>220</v>
+      <c r="Q3" s="145" t="s">
+        <v>112</v>
       </c>
-      <c r="P3" s="120" t="s">
-        <v>186</v>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="89"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="132" t="s">
+        <v>190</v>
       </c>
-      <c r="Q3" s="148" t="s">
-        <v>118</v>
+      <c r="D4" s="106" t="s">
+        <v>177</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="92"/>
-      <c r="C4" s="135" t="s">
-        <v>196</v>
+      <c r="E4" s="108"/>
+      <c r="F4" s="132" t="s">
+        <v>190</v>
       </c>
-      <c r="D4" s="109" t="s">
-        <v>183</v>
+      <c r="G4" s="106" t="s">
+        <v>177</v>
       </c>
-      <c r="E4" s="111"/>
-      <c r="F4" s="135" t="s">
-        <v>196</v>
-      </c>
-      <c r="G4" s="109" t="s">
-        <v>183</v>
-      </c>
-      <c r="H4" s="111"/>
-      <c r="I4" s="124"/>
-      <c r="J4" s="119"/>
-      <c r="K4" s="119"/>
-      <c r="L4" s="119"/>
-      <c r="M4" s="119"/>
-      <c r="N4" s="120"/>
-      <c r="O4" s="120"/>
-      <c r="P4" s="120"/>
-      <c r="Q4" s="148"/>
+      <c r="H4" s="108"/>
+      <c r="I4" s="121"/>
+      <c r="J4" s="116"/>
+      <c r="K4" s="116"/>
+      <c r="L4" s="116"/>
+      <c r="M4" s="116"/>
+      <c r="N4" s="117"/>
+      <c r="O4" s="117"/>
+      <c r="P4" s="117"/>
+      <c r="Q4" s="145"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="92"/>
-      <c r="C5" s="136"/>
-      <c r="D5" s="67" t="s">
+      <c r="A5" s="89"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="133"/>
+      <c r="D5" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="67" t="s">
+      <c r="E5" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="136"/>
-      <c r="G5" s="67" t="s">
+      <c r="F5" s="133"/>
+      <c r="G5" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="H5" s="67" t="s">
+      <c r="H5" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="I5" s="124"/>
+      <c r="I5" s="121"/>
       <c r="J5" s="19" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
-      <c r="N5" s="120"/>
-      <c r="O5" s="120"/>
-      <c r="P5" s="120"/>
-      <c r="Q5" s="148"/>
+      <c r="N5" s="117"/>
+      <c r="O5" s="117"/>
+      <c r="P5" s="117"/>
+      <c r="Q5" s="145"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -15037,48 +15055,48 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
       <c r="D1" s="16"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
-        <v>211</v>
+      <c r="A2" s="89" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="92" t="s">
-        <v>216</v>
+      <c r="B2" s="89" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="120" t="s">
-        <v>119</v>
+      <c r="C2" s="117" t="s">
+        <v>113</v>
       </c>
-      <c r="D2" s="120"/>
+      <c r="D2" s="117"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
-      <c r="B3" s="92"/>
-      <c r="C3" s="149" t="s">
-        <v>156</v>
+      <c r="A3" s="89"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="146" t="s">
+        <v>150</v>
       </c>
-      <c r="D3" s="150"/>
+      <c r="D3" s="147"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="92"/>
-      <c r="C4" s="149" t="s">
-        <v>82</v>
+      <c r="A4" s="89"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="146" t="s">
+        <v>76</v>
       </c>
-      <c r="D4" s="150"/>
+      <c r="D4" s="147"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="92"/>
+      <c r="A5" s="89"/>
+      <c r="B5" s="89"/>
       <c r="C5" s="6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -16317,7 +16335,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -16332,89 +16350,89 @@
       <c r="L1" s="16"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
-        <v>211</v>
+      <c r="A2" s="89" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="92" t="s">
-        <v>216</v>
+      <c r="B2" s="89" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="92" t="s">
-        <v>221</v>
+      <c r="C2" s="89" t="s">
+        <v>214</v>
       </c>
-      <c r="D2" s="94" t="s">
-        <v>121</v>
+      <c r="D2" s="91" t="s">
+        <v>115</v>
       </c>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="91"/>
+      <c r="L2" s="91"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
-      <c r="B3" s="92"/>
-      <c r="C3" s="92"/>
-      <c r="D3" s="148" t="s">
-        <v>93</v>
+      <c r="A3" s="89"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="145" t="s">
+        <v>87</v>
       </c>
-      <c r="E3" s="151" t="s">
-        <v>210</v>
+      <c r="E3" s="148" t="s">
+        <v>204</v>
       </c>
-      <c r="F3" s="152"/>
-      <c r="G3" s="148" t="s">
-        <v>158</v>
+      <c r="F3" s="149"/>
+      <c r="G3" s="145" t="s">
+        <v>152</v>
       </c>
-      <c r="H3" s="120" t="s">
-        <v>195</v>
+      <c r="H3" s="117" t="s">
+        <v>189</v>
       </c>
-      <c r="I3" s="119" t="s">
-        <v>122</v>
+      <c r="I3" s="116" t="s">
+        <v>116</v>
       </c>
-      <c r="J3" s="119"/>
-      <c r="K3" s="119"/>
-      <c r="L3" s="119"/>
+      <c r="J3" s="116"/>
+      <c r="K3" s="116"/>
+      <c r="L3" s="116"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="92"/>
-      <c r="C4" s="92"/>
-      <c r="D4" s="148"/>
-      <c r="E4" s="153"/>
-      <c r="F4" s="154"/>
-      <c r="G4" s="148"/>
-      <c r="H4" s="120"/>
-      <c r="I4" s="119"/>
-      <c r="J4" s="119"/>
-      <c r="K4" s="119"/>
-      <c r="L4" s="119"/>
+      <c r="A4" s="89"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="145"/>
+      <c r="E4" s="150"/>
+      <c r="F4" s="151"/>
+      <c r="G4" s="145"/>
+      <c r="H4" s="117"/>
+      <c r="I4" s="116"/>
+      <c r="J4" s="116"/>
+      <c r="K4" s="116"/>
+      <c r="L4" s="116"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="148"/>
-      <c r="E5" s="73" t="s">
+      <c r="A5" s="89"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="145"/>
+      <c r="E5" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="74" t="s">
-        <v>209</v>
+      <c r="F5" s="71" t="s">
+        <v>203</v>
       </c>
-      <c r="G5" s="148"/>
-      <c r="H5" s="120"/>
+      <c r="G5" s="145"/>
+      <c r="H5" s="117"/>
       <c r="I5" s="12" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>30</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -19283,7 +19301,7 @@
   <sheetData>
     <row r="1" spans="1:24" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -19310,143 +19328,143 @@
       <c r="X1" s="15"/>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A2" s="157" t="s">
-        <v>211</v>
+      <c r="A2" s="154" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="157" t="s">
-        <v>216</v>
+      <c r="B2" s="154" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="157" t="s">
-        <v>221</v>
+      <c r="C2" s="154" t="s">
+        <v>214</v>
       </c>
-      <c r="D2" s="157" t="s">
-        <v>222</v>
+      <c r="D2" s="154" t="s">
+        <v>215</v>
       </c>
       <c r="E2" s="28" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="F2" s="26"/>
       <c r="G2" s="26"/>
       <c r="H2" s="26"/>
       <c r="I2" s="26"/>
       <c r="J2" s="26"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
-      <c r="T2" s="36"/>
-      <c r="U2" s="36"/>
-      <c r="V2" s="36"/>
-      <c r="W2" s="36"/>
-      <c r="X2" s="36"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="35"/>
+      <c r="W2" s="35"/>
+      <c r="X2" s="35"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="158"/>
-      <c r="B3" s="158"/>
-      <c r="C3" s="158"/>
-      <c r="D3" s="158"/>
-      <c r="E3" s="160" t="s">
-        <v>157</v>
+      <c r="A3" s="155"/>
+      <c r="B3" s="155"/>
+      <c r="C3" s="155"/>
+      <c r="D3" s="155"/>
+      <c r="E3" s="157" t="s">
+        <v>151</v>
       </c>
-      <c r="F3" s="160" t="s">
-        <v>158</v>
+      <c r="F3" s="157" t="s">
+        <v>152</v>
       </c>
-      <c r="G3" s="92" t="s">
+      <c r="G3" s="89" t="s">
+        <v>118</v>
+      </c>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="89"/>
+      <c r="K3" s="90" t="s">
+        <v>119</v>
+      </c>
+      <c r="L3" s="90"/>
+      <c r="M3" s="90"/>
+      <c r="N3" s="90"/>
+      <c r="O3" s="90" t="s">
+        <v>116</v>
+      </c>
+      <c r="P3" s="90"/>
+      <c r="Q3" s="90"/>
+      <c r="R3" s="152" t="s">
+        <v>123</v>
+      </c>
+      <c r="S3" s="103" t="s">
+        <v>198</v>
+      </c>
+      <c r="T3" s="105"/>
+      <c r="U3" s="90" t="s">
+        <v>129</v>
+      </c>
+      <c r="V3" s="90"/>
+      <c r="W3" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="H3" s="92"/>
-      <c r="I3" s="92"/>
-      <c r="J3" s="92"/>
-      <c r="K3" s="93" t="s">
-        <v>125</v>
-      </c>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93" t="s">
-        <v>122</v>
-      </c>
-      <c r="P3" s="93"/>
-      <c r="Q3" s="93"/>
-      <c r="R3" s="155" t="s">
-        <v>129</v>
-      </c>
-      <c r="S3" s="106" t="s">
-        <v>204</v>
-      </c>
-      <c r="T3" s="108"/>
-      <c r="U3" s="93" t="s">
-        <v>135</v>
-      </c>
-      <c r="V3" s="93"/>
-      <c r="W3" s="93" t="s">
-        <v>130</v>
-      </c>
-      <c r="X3" s="93"/>
+      <c r="X3" s="90"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="159"/>
-      <c r="B4" s="159"/>
-      <c r="C4" s="159"/>
-      <c r="D4" s="159"/>
-      <c r="E4" s="161"/>
-      <c r="F4" s="161"/>
+      <c r="A4" s="156"/>
+      <c r="B4" s="156"/>
+      <c r="C4" s="156"/>
+      <c r="D4" s="156"/>
+      <c r="E4" s="158"/>
+      <c r="F4" s="158"/>
       <c r="G4" s="23" t="s">
         <v>32</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J4" s="24" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="K4" s="12" t="s">
         <v>32</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="O4" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="P4" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="P4" s="6" t="s">
-        <v>126</v>
+      <c r="Q4" s="12" t="s">
+        <v>121</v>
       </c>
-      <c r="Q4" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="R4" s="156"/>
+      <c r="R4" s="153"/>
       <c r="S4" s="9" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="T4" s="7" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="U4" s="8" t="s">
         <v>31</v>
       </c>
       <c r="V4" s="6" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
@@ -24718,7 +24736,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -24736,101 +24754,101 @@
       <c r="O1" s="15"/>
       <c r="P1" s="15"/>
       <c r="Q1" s="15"/>
-      <c r="R1" s="39"/>
-      <c r="S1" s="39"/>
-      <c r="T1" s="39"/>
+      <c r="R1" s="38"/>
+      <c r="S1" s="38"/>
+      <c r="T1" s="38"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="157" t="s">
-        <v>211</v>
+      <c r="A2" s="154" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="157" t="s">
-        <v>216</v>
+      <c r="B2" s="154" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="157" t="s">
-        <v>221</v>
+      <c r="C2" s="154" t="s">
+        <v>214</v>
       </c>
-      <c r="D2" s="157" t="s">
-        <v>222</v>
+      <c r="D2" s="154" t="s">
+        <v>215</v>
       </c>
-      <c r="E2" s="162" t="s">
-        <v>150</v>
+      <c r="E2" s="159" t="s">
+        <v>144</v>
       </c>
-      <c r="F2" s="163"/>
-      <c r="G2" s="163"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="37"/>
-      <c r="M2" s="37"/>
-      <c r="N2" s="37"/>
-      <c r="O2" s="37"/>
-      <c r="P2" s="37"/>
-      <c r="Q2" s="37"/>
-      <c r="R2" s="37"/>
-      <c r="S2" s="38"/>
-      <c r="T2" s="38"/>
+      <c r="F2" s="160"/>
+      <c r="G2" s="160"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="36"/>
+      <c r="P2" s="36"/>
+      <c r="Q2" s="36"/>
+      <c r="R2" s="36"/>
+      <c r="S2" s="37"/>
+      <c r="T2" s="37"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="158"/>
-      <c r="B3" s="158"/>
-      <c r="C3" s="158"/>
-      <c r="D3" s="158"/>
-      <c r="E3" s="164" t="s">
-        <v>132</v>
+      <c r="A3" s="155"/>
+      <c r="B3" s="155"/>
+      <c r="C3" s="155"/>
+      <c r="D3" s="155"/>
+      <c r="E3" s="161" t="s">
+        <v>126</v>
       </c>
-      <c r="F3" s="164" t="s">
-        <v>133</v>
+      <c r="F3" s="161" t="s">
+        <v>127</v>
       </c>
-      <c r="G3" s="166" t="s">
+      <c r="G3" s="163" t="s">
+        <v>136</v>
+      </c>
+      <c r="H3" s="165" t="s">
+        <v>137</v>
+      </c>
+      <c r="I3" s="92" t="s">
+        <v>145</v>
+      </c>
+      <c r="J3" s="93"/>
+      <c r="K3" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="L3" s="93"/>
+      <c r="M3" s="165" t="s">
+        <v>140</v>
+      </c>
+      <c r="N3" s="167" t="s">
+        <v>154</v>
+      </c>
+      <c r="O3" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="P3" s="165" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q3" s="167" t="s">
         <v>142</v>
       </c>
-      <c r="H3" s="168" t="s">
+      <c r="R3" s="167" t="s">
         <v>143</v>
       </c>
-      <c r="I3" s="95" t="s">
-        <v>151</v>
+      <c r="S3" s="122" t="s">
+        <v>124</v>
       </c>
-      <c r="J3" s="96"/>
-      <c r="K3" s="95" t="s">
-        <v>152</v>
-      </c>
-      <c r="L3" s="96"/>
-      <c r="M3" s="168" t="s">
-        <v>146</v>
-      </c>
-      <c r="N3" s="170" t="s">
-        <v>160</v>
-      </c>
-      <c r="O3" s="170" t="s">
-        <v>147</v>
-      </c>
-      <c r="P3" s="168" t="s">
-        <v>200</v>
-      </c>
-      <c r="Q3" s="170" t="s">
-        <v>148</v>
-      </c>
-      <c r="R3" s="170" t="s">
-        <v>149</v>
-      </c>
-      <c r="S3" s="125" t="s">
-        <v>130</v>
-      </c>
-      <c r="T3" s="125"/>
+      <c r="T3" s="122"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" s="159"/>
-      <c r="B4" s="159"/>
-      <c r="C4" s="159"/>
-      <c r="D4" s="159"/>
-      <c r="E4" s="165"/>
-      <c r="F4" s="165"/>
-      <c r="G4" s="167"/>
-      <c r="H4" s="169"/>
+      <c r="A4" s="156"/>
+      <c r="B4" s="156"/>
+      <c r="C4" s="156"/>
+      <c r="D4" s="156"/>
+      <c r="E4" s="162"/>
+      <c r="F4" s="162"/>
+      <c r="G4" s="164"/>
+      <c r="H4" s="166"/>
       <c r="I4" s="12" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="J4" s="12" t="s">
         <v>32</v>
@@ -24839,19 +24857,19 @@
         <v>65</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
-      <c r="M4" s="169"/>
-      <c r="N4" s="114"/>
-      <c r="O4" s="114"/>
-      <c r="P4" s="169"/>
-      <c r="Q4" s="114"/>
-      <c r="R4" s="114"/>
-      <c r="S4" s="35" t="s">
-        <v>131</v>
+      <c r="M4" s="166"/>
+      <c r="N4" s="111"/>
+      <c r="O4" s="111"/>
+      <c r="P4" s="166"/>
+      <c r="Q4" s="111"/>
+      <c r="R4" s="111"/>
+      <c r="S4" s="34" t="s">
+        <v>125</v>
       </c>
-      <c r="T4" s="35" t="s">
-        <v>201</v>
+      <c r="T4" s="34" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
@@ -29318,7 +29336,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -29332,53 +29350,53 @@
       <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="157" t="s">
-        <v>211</v>
+      <c r="A2" s="154" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="157" t="s">
-        <v>216</v>
+      <c r="B2" s="154" t="s">
+        <v>209</v>
       </c>
-      <c r="C2" s="157" t="s">
-        <v>221</v>
+      <c r="C2" s="154" t="s">
+        <v>214</v>
       </c>
-      <c r="D2" s="157" t="s">
-        <v>222</v>
+      <c r="D2" s="154" t="s">
+        <v>215</v>
       </c>
-      <c r="E2" s="171" t="s">
-        <v>140</v>
+      <c r="E2" s="168" t="s">
+        <v>134</v>
       </c>
-      <c r="F2" s="172"/>
-      <c r="G2" s="172"/>
-      <c r="H2" s="172"/>
-      <c r="I2" s="172"/>
-      <c r="J2" s="172"/>
-      <c r="K2" s="173"/>
+      <c r="F2" s="169"/>
+      <c r="G2" s="169"/>
+      <c r="H2" s="169"/>
+      <c r="I2" s="169"/>
+      <c r="J2" s="169"/>
+      <c r="K2" s="170"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="159"/>
-      <c r="B3" s="159"/>
-      <c r="C3" s="159"/>
-      <c r="D3" s="159"/>
+      <c r="A3" s="156"/>
+      <c r="B3" s="156"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
       <c r="E3" s="25" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
-      <c r="G3" s="35" t="s">
+      <c r="G3" s="34" t="s">
         <v>32</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="I3" s="25" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="J3" s="25" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="K3" s="25" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -32038,7 +32056,7 @@
   <sheetData>
     <row r="1" spans="1:25" s="17" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -32065,181 +32083,181 @@
       <c r="X1" s="16"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" s="89" t="s">
-        <v>211</v>
+      <c r="A2" s="86" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="97" t="s">
-        <v>288</v>
+      <c r="B2" s="94" t="s">
+        <v>277</v>
       </c>
-      <c r="C2" s="97"/>
-      <c r="D2" s="98" t="s">
-        <v>289</v>
+      <c r="C2" s="94"/>
+      <c r="D2" s="95" t="s">
+        <v>278</v>
       </c>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98"/>
-      <c r="N2" s="138" t="s">
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="135" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="193"/>
-      <c r="P2" s="193"/>
-      <c r="Q2" s="193"/>
-      <c r="R2" s="193"/>
-      <c r="S2" s="193"/>
-      <c r="T2" s="193"/>
-      <c r="U2" s="193"/>
-      <c r="V2" s="193"/>
-      <c r="W2" s="193"/>
-      <c r="X2" s="139"/>
+      <c r="O2" s="190"/>
+      <c r="P2" s="190"/>
+      <c r="Q2" s="190"/>
+      <c r="R2" s="190"/>
+      <c r="S2" s="190"/>
+      <c r="T2" s="190"/>
+      <c r="U2" s="190"/>
+      <c r="V2" s="190"/>
+      <c r="W2" s="190"/>
+      <c r="X2" s="136"/>
       <c r="Y2" s="4"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="90"/>
-      <c r="B3" s="97"/>
-      <c r="C3" s="97"/>
-      <c r="D3" s="99" t="s">
-        <v>179</v>
+      <c r="A3" s="87"/>
+      <c r="B3" s="94"/>
+      <c r="C3" s="94"/>
+      <c r="D3" s="96" t="s">
+        <v>173</v>
       </c>
-      <c r="E3" s="100"/>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="103"/>
-      <c r="I3" s="99" t="s">
-        <v>180</v>
+      <c r="E3" s="97"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="97"/>
+      <c r="H3" s="100"/>
+      <c r="I3" s="96" t="s">
+        <v>174</v>
       </c>
-      <c r="J3" s="100"/>
-      <c r="K3" s="100"/>
-      <c r="L3" s="100"/>
-      <c r="M3" s="100"/>
-      <c r="N3" s="140"/>
-      <c r="O3" s="194"/>
-      <c r="P3" s="194"/>
-      <c r="Q3" s="194"/>
-      <c r="R3" s="194"/>
-      <c r="S3" s="194"/>
-      <c r="T3" s="194"/>
-      <c r="U3" s="194"/>
-      <c r="V3" s="194"/>
-      <c r="W3" s="194"/>
-      <c r="X3" s="141"/>
+      <c r="J3" s="97"/>
+      <c r="K3" s="97"/>
+      <c r="L3" s="97"/>
+      <c r="M3" s="97"/>
+      <c r="N3" s="137"/>
+      <c r="O3" s="191"/>
+      <c r="P3" s="191"/>
+      <c r="Q3" s="191"/>
+      <c r="R3" s="191"/>
+      <c r="S3" s="191"/>
+      <c r="T3" s="191"/>
+      <c r="U3" s="191"/>
+      <c r="V3" s="191"/>
+      <c r="W3" s="191"/>
+      <c r="X3" s="138"/>
       <c r="Y3" s="4"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="90"/>
-      <c r="B4" s="97"/>
-      <c r="C4" s="97"/>
-      <c r="D4" s="95" t="s">
-        <v>177</v>
+      <c r="A4" s="87"/>
+      <c r="B4" s="94"/>
+      <c r="C4" s="94"/>
+      <c r="D4" s="92" t="s">
+        <v>171</v>
       </c>
-      <c r="E4" s="96"/>
-      <c r="F4" s="95" t="s">
-        <v>178</v>
+      <c r="E4" s="93"/>
+      <c r="F4" s="92" t="s">
+        <v>172</v>
       </c>
-      <c r="G4" s="96"/>
-      <c r="H4" s="104" t="s">
-        <v>196</v>
+      <c r="G4" s="93"/>
+      <c r="H4" s="101" t="s">
+        <v>190</v>
       </c>
-      <c r="I4" s="95" t="s">
-        <v>177</v>
+      <c r="I4" s="92" t="s">
+        <v>171</v>
       </c>
-      <c r="J4" s="96"/>
-      <c r="K4" s="95" t="s">
-        <v>178</v>
+      <c r="J4" s="93"/>
+      <c r="K4" s="92" t="s">
+        <v>172</v>
       </c>
-      <c r="L4" s="96"/>
-      <c r="M4" s="101" t="s">
-        <v>196</v>
+      <c r="L4" s="93"/>
+      <c r="M4" s="98" t="s">
+        <v>190</v>
       </c>
-      <c r="N4" s="92" t="s">
-        <v>290</v>
+      <c r="N4" s="89" t="s">
+        <v>279</v>
       </c>
-      <c r="O4" s="92"/>
-      <c r="P4" s="93" t="s">
+      <c r="O4" s="89"/>
+      <c r="P4" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="Q4" s="93"/>
-      <c r="R4" s="93"/>
-      <c r="S4" s="93"/>
-      <c r="T4" s="93"/>
-      <c r="U4" s="93" t="s">
+      <c r="Q4" s="90"/>
+      <c r="R4" s="90"/>
+      <c r="S4" s="90"/>
+      <c r="T4" s="90"/>
+      <c r="U4" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="V4" s="93"/>
-      <c r="W4" s="93"/>
-      <c r="X4" s="93"/>
+      <c r="V4" s="90"/>
+      <c r="W4" s="90"/>
+      <c r="X4" s="90"/>
     </row>
     <row r="5" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="91"/>
-      <c r="B5" s="66" t="s">
-        <v>236</v>
+      <c r="A5" s="88"/>
+      <c r="B5" s="65" t="s">
+        <v>229</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="178" t="s">
-        <v>247</v>
+      <c r="D5" s="175" t="s">
+        <v>236</v>
       </c>
-      <c r="E5" s="178" t="s">
+      <c r="E5" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="41" t="s">
+      <c r="F5" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="G5" s="41" t="s">
+      <c r="G5" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="H5" s="105"/>
-      <c r="I5" s="178" t="s">
-        <v>247</v>
+      <c r="H5" s="102"/>
+      <c r="I5" s="175" t="s">
+        <v>236</v>
       </c>
-      <c r="J5" s="178" t="s">
+      <c r="J5" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="41" t="s">
+      <c r="K5" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="L5" s="41" t="s">
+      <c r="L5" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="M5" s="102"/>
-      <c r="N5" s="66" t="s">
+      <c r="M5" s="99"/>
+      <c r="N5" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="O5" s="66" t="s">
+      <c r="O5" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="P5" s="41" t="s">
+      <c r="P5" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="Q5" s="41" t="s">
+      <c r="Q5" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="41" t="s">
+      <c r="R5" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="S5" s="41" t="s">
+      <c r="S5" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="T5" s="41" t="s">
+      <c r="T5" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="U5" s="179" t="s">
-        <v>248</v>
+      <c r="U5" s="176" t="s">
+        <v>237</v>
       </c>
-      <c r="V5" s="179" t="s">
-        <v>249</v>
+      <c r="V5" s="176" t="s">
+        <v>238</v>
       </c>
-      <c r="W5" s="179" t="s">
-        <v>250</v>
+      <c r="W5" s="176" t="s">
+        <v>239</v>
       </c>
-      <c r="X5" s="179" t="s">
-        <v>251</v>
+      <c r="X5" s="176" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -37483,7 +37501,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -37502,8 +37520,8 @@
       <c r="P1" s="16"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="97" t="s">
-        <v>211</v>
+      <c r="A2" s="94" t="s">
+        <v>205</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>26</v>
@@ -37524,102 +37542,102 @@
       <c r="P2" s="27"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="97"/>
-      <c r="B3" s="109" t="s">
+      <c r="A3" s="94"/>
+      <c r="B3" s="106" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="110"/>
-      <c r="D3" s="110"/>
-      <c r="E3" s="110"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="106" t="s">
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="107"/>
-      <c r="I3" s="108"/>
-      <c r="J3" s="187" t="s">
+      <c r="H3" s="104"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="40" t="s">
-        <v>212</v>
+      <c r="K3" s="39" t="s">
+        <v>206</v>
       </c>
-      <c r="L3" s="109" t="s">
+      <c r="L3" s="106" t="s">
+        <v>230</v>
+      </c>
+      <c r="M3" s="107"/>
+      <c r="N3" s="107"/>
+      <c r="O3" s="107"/>
+      <c r="P3" s="108"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="94"/>
+      <c r="B4" s="94" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="177" t="s">
         <v>241</v>
       </c>
-      <c r="M3" s="110"/>
-      <c r="N3" s="110"/>
-      <c r="O3" s="110"/>
-      <c r="P3" s="111"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="97"/>
-      <c r="B4" s="97" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="180" t="s">
-        <v>252</v>
-      </c>
-      <c r="D4" s="94" t="s">
+      <c r="D4" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="104" t="s">
+      <c r="E4" s="101" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="98" t="s">
+      <c r="F4" s="95" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="181" t="s">
-        <v>247</v>
+      <c r="G4" s="178" t="s">
+        <v>236</v>
       </c>
-      <c r="H4" s="182" t="s">
+      <c r="H4" s="179" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="195" t="s">
-        <v>291</v>
+      <c r="I4" s="192" t="s">
+        <v>280</v>
       </c>
-      <c r="J4" s="181" t="s">
-        <v>253</v>
+      <c r="J4" s="178" t="s">
+        <v>242</v>
       </c>
-      <c r="K4" s="184" t="s">
-        <v>254</v>
+      <c r="K4" s="181" t="s">
+        <v>243</v>
       </c>
-      <c r="L4" s="92" t="s">
+      <c r="L4" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="M4" s="92"/>
-      <c r="N4" s="92" t="s">
+      <c r="M4" s="89"/>
+      <c r="N4" s="89" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="92"/>
-      <c r="P4" s="98" t="s">
+      <c r="O4" s="89"/>
+      <c r="P4" s="95" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="97"/>
-      <c r="B5" s="97"/>
-      <c r="C5" s="180"/>
-      <c r="D5" s="94"/>
-      <c r="E5" s="105"/>
-      <c r="F5" s="98"/>
-      <c r="G5" s="181"/>
-      <c r="H5" s="183"/>
-      <c r="I5" s="195"/>
-      <c r="J5" s="181"/>
-      <c r="K5" s="185"/>
+      <c r="A5" s="94"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="177"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="95"/>
+      <c r="G5" s="178"/>
+      <c r="H5" s="180"/>
+      <c r="I5" s="192"/>
+      <c r="J5" s="178"/>
+      <c r="K5" s="182"/>
       <c r="L5" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="M5" s="186" t="s">
+      <c r="M5" s="183" t="s">
         <v>5</v>
       </c>
       <c r="N5" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="O5" s="186" t="s">
+      <c r="O5" s="183" t="s">
         <v>5</v>
       </c>
-      <c r="P5" s="98"/>
+      <c r="P5" s="95"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -41285,7 +41303,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -41299,88 +41317,88 @@
       <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="97" t="s">
-        <v>211</v>
+      <c r="A2" s="94" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="98" t="s">
+      <c r="B2" s="95" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="97"/>
-      <c r="B3" s="98" t="s">
+      <c r="A3" s="94"/>
+      <c r="B3" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="98"/>
-      <c r="D3" s="98"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98" t="s">
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="95" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="98"/>
-      <c r="I3" s="98"/>
-      <c r="J3" s="98"/>
-      <c r="K3" s="98"/>
+      <c r="H3" s="95"/>
+      <c r="I3" s="95"/>
+      <c r="J3" s="95"/>
+      <c r="K3" s="95"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="97"/>
-      <c r="B4" s="99" t="s">
+      <c r="A4" s="94"/>
+      <c r="B4" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="100"/>
-      <c r="D4" s="100"/>
-      <c r="E4" s="100"/>
-      <c r="F4" s="104" t="s">
-        <v>196</v>
+      <c r="C4" s="97"/>
+      <c r="D4" s="97"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="101" t="s">
+        <v>190</v>
       </c>
-      <c r="G4" s="99" t="s">
+      <c r="G4" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="100"/>
-      <c r="I4" s="100"/>
-      <c r="J4" s="103"/>
-      <c r="K4" s="101" t="s">
-        <v>196</v>
+      <c r="H4" s="97"/>
+      <c r="I4" s="97"/>
+      <c r="J4" s="100"/>
+      <c r="K4" s="98" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="97"/>
-      <c r="B5" s="178" t="s">
-        <v>247</v>
+      <c r="A5" s="94"/>
+      <c r="B5" s="175" t="s">
+        <v>236</v>
       </c>
-      <c r="C5" s="178" t="s">
+      <c r="C5" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="191" t="s">
+      <c r="D5" s="188" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="191" t="s">
+      <c r="E5" s="188" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="105"/>
-      <c r="G5" s="178" t="s">
-        <v>247</v>
+      <c r="F5" s="102"/>
+      <c r="G5" s="175" t="s">
+        <v>236</v>
       </c>
-      <c r="H5" s="178" t="s">
+      <c r="H5" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="191" t="s">
+      <c r="I5" s="188" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="191" t="s">
+      <c r="J5" s="188" t="s">
         <v>1</v>
       </c>
-      <c r="K5" s="102"/>
+      <c r="K5" s="99"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -44061,7 +44079,7 @@
   <sheetData>
     <row r="1" spans="1:41" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -44105,207 +44123,207 @@
       <c r="AO1" s="15"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A2" s="97" t="s">
-        <v>211</v>
+      <c r="A2" s="94" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="119" t="s">
+      <c r="B2" s="116" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
-      <c r="I2" s="119"/>
-      <c r="J2" s="119"/>
-      <c r="K2" s="119"/>
-      <c r="L2" s="119"/>
-      <c r="M2" s="119"/>
-      <c r="N2" s="119"/>
-      <c r="O2" s="119"/>
-      <c r="P2" s="119"/>
-      <c r="Q2" s="119"/>
-      <c r="R2" s="119"/>
-      <c r="S2" s="119"/>
-      <c r="T2" s="119"/>
-      <c r="U2" s="115" t="s">
+      <c r="C2" s="116"/>
+      <c r="D2" s="116"/>
+      <c r="E2" s="116"/>
+      <c r="F2" s="116"/>
+      <c r="G2" s="116"/>
+      <c r="H2" s="116"/>
+      <c r="I2" s="116"/>
+      <c r="J2" s="116"/>
+      <c r="K2" s="116"/>
+      <c r="L2" s="116"/>
+      <c r="M2" s="116"/>
+      <c r="N2" s="116"/>
+      <c r="O2" s="116"/>
+      <c r="P2" s="116"/>
+      <c r="Q2" s="116"/>
+      <c r="R2" s="116"/>
+      <c r="S2" s="116"/>
+      <c r="T2" s="116"/>
+      <c r="U2" s="112" t="s">
         <v>56</v>
       </c>
-      <c r="V2" s="116"/>
-      <c r="W2" s="116"/>
-      <c r="X2" s="116"/>
-      <c r="Y2" s="116"/>
-      <c r="Z2" s="116"/>
-      <c r="AA2" s="116"/>
-      <c r="AB2" s="116"/>
-      <c r="AC2" s="116"/>
-      <c r="AD2" s="116"/>
-      <c r="AE2" s="116"/>
-      <c r="AF2" s="116"/>
-      <c r="AG2" s="117"/>
-      <c r="AH2" s="115" t="s">
+      <c r="V2" s="113"/>
+      <c r="W2" s="113"/>
+      <c r="X2" s="113"/>
+      <c r="Y2" s="113"/>
+      <c r="Z2" s="113"/>
+      <c r="AA2" s="113"/>
+      <c r="AB2" s="113"/>
+      <c r="AC2" s="113"/>
+      <c r="AD2" s="113"/>
+      <c r="AE2" s="113"/>
+      <c r="AF2" s="113"/>
+      <c r="AG2" s="114"/>
+      <c r="AH2" s="112" t="s">
         <v>61</v>
       </c>
-      <c r="AI2" s="116"/>
-      <c r="AJ2" s="116"/>
-      <c r="AK2" s="116"/>
-      <c r="AL2" s="116"/>
-      <c r="AM2" s="116"/>
-      <c r="AN2" s="116"/>
-      <c r="AO2" s="117"/>
+      <c r="AI2" s="113"/>
+      <c r="AJ2" s="113"/>
+      <c r="AK2" s="113"/>
+      <c r="AL2" s="113"/>
+      <c r="AM2" s="113"/>
+      <c r="AN2" s="113"/>
+      <c r="AO2" s="114"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A3" s="97"/>
-      <c r="B3" s="119"/>
-      <c r="C3" s="119"/>
-      <c r="D3" s="119"/>
-      <c r="E3" s="119"/>
-      <c r="F3" s="119"/>
-      <c r="G3" s="119"/>
-      <c r="H3" s="119"/>
-      <c r="I3" s="119"/>
-      <c r="J3" s="119"/>
-      <c r="K3" s="119"/>
-      <c r="L3" s="119"/>
-      <c r="M3" s="119"/>
-      <c r="N3" s="119"/>
-      <c r="O3" s="119"/>
-      <c r="P3" s="119"/>
-      <c r="Q3" s="119"/>
-      <c r="R3" s="119"/>
-      <c r="S3" s="119"/>
-      <c r="T3" s="119"/>
-      <c r="U3" s="95"/>
-      <c r="V3" s="118"/>
-      <c r="W3" s="118"/>
-      <c r="X3" s="118"/>
-      <c r="Y3" s="118"/>
-      <c r="Z3" s="118"/>
-      <c r="AA3" s="118"/>
-      <c r="AB3" s="118"/>
-      <c r="AC3" s="118"/>
-      <c r="AD3" s="118"/>
-      <c r="AE3" s="118"/>
-      <c r="AF3" s="118"/>
-      <c r="AG3" s="96"/>
-      <c r="AH3" s="95"/>
-      <c r="AI3" s="118"/>
-      <c r="AJ3" s="118"/>
-      <c r="AK3" s="118"/>
-      <c r="AL3" s="118"/>
-      <c r="AM3" s="118"/>
-      <c r="AN3" s="118"/>
-      <c r="AO3" s="96"/>
+      <c r="A3" s="94"/>
+      <c r="B3" s="116"/>
+      <c r="C3" s="116"/>
+      <c r="D3" s="116"/>
+      <c r="E3" s="116"/>
+      <c r="F3" s="116"/>
+      <c r="G3" s="116"/>
+      <c r="H3" s="116"/>
+      <c r="I3" s="116"/>
+      <c r="J3" s="116"/>
+      <c r="K3" s="116"/>
+      <c r="L3" s="116"/>
+      <c r="M3" s="116"/>
+      <c r="N3" s="116"/>
+      <c r="O3" s="116"/>
+      <c r="P3" s="116"/>
+      <c r="Q3" s="116"/>
+      <c r="R3" s="116"/>
+      <c r="S3" s="116"/>
+      <c r="T3" s="116"/>
+      <c r="U3" s="92"/>
+      <c r="V3" s="115"/>
+      <c r="W3" s="115"/>
+      <c r="X3" s="115"/>
+      <c r="Y3" s="115"/>
+      <c r="Z3" s="115"/>
+      <c r="AA3" s="115"/>
+      <c r="AB3" s="115"/>
+      <c r="AC3" s="115"/>
+      <c r="AD3" s="115"/>
+      <c r="AE3" s="115"/>
+      <c r="AF3" s="115"/>
+      <c r="AG3" s="93"/>
+      <c r="AH3" s="92"/>
+      <c r="AI3" s="115"/>
+      <c r="AJ3" s="115"/>
+      <c r="AK3" s="115"/>
+      <c r="AL3" s="115"/>
+      <c r="AM3" s="115"/>
+      <c r="AN3" s="115"/>
+      <c r="AO3" s="93"/>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A4" s="97"/>
-      <c r="B4" s="104" t="s">
-        <v>256</v>
+      <c r="A4" s="94"/>
+      <c r="B4" s="101" t="s">
+        <v>245</v>
       </c>
-      <c r="C4" s="104" t="s">
+      <c r="C4" s="101" t="s">
+        <v>246</v>
+      </c>
+      <c r="D4" s="186" t="s">
+        <v>247</v>
+      </c>
+      <c r="E4" s="90" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="101" t="s">
+        <v>276</v>
+      </c>
+      <c r="L4" s="90" t="s">
+        <v>41</v>
+      </c>
+      <c r="M4" s="90"/>
+      <c r="N4" s="90"/>
+      <c r="O4" s="90"/>
+      <c r="P4" s="90" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q4" s="90"/>
+      <c r="R4" s="90"/>
+      <c r="S4" s="90" t="s">
+        <v>42</v>
+      </c>
+      <c r="T4" s="90"/>
+      <c r="U4" s="95" t="s">
         <v>257</v>
       </c>
-      <c r="D4" s="189" t="s">
-        <v>258</v>
-      </c>
-      <c r="E4" s="93" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="93"/>
-      <c r="G4" s="93"/>
-      <c r="H4" s="93" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" s="93"/>
-      <c r="J4" s="93"/>
-      <c r="K4" s="104" t="s">
-        <v>287</v>
-      </c>
-      <c r="L4" s="93" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="93"/>
-      <c r="N4" s="93"/>
-      <c r="O4" s="93"/>
-      <c r="P4" s="93" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q4" s="93"/>
-      <c r="R4" s="93"/>
-      <c r="S4" s="93" t="s">
-        <v>42</v>
-      </c>
-      <c r="T4" s="93"/>
-      <c r="U4" s="98" t="s">
-        <v>268</v>
-      </c>
-      <c r="V4" s="98" t="s">
+      <c r="V4" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="W4" s="98" t="s">
+      <c r="W4" s="95" t="s">
         <v>55</v>
       </c>
-      <c r="X4" s="98" t="s">
+      <c r="X4" s="95" t="s">
         <v>46</v>
       </c>
-      <c r="Y4" s="98" t="s">
+      <c r="Y4" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="Z4" s="98" t="s">
+      <c r="Z4" s="95" t="s">
         <v>48</v>
       </c>
-      <c r="AA4" s="98" t="s">
+      <c r="AA4" s="95" t="s">
         <v>49</v>
       </c>
-      <c r="AB4" s="98" t="s">
+      <c r="AB4" s="95" t="s">
         <v>50</v>
       </c>
-      <c r="AC4" s="98" t="s">
+      <c r="AC4" s="95" t="s">
         <v>51</v>
       </c>
-      <c r="AD4" s="98" t="s">
+      <c r="AD4" s="95" t="s">
         <v>52</v>
       </c>
-      <c r="AE4" s="98" t="s">
+      <c r="AE4" s="95" t="s">
         <v>53</v>
       </c>
-      <c r="AF4" s="98" t="s">
-        <v>260</v>
+      <c r="AF4" s="95" t="s">
+        <v>249</v>
       </c>
-      <c r="AG4" s="98" t="s">
+      <c r="AG4" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="AH4" s="106" t="s">
+      <c r="AH4" s="103" t="s">
         <v>57</v>
       </c>
-      <c r="AI4" s="108"/>
-      <c r="AJ4" s="93" t="s">
+      <c r="AI4" s="105"/>
+      <c r="AJ4" s="90" t="s">
         <v>60</v>
       </c>
-      <c r="AK4" s="93"/>
-      <c r="AL4" s="93" t="s">
+      <c r="AK4" s="90"/>
+      <c r="AL4" s="90" t="s">
         <v>58</v>
       </c>
-      <c r="AM4" s="93"/>
-      <c r="AN4" s="93" t="s">
+      <c r="AM4" s="90"/>
+      <c r="AN4" s="90" t="s">
         <v>59</v>
       </c>
-      <c r="AO4" s="93"/>
+      <c r="AO4" s="90"/>
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A5" s="97"/>
-      <c r="B5" s="105"/>
-      <c r="C5" s="105"/>
-      <c r="D5" s="190"/>
+      <c r="A5" s="94"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="187"/>
       <c r="E5" s="25" t="s">
         <v>37</v>
       </c>
       <c r="F5" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="188" t="s">
-        <v>255</v>
+      <c r="G5" s="185" t="s">
+        <v>244</v>
       </c>
       <c r="H5" s="25" t="s">
         <v>37</v>
@@ -44313,73 +44331,73 @@
       <c r="I5" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="J5" s="188" t="s">
+      <c r="J5" s="185" t="s">
+        <v>244</v>
+      </c>
+      <c r="K5" s="102"/>
+      <c r="L5" s="176" t="s">
+        <v>248</v>
+      </c>
+      <c r="M5" s="176" t="s">
+        <v>251</v>
+      </c>
+      <c r="N5" s="176" t="s">
+        <v>252</v>
+      </c>
+      <c r="O5" s="176" t="s">
+        <v>253</v>
+      </c>
+      <c r="P5" s="176" t="s">
+        <v>254</v>
+      </c>
+      <c r="Q5" s="176" t="s">
         <v>255</v>
       </c>
-      <c r="K5" s="105"/>
-      <c r="L5" s="179" t="s">
-        <v>259</v>
-      </c>
-      <c r="M5" s="179" t="s">
-        <v>262</v>
-      </c>
-      <c r="N5" s="179" t="s">
-        <v>263</v>
-      </c>
-      <c r="O5" s="179" t="s">
-        <v>264</v>
-      </c>
-      <c r="P5" s="179" t="s">
-        <v>265</v>
-      </c>
-      <c r="Q5" s="179" t="s">
-        <v>266</v>
-      </c>
-      <c r="R5" s="179" t="s">
-        <v>267</v>
+      <c r="R5" s="176" t="s">
+        <v>256</v>
       </c>
       <c r="S5" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="T5" s="188" t="s">
+      <c r="T5" s="185" t="s">
+        <v>250</v>
+      </c>
+      <c r="U5" s="95"/>
+      <c r="V5" s="95"/>
+      <c r="W5" s="95"/>
+      <c r="X5" s="95"/>
+      <c r="Y5" s="95"/>
+      <c r="Z5" s="95"/>
+      <c r="AA5" s="95"/>
+      <c r="AB5" s="95"/>
+      <c r="AC5" s="95"/>
+      <c r="AD5" s="95"/>
+      <c r="AE5" s="95"/>
+      <c r="AF5" s="95"/>
+      <c r="AG5" s="95"/>
+      <c r="AH5" s="176" t="s">
+        <v>258</v>
+      </c>
+      <c r="AI5" s="176" t="s">
+        <v>259</v>
+      </c>
+      <c r="AJ5" s="176" t="s">
+        <v>260</v>
+      </c>
+      <c r="AK5" s="176" t="s">
         <v>261</v>
       </c>
-      <c r="U5" s="98"/>
-      <c r="V5" s="98"/>
-      <c r="W5" s="98"/>
-      <c r="X5" s="98"/>
-      <c r="Y5" s="98"/>
-      <c r="Z5" s="98"/>
-      <c r="AA5" s="98"/>
-      <c r="AB5" s="98"/>
-      <c r="AC5" s="98"/>
-      <c r="AD5" s="98"/>
-      <c r="AE5" s="98"/>
-      <c r="AF5" s="98"/>
-      <c r="AG5" s="98"/>
-      <c r="AH5" s="179" t="s">
-        <v>269</v>
+      <c r="AL5" s="176" t="s">
+        <v>262</v>
       </c>
-      <c r="AI5" s="179" t="s">
-        <v>270</v>
+      <c r="AM5" s="176" t="s">
+        <v>263</v>
       </c>
-      <c r="AJ5" s="179" t="s">
-        <v>271</v>
+      <c r="AN5" s="176" t="s">
+        <v>264</v>
       </c>
-      <c r="AK5" s="179" t="s">
-        <v>272</v>
-      </c>
-      <c r="AL5" s="179" t="s">
-        <v>273</v>
-      </c>
-      <c r="AM5" s="179" t="s">
-        <v>274</v>
-      </c>
-      <c r="AN5" s="179" t="s">
-        <v>275</v>
-      </c>
-      <c r="AO5" s="179" t="s">
-        <v>276</v>
+      <c r="AO5" s="176" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.25">
@@ -52983,7 +53001,7 @@
       <c r="AO205" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="bdyCQ1qbwvPeawoc8hB7j1eM3+0at+J/KVx8jfWYor+mGz6e52Vxp8Kxhppii9kljlqncXdac0Stj3/E8g2WWA==" saltValue="Ul4zYB9s4JdZdrH9J5pmTw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AH2:AO3"/>
@@ -53059,49 +53077,49 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="97" t="s">
-        <v>211</v>
+      <c r="A2" s="94" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="97" t="s">
+      <c r="B2" s="94" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="97"/>
-      <c r="D2" s="97"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="133"/>
-      <c r="B3" s="97" t="s">
-        <v>213</v>
+      <c r="A3" s="130"/>
+      <c r="B3" s="94" t="s">
+        <v>287</v>
       </c>
-      <c r="C3" s="134" t="s">
+      <c r="C3" s="131" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="97" t="s">
+      <c r="D3" s="94" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="133"/>
-      <c r="B4" s="97"/>
-      <c r="C4" s="134"/>
-      <c r="D4" s="97"/>
+      <c r="A4" s="130"/>
+      <c r="B4" s="94"/>
+      <c r="C4" s="131"/>
+      <c r="D4" s="94"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="133"/>
-      <c r="B5" s="97"/>
-      <c r="C5" s="134"/>
-      <c r="D5" s="97"/>
+      <c r="A5" s="130"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="131"/>
+      <c r="D5" s="94"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="192"/>
+      <c r="B6" s="189"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
@@ -54300,7 +54318,7 @@
       <c r="D205" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="nrA/J4zBGR80COd2iPCeyQKzj6apxsLrJ+dUy7JPrvb7JclMTfUI4MLaxhlDQ6TMG8+ikPCi0bHA9yGu34hY+A==" saltValue="VjnPj9tjX0orMQKjAOrpTA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="uvTpkrLsktAunA9S+XlYlTnvwA2HnPU9YSSMq5ZpoUHDC+2Hym15nxRB2vQ8B4b7AViQn0daTOn9hKRllZBaLg==" saltValue="Q9Dmn/rAHhKzakhl7MM4DQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="5">
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="B3:B5"/>
@@ -54334,7 +54352,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -54347,63 +54365,63 @@
       <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="89" t="s">
-        <v>211</v>
+      <c r="A2" s="86" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="98" t="s">
-        <v>80</v>
+      <c r="B2" s="95" t="s">
+        <v>74</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="115" t="s">
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="112" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="116"/>
-      <c r="I2" s="116"/>
-      <c r="J2" s="117"/>
+      <c r="H2" s="113"/>
+      <c r="I2" s="113"/>
+      <c r="J2" s="114"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="90"/>
-      <c r="B3" s="104" t="s">
-        <v>277</v>
+      <c r="A3" s="87"/>
+      <c r="B3" s="101" t="s">
+        <v>266</v>
       </c>
-      <c r="C3" s="104" t="s">
-        <v>278</v>
+      <c r="C3" s="101" t="s">
+        <v>267</v>
       </c>
-      <c r="D3" s="181" t="s">
-        <v>279</v>
+      <c r="D3" s="178" t="s">
+        <v>268</v>
       </c>
-      <c r="E3" s="98" t="s">
-        <v>284</v>
+      <c r="E3" s="95" t="s">
+        <v>273</v>
       </c>
-      <c r="F3" s="117" t="s">
-        <v>285</v>
+      <c r="F3" s="114" t="s">
+        <v>274</v>
       </c>
-      <c r="G3" s="95"/>
-      <c r="H3" s="118"/>
-      <c r="I3" s="118"/>
-      <c r="J3" s="96"/>
+      <c r="G3" s="92"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="93"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="91"/>
-      <c r="B4" s="105"/>
-      <c r="C4" s="105"/>
-      <c r="D4" s="181"/>
-      <c r="E4" s="98"/>
-      <c r="F4" s="96"/>
-      <c r="G4" s="178" t="s">
-        <v>280</v>
+      <c r="A4" s="88"/>
+      <c r="B4" s="102"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="178"/>
+      <c r="E4" s="95"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="175" t="s">
+        <v>269</v>
       </c>
-      <c r="H4" s="178" t="s">
-        <v>281</v>
+      <c r="H4" s="175" t="s">
+        <v>270</v>
       </c>
-      <c r="I4" s="178" t="s">
-        <v>282</v>
+      <c r="I4" s="175" t="s">
+        <v>271</v>
       </c>
-      <c r="J4" s="178" t="s">
-        <v>283</v>
+      <c r="J4" s="175" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -56856,7 +56874,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="31"/>
@@ -56875,97 +56893,97 @@
       <c r="P1" s="30"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="89" t="s">
-        <v>211</v>
+      <c r="A2" s="86" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="133" t="s">
-        <v>78</v>
+      <c r="B2" s="130" t="s">
+        <v>281</v>
       </c>
-      <c r="C2" s="137"/>
-      <c r="D2" s="137"/>
-      <c r="E2" s="137"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="137"/>
-      <c r="H2" s="137"/>
-      <c r="I2" s="137"/>
-      <c r="J2" s="137"/>
-      <c r="K2" s="134"/>
-      <c r="L2" s="115" t="s">
-        <v>215</v>
+      <c r="C2" s="134"/>
+      <c r="D2" s="134"/>
+      <c r="E2" s="134"/>
+      <c r="F2" s="134"/>
+      <c r="G2" s="134"/>
+      <c r="H2" s="134"/>
+      <c r="I2" s="134"/>
+      <c r="J2" s="134"/>
+      <c r="K2" s="131"/>
+      <c r="L2" s="112" t="s">
+        <v>208</v>
       </c>
-      <c r="M2" s="116"/>
-      <c r="N2" s="116"/>
-      <c r="O2" s="116"/>
-      <c r="P2" s="117"/>
+      <c r="M2" s="113"/>
+      <c r="N2" s="113"/>
+      <c r="O2" s="113"/>
+      <c r="P2" s="114"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="90"/>
-      <c r="B3" s="176" t="s">
+      <c r="A3" s="87"/>
+      <c r="B3" s="173" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="196" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="197"/>
+      <c r="E3" s="197"/>
+      <c r="F3" s="197"/>
+      <c r="G3" s="198"/>
+      <c r="H3" s="171" t="s">
+        <v>284</v>
+      </c>
+      <c r="I3" s="173" t="s">
+        <v>285</v>
+      </c>
+      <c r="J3" s="123" t="s">
+        <v>72</v>
+      </c>
+      <c r="K3" s="124"/>
+      <c r="L3" s="92"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="93"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="88"/>
+      <c r="B4" s="174"/>
+      <c r="C4" s="193" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="194" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" s="195" t="s">
+        <v>282</v>
+      </c>
+      <c r="F4" s="194" t="s">
+        <v>283</v>
+      </c>
+      <c r="G4" s="195" t="s">
+        <v>70</v>
+      </c>
+      <c r="H4" s="172"/>
+      <c r="I4" s="174"/>
+      <c r="J4" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" s="200" t="s">
         <v>286</v>
       </c>
-      <c r="C3" s="69" t="s">
-        <v>74</v>
+      <c r="M4" s="199" t="s">
+        <v>288</v>
       </c>
-      <c r="D3" s="174" t="s">
-        <v>76</v>
+      <c r="N4" s="199" t="s">
+        <v>289</v>
       </c>
-      <c r="E3" s="176" t="s">
-        <v>237</v>
+      <c r="O4" s="199" t="s">
+        <v>290</v>
       </c>
-      <c r="F3" s="174" t="s">
-        <v>238</v>
-      </c>
-      <c r="G3" s="176" t="s">
-        <v>75</v>
-      </c>
-      <c r="H3" s="174" t="s">
-        <v>239</v>
-      </c>
-      <c r="I3" s="176" t="s">
-        <v>240</v>
-      </c>
-      <c r="J3" s="126" t="s">
-        <v>77</v>
-      </c>
-      <c r="K3" s="127"/>
-      <c r="L3" s="95"/>
-      <c r="M3" s="118"/>
-      <c r="N3" s="118"/>
-      <c r="O3" s="118"/>
-      <c r="P3" s="96"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="91"/>
-      <c r="B4" s="177"/>
-      <c r="C4" s="70" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="175"/>
-      <c r="E4" s="177"/>
-      <c r="F4" s="175"/>
-      <c r="G4" s="177"/>
-      <c r="H4" s="175"/>
-      <c r="I4" s="177"/>
-      <c r="J4" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="L4" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="M4" s="32" t="s">
-        <v>70</v>
-      </c>
-      <c r="N4" s="32" t="s">
-        <v>71</v>
-      </c>
-      <c r="O4" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="P4" s="32" t="s">
-        <v>73</v>
+      <c r="P4" s="199" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -60570,31 +60588,28 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
-  <mergeCells count="11">
+  <mergeCells count="8">
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="L2:P3"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="G3:G4"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="F3:F4"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="I3:I4"/>
-    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="C3:G3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4:P4 C4" xr:uid="{CD6651F3-A46F-4145-A884-D4B65D9D832A}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 N4 O4 P4" xr:uid="{CD6651F3-A46F-4145-A884-D4B65D9D832A}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" location="streamerTypes" xr:uid="{F5B00754-CAA7-4970-9267-C564E10BAB15}"/>
-    <hyperlink ref="L4" r:id="rId2" location="mitigationDevices" xr:uid="{E64F730D-939F-45B5-880D-5F6B514D9768}"/>
-    <hyperlink ref="M4" r:id="rId3" location="mitigationDevices" xr:uid="{9ED9D614-FD6F-49CD-865E-6F4E2F134AB8}"/>
-    <hyperlink ref="N4" r:id="rId4" location="mitigationDevices" xr:uid="{FD249156-8181-4617-AA2E-7D78285B2BA7}"/>
-    <hyperlink ref="O4" r:id="rId5" location="mitigationDevices" xr:uid="{93C2D1ED-DD7E-4C3A-94FD-7C83A902B4EA}"/>
-    <hyperlink ref="P4" r:id="rId6" location="mitigationDevices" xr:uid="{468402CE-24B4-4147-BA53-73E2855BBFD5}"/>
+    <hyperlink ref="C4" r:id="rId1" location="streamerTypes" display="TYPE_CODE" xr:uid="{F5B00754-CAA7-4970-9267-C564E10BAB15}"/>
+    <hyperlink ref="L4" r:id="rId2" location="mitigationDevices" display="DEVICE_1_CODE" xr:uid="{E64F730D-939F-45B5-880D-5F6B514D9768}"/>
+    <hyperlink ref="M4" r:id="rId3" location="mitigationDevices" display="DEVICE_2_CODE" xr:uid="{9ED9D614-FD6F-49CD-865E-6F4E2F134AB8}"/>
+    <hyperlink ref="N4" r:id="rId4" location="mitigationDevices" display="DEVICE_3_CODE" xr:uid="{FD249156-8181-4617-AA2E-7D78285B2BA7}"/>
+    <hyperlink ref="O4" r:id="rId5" location="mitigationDevices" display="DEVICE_4_CODE" xr:uid="{93C2D1ED-DD7E-4C3A-94FD-7C83A902B4EA}"/>
+    <hyperlink ref="P4" r:id="rId6" location="mitigationDevices" display="DEVICE_5_CODE" xr:uid="{468402CE-24B4-4147-BA53-73E2855BBFD5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -60637,7 +60652,7 @@
   <sheetData>
     <row r="1" spans="1:29" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -60669,14 +60684,14 @@
       <c r="AC1" s="16"/>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
-        <v>211</v>
+      <c r="A2" s="89" t="s">
+        <v>205</v>
       </c>
-      <c r="B2" s="121" t="s">
-        <v>216</v>
+      <c r="B2" s="118" t="s">
+        <v>209</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="D2" s="26"/>
       <c r="E2" s="26"/>
@@ -60706,127 +60721,127 @@
       <c r="AC2" s="27"/>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
-      <c r="B3" s="122"/>
-      <c r="C3" s="133" t="s">
-        <v>181</v>
+      <c r="A3" s="89"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="130" t="s">
+        <v>175</v>
       </c>
-      <c r="D3" s="137"/>
-      <c r="E3" s="134"/>
-      <c r="F3" s="133" t="s">
-        <v>182</v>
+      <c r="D3" s="134"/>
+      <c r="E3" s="131"/>
+      <c r="F3" s="130" t="s">
+        <v>176</v>
       </c>
-      <c r="G3" s="137"/>
-      <c r="H3" s="134"/>
+      <c r="G3" s="134"/>
+      <c r="H3" s="131"/>
       <c r="I3" s="24" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="J3" s="24"/>
-      <c r="K3" s="115" t="s">
+      <c r="K3" s="112" t="s">
         <v>66</v>
       </c>
-      <c r="L3" s="116"/>
-      <c r="M3" s="117"/>
-      <c r="N3" s="115" t="s">
-        <v>84</v>
+      <c r="L3" s="113"/>
+      <c r="M3" s="114"/>
+      <c r="N3" s="112" t="s">
+        <v>78</v>
       </c>
-      <c r="O3" s="117"/>
-      <c r="P3" s="92" t="s">
+      <c r="O3" s="114"/>
+      <c r="P3" s="89" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q3" s="90" t="s">
+        <v>185</v>
+      </c>
+      <c r="R3" s="89" t="s">
+        <v>186</v>
+      </c>
+      <c r="S3" s="94" t="s">
+        <v>80</v>
+      </c>
+      <c r="T3" s="94"/>
+      <c r="U3" s="135" t="s">
+        <v>211</v>
+      </c>
+      <c r="V3" s="136"/>
+      <c r="W3" s="135" t="s">
+        <v>210</v>
+      </c>
+      <c r="X3" s="136"/>
+      <c r="Y3" s="94" t="s">
+        <v>81</v>
+      </c>
+      <c r="Z3" s="94"/>
+      <c r="AA3" s="94"/>
+      <c r="AB3" s="94"/>
+      <c r="AC3" s="109" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A4" s="89"/>
+      <c r="B4" s="119"/>
+      <c r="C4" s="128" t="s">
         <v>190</v>
       </c>
-      <c r="Q3" s="93" t="s">
-        <v>191</v>
+      <c r="D4" s="130" t="s">
+        <v>177</v>
       </c>
-      <c r="R3" s="92" t="s">
-        <v>192</v>
+      <c r="E4" s="131"/>
+      <c r="F4" s="132" t="s">
+        <v>190</v>
       </c>
-      <c r="S3" s="97" t="s">
-        <v>86</v>
+      <c r="G4" s="130" t="s">
+        <v>177</v>
       </c>
-      <c r="T3" s="97"/>
-      <c r="U3" s="138" t="s">
-        <v>218</v>
+      <c r="H4" s="131"/>
+      <c r="I4" s="39" t="s">
+        <v>89</v>
       </c>
-      <c r="V3" s="139"/>
-      <c r="W3" s="138" t="s">
-        <v>217</v>
-      </c>
-      <c r="X3" s="139"/>
-      <c r="Y3" s="97" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z3" s="97"/>
-      <c r="AA3" s="97"/>
-      <c r="AB3" s="97"/>
-      <c r="AC3" s="112" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="122"/>
-      <c r="C4" s="131" t="s">
-        <v>196</v>
-      </c>
-      <c r="D4" s="133" t="s">
-        <v>183</v>
-      </c>
-      <c r="E4" s="134"/>
-      <c r="F4" s="135" t="s">
-        <v>196</v>
-      </c>
-      <c r="G4" s="133" t="s">
-        <v>183</v>
-      </c>
-      <c r="H4" s="134"/>
-      <c r="I4" s="40" t="s">
-        <v>95</v>
-      </c>
-      <c r="J4" s="68" t="s">
+      <c r="J4" s="67" t="s">
         <v>62</v>
       </c>
-      <c r="K4" s="95"/>
-      <c r="L4" s="118"/>
-      <c r="M4" s="96"/>
-      <c r="N4" s="95"/>
-      <c r="O4" s="96"/>
-      <c r="P4" s="92"/>
-      <c r="Q4" s="93"/>
-      <c r="R4" s="92"/>
-      <c r="S4" s="97"/>
-      <c r="T4" s="97"/>
-      <c r="U4" s="140"/>
-      <c r="V4" s="141"/>
-      <c r="W4" s="140"/>
-      <c r="X4" s="141"/>
-      <c r="Y4" s="97"/>
-      <c r="Z4" s="97"/>
-      <c r="AA4" s="97"/>
-      <c r="AB4" s="97"/>
-      <c r="AC4" s="112"/>
+      <c r="K4" s="92"/>
+      <c r="L4" s="115"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="92"/>
+      <c r="O4" s="93"/>
+      <c r="P4" s="89"/>
+      <c r="Q4" s="90"/>
+      <c r="R4" s="89"/>
+      <c r="S4" s="94"/>
+      <c r="T4" s="94"/>
+      <c r="U4" s="137"/>
+      <c r="V4" s="138"/>
+      <c r="W4" s="137"/>
+      <c r="X4" s="138"/>
+      <c r="Y4" s="94"/>
+      <c r="Z4" s="94"/>
+      <c r="AA4" s="94"/>
+      <c r="AB4" s="94"/>
+      <c r="AC4" s="109"/>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="123"/>
-      <c r="C5" s="132"/>
-      <c r="D5" s="67" t="s">
+      <c r="A5" s="89"/>
+      <c r="B5" s="120"/>
+      <c r="C5" s="129"/>
+      <c r="D5" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="67" t="s">
+      <c r="E5" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="136"/>
-      <c r="G5" s="67" t="s">
+      <c r="F5" s="133"/>
+      <c r="G5" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="H5" s="67" t="s">
+      <c r="H5" s="66" t="s">
         <v>1</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
-      <c r="J5" s="67" t="s">
-        <v>207</v>
+      <c r="J5" s="66" t="s">
+        <v>201</v>
       </c>
       <c r="K5" s="21" t="s">
         <v>65</v>
@@ -60834,35 +60849,35 @@
       <c r="L5" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="M5" s="34" t="s">
-        <v>205</v>
+      <c r="M5" s="33" t="s">
+        <v>199</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="O5" s="13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
-      <c r="P5" s="92"/>
-      <c r="Q5" s="93"/>
-      <c r="R5" s="92"/>
-      <c r="S5" s="40" t="s">
+      <c r="P5" s="89"/>
+      <c r="Q5" s="90"/>
+      <c r="R5" s="89"/>
+      <c r="S5" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="T5" s="25" t="s">
+        <v>183</v>
+      </c>
+      <c r="U5" s="65" t="s">
+        <v>32</v>
+      </c>
+      <c r="V5" s="65" t="s">
         <v>85</v>
       </c>
-      <c r="T5" s="25" t="s">
-        <v>189</v>
-      </c>
-      <c r="U5" s="66" t="s">
-        <v>32</v>
-      </c>
-      <c r="V5" s="66" t="s">
-        <v>91</v>
-      </c>
-      <c r="W5" s="40" t="s">
+      <c r="W5" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="X5" s="71" t="s">
-        <v>206</v>
+      <c r="X5" s="68" t="s">
+        <v>200</v>
       </c>
       <c r="Y5" s="23" t="s">
         <v>33</v>
@@ -60876,7 +60891,7 @@
       <c r="AB5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="AC5" s="112"/>
+      <c r="AC5" s="109"/>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>

</xml_diff>

<commit_message>
Details of the changes made to ROS LL description and final corrections (inshallah)
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -5,13 +5,13 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schirico\Repositories\iotc-reference-forms\form_reporting_templates\ros\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{245EE23D-1A7D-44F3-9CA1-EF893FD22309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69718F07-E18E-47F4-97CE-F6ADAE11F97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28755" yWindow="315" windowWidth="27705" windowHeight="15090" tabRatio="879" firstSheet="11" activeTab="18" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" firstSheet="5" activeTab="8" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -1449,6 +1449,12 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1542,6 +1548,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1589,22 +1612,8 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1631,9 +1640,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1695,12 +1701,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2039,24 +2039,24 @@
   <sheetData>
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="66" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="66"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="68"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="67"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="69"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="71"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="12"/>
@@ -2106,15 +2106,15 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="18"/>
-      <c r="C8" s="70" t="s">
+      <c r="C8" s="72" t="s">
         <v>133</v>
       </c>
-      <c r="D8" s="70"/>
+      <c r="D8" s="72"/>
       <c r="E8" s="19"/>
-      <c r="F8" s="70" t="s">
+      <c r="F8" s="72" t="s">
         <v>132</v>
       </c>
-      <c r="G8" s="70"/>
+      <c r="G8" s="72"/>
       <c r="H8" s="20"/>
     </row>
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2296,11 +2296,11 @@
     </row>
     <row r="26" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="18"/>
-      <c r="C26" s="71"/>
-      <c r="D26" s="72"/>
-      <c r="E26" s="72"/>
-      <c r="F26" s="72"/>
-      <c r="G26" s="73"/>
+      <c r="C26" s="73"/>
+      <c r="D26" s="74"/>
+      <c r="E26" s="74"/>
+      <c r="F26" s="74"/>
+      <c r="G26" s="75"/>
       <c r="H26" s="20"/>
     </row>
     <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2363,10 +2363,10 @@
       <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="141" t="s">
+      <c r="A2" s="64" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="141" t="s">
+      <c r="B2" s="64" t="s">
         <v>110</v>
       </c>
       <c r="C2" s="56" t="s">
@@ -3835,54 +3835,54 @@
       <c r="O1" s="6"/>
     </row>
     <row r="2" spans="1:15" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="120" t="s">
+      <c r="B2" s="114" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="120" t="s">
+      <c r="C2" s="114" t="s">
         <v>251</v>
       </c>
-      <c r="D2" s="120" t="s">
+      <c r="D2" s="114" t="s">
         <v>252</v>
       </c>
-      <c r="E2" s="93" t="s">
+      <c r="E2" s="95" t="s">
         <v>55</v>
       </c>
-      <c r="F2" s="120" t="s">
+      <c r="F2" s="114" t="s">
         <v>253</v>
       </c>
-      <c r="G2" s="120" t="s">
+      <c r="G2" s="114" t="s">
         <v>250</v>
       </c>
-      <c r="H2" s="120" t="s">
+      <c r="H2" s="114" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="120" t="s">
+      <c r="I2" s="114" t="s">
         <v>111</v>
       </c>
-      <c r="J2" s="88" t="s">
+      <c r="J2" s="90" t="s">
         <v>244</v>
       </c>
-      <c r="K2" s="92"/>
-      <c r="L2" s="116" t="s">
+      <c r="K2" s="94"/>
+      <c r="L2" s="119" t="s">
         <v>245</v>
       </c>
-      <c r="M2" s="123"/>
-      <c r="N2" s="123"/>
-      <c r="O2" s="117"/>
+      <c r="M2" s="125"/>
+      <c r="N2" s="125"/>
+      <c r="O2" s="120"/>
     </row>
     <row r="3" spans="1:15" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75"/>
-      <c r="B3" s="75"/>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="75"/>
+      <c r="A3" s="77"/>
+      <c r="B3" s="77"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
       <c r="J3" s="42" t="s">
         <v>47</v>
       </c>
@@ -7304,17 +7304,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="ZHZ61xEMWo2GozKFDfIGwtbJZnm3eVYJpvIE2b76e/O5EaOFEu4qUPnEZ+3+QLMo4fMOZjuAZJWBGppNj6h0fg==" saltValue="p7UsgbvwfBAQ3S2mqNofIA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="E2:E3"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="J2:K2"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="I2:I3"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="E2:E3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3 M3 N3 O3" xr:uid="{35387E2C-FBDF-4B0A-A0B5-EF76A6744ABB}">
@@ -7356,21 +7356,21 @@
       <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="120" t="s">
+      <c r="B2" s="114" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="116" t="s">
+      <c r="C2" s="119" t="s">
         <v>221</v>
       </c>
-      <c r="D2" s="123"/>
-      <c r="E2" s="117"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="120"/>
     </row>
     <row r="3" spans="1:5" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75"/>
-      <c r="B3" s="75"/>
+      <c r="A3" s="77"/>
+      <c r="B3" s="77"/>
       <c r="C3" s="56" t="s">
         <v>23</v>
       </c>
@@ -8822,22 +8822,22 @@
       <c r="F1" s="6"/>
     </row>
     <row r="2" spans="1:6" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="120" t="s">
+      <c r="B2" s="114" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="116" t="s">
+      <c r="C2" s="119" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="123"/>
-      <c r="E2" s="123"/>
-      <c r="F2" s="117"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="120"/>
     </row>
     <row r="3" spans="1:6" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75"/>
-      <c r="B3" s="75"/>
+      <c r="A3" s="77"/>
+      <c r="B3" s="77"/>
       <c r="C3" s="56" t="s">
         <v>197</v>
       </c>
@@ -10517,89 +10517,89 @@
       <c r="Q1" s="6"/>
     </row>
     <row r="2" spans="1:17" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="120" t="s">
+      <c r="B2" s="114" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="116" t="s">
+      <c r="C2" s="119" t="s">
         <v>227</v>
       </c>
-      <c r="D2" s="123"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="116" t="s">
+      <c r="D2" s="125"/>
+      <c r="E2" s="120"/>
+      <c r="F2" s="119" t="s">
         <v>228</v>
       </c>
-      <c r="G2" s="123"/>
-      <c r="H2" s="117"/>
-      <c r="I2" s="99" t="s">
+      <c r="G2" s="125"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="106" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="98" t="s">
+      <c r="J2" s="105" t="s">
         <v>214</v>
       </c>
-      <c r="K2" s="98"/>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98"/>
-      <c r="N2" s="86" t="s">
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="88" t="s">
         <v>58</v>
       </c>
-      <c r="O2" s="86" t="s">
+      <c r="O2" s="88" t="s">
         <v>219</v>
       </c>
-      <c r="P2" s="86" t="s">
+      <c r="P2" s="88" t="s">
         <v>220</v>
       </c>
-      <c r="Q2" s="133" t="s">
+      <c r="Q2" s="135" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:17" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="74"/>
-      <c r="C3" s="120" t="s">
+      <c r="A3" s="76"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="114" t="s">
         <v>98</v>
       </c>
-      <c r="D3" s="116" t="s">
+      <c r="D3" s="119" t="s">
         <v>96</v>
       </c>
-      <c r="E3" s="117"/>
-      <c r="F3" s="120" t="s">
+      <c r="E3" s="120"/>
+      <c r="F3" s="114" t="s">
         <v>98</v>
       </c>
-      <c r="G3" s="116" t="s">
+      <c r="G3" s="119" t="s">
         <v>96</v>
       </c>
-      <c r="H3" s="117"/>
-      <c r="I3" s="99"/>
-      <c r="J3" s="98"/>
-      <c r="K3" s="98"/>
-      <c r="L3" s="98"/>
-      <c r="M3" s="98"/>
-      <c r="N3" s="86"/>
-      <c r="O3" s="86"/>
-      <c r="P3" s="86"/>
-      <c r="Q3" s="133"/>
+      <c r="H3" s="120"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="105"/>
+      <c r="L3" s="105"/>
+      <c r="M3" s="105"/>
+      <c r="N3" s="88"/>
+      <c r="O3" s="88"/>
+      <c r="P3" s="88"/>
+      <c r="Q3" s="135"/>
     </row>
     <row r="4" spans="1:17" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
+      <c r="A4" s="77"/>
+      <c r="B4" s="77"/>
+      <c r="C4" s="77"/>
       <c r="D4" s="39" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="75"/>
+      <c r="F4" s="77"/>
       <c r="G4" s="39" t="s">
         <v>0</v>
       </c>
       <c r="H4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="99"/>
+      <c r="I4" s="106"/>
       <c r="J4" s="50" t="s">
         <v>213</v>
       </c>
@@ -10612,10 +10612,10 @@
       <c r="M4" s="50" t="s">
         <v>217</v>
       </c>
-      <c r="N4" s="86"/>
-      <c r="O4" s="86"/>
-      <c r="P4" s="86"/>
-      <c r="Q4" s="133"/>
+      <c r="N4" s="88"/>
+      <c r="O4" s="88"/>
+      <c r="P4" s="88"/>
+      <c r="Q4" s="135"/>
     </row>
     <row r="5" spans="1:17" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
@@ -14420,6 +14420,7 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="6+yDI0OgPd4WYm3G6Z5geZ6OVSItsmzuI6pvXBhnqIBLkRwqZYhw/9myNYQcHogXrON+p0Vn9Al4arNGxWcvhQ==" saltValue="yoKDrVsoZTsh8FbYtsclwg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="C3:C4"/>
@@ -14433,7 +14434,6 @@
     <mergeCell ref="I2:I4"/>
     <mergeCell ref="J2:M3"/>
     <mergeCell ref="N2:N4"/>
-    <mergeCell ref="A2:A4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I4 M4 J4 K4 L4 Q2:Q4" xr:uid="{2FBCC481-6114-481E-B036-95624C9F7883}">
@@ -14475,20 +14475,20 @@
       <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:4" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="120" t="s">
+      <c r="B2" s="114" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="88" t="s">
+      <c r="C2" s="90" t="s">
         <v>48</v>
       </c>
-      <c r="D2" s="92"/>
+      <c r="D2" s="94"/>
     </row>
     <row r="3" spans="1:4" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75"/>
-      <c r="B3" s="75"/>
+      <c r="A3" s="77"/>
+      <c r="B3" s="77"/>
       <c r="C3" s="42" t="s">
         <v>164</v>
       </c>
@@ -15743,60 +15743,60 @@
       <c r="K1" s="6"/>
     </row>
     <row r="2" spans="1:11" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="120" t="s">
+      <c r="B2" s="114" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="120" t="s">
+      <c r="C2" s="114" t="s">
         <v>112</v>
       </c>
-      <c r="D2" s="133" t="s">
+      <c r="D2" s="135" t="s">
         <v>140</v>
       </c>
-      <c r="E2" s="134" t="s">
+      <c r="E2" s="136" t="s">
         <v>106</v>
       </c>
-      <c r="F2" s="135"/>
-      <c r="G2" s="133" t="s">
+      <c r="F2" s="137"/>
+      <c r="G2" s="135" t="s">
         <v>203</v>
       </c>
-      <c r="H2" s="86" t="s">
+      <c r="H2" s="88" t="s">
         <v>230</v>
       </c>
-      <c r="I2" s="112" t="s">
+      <c r="I2" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="113"/>
-      <c r="K2" s="114"/>
+      <c r="J2" s="116"/>
+      <c r="K2" s="117"/>
     </row>
     <row r="3" spans="1:11" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="133"/>
-      <c r="E3" s="136"/>
-      <c r="F3" s="137"/>
-      <c r="G3" s="133"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="84"/>
-      <c r="J3" s="115"/>
-      <c r="K3" s="85"/>
+      <c r="A3" s="76"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="135"/>
+      <c r="E3" s="138"/>
+      <c r="F3" s="139"/>
+      <c r="G3" s="135"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="118"/>
+      <c r="K3" s="87"/>
     </row>
     <row r="4" spans="1:11" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="133"/>
+      <c r="A4" s="77"/>
+      <c r="B4" s="77"/>
+      <c r="C4" s="77"/>
+      <c r="D4" s="135"/>
       <c r="E4" s="56" t="s">
         <v>23</v>
       </c>
       <c r="F4" s="56" t="s">
         <v>105</v>
       </c>
-      <c r="G4" s="133"/>
-      <c r="H4" s="86"/>
+      <c r="G4" s="135"/>
+      <c r="H4" s="88"/>
       <c r="I4" s="50" t="s">
         <v>205</v>
       </c>
@@ -18502,65 +18502,65 @@
       <c r="Y1" s="6"/>
     </row>
     <row r="2" spans="1:25" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="138" t="s">
+      <c r="A2" s="140" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="138" t="s">
+      <c r="B2" s="140" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="138" t="s">
+      <c r="C2" s="140" t="s">
         <v>112</v>
       </c>
-      <c r="D2" s="138" t="s">
+      <c r="D2" s="140" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="107" t="s">
+      <c r="E2" s="96" t="s">
         <v>202</v>
       </c>
-      <c r="F2" s="107" t="s">
+      <c r="F2" s="96" t="s">
         <v>203</v>
       </c>
-      <c r="G2" s="86" t="s">
+      <c r="G2" s="88" t="s">
         <v>206</v>
       </c>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="98" t="s">
+      <c r="H2" s="88"/>
+      <c r="I2" s="88"/>
+      <c r="J2" s="88"/>
+      <c r="K2" s="105" t="s">
         <v>208</v>
       </c>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98"/>
-      <c r="N2" s="98"/>
-      <c r="O2" s="98" t="s">
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105" t="s">
         <v>59</v>
       </c>
-      <c r="P2" s="98"/>
-      <c r="Q2" s="98"/>
-      <c r="R2" s="104" t="s">
+      <c r="P2" s="105"/>
+      <c r="Q2" s="105"/>
+      <c r="R2" s="111" t="s">
         <v>62</v>
       </c>
-      <c r="S2" s="88" t="s">
+      <c r="S2" s="90" t="s">
         <v>104</v>
       </c>
-      <c r="T2" s="92"/>
-      <c r="U2" s="88" t="s">
+      <c r="T2" s="94"/>
+      <c r="U2" s="90" t="s">
         <v>211</v>
       </c>
-      <c r="V2" s="89"/>
-      <c r="W2" s="92"/>
-      <c r="X2" s="98" t="s">
+      <c r="V2" s="91"/>
+      <c r="W2" s="94"/>
+      <c r="X2" s="105" t="s">
         <v>210</v>
       </c>
-      <c r="Y2" s="98"/>
+      <c r="Y2" s="105"/>
     </row>
     <row r="3" spans="1:25" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="139"/>
-      <c r="B3" s="139"/>
-      <c r="C3" s="139"/>
-      <c r="D3" s="139"/>
-      <c r="E3" s="108"/>
-      <c r="F3" s="108"/>
+      <c r="A3" s="141"/>
+      <c r="B3" s="141"/>
+      <c r="C3" s="141"/>
+      <c r="D3" s="141"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="97"/>
       <c r="G3" s="56" t="s">
         <v>23</v>
       </c>
@@ -18594,7 +18594,7 @@
       <c r="Q3" s="50" t="s">
         <v>224</v>
       </c>
-      <c r="R3" s="106"/>
+      <c r="R3" s="113"/>
       <c r="S3" s="43" t="s">
         <v>102</v>
       </c>
@@ -24109,70 +24109,70 @@
       <c r="T1" s="6"/>
     </row>
     <row r="2" spans="1:20" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="138" t="s">
+      <c r="A2" s="140" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="138" t="s">
+      <c r="B2" s="140" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="138" t="s">
+      <c r="C2" s="140" t="s">
         <v>112</v>
       </c>
-      <c r="D2" s="138" t="s">
+      <c r="D2" s="140" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="107" t="s">
+      <c r="E2" s="96" t="s">
         <v>193</v>
       </c>
-      <c r="F2" s="107" t="s">
+      <c r="F2" s="96" t="s">
         <v>194</v>
       </c>
-      <c r="G2" s="107" t="s">
+      <c r="G2" s="96" t="s">
         <v>195</v>
       </c>
-      <c r="H2" s="105" t="s">
+      <c r="H2" s="112" t="s">
         <v>196</v>
       </c>
-      <c r="I2" s="84" t="s">
+      <c r="I2" s="86" t="s">
         <v>72</v>
       </c>
-      <c r="J2" s="85"/>
-      <c r="K2" s="81" t="s">
+      <c r="J2" s="87"/>
+      <c r="K2" s="83" t="s">
         <v>73</v>
       </c>
-      <c r="L2" s="83"/>
-      <c r="M2" s="105" t="s">
+      <c r="L2" s="85"/>
+      <c r="M2" s="112" t="s">
         <v>201</v>
       </c>
-      <c r="N2" s="140" t="s">
+      <c r="N2" s="142" t="s">
         <v>75</v>
       </c>
-      <c r="O2" s="140" t="s">
+      <c r="O2" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="P2" s="105" t="s">
+      <c r="P2" s="112" t="s">
         <v>200</v>
       </c>
-      <c r="Q2" s="140" t="s">
+      <c r="Q2" s="142" t="s">
         <v>70</v>
       </c>
-      <c r="R2" s="140" t="s">
+      <c r="R2" s="142" t="s">
         <v>71</v>
       </c>
-      <c r="S2" s="87" t="s">
+      <c r="S2" s="89" t="s">
         <v>210</v>
       </c>
-      <c r="T2" s="87"/>
+      <c r="T2" s="89"/>
     </row>
     <row r="3" spans="1:20" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="139"/>
-      <c r="B3" s="139"/>
-      <c r="C3" s="139"/>
-      <c r="D3" s="139"/>
-      <c r="E3" s="108"/>
-      <c r="F3" s="108"/>
-      <c r="G3" s="108"/>
-      <c r="H3" s="106"/>
+      <c r="A3" s="141"/>
+      <c r="B3" s="141"/>
+      <c r="C3" s="141"/>
+      <c r="D3" s="141"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="97"/>
+      <c r="H3" s="113"/>
       <c r="I3" s="50" t="s">
         <v>197</v>
       </c>
@@ -24185,12 +24185,12 @@
       <c r="L3" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="M3" s="106"/>
-      <c r="N3" s="87"/>
-      <c r="O3" s="87"/>
-      <c r="P3" s="106"/>
-      <c r="Q3" s="87"/>
-      <c r="R3" s="87"/>
+      <c r="M3" s="113"/>
+      <c r="N3" s="89"/>
+      <c r="O3" s="89"/>
+      <c r="P3" s="113"/>
+      <c r="Q3" s="89"/>
+      <c r="R3" s="89"/>
       <c r="S3" s="50" t="s">
         <v>199</v>
       </c>
@@ -28601,16 +28601,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="owrGYnA0RoV/U9MjDeglShzyfAHibWrOJ91U+dfsJvx7FpXhtP7KXYqD/XawmrJ8WUgOAZj9nC2wQr9dD2KQZw==" saltValue="h+hFQsEVq78bir+WDv8nRA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="S2:T2"/>
     <mergeCell ref="H2:H3"/>
@@ -28618,6 +28608,16 @@
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="K2:L2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F3 H2:H3 P2:P3 S3 J3 E2:E3 G2:G3 I3 M2:M3 T3" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -28675,16 +28675,16 @@
       <c r="K1" s="7"/>
     </row>
     <row r="2" spans="1:11" s="53" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="142" t="s">
+      <c r="A2" s="65" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="142" t="s">
+      <c r="B2" s="65" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="142" t="s">
+      <c r="C2" s="65" t="s">
         <v>112</v>
       </c>
-      <c r="D2" s="142" t="s">
+      <c r="D2" s="65" t="s">
         <v>113</v>
       </c>
       <c r="E2" s="42" t="s">
@@ -31386,117 +31386,117 @@
       <c r="X1" s="63"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" s="74" t="s">
+      <c r="A2" s="76" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="75" t="s">
+      <c r="B2" s="77" t="s">
         <v>175</v>
       </c>
-      <c r="C2" s="75"/>
-      <c r="D2" s="87" t="s">
+      <c r="C2" s="77"/>
+      <c r="D2" s="89" t="s">
         <v>176</v>
       </c>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="87"/>
-      <c r="I2" s="87"/>
-      <c r="J2" s="87"/>
-      <c r="K2" s="87"/>
-      <c r="L2" s="87"/>
-      <c r="M2" s="87"/>
-      <c r="N2" s="78" t="s">
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
+      <c r="K2" s="89"/>
+      <c r="L2" s="89"/>
+      <c r="M2" s="89"/>
+      <c r="N2" s="80" t="s">
         <v>232</v>
       </c>
-      <c r="O2" s="79"/>
-      <c r="P2" s="79"/>
-      <c r="Q2" s="79"/>
-      <c r="R2" s="79"/>
-      <c r="S2" s="79"/>
-      <c r="T2" s="79"/>
-      <c r="U2" s="79"/>
-      <c r="V2" s="79"/>
-      <c r="W2" s="79"/>
-      <c r="X2" s="80"/>
+      <c r="O2" s="81"/>
+      <c r="P2" s="81"/>
+      <c r="Q2" s="81"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
       <c r="Y2" s="53"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="86"/>
-      <c r="C3" s="86"/>
-      <c r="D3" s="88" t="s">
+      <c r="A3" s="76"/>
+      <c r="B3" s="88"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="90" t="s">
         <v>92</v>
       </c>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="92"/>
-      <c r="I3" s="88" t="s">
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="94"/>
+      <c r="I3" s="90" t="s">
         <v>93</v>
       </c>
-      <c r="J3" s="89"/>
-      <c r="K3" s="89"/>
-      <c r="L3" s="89"/>
-      <c r="M3" s="89"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="82"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="82"/>
-      <c r="R3" s="82"/>
-      <c r="S3" s="82"/>
-      <c r="T3" s="82"/>
-      <c r="U3" s="82"/>
-      <c r="V3" s="82"/>
-      <c r="W3" s="82"/>
-      <c r="X3" s="83"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="91"/>
+      <c r="L3" s="91"/>
+      <c r="M3" s="91"/>
+      <c r="N3" s="83"/>
+      <c r="O3" s="84"/>
+      <c r="P3" s="84"/>
+      <c r="Q3" s="84"/>
+      <c r="R3" s="84"/>
+      <c r="S3" s="84"/>
+      <c r="T3" s="84"/>
+      <c r="U3" s="84"/>
+      <c r="V3" s="84"/>
+      <c r="W3" s="84"/>
+      <c r="X3" s="85"/>
       <c r="Y3" s="53"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="74"/>
-      <c r="B4" s="86"/>
-      <c r="C4" s="86"/>
-      <c r="D4" s="84" t="s">
+      <c r="A4" s="76"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="88"/>
+      <c r="D4" s="86" t="s">
         <v>90</v>
       </c>
-      <c r="E4" s="85"/>
-      <c r="F4" s="84" t="s">
+      <c r="E4" s="87"/>
+      <c r="F4" s="86" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="85"/>
-      <c r="H4" s="93" t="s">
+      <c r="G4" s="87"/>
+      <c r="H4" s="95" t="s">
         <v>98</v>
       </c>
-      <c r="I4" s="84" t="s">
+      <c r="I4" s="86" t="s">
         <v>90</v>
       </c>
-      <c r="J4" s="85"/>
-      <c r="K4" s="84" t="s">
+      <c r="J4" s="87"/>
+      <c r="K4" s="86" t="s">
         <v>91</v>
       </c>
-      <c r="L4" s="85"/>
-      <c r="M4" s="90" t="s">
+      <c r="L4" s="87"/>
+      <c r="M4" s="92" t="s">
         <v>98</v>
       </c>
-      <c r="N4" s="76" t="s">
+      <c r="N4" s="78" t="s">
         <v>257</v>
       </c>
-      <c r="O4" s="76"/>
-      <c r="P4" s="77" t="s">
+      <c r="O4" s="78"/>
+      <c r="P4" s="79" t="s">
         <v>255</v>
       </c>
-      <c r="Q4" s="77"/>
-      <c r="R4" s="77"/>
-      <c r="S4" s="77"/>
-      <c r="T4" s="77"/>
-      <c r="U4" s="77" t="s">
+      <c r="Q4" s="79"/>
+      <c r="R4" s="79"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="79"/>
+      <c r="U4" s="79" t="s">
         <v>256</v>
       </c>
-      <c r="V4" s="77"/>
-      <c r="W4" s="77"/>
-      <c r="X4" s="77"/>
+      <c r="V4" s="79"/>
+      <c r="W4" s="79"/>
+      <c r="X4" s="79"/>
     </row>
     <row r="5" spans="1:25" s="54" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="75"/>
+      <c r="A5" s="77"/>
       <c r="B5" s="39" t="s">
         <v>127</v>
       </c>
@@ -31515,7 +31515,7 @@
       <c r="G5" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="H5" s="87"/>
+      <c r="H5" s="89"/>
       <c r="I5" s="50" t="s">
         <v>134</v>
       </c>
@@ -31528,7 +31528,7 @@
       <c r="L5" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="M5" s="91"/>
+      <c r="M5" s="93"/>
       <c r="N5" s="39" t="s">
         <v>5</v>
       </c>
@@ -36823,109 +36823,109 @@
       <c r="P1" s="6"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="88" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="95" t="s">
+      <c r="B2" s="102" t="s">
         <v>241</v>
       </c>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
-      <c r="L2" s="96"/>
-      <c r="M2" s="96"/>
-      <c r="N2" s="96"/>
-      <c r="O2" s="96"/>
-      <c r="P2" s="97"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="103"/>
+      <c r="P2" s="104"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="86"/>
-      <c r="B3" s="95" t="s">
+      <c r="A3" s="88"/>
+      <c r="B3" s="102" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="97"/>
-      <c r="G3" s="109" t="s">
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="98" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="110"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="104" t="s">
+      <c r="H3" s="99"/>
+      <c r="I3" s="100"/>
+      <c r="J3" s="111" t="s">
         <v>17</v>
       </c>
       <c r="K3" s="52" t="s">
         <v>108</v>
       </c>
-      <c r="L3" s="95" t="s">
+      <c r="L3" s="102" t="s">
         <v>128</v>
       </c>
-      <c r="M3" s="96"/>
-      <c r="N3" s="96"/>
-      <c r="O3" s="96"/>
-      <c r="P3" s="97"/>
+      <c r="M3" s="103"/>
+      <c r="N3" s="103"/>
+      <c r="O3" s="103"/>
+      <c r="P3" s="104"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="86"/>
-      <c r="B4" s="86" t="s">
+      <c r="A4" s="88"/>
+      <c r="B4" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="102" t="s">
+      <c r="C4" s="109" t="s">
         <v>139</v>
       </c>
-      <c r="D4" s="103" t="s">
+      <c r="D4" s="110" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="93" t="s">
+      <c r="E4" s="95" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="98" t="s">
+      <c r="F4" s="105" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="99" t="s">
+      <c r="G4" s="106" t="s">
         <v>134</v>
       </c>
-      <c r="H4" s="100" t="s">
+      <c r="H4" s="107" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="94" t="s">
+      <c r="I4" s="101" t="s">
         <v>177</v>
       </c>
-      <c r="J4" s="105"/>
-      <c r="K4" s="107" t="s">
+      <c r="J4" s="112"/>
+      <c r="K4" s="96" t="s">
         <v>141</v>
       </c>
-      <c r="L4" s="76" t="s">
+      <c r="L4" s="78" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="76"/>
-      <c r="N4" s="76" t="s">
+      <c r="M4" s="78"/>
+      <c r="N4" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="O4" s="76"/>
-      <c r="P4" s="98" t="s">
+      <c r="O4" s="78"/>
+      <c r="P4" s="105" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="86"/>
-      <c r="B5" s="86"/>
-      <c r="C5" s="102"/>
-      <c r="D5" s="103"/>
-      <c r="E5" s="87"/>
-      <c r="F5" s="98"/>
-      <c r="G5" s="99"/>
-      <c r="H5" s="101"/>
-      <c r="I5" s="94"/>
-      <c r="J5" s="106"/>
-      <c r="K5" s="108"/>
+      <c r="A5" s="88"/>
+      <c r="B5" s="88"/>
+      <c r="C5" s="109"/>
+      <c r="D5" s="110"/>
+      <c r="E5" s="89"/>
+      <c r="F5" s="105"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="108"/>
+      <c r="I5" s="101"/>
+      <c r="J5" s="113"/>
+      <c r="K5" s="97"/>
       <c r="L5" s="39" t="s">
         <v>3</v>
       </c>
@@ -36938,7 +36938,7 @@
       <c r="O5" s="56" t="s">
         <v>254</v>
       </c>
-      <c r="P5" s="98"/>
+      <c r="P5" s="105"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -40543,6 +40543,8 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="9TADddINtH3/s8+B+YSEyrbqN3sXm6gNvmsaihCGVKf7Pla3vF7K/W63Z2DPtXhM7gpZzMQTmkRfISjjfsW2DA==" saltValue="PE4zbTBOxopTV3TBfcOFrw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="18">
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="F4:F5"/>
     <mergeCell ref="K4:K5"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="I4:I5"/>
@@ -40559,8 +40561,6 @@
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="B2:P2"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="F4:F5"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M5 J6 K4:K5 G4:I5 O5" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40618,47 +40618,47 @@
       <c r="K1" s="6"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="98" t="s">
+      <c r="B2" s="105" t="s">
         <v>233</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98" t="s">
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105" t="s">
         <v>234</v>
       </c>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="88" t="s">
+      <c r="A3" s="76"/>
+      <c r="B3" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="89"/>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="93" t="s">
+      <c r="C3" s="91"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="95" t="s">
         <v>98</v>
       </c>
-      <c r="G3" s="88" t="s">
+      <c r="G3" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="92"/>
-      <c r="K3" s="93" t="s">
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="94"/>
+      <c r="K3" s="95" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
+      <c r="A4" s="77"/>
       <c r="B4" s="50" t="s">
         <v>134</v>
       </c>
@@ -40671,7 +40671,7 @@
       <c r="E4" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="87"/>
+      <c r="F4" s="89"/>
       <c r="G4" s="50" t="s">
         <v>134</v>
       </c>
@@ -40684,7 +40684,7 @@
       <c r="J4" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="K4" s="87"/>
+      <c r="K4" s="89"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
@@ -43289,13 +43289,13 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="u8pXLSYhOVbviCjMnAbnq7QuW/5rhXgGJG1eFeVlUlduAeybGPslcLzuVz4XyLFP1j/6v1ftio6sP6s2dukYSA==" saltValue="CawdL5I7cgplaq9Fy5TfQw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="7">
+    <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="G2:K2"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="G3:J3"/>
-    <mergeCell ref="A2:A4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4:C4 G4:H4" xr:uid="{E97A6FE4-6BFF-4959-9F92-FB6DF23A11A6}">
@@ -43405,199 +43405,199 @@
       <c r="AO1" s="5"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="88" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="98" t="s">
+      <c r="B2" s="105" t="s">
         <v>190</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98"/>
-      <c r="N2" s="98"/>
-      <c r="O2" s="98"/>
-      <c r="P2" s="98"/>
-      <c r="Q2" s="98"/>
-      <c r="R2" s="98"/>
-      <c r="S2" s="98"/>
-      <c r="T2" s="98"/>
-      <c r="U2" s="112" t="s">
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
+      <c r="P2" s="105"/>
+      <c r="Q2" s="105"/>
+      <c r="R2" s="105"/>
+      <c r="S2" s="105"/>
+      <c r="T2" s="105"/>
+      <c r="U2" s="115" t="s">
         <v>235</v>
       </c>
-      <c r="V2" s="113"/>
-      <c r="W2" s="113"/>
-      <c r="X2" s="113"/>
-      <c r="Y2" s="113"/>
-      <c r="Z2" s="113"/>
-      <c r="AA2" s="113"/>
-      <c r="AB2" s="113"/>
-      <c r="AC2" s="113"/>
-      <c r="AD2" s="113"/>
-      <c r="AE2" s="113"/>
-      <c r="AF2" s="113"/>
-      <c r="AG2" s="114"/>
-      <c r="AH2" s="112" t="s">
+      <c r="V2" s="116"/>
+      <c r="W2" s="116"/>
+      <c r="X2" s="116"/>
+      <c r="Y2" s="116"/>
+      <c r="Z2" s="116"/>
+      <c r="AA2" s="116"/>
+      <c r="AB2" s="116"/>
+      <c r="AC2" s="116"/>
+      <c r="AD2" s="116"/>
+      <c r="AE2" s="116"/>
+      <c r="AF2" s="116"/>
+      <c r="AG2" s="117"/>
+      <c r="AH2" s="115" t="s">
         <v>236</v>
       </c>
-      <c r="AI2" s="113"/>
-      <c r="AJ2" s="113"/>
-      <c r="AK2" s="113"/>
-      <c r="AL2" s="113"/>
-      <c r="AM2" s="113"/>
-      <c r="AN2" s="113"/>
-      <c r="AO2" s="114"/>
+      <c r="AI2" s="116"/>
+      <c r="AJ2" s="116"/>
+      <c r="AK2" s="116"/>
+      <c r="AL2" s="116"/>
+      <c r="AM2" s="116"/>
+      <c r="AN2" s="116"/>
+      <c r="AO2" s="117"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A3" s="86"/>
-      <c r="B3" s="98"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="98"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="98"/>
-      <c r="I3" s="98"/>
-      <c r="J3" s="98"/>
-      <c r="K3" s="98"/>
-      <c r="L3" s="98"/>
-      <c r="M3" s="98"/>
-      <c r="N3" s="98"/>
-      <c r="O3" s="98"/>
-      <c r="P3" s="98"/>
-      <c r="Q3" s="98"/>
-      <c r="R3" s="98"/>
-      <c r="S3" s="98"/>
-      <c r="T3" s="98"/>
-      <c r="U3" s="84"/>
-      <c r="V3" s="115"/>
-      <c r="W3" s="115"/>
-      <c r="X3" s="115"/>
-      <c r="Y3" s="115"/>
-      <c r="Z3" s="115"/>
-      <c r="AA3" s="115"/>
-      <c r="AB3" s="115"/>
-      <c r="AC3" s="115"/>
-      <c r="AD3" s="115"/>
-      <c r="AE3" s="115"/>
-      <c r="AF3" s="115"/>
-      <c r="AG3" s="85"/>
-      <c r="AH3" s="84"/>
-      <c r="AI3" s="115"/>
-      <c r="AJ3" s="115"/>
-      <c r="AK3" s="115"/>
-      <c r="AL3" s="115"/>
-      <c r="AM3" s="115"/>
-      <c r="AN3" s="115"/>
-      <c r="AO3" s="85"/>
+      <c r="A3" s="88"/>
+      <c r="B3" s="105"/>
+      <c r="C3" s="105"/>
+      <c r="D3" s="105"/>
+      <c r="E3" s="105"/>
+      <c r="F3" s="105"/>
+      <c r="G3" s="105"/>
+      <c r="H3" s="105"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="105"/>
+      <c r="L3" s="105"/>
+      <c r="M3" s="105"/>
+      <c r="N3" s="105"/>
+      <c r="O3" s="105"/>
+      <c r="P3" s="105"/>
+      <c r="Q3" s="105"/>
+      <c r="R3" s="105"/>
+      <c r="S3" s="105"/>
+      <c r="T3" s="105"/>
+      <c r="U3" s="86"/>
+      <c r="V3" s="118"/>
+      <c r="W3" s="118"/>
+      <c r="X3" s="118"/>
+      <c r="Y3" s="118"/>
+      <c r="Z3" s="118"/>
+      <c r="AA3" s="118"/>
+      <c r="AB3" s="118"/>
+      <c r="AC3" s="118"/>
+      <c r="AD3" s="118"/>
+      <c r="AE3" s="118"/>
+      <c r="AF3" s="118"/>
+      <c r="AG3" s="87"/>
+      <c r="AH3" s="86"/>
+      <c r="AI3" s="118"/>
+      <c r="AJ3" s="118"/>
+      <c r="AK3" s="118"/>
+      <c r="AL3" s="118"/>
+      <c r="AM3" s="118"/>
+      <c r="AN3" s="118"/>
+      <c r="AO3" s="87"/>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A4" s="86"/>
-      <c r="B4" s="93" t="s">
+      <c r="A4" s="88"/>
+      <c r="B4" s="95" t="s">
         <v>143</v>
       </c>
-      <c r="C4" s="93" t="s">
+      <c r="C4" s="95" t="s">
         <v>144</v>
       </c>
-      <c r="D4" s="104" t="s">
+      <c r="D4" s="111" t="s">
         <v>145</v>
       </c>
-      <c r="E4" s="77" t="s">
+      <c r="E4" s="79" t="s">
         <v>191</v>
       </c>
-      <c r="F4" s="77"/>
-      <c r="G4" s="77"/>
-      <c r="H4" s="77" t="s">
+      <c r="F4" s="79"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="79" t="s">
         <v>192</v>
       </c>
-      <c r="I4" s="77"/>
-      <c r="J4" s="77"/>
-      <c r="K4" s="93" t="s">
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="95" t="s">
         <v>174</v>
       </c>
-      <c r="L4" s="77" t="s">
+      <c r="L4" s="79" t="s">
         <v>27</v>
       </c>
-      <c r="M4" s="77"/>
-      <c r="N4" s="77"/>
-      <c r="O4" s="77"/>
-      <c r="P4" s="77" t="s">
+      <c r="M4" s="79"/>
+      <c r="N4" s="79"/>
+      <c r="O4" s="79"/>
+      <c r="P4" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="Q4" s="77"/>
-      <c r="R4" s="77"/>
-      <c r="S4" s="77" t="s">
+      <c r="Q4" s="79"/>
+      <c r="R4" s="79"/>
+      <c r="S4" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="T4" s="77"/>
-      <c r="U4" s="98" t="s">
+      <c r="T4" s="79"/>
+      <c r="U4" s="105" t="s">
         <v>155</v>
       </c>
-      <c r="V4" s="98" t="s">
+      <c r="V4" s="105" t="s">
         <v>30</v>
       </c>
-      <c r="W4" s="98" t="s">
+      <c r="W4" s="105" t="s">
         <v>40</v>
       </c>
-      <c r="X4" s="98" t="s">
+      <c r="X4" s="105" t="s">
         <v>31</v>
       </c>
-      <c r="Y4" s="98" t="s">
+      <c r="Y4" s="105" t="s">
         <v>32</v>
       </c>
-      <c r="Z4" s="98" t="s">
+      <c r="Z4" s="105" t="s">
         <v>33</v>
       </c>
-      <c r="AA4" s="98" t="s">
+      <c r="AA4" s="105" t="s">
         <v>34</v>
       </c>
-      <c r="AB4" s="98" t="s">
+      <c r="AB4" s="105" t="s">
         <v>35</v>
       </c>
-      <c r="AC4" s="98" t="s">
+      <c r="AC4" s="105" t="s">
         <v>36</v>
       </c>
-      <c r="AD4" s="98" t="s">
+      <c r="AD4" s="105" t="s">
         <v>37</v>
       </c>
-      <c r="AE4" s="98" t="s">
+      <c r="AE4" s="105" t="s">
         <v>38</v>
       </c>
-      <c r="AF4" s="98" t="s">
+      <c r="AF4" s="105" t="s">
         <v>147</v>
       </c>
-      <c r="AG4" s="98" t="s">
+      <c r="AG4" s="105" t="s">
         <v>39</v>
       </c>
-      <c r="AH4" s="109" t="s">
+      <c r="AH4" s="98" t="s">
         <v>237</v>
       </c>
-      <c r="AI4" s="111"/>
-      <c r="AJ4" s="77" t="s">
+      <c r="AI4" s="100"/>
+      <c r="AJ4" s="79" t="s">
         <v>238</v>
       </c>
-      <c r="AK4" s="77"/>
-      <c r="AL4" s="77" t="s">
+      <c r="AK4" s="79"/>
+      <c r="AL4" s="79" t="s">
         <v>239</v>
       </c>
-      <c r="AM4" s="77"/>
-      <c r="AN4" s="77" t="s">
+      <c r="AM4" s="79"/>
+      <c r="AN4" s="79" t="s">
         <v>240</v>
       </c>
-      <c r="AO4" s="77"/>
+      <c r="AO4" s="79"/>
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A5" s="86"/>
-      <c r="B5" s="87"/>
-      <c r="C5" s="87"/>
-      <c r="D5" s="106"/>
+      <c r="A5" s="88"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="113"/>
       <c r="E5" s="41" t="s">
         <v>25</v>
       </c>
@@ -43616,7 +43616,7 @@
       <c r="J5" s="44" t="s">
         <v>142</v>
       </c>
-      <c r="K5" s="87"/>
+      <c r="K5" s="89"/>
       <c r="L5" s="38" t="s">
         <v>146</v>
       </c>
@@ -43644,19 +43644,19 @@
       <c r="T5" s="44" t="s">
         <v>148</v>
       </c>
-      <c r="U5" s="98"/>
-      <c r="V5" s="98"/>
-      <c r="W5" s="98"/>
-      <c r="X5" s="98"/>
-      <c r="Y5" s="98"/>
-      <c r="Z5" s="98"/>
-      <c r="AA5" s="98"/>
-      <c r="AB5" s="98"/>
-      <c r="AC5" s="98"/>
-      <c r="AD5" s="98"/>
-      <c r="AE5" s="98"/>
-      <c r="AF5" s="98"/>
-      <c r="AG5" s="98"/>
+      <c r="U5" s="105"/>
+      <c r="V5" s="105"/>
+      <c r="W5" s="105"/>
+      <c r="X5" s="105"/>
+      <c r="Y5" s="105"/>
+      <c r="Z5" s="105"/>
+      <c r="AA5" s="105"/>
+      <c r="AB5" s="105"/>
+      <c r="AC5" s="105"/>
+      <c r="AD5" s="105"/>
+      <c r="AE5" s="105"/>
+      <c r="AF5" s="105"/>
+      <c r="AG5" s="105"/>
       <c r="AH5" s="38" t="s">
         <v>156</v>
       </c>
@@ -52285,6 +52285,20 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="NiKKXtjpQMePcsqc5jjUDaSQ7PwYr9+sjfqfZD87x0KbSUAFE8Baue/7fXFs4bMxVWpKhzgpmVEg8+jmkTDZbw==" saltValue="/cWUcVxNNlNaEWVwXWfzkw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="U2:AG3"/>
+    <mergeCell ref="AB4:AB5"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="B2:T3"/>
+    <mergeCell ref="U4:U5"/>
+    <mergeCell ref="V4:V5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AH2:AO3"/>
     <mergeCell ref="D4:D5"/>
@@ -52301,20 +52315,6 @@
     <mergeCell ref="AG4:AG5"/>
     <mergeCell ref="L4:O4"/>
     <mergeCell ref="AL4:AM4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="U2:AG3"/>
-    <mergeCell ref="AB4:AB5"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="P4:R4"/>
-    <mergeCell ref="B2:T3"/>
-    <mergeCell ref="U4:U5"/>
-    <mergeCell ref="V4:V5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:D5 R5 AI5 AK5 AM5 L5 M5 N5 O5 P5 Q5 AO5 AJ5 AL5 AN5 AH5" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -52366,38 +52366,38 @@
       <c r="D1" s="5"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="88" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="86" t="s">
+      <c r="B2" s="88" t="s">
         <v>189</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="88"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="116"/>
-      <c r="B3" s="86" t="s">
+      <c r="A3" s="119"/>
+      <c r="B3" s="88" t="s">
         <v>184</v>
       </c>
-      <c r="C3" s="117" t="s">
+      <c r="C3" s="120" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="86" t="s">
+      <c r="D3" s="88" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="116"/>
-      <c r="B4" s="86"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="86"/>
+      <c r="A4" s="119"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="120"/>
+      <c r="D4" s="88"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="116"/>
-      <c r="B5" s="86"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="86"/>
+      <c r="A5" s="119"/>
+      <c r="B5" s="88"/>
+      <c r="C5" s="120"/>
+      <c r="D5" s="88"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -53647,64 +53647,64 @@
       <c r="J1" s="7"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="98" t="s">
+      <c r="B2" s="105" t="s">
         <v>225</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="88" t="s">
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="90" t="s">
         <v>226</v>
       </c>
-      <c r="H2" s="89"/>
-      <c r="I2" s="89"/>
-      <c r="J2" s="92"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="94"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="93" t="s">
+      <c r="A3" s="76"/>
+      <c r="B3" s="95" t="s">
         <v>164</v>
       </c>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="95" t="s">
         <v>165</v>
       </c>
-      <c r="D3" s="99" t="s">
+      <c r="D3" s="106" t="s">
         <v>166</v>
       </c>
-      <c r="E3" s="98" t="s">
+      <c r="E3" s="105" t="s">
         <v>171</v>
       </c>
-      <c r="F3" s="114" t="s">
+      <c r="F3" s="117" t="s">
         <v>172</v>
       </c>
-      <c r="G3" s="104" t="s">
+      <c r="G3" s="111" t="s">
         <v>167</v>
       </c>
-      <c r="H3" s="104" t="s">
+      <c r="H3" s="111" t="s">
         <v>168</v>
       </c>
-      <c r="I3" s="104" t="s">
+      <c r="I3" s="111" t="s">
         <v>169</v>
       </c>
-      <c r="J3" s="118" t="s">
+      <c r="J3" s="121" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="87"/>
-      <c r="C4" s="87"/>
-      <c r="D4" s="99"/>
-      <c r="E4" s="98"/>
-      <c r="F4" s="85"/>
-      <c r="G4" s="106"/>
-      <c r="H4" s="106"/>
-      <c r="I4" s="106"/>
-      <c r="J4" s="119"/>
+      <c r="A4" s="77"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="106"/>
+      <c r="E4" s="105"/>
+      <c r="F4" s="87"/>
+      <c r="G4" s="113"/>
+      <c r="H4" s="113"/>
+      <c r="I4" s="113"/>
+      <c r="J4" s="122"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
@@ -56109,6 +56109,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="rbaELUtMLiFIUzK2Lo99z9d9U/+7pUd8ywEap5Et9u8xKeEcXwzK/YHzlDzNf0b31XcPQzpRtM0zLEm0RaQL/w==" saltValue="qBVdEFs3JSBOU1K55aehjA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="12">
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="G2:J2"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
@@ -56116,11 +56121,6 @@
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="G2:J2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D4 G3 H3 I3 J3" xr:uid="{17D462F2-8B43-4EF8-AF0E-D9F26228FDD4}">
@@ -56179,60 +56179,60 @@
       <c r="P1" s="10"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="116" t="s">
+      <c r="B2" s="119" t="s">
         <v>178</v>
       </c>
-      <c r="C2" s="123"/>
-      <c r="D2" s="123"/>
-      <c r="E2" s="123"/>
-      <c r="F2" s="123"/>
-      <c r="G2" s="123"/>
-      <c r="H2" s="123"/>
-      <c r="I2" s="123"/>
-      <c r="J2" s="123"/>
-      <c r="K2" s="117"/>
-      <c r="L2" s="112" t="s">
+      <c r="C2" s="125"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="125"/>
+      <c r="G2" s="125"/>
+      <c r="H2" s="125"/>
+      <c r="I2" s="125"/>
+      <c r="J2" s="125"/>
+      <c r="K2" s="120"/>
+      <c r="L2" s="115" t="s">
         <v>242</v>
       </c>
-      <c r="M2" s="113"/>
-      <c r="N2" s="113"/>
-      <c r="O2" s="113"/>
-      <c r="P2" s="114"/>
+      <c r="M2" s="116"/>
+      <c r="N2" s="116"/>
+      <c r="O2" s="116"/>
+      <c r="P2" s="117"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="124" t="s">
+      <c r="A3" s="76"/>
+      <c r="B3" s="126" t="s">
         <v>173</v>
       </c>
-      <c r="C3" s="128" t="s">
+      <c r="C3" s="130" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="129"/>
-      <c r="E3" s="129"/>
-      <c r="F3" s="129"/>
-      <c r="G3" s="130"/>
-      <c r="H3" s="126" t="s">
+      <c r="D3" s="131"/>
+      <c r="E3" s="131"/>
+      <c r="F3" s="131"/>
+      <c r="G3" s="132"/>
+      <c r="H3" s="128" t="s">
         <v>181</v>
       </c>
-      <c r="I3" s="124" t="s">
+      <c r="I3" s="126" t="s">
         <v>182</v>
       </c>
-      <c r="J3" s="121" t="s">
+      <c r="J3" s="123" t="s">
         <v>243</v>
       </c>
-      <c r="K3" s="122"/>
-      <c r="L3" s="84"/>
-      <c r="M3" s="115"/>
-      <c r="N3" s="115"/>
-      <c r="O3" s="115"/>
-      <c r="P3" s="85"/>
+      <c r="K3" s="124"/>
+      <c r="L3" s="86"/>
+      <c r="M3" s="118"/>
+      <c r="N3" s="118"/>
+      <c r="O3" s="118"/>
+      <c r="P3" s="87"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="125"/>
+      <c r="A4" s="77"/>
+      <c r="B4" s="127"/>
       <c r="C4" s="47" t="s">
         <v>23</v>
       </c>
@@ -56248,8 +56248,8 @@
       <c r="G4" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="H4" s="127"/>
-      <c r="I4" s="125"/>
+      <c r="H4" s="129"/>
+      <c r="I4" s="127"/>
       <c r="J4" s="48" t="s">
         <v>23</v>
       </c>
@@ -59906,7 +59906,7 @@
   <sheetPr>
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:AD205"/>
+  <dimension ref="A1:AD204"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="3" customWidth="1"/>
@@ -59973,128 +59973,128 @@
       <c r="AD1" s="5"/>
     </row>
     <row r="2" spans="1:30" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="86" t="s">
+      <c r="B2" s="114" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="86" t="s">
+      <c r="C2" s="88" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="116" t="s">
+      <c r="D2" s="88"/>
+      <c r="E2" s="88"/>
+      <c r="F2" s="119" t="s">
         <v>95</v>
       </c>
-      <c r="G2" s="123"/>
-      <c r="H2" s="117"/>
-      <c r="I2" s="120" t="s">
+      <c r="G2" s="125"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="114" t="s">
         <v>260</v>
       </c>
-      <c r="J2" s="120" t="s">
+      <c r="J2" s="114" t="s">
         <v>261</v>
       </c>
-      <c r="K2" s="112" t="s">
+      <c r="K2" s="115" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="113"/>
-      <c r="M2" s="114"/>
-      <c r="N2" s="112" t="s">
+      <c r="L2" s="116"/>
+      <c r="M2" s="117"/>
+      <c r="N2" s="115" t="s">
         <v>50</v>
       </c>
-      <c r="O2" s="114"/>
-      <c r="P2" s="86" t="s">
+      <c r="O2" s="117"/>
+      <c r="P2" s="88" t="s">
         <v>262</v>
       </c>
-      <c r="Q2" s="98" t="s">
+      <c r="Q2" s="105" t="s">
         <v>263</v>
       </c>
-      <c r="R2" s="86" t="s">
+      <c r="R2" s="88" t="s">
         <v>264</v>
       </c>
-      <c r="S2" s="86" t="s">
+      <c r="S2" s="88" t="s">
         <v>271</v>
       </c>
-      <c r="T2" s="86"/>
-      <c r="U2" s="131" t="s">
+      <c r="T2" s="88"/>
+      <c r="U2" s="133" t="s">
         <v>272</v>
       </c>
-      <c r="V2" s="132"/>
-      <c r="W2" s="131" t="s">
+      <c r="V2" s="134"/>
+      <c r="W2" s="133" t="s">
         <v>273</v>
       </c>
-      <c r="X2" s="132"/>
-      <c r="Y2" s="131" t="s">
+      <c r="X2" s="134"/>
+      <c r="Y2" s="133" t="s">
         <v>274</v>
       </c>
-      <c r="Z2" s="132"/>
-      <c r="AA2" s="86" t="s">
+      <c r="Z2" s="134"/>
+      <c r="AA2" s="88" t="s">
         <v>270</v>
       </c>
-      <c r="AB2" s="86"/>
-      <c r="AC2" s="86"/>
-      <c r="AD2" s="86"/>
+      <c r="AB2" s="88"/>
+      <c r="AC2" s="88"/>
+      <c r="AD2" s="88"/>
     </row>
     <row r="3" spans="1:30" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="86"/>
-      <c r="B3" s="86"/>
-      <c r="C3" s="78" t="s">
+      <c r="A3" s="76"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="80" t="s">
         <v>98</v>
       </c>
-      <c r="D3" s="116" t="s">
+      <c r="D3" s="119" t="s">
         <v>96</v>
       </c>
-      <c r="E3" s="117"/>
-      <c r="F3" s="120" t="s">
+      <c r="E3" s="120"/>
+      <c r="F3" s="114" t="s">
         <v>98</v>
       </c>
-      <c r="G3" s="116" t="s">
+      <c r="G3" s="119" t="s">
         <v>96</v>
       </c>
-      <c r="H3" s="117"/>
-      <c r="I3" s="74"/>
-      <c r="J3" s="74"/>
-      <c r="K3" s="84"/>
-      <c r="L3" s="115"/>
-      <c r="M3" s="85"/>
-      <c r="N3" s="84"/>
-      <c r="O3" s="85"/>
-      <c r="P3" s="86"/>
-      <c r="Q3" s="98"/>
-      <c r="R3" s="86"/>
-      <c r="S3" s="86"/>
-      <c r="T3" s="86"/>
-      <c r="U3" s="81"/>
-      <c r="V3" s="83"/>
-      <c r="W3" s="81"/>
-      <c r="X3" s="83"/>
-      <c r="Y3" s="81"/>
-      <c r="Z3" s="83"/>
-      <c r="AA3" s="86"/>
-      <c r="AB3" s="86"/>
-      <c r="AC3" s="86"/>
-      <c r="AD3" s="86"/>
+      <c r="H3" s="120"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="86"/>
+      <c r="L3" s="118"/>
+      <c r="M3" s="87"/>
+      <c r="N3" s="86"/>
+      <c r="O3" s="87"/>
+      <c r="P3" s="88"/>
+      <c r="Q3" s="105"/>
+      <c r="R3" s="88"/>
+      <c r="S3" s="88"/>
+      <c r="T3" s="88"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="85"/>
+      <c r="W3" s="83"/>
+      <c r="X3" s="85"/>
+      <c r="Y3" s="83"/>
+      <c r="Z3" s="85"/>
+      <c r="AA3" s="88"/>
+      <c r="AB3" s="88"/>
+      <c r="AC3" s="88"/>
+      <c r="AD3" s="88"/>
     </row>
     <row r="4" spans="1:30" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="86"/>
-      <c r="B4" s="86"/>
-      <c r="C4" s="81"/>
+      <c r="A4" s="77"/>
+      <c r="B4" s="77"/>
+      <c r="C4" s="83"/>
       <c r="D4" s="39" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="75"/>
+      <c r="F4" s="77"/>
       <c r="G4" s="39" t="s">
         <v>0</v>
       </c>
       <c r="H4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="75"/>
-      <c r="J4" s="75"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="77"/>
       <c r="K4" s="50" t="s">
         <v>212</v>
       </c>
@@ -60110,9 +60110,9 @@
       <c r="O4" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="P4" s="86"/>
-      <c r="Q4" s="98"/>
-      <c r="R4" s="86"/>
+      <c r="P4" s="88"/>
+      <c r="Q4" s="105"/>
+      <c r="R4" s="88"/>
       <c r="S4" s="39" t="s">
         <v>51</v>
       </c>
@@ -60150,9 +60150,9 @@
         <v>269</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="86"/>
-      <c r="B5" s="86"/>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -66521,62 +66521,30 @@
     <row r="204" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A204" s="2"/>
       <c r="B204" s="2"/>
-      <c r="C204" s="2"/>
-      <c r="D204" s="2"/>
-      <c r="E204" s="2"/>
-      <c r="F204" s="2"/>
-      <c r="G204" s="2"/>
-      <c r="H204" s="2"/>
-      <c r="I204" s="2"/>
-      <c r="J204" s="2"/>
-      <c r="K204" s="2"/>
-      <c r="L204" s="2"/>
-      <c r="M204" s="2"/>
-      <c r="N204" s="2"/>
-      <c r="O204" s="2"/>
-      <c r="P204" s="2"/>
-      <c r="Q204" s="2"/>
-      <c r="R204" s="2"/>
-      <c r="S204" s="2"/>
-      <c r="T204" s="2"/>
-      <c r="U204" s="2"/>
-      <c r="V204" s="2"/>
-      <c r="W204" s="2"/>
-      <c r="X204" s="2"/>
-      <c r="Y204" s="2"/>
-      <c r="Z204" s="2"/>
-      <c r="AA204" s="2"/>
-      <c r="AB204" s="2"/>
-      <c r="AC204" s="2"/>
-      <c r="AD204" s="2"/>
-    </row>
-    <row r="205" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A205" s="2"/>
-      <c r="B205" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="zQSoqCh6NklK+XOlfBHn5L/gkA8bUhEBpKNPR/UWtjP7LqyKJ82YTrw2gHO9hiqZ9v7JIRNMdfA8g75dUAbLKw==" saltValue="Ukda4p/GuI/wk/l5mCii6g==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="Npdc6hR1jWNwlUd78HFJSJlOVnyVZEkwE3li2w9MaNYbr3qpWORdGSkVHRoIs6ZmqiHg7fNUc25lo9m1DLSPvg==" saltValue="CpsBwfeTpFYKyUOX8eB08w==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="Y2:Z3"/>
+    <mergeCell ref="AA2:AD3"/>
+    <mergeCell ref="U2:V3"/>
+    <mergeCell ref="W2:X3"/>
+    <mergeCell ref="K2:M3"/>
+    <mergeCell ref="P2:P4"/>
+    <mergeCell ref="Q2:Q4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="S2:T3"/>
+    <mergeCell ref="I2:I4"/>
+    <mergeCell ref="J2:J4"/>
     <mergeCell ref="N2:O3"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B2:B5"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="C2:E2"/>
-    <mergeCell ref="P2:P4"/>
-    <mergeCell ref="Q2:Q4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="S2:T3"/>
-    <mergeCell ref="I2:I4"/>
-    <mergeCell ref="J2:J4"/>
-    <mergeCell ref="Y2:Z3"/>
-    <mergeCell ref="AA2:AD3"/>
-    <mergeCell ref="U2:V3"/>
-    <mergeCell ref="W2:X3"/>
-    <mergeCell ref="K2:M3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 AA4:AD4" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">

</xml_diff>

<commit_message>
Description of all changes to the Form LL
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69718F07-E18E-47F4-97CE-F6ADAE11F97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE237DD-1B0B-44E3-951A-85282E8A3179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" firstSheet="5" activeTab="8" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="274">
   <si>
     <t>LATITUDE</t>
   </si>
@@ -715,9 +715,6 @@
   </si>
   <si>
     <t>NUMBER_BRANCHLINE_HAULINGS_OBSERVED</t>
-  </si>
-  <si>
-    <t>NUMBER_HOOKS_RETRIEVED_DURING_OBSERVATION</t>
   </si>
   <si>
     <t>HOOKS</t>
@@ -1548,6 +1545,21 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1578,9 +1590,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1599,18 +1608,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2373,10 +2370,10 @@
         <v>23</v>
       </c>
       <c r="D2" s="56" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E2" s="60" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="55" customFormat="1" x14ac:dyDescent="0.25">
@@ -3842,19 +3839,19 @@
         <v>110</v>
       </c>
       <c r="C2" s="114" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D2" s="114" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E2" s="95" t="s">
         <v>55</v>
       </c>
       <c r="F2" s="114" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G2" s="114" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H2" s="114" t="s">
         <v>56</v>
@@ -3863,11 +3860,11 @@
         <v>111</v>
       </c>
       <c r="J2" s="90" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="K2" s="94"/>
       <c r="L2" s="119" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="M2" s="125"/>
       <c r="N2" s="125"/>
@@ -3890,16 +3887,16 @@
         <v>97</v>
       </c>
       <c r="L3" s="56" t="s">
+        <v>245</v>
+      </c>
+      <c r="M3" s="56" t="s">
         <v>246</v>
       </c>
-      <c r="M3" s="56" t="s">
+      <c r="N3" s="56" t="s">
         <v>247</v>
       </c>
-      <c r="N3" s="56" t="s">
+      <c r="O3" s="56" t="s">
         <v>248</v>
-      </c>
-      <c r="O3" s="56" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -7304,17 +7301,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="ZHZ61xEMWo2GozKFDfIGwtbJZnm3eVYJpvIE2b76e/O5EaOFEu4qUPnEZ+3+QLMo4fMOZjuAZJWBGppNj6h0fg==" saltValue="p7UsgbvwfBAQ3S2mqNofIA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="E2:E3"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="J2:K2"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="I2:I3"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="E2:E3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3 M3 N3 O3" xr:uid="{35387E2C-FBDF-4B0A-A0B5-EF76A6744ABB}">
@@ -7363,7 +7360,7 @@
         <v>110</v>
       </c>
       <c r="C2" s="119" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D2" s="125"/>
       <c r="E2" s="120"/>
@@ -8813,7 +8810,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -10476,7 +10473,7 @@
   <sheetPr>
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:Q204"/>
+  <dimension ref="A1:P204"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.28515625" style="3" bestFit="1" customWidth="1"/>
@@ -10491,11 +10488,10 @@
     <col min="10" max="13" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="33.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="42.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="49.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>85</v>
       </c>
@@ -10513,10 +10509,9 @@
       <c r="M1" s="5"/>
       <c r="N1" s="5"/>
       <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="6"/>
-    </row>
-    <row r="2" spans="1:17" s="55" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="P1" s="6"/>
+    </row>
+    <row r="2" spans="1:16" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
@@ -10524,38 +10519,35 @@
         <v>110</v>
       </c>
       <c r="C2" s="119" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D2" s="125"/>
       <c r="E2" s="120"/>
       <c r="F2" s="119" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G2" s="125"/>
       <c r="H2" s="120"/>
-      <c r="I2" s="106" t="s">
+      <c r="I2" s="109" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="105" t="s">
+      <c r="J2" s="99" t="s">
         <v>214</v>
       </c>
-      <c r="K2" s="105"/>
-      <c r="L2" s="105"/>
-      <c r="M2" s="105"/>
+      <c r="K2" s="99"/>
+      <c r="L2" s="99"/>
+      <c r="M2" s="99"/>
       <c r="N2" s="88" t="s">
         <v>58</v>
       </c>
       <c r="O2" s="88" t="s">
         <v>219</v>
       </c>
-      <c r="P2" s="88" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q2" s="135" t="s">
+      <c r="P2" s="135" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="3" spans="1:17" s="55" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
       <c r="B3" s="76"/>
       <c r="C3" s="114" t="s">
@@ -10572,17 +10564,16 @@
         <v>96</v>
       </c>
       <c r="H3" s="120"/>
-      <c r="I3" s="106"/>
-      <c r="J3" s="105"/>
-      <c r="K3" s="105"/>
-      <c r="L3" s="105"/>
-      <c r="M3" s="105"/>
+      <c r="I3" s="109"/>
+      <c r="J3" s="99"/>
+      <c r="K3" s="99"/>
+      <c r="L3" s="99"/>
+      <c r="M3" s="99"/>
       <c r="N3" s="88"/>
       <c r="O3" s="88"/>
-      <c r="P3" s="88"/>
-      <c r="Q3" s="135"/>
-    </row>
-    <row r="4" spans="1:17" s="55" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="P3" s="135"/>
+    </row>
+    <row r="4" spans="1:16" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="77"/>
       <c r="B4" s="77"/>
       <c r="C4" s="77"/>
@@ -10599,7 +10590,7 @@
       <c r="H4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="106"/>
+      <c r="I4" s="109"/>
       <c r="J4" s="50" t="s">
         <v>213</v>
       </c>
@@ -10614,10 +10605,9 @@
       </c>
       <c r="N4" s="88"/>
       <c r="O4" s="88"/>
-      <c r="P4" s="88"/>
-      <c r="Q4" s="135"/>
-    </row>
-    <row r="5" spans="1:17" s="55" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="P4" s="135"/>
+    </row>
+    <row r="5" spans="1:16" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -10634,9 +10624,8 @@
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -10653,9 +10642,8 @@
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10672,9 +10660,8 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -10691,9 +10678,8 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -10710,9 +10696,8 @@
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -10729,9 +10714,8 @@
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -10748,9 +10732,8 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -10767,9 +10750,8 @@
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -10786,9 +10768,8 @@
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -10805,9 +10786,8 @@
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -10824,9 +10804,8 @@
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -10843,9 +10822,8 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -10862,9 +10840,8 @@
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -10881,9 +10858,8 @@
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -10900,9 +10876,8 @@
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -10919,9 +10894,8 @@
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -10938,9 +10912,8 @@
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -10957,9 +10930,8 @@
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -10976,9 +10948,8 @@
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -10995,9 +10966,8 @@
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -11014,9 +10984,8 @@
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
       <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -11033,9 +11002,8 @@
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
-      <c r="Q26" s="2"/>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -11052,9 +11020,8 @@
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
-      <c r="Q27" s="2"/>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -11071,9 +11038,8 @@
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
       <c r="P28" s="2"/>
-      <c r="Q28" s="2"/>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -11090,9 +11056,8 @@
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
-      <c r="Q29" s="2"/>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -11109,9 +11074,8 @@
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -11128,9 +11092,8 @@
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
-      <c r="Q31" s="2"/>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -11147,9 +11110,8 @@
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
-      <c r="Q32" s="2"/>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -11166,9 +11128,8 @@
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
-      <c r="Q33" s="2"/>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -11185,9 +11146,8 @@
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
-      <c r="Q34" s="2"/>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -11204,9 +11164,8 @@
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
-      <c r="Q35" s="2"/>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -11223,9 +11182,8 @@
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -11242,9 +11200,8 @@
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
-      <c r="Q37" s="2"/>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -11261,9 +11218,8 @@
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" s="2"/>
-      <c r="Q38" s="2"/>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -11280,9 +11236,8 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
-      <c r="Q39" s="2"/>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -11299,9 +11254,8 @@
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
-      <c r="Q40" s="2"/>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -11318,9 +11272,8 @@
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
-      <c r="Q41" s="2"/>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -11337,9 +11290,8 @@
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
-      <c r="Q42" s="2"/>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -11356,9 +11308,8 @@
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
-      <c r="Q43" s="2"/>
-    </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -11375,9 +11326,8 @@
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
-      <c r="Q44" s="2"/>
-    </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -11394,9 +11344,8 @@
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
-      <c r="Q45" s="2"/>
-    </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -11413,9 +11362,8 @@
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
-      <c r="Q46" s="2"/>
-    </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -11432,9 +11380,8 @@
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
-      <c r="Q47" s="2"/>
-    </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -11451,9 +11398,8 @@
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
-      <c r="Q48" s="2"/>
-    </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -11470,9 +11416,8 @@
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
-      <c r="Q49" s="2"/>
-    </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -11489,9 +11434,8 @@
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
-      <c r="Q50" s="2"/>
-    </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -11508,9 +11452,8 @@
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
-      <c r="Q51" s="2"/>
-    </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -11527,9 +11470,8 @@
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
       <c r="P52" s="2"/>
-      <c r="Q52" s="2"/>
-    </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -11546,9 +11488,8 @@
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
       <c r="P53" s="2"/>
-      <c r="Q53" s="2"/>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -11565,9 +11506,8 @@
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
-      <c r="Q54" s="2"/>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -11584,9 +11524,8 @@
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
       <c r="P55" s="2"/>
-      <c r="Q55" s="2"/>
-    </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -11603,9 +11542,8 @@
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
       <c r="P56" s="2"/>
-      <c r="Q56" s="2"/>
-    </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -11622,9 +11560,8 @@
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
       <c r="P57" s="2"/>
-      <c r="Q57" s="2"/>
-    </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -11641,9 +11578,8 @@
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
-      <c r="Q58" s="2"/>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -11660,9 +11596,8 @@
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
-      <c r="Q59" s="2"/>
-    </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -11679,9 +11614,8 @@
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
-      <c r="Q60" s="2"/>
-    </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -11698,9 +11632,8 @@
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
-      <c r="Q61" s="2"/>
-    </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -11717,9 +11650,8 @@
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
-      <c r="Q62" s="2"/>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -11736,9 +11668,8 @@
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
-      <c r="Q63" s="2"/>
-    </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -11755,9 +11686,8 @@
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
-      <c r="Q64" s="2"/>
-    </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -11774,9 +11704,8 @@
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
-      <c r="Q65" s="2"/>
-    </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -11793,9 +11722,8 @@
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
-      <c r="Q66" s="2"/>
-    </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -11812,9 +11740,8 @@
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
       <c r="P67" s="2"/>
-      <c r="Q67" s="2"/>
-    </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -11831,9 +11758,8 @@
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
-      <c r="Q68" s="2"/>
-    </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -11850,9 +11776,8 @@
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
-      <c r="Q69" s="2"/>
-    </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -11869,9 +11794,8 @@
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
-      <c r="Q70" s="2"/>
-    </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -11888,9 +11812,8 @@
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
       <c r="P71" s="2"/>
-      <c r="Q71" s="2"/>
-    </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -11907,9 +11830,8 @@
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
-      <c r="Q72" s="2"/>
-    </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -11926,9 +11848,8 @@
       <c r="N73" s="2"/>
       <c r="O73" s="2"/>
       <c r="P73" s="2"/>
-      <c r="Q73" s="2"/>
-    </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -11945,9 +11866,8 @@
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
       <c r="P74" s="2"/>
-      <c r="Q74" s="2"/>
-    </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -11964,9 +11884,8 @@
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
-      <c r="Q75" s="2"/>
-    </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -11983,9 +11902,8 @@
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
-      <c r="Q76" s="2"/>
-    </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -12002,9 +11920,8 @@
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>
-      <c r="Q77" s="2"/>
-    </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -12021,9 +11938,8 @@
       <c r="N78" s="2"/>
       <c r="O78" s="2"/>
       <c r="P78" s="2"/>
-      <c r="Q78" s="2"/>
-    </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -12040,9 +11956,8 @@
       <c r="N79" s="2"/>
       <c r="O79" s="2"/>
       <c r="P79" s="2"/>
-      <c r="Q79" s="2"/>
-    </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -12059,9 +11974,8 @@
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
       <c r="P80" s="2"/>
-      <c r="Q80" s="2"/>
-    </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -12078,9 +11992,8 @@
       <c r="N81" s="2"/>
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
-      <c r="Q81" s="2"/>
-    </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -12097,9 +12010,8 @@
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
       <c r="P82" s="2"/>
-      <c r="Q82" s="2"/>
-    </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -12116,9 +12028,8 @@
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
       <c r="P83" s="2"/>
-      <c r="Q83" s="2"/>
-    </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -12135,9 +12046,8 @@
       <c r="N84" s="2"/>
       <c r="O84" s="2"/>
       <c r="P84" s="2"/>
-      <c r="Q84" s="2"/>
-    </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -12154,9 +12064,8 @@
       <c r="N85" s="2"/>
       <c r="O85" s="2"/>
       <c r="P85" s="2"/>
-      <c r="Q85" s="2"/>
-    </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -12173,9 +12082,8 @@
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
       <c r="P86" s="2"/>
-      <c r="Q86" s="2"/>
-    </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -12192,9 +12100,8 @@
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
       <c r="P87" s="2"/>
-      <c r="Q87" s="2"/>
-    </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -12211,9 +12118,8 @@
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
       <c r="P88" s="2"/>
-      <c r="Q88" s="2"/>
-    </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -12230,9 +12136,8 @@
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
       <c r="P89" s="2"/>
-      <c r="Q89" s="2"/>
-    </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -12249,9 +12154,8 @@
       <c r="N90" s="2"/>
       <c r="O90" s="2"/>
       <c r="P90" s="2"/>
-      <c r="Q90" s="2"/>
-    </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -12268,9 +12172,8 @@
       <c r="N91" s="2"/>
       <c r="O91" s="2"/>
       <c r="P91" s="2"/>
-      <c r="Q91" s="2"/>
-    </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -12287,9 +12190,8 @@
       <c r="N92" s="2"/>
       <c r="O92" s="2"/>
       <c r="P92" s="2"/>
-      <c r="Q92" s="2"/>
-    </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -12306,9 +12208,8 @@
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
       <c r="P93" s="2"/>
-      <c r="Q93" s="2"/>
-    </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -12325,9 +12226,8 @@
       <c r="N94" s="2"/>
       <c r="O94" s="2"/>
       <c r="P94" s="2"/>
-      <c r="Q94" s="2"/>
-    </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -12344,9 +12244,8 @@
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
       <c r="P95" s="2"/>
-      <c r="Q95" s="2"/>
-    </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -12363,9 +12262,8 @@
       <c r="N96" s="2"/>
       <c r="O96" s="2"/>
       <c r="P96" s="2"/>
-      <c r="Q96" s="2"/>
-    </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -12382,9 +12280,8 @@
       <c r="N97" s="2"/>
       <c r="O97" s="2"/>
       <c r="P97" s="2"/>
-      <c r="Q97" s="2"/>
-    </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -12401,9 +12298,8 @@
       <c r="N98" s="2"/>
       <c r="O98" s="2"/>
       <c r="P98" s="2"/>
-      <c r="Q98" s="2"/>
-    </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -12420,9 +12316,8 @@
       <c r="N99" s="2"/>
       <c r="O99" s="2"/>
       <c r="P99" s="2"/>
-      <c r="Q99" s="2"/>
-    </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -12439,9 +12334,8 @@
       <c r="N100" s="2"/>
       <c r="O100" s="2"/>
       <c r="P100" s="2"/>
-      <c r="Q100" s="2"/>
-    </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
@@ -12458,9 +12352,8 @@
       <c r="N101" s="2"/>
       <c r="O101" s="2"/>
       <c r="P101" s="2"/>
-      <c r="Q101" s="2"/>
-    </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -12477,9 +12370,8 @@
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
       <c r="P102" s="2"/>
-      <c r="Q102" s="2"/>
-    </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -12496,9 +12388,8 @@
       <c r="N103" s="2"/>
       <c r="O103" s="2"/>
       <c r="P103" s="2"/>
-      <c r="Q103" s="2"/>
-    </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -12515,9 +12406,8 @@
       <c r="N104" s="2"/>
       <c r="O104" s="2"/>
       <c r="P104" s="2"/>
-      <c r="Q104" s="2"/>
-    </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="2"/>
@@ -12534,9 +12424,8 @@
       <c r="N105" s="2"/>
       <c r="O105" s="2"/>
       <c r="P105" s="2"/>
-      <c r="Q105" s="2"/>
-    </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2"/>
@@ -12553,9 +12442,8 @@
       <c r="N106" s="2"/>
       <c r="O106" s="2"/>
       <c r="P106" s="2"/>
-      <c r="Q106" s="2"/>
-    </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
@@ -12572,9 +12460,8 @@
       <c r="N107" s="2"/>
       <c r="O107" s="2"/>
       <c r="P107" s="2"/>
-      <c r="Q107" s="2"/>
-    </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="2"/>
@@ -12591,9 +12478,8 @@
       <c r="N108" s="2"/>
       <c r="O108" s="2"/>
       <c r="P108" s="2"/>
-      <c r="Q108" s="2"/>
-    </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
@@ -12610,9 +12496,8 @@
       <c r="N109" s="2"/>
       <c r="O109" s="2"/>
       <c r="P109" s="2"/>
-      <c r="Q109" s="2"/>
-    </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
@@ -12629,9 +12514,8 @@
       <c r="N110" s="2"/>
       <c r="O110" s="2"/>
       <c r="P110" s="2"/>
-      <c r="Q110" s="2"/>
-    </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
@@ -12648,9 +12532,8 @@
       <c r="N111" s="2"/>
       <c r="O111" s="2"/>
       <c r="P111" s="2"/>
-      <c r="Q111" s="2"/>
-    </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
@@ -12667,9 +12550,8 @@
       <c r="N112" s="2"/>
       <c r="O112" s="2"/>
       <c r="P112" s="2"/>
-      <c r="Q112" s="2"/>
-    </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
@@ -12686,9 +12568,8 @@
       <c r="N113" s="2"/>
       <c r="O113" s="2"/>
       <c r="P113" s="2"/>
-      <c r="Q113" s="2"/>
-    </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
@@ -12705,9 +12586,8 @@
       <c r="N114" s="2"/>
       <c r="O114" s="2"/>
       <c r="P114" s="2"/>
-      <c r="Q114" s="2"/>
-    </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -12724,9 +12604,8 @@
       <c r="N115" s="2"/>
       <c r="O115" s="2"/>
       <c r="P115" s="2"/>
-      <c r="Q115" s="2"/>
-    </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
@@ -12743,9 +12622,8 @@
       <c r="N116" s="2"/>
       <c r="O116" s="2"/>
       <c r="P116" s="2"/>
-      <c r="Q116" s="2"/>
-    </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
@@ -12762,9 +12640,8 @@
       <c r="N117" s="2"/>
       <c r="O117" s="2"/>
       <c r="P117" s="2"/>
-      <c r="Q117" s="2"/>
-    </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="2"/>
@@ -12781,9 +12658,8 @@
       <c r="N118" s="2"/>
       <c r="O118" s="2"/>
       <c r="P118" s="2"/>
-      <c r="Q118" s="2"/>
-    </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
@@ -12800,9 +12676,8 @@
       <c r="N119" s="2"/>
       <c r="O119" s="2"/>
       <c r="P119" s="2"/>
-      <c r="Q119" s="2"/>
-    </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
@@ -12819,9 +12694,8 @@
       <c r="N120" s="2"/>
       <c r="O120" s="2"/>
       <c r="P120" s="2"/>
-      <c r="Q120" s="2"/>
-    </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
@@ -12838,9 +12712,8 @@
       <c r="N121" s="2"/>
       <c r="O121" s="2"/>
       <c r="P121" s="2"/>
-      <c r="Q121" s="2"/>
-    </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
@@ -12857,9 +12730,8 @@
       <c r="N122" s="2"/>
       <c r="O122" s="2"/>
       <c r="P122" s="2"/>
-      <c r="Q122" s="2"/>
-    </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -12876,9 +12748,8 @@
       <c r="N123" s="2"/>
       <c r="O123" s="2"/>
       <c r="P123" s="2"/>
-      <c r="Q123" s="2"/>
-    </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="2"/>
@@ -12895,9 +12766,8 @@
       <c r="N124" s="2"/>
       <c r="O124" s="2"/>
       <c r="P124" s="2"/>
-      <c r="Q124" s="2"/>
-    </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -12914,9 +12784,8 @@
       <c r="N125" s="2"/>
       <c r="O125" s="2"/>
       <c r="P125" s="2"/>
-      <c r="Q125" s="2"/>
-    </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
@@ -12933,9 +12802,8 @@
       <c r="N126" s="2"/>
       <c r="O126" s="2"/>
       <c r="P126" s="2"/>
-      <c r="Q126" s="2"/>
-    </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
@@ -12952,9 +12820,8 @@
       <c r="N127" s="2"/>
       <c r="O127" s="2"/>
       <c r="P127" s="2"/>
-      <c r="Q127" s="2"/>
-    </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="2"/>
@@ -12971,9 +12838,8 @@
       <c r="N128" s="2"/>
       <c r="O128" s="2"/>
       <c r="P128" s="2"/>
-      <c r="Q128" s="2"/>
-    </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
@@ -12990,9 +12856,8 @@
       <c r="N129" s="2"/>
       <c r="O129" s="2"/>
       <c r="P129" s="2"/>
-      <c r="Q129" s="2"/>
-    </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
@@ -13009,9 +12874,8 @@
       <c r="N130" s="2"/>
       <c r="O130" s="2"/>
       <c r="P130" s="2"/>
-      <c r="Q130" s="2"/>
-    </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
@@ -13028,9 +12892,8 @@
       <c r="N131" s="2"/>
       <c r="O131" s="2"/>
       <c r="P131" s="2"/>
-      <c r="Q131" s="2"/>
-    </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -13047,9 +12910,8 @@
       <c r="N132" s="2"/>
       <c r="O132" s="2"/>
       <c r="P132" s="2"/>
-      <c r="Q132" s="2"/>
-    </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
@@ -13066,9 +12928,8 @@
       <c r="N133" s="2"/>
       <c r="O133" s="2"/>
       <c r="P133" s="2"/>
-      <c r="Q133" s="2"/>
-    </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -13085,9 +12946,8 @@
       <c r="N134" s="2"/>
       <c r="O134" s="2"/>
       <c r="P134" s="2"/>
-      <c r="Q134" s="2"/>
-    </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
@@ -13104,9 +12964,8 @@
       <c r="N135" s="2"/>
       <c r="O135" s="2"/>
       <c r="P135" s="2"/>
-      <c r="Q135" s="2"/>
-    </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -13123,9 +12982,8 @@
       <c r="N136" s="2"/>
       <c r="O136" s="2"/>
       <c r="P136" s="2"/>
-      <c r="Q136" s="2"/>
-    </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
@@ -13142,9 +13000,8 @@
       <c r="N137" s="2"/>
       <c r="O137" s="2"/>
       <c r="P137" s="2"/>
-      <c r="Q137" s="2"/>
-    </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
@@ -13161,9 +13018,8 @@
       <c r="N138" s="2"/>
       <c r="O138" s="2"/>
       <c r="P138" s="2"/>
-      <c r="Q138" s="2"/>
-    </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
@@ -13180,9 +13036,8 @@
       <c r="N139" s="2"/>
       <c r="O139" s="2"/>
       <c r="P139" s="2"/>
-      <c r="Q139" s="2"/>
-    </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
@@ -13199,9 +13054,8 @@
       <c r="N140" s="2"/>
       <c r="O140" s="2"/>
       <c r="P140" s="2"/>
-      <c r="Q140" s="2"/>
-    </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
       <c r="C141" s="2"/>
@@ -13218,9 +13072,8 @@
       <c r="N141" s="2"/>
       <c r="O141" s="2"/>
       <c r="P141" s="2"/>
-      <c r="Q141" s="2"/>
-    </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A142" s="2"/>
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
@@ -13237,9 +13090,8 @@
       <c r="N142" s="2"/>
       <c r="O142" s="2"/>
       <c r="P142" s="2"/>
-      <c r="Q142" s="2"/>
-    </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
@@ -13256,9 +13108,8 @@
       <c r="N143" s="2"/>
       <c r="O143" s="2"/>
       <c r="P143" s="2"/>
-      <c r="Q143" s="2"/>
-    </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A144" s="2"/>
       <c r="B144" s="2"/>
       <c r="C144" s="2"/>
@@ -13275,9 +13126,8 @@
       <c r="N144" s="2"/>
       <c r="O144" s="2"/>
       <c r="P144" s="2"/>
-      <c r="Q144" s="2"/>
-    </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
@@ -13294,9 +13144,8 @@
       <c r="N145" s="2"/>
       <c r="O145" s="2"/>
       <c r="P145" s="2"/>
-      <c r="Q145" s="2"/>
-    </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="2"/>
@@ -13313,9 +13162,8 @@
       <c r="N146" s="2"/>
       <c r="O146" s="2"/>
       <c r="P146" s="2"/>
-      <c r="Q146" s="2"/>
-    </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
@@ -13332,9 +13180,8 @@
       <c r="N147" s="2"/>
       <c r="O147" s="2"/>
       <c r="P147" s="2"/>
-      <c r="Q147" s="2"/>
-    </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
       <c r="C148" s="2"/>
@@ -13351,9 +13198,8 @@
       <c r="N148" s="2"/>
       <c r="O148" s="2"/>
       <c r="P148" s="2"/>
-      <c r="Q148" s="2"/>
-    </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
@@ -13370,9 +13216,8 @@
       <c r="N149" s="2"/>
       <c r="O149" s="2"/>
       <c r="P149" s="2"/>
-      <c r="Q149" s="2"/>
-    </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
@@ -13389,9 +13234,8 @@
       <c r="N150" s="2"/>
       <c r="O150" s="2"/>
       <c r="P150" s="2"/>
-      <c r="Q150" s="2"/>
-    </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
@@ -13408,9 +13252,8 @@
       <c r="N151" s="2"/>
       <c r="O151" s="2"/>
       <c r="P151" s="2"/>
-      <c r="Q151" s="2"/>
-    </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
@@ -13427,9 +13270,8 @@
       <c r="N152" s="2"/>
       <c r="O152" s="2"/>
       <c r="P152" s="2"/>
-      <c r="Q152" s="2"/>
-    </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="153" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -13446,9 +13288,8 @@
       <c r="N153" s="2"/>
       <c r="O153" s="2"/>
       <c r="P153" s="2"/>
-      <c r="Q153" s="2"/>
-    </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
@@ -13465,9 +13306,8 @@
       <c r="N154" s="2"/>
       <c r="O154" s="2"/>
       <c r="P154" s="2"/>
-      <c r="Q154" s="2"/>
-    </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
@@ -13484,9 +13324,8 @@
       <c r="N155" s="2"/>
       <c r="O155" s="2"/>
       <c r="P155" s="2"/>
-      <c r="Q155" s="2"/>
-    </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
@@ -13503,9 +13342,8 @@
       <c r="N156" s="2"/>
       <c r="O156" s="2"/>
       <c r="P156" s="2"/>
-      <c r="Q156" s="2"/>
-    </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="157" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
@@ -13522,9 +13360,8 @@
       <c r="N157" s="2"/>
       <c r="O157" s="2"/>
       <c r="P157" s="2"/>
-      <c r="Q157" s="2"/>
-    </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="158" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
@@ -13541,9 +13378,8 @@
       <c r="N158" s="2"/>
       <c r="O158" s="2"/>
       <c r="P158" s="2"/>
-      <c r="Q158" s="2"/>
-    </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
@@ -13560,9 +13396,8 @@
       <c r="N159" s="2"/>
       <c r="O159" s="2"/>
       <c r="P159" s="2"/>
-      <c r="Q159" s="2"/>
-    </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
@@ -13579,9 +13414,8 @@
       <c r="N160" s="2"/>
       <c r="O160" s="2"/>
       <c r="P160" s="2"/>
-      <c r="Q160" s="2"/>
-    </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="161" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
@@ -13598,9 +13432,8 @@
       <c r="N161" s="2"/>
       <c r="O161" s="2"/>
       <c r="P161" s="2"/>
-      <c r="Q161" s="2"/>
-    </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="162" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
@@ -13617,9 +13450,8 @@
       <c r="N162" s="2"/>
       <c r="O162" s="2"/>
       <c r="P162" s="2"/>
-      <c r="Q162" s="2"/>
-    </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="163" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
@@ -13636,9 +13468,8 @@
       <c r="N163" s="2"/>
       <c r="O163" s="2"/>
       <c r="P163" s="2"/>
-      <c r="Q163" s="2"/>
-    </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="164" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
@@ -13655,9 +13486,8 @@
       <c r="N164" s="2"/>
       <c r="O164" s="2"/>
       <c r="P164" s="2"/>
-      <c r="Q164" s="2"/>
-    </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="165" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
@@ -13674,9 +13504,8 @@
       <c r="N165" s="2"/>
       <c r="O165" s="2"/>
       <c r="P165" s="2"/>
-      <c r="Q165" s="2"/>
-    </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="166" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
@@ -13693,9 +13522,8 @@
       <c r="N166" s="2"/>
       <c r="O166" s="2"/>
       <c r="P166" s="2"/>
-      <c r="Q166" s="2"/>
-    </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="167" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A167" s="2"/>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
@@ -13712,9 +13540,8 @@
       <c r="N167" s="2"/>
       <c r="O167" s="2"/>
       <c r="P167" s="2"/>
-      <c r="Q167" s="2"/>
-    </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="168" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A168" s="2"/>
       <c r="B168" s="2"/>
       <c r="C168" s="2"/>
@@ -13731,9 +13558,8 @@
       <c r="N168" s="2"/>
       <c r="O168" s="2"/>
       <c r="P168" s="2"/>
-      <c r="Q168" s="2"/>
-    </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="169" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
@@ -13750,9 +13576,8 @@
       <c r="N169" s="2"/>
       <c r="O169" s="2"/>
       <c r="P169" s="2"/>
-      <c r="Q169" s="2"/>
-    </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A170" s="2"/>
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
@@ -13769,9 +13594,8 @@
       <c r="N170" s="2"/>
       <c r="O170" s="2"/>
       <c r="P170" s="2"/>
-      <c r="Q170" s="2"/>
-    </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="171" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
@@ -13788,9 +13612,8 @@
       <c r="N171" s="2"/>
       <c r="O171" s="2"/>
       <c r="P171" s="2"/>
-      <c r="Q171" s="2"/>
-    </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="172" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A172" s="2"/>
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
@@ -13807,9 +13630,8 @@
       <c r="N172" s="2"/>
       <c r="O172" s="2"/>
       <c r="P172" s="2"/>
-      <c r="Q172" s="2"/>
-    </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="173" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A173" s="2"/>
       <c r="B173" s="2"/>
       <c r="C173" s="2"/>
@@ -13826,9 +13648,8 @@
       <c r="N173" s="2"/>
       <c r="O173" s="2"/>
       <c r="P173" s="2"/>
-      <c r="Q173" s="2"/>
-    </row>
-    <row r="174" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="174" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A174" s="2"/>
       <c r="B174" s="2"/>
       <c r="C174" s="2"/>
@@ -13845,9 +13666,8 @@
       <c r="N174" s="2"/>
       <c r="O174" s="2"/>
       <c r="P174" s="2"/>
-      <c r="Q174" s="2"/>
-    </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="175" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A175" s="2"/>
       <c r="B175" s="2"/>
       <c r="C175" s="2"/>
@@ -13864,9 +13684,8 @@
       <c r="N175" s="2"/>
       <c r="O175" s="2"/>
       <c r="P175" s="2"/>
-      <c r="Q175" s="2"/>
-    </row>
-    <row r="176" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="176" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A176" s="2"/>
       <c r="B176" s="2"/>
       <c r="C176" s="2"/>
@@ -13883,9 +13702,8 @@
       <c r="N176" s="2"/>
       <c r="O176" s="2"/>
       <c r="P176" s="2"/>
-      <c r="Q176" s="2"/>
-    </row>
-    <row r="177" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A177" s="2"/>
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
@@ -13902,9 +13720,8 @@
       <c r="N177" s="2"/>
       <c r="O177" s="2"/>
       <c r="P177" s="2"/>
-      <c r="Q177" s="2"/>
-    </row>
-    <row r="178" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A178" s="2"/>
       <c r="B178" s="2"/>
       <c r="C178" s="2"/>
@@ -13921,9 +13738,8 @@
       <c r="N178" s="2"/>
       <c r="O178" s="2"/>
       <c r="P178" s="2"/>
-      <c r="Q178" s="2"/>
-    </row>
-    <row r="179" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A179" s="2"/>
       <c r="B179" s="2"/>
       <c r="C179" s="2"/>
@@ -13940,9 +13756,8 @@
       <c r="N179" s="2"/>
       <c r="O179" s="2"/>
       <c r="P179" s="2"/>
-      <c r="Q179" s="2"/>
-    </row>
-    <row r="180" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A180" s="2"/>
       <c r="B180" s="2"/>
       <c r="C180" s="2"/>
@@ -13959,9 +13774,8 @@
       <c r="N180" s="2"/>
       <c r="O180" s="2"/>
       <c r="P180" s="2"/>
-      <c r="Q180" s="2"/>
-    </row>
-    <row r="181" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A181" s="2"/>
       <c r="B181" s="2"/>
       <c r="C181" s="2"/>
@@ -13978,9 +13792,8 @@
       <c r="N181" s="2"/>
       <c r="O181" s="2"/>
       <c r="P181" s="2"/>
-      <c r="Q181" s="2"/>
-    </row>
-    <row r="182" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A182" s="2"/>
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
@@ -13997,9 +13810,8 @@
       <c r="N182" s="2"/>
       <c r="O182" s="2"/>
       <c r="P182" s="2"/>
-      <c r="Q182" s="2"/>
-    </row>
-    <row r="183" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A183" s="2"/>
       <c r="B183" s="2"/>
       <c r="C183" s="2"/>
@@ -14016,9 +13828,8 @@
       <c r="N183" s="2"/>
       <c r="O183" s="2"/>
       <c r="P183" s="2"/>
-      <c r="Q183" s="2"/>
-    </row>
-    <row r="184" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A184" s="2"/>
       <c r="B184" s="2"/>
       <c r="C184" s="2"/>
@@ -14035,9 +13846,8 @@
       <c r="N184" s="2"/>
       <c r="O184" s="2"/>
       <c r="P184" s="2"/>
-      <c r="Q184" s="2"/>
-    </row>
-    <row r="185" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A185" s="2"/>
       <c r="B185" s="2"/>
       <c r="C185" s="2"/>
@@ -14054,9 +13864,8 @@
       <c r="N185" s="2"/>
       <c r="O185" s="2"/>
       <c r="P185" s="2"/>
-      <c r="Q185" s="2"/>
-    </row>
-    <row r="186" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A186" s="2"/>
       <c r="B186" s="2"/>
       <c r="C186" s="2"/>
@@ -14073,9 +13882,8 @@
       <c r="N186" s="2"/>
       <c r="O186" s="2"/>
       <c r="P186" s="2"/>
-      <c r="Q186" s="2"/>
-    </row>
-    <row r="187" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="2"/>
@@ -14092,9 +13900,8 @@
       <c r="N187" s="2"/>
       <c r="O187" s="2"/>
       <c r="P187" s="2"/>
-      <c r="Q187" s="2"/>
-    </row>
-    <row r="188" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A188" s="2"/>
       <c r="B188" s="2"/>
       <c r="C188" s="2"/>
@@ -14111,9 +13918,8 @@
       <c r="N188" s="2"/>
       <c r="O188" s="2"/>
       <c r="P188" s="2"/>
-      <c r="Q188" s="2"/>
-    </row>
-    <row r="189" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
       <c r="C189" s="2"/>
@@ -14130,9 +13936,8 @@
       <c r="N189" s="2"/>
       <c r="O189" s="2"/>
       <c r="P189" s="2"/>
-      <c r="Q189" s="2"/>
-    </row>
-    <row r="190" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A190" s="2"/>
       <c r="B190" s="2"/>
       <c r="C190" s="2"/>
@@ -14149,9 +13954,8 @@
       <c r="N190" s="2"/>
       <c r="O190" s="2"/>
       <c r="P190" s="2"/>
-      <c r="Q190" s="2"/>
-    </row>
-    <row r="191" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A191" s="2"/>
       <c r="B191" s="2"/>
       <c r="C191" s="2"/>
@@ -14168,9 +13972,8 @@
       <c r="N191" s="2"/>
       <c r="O191" s="2"/>
       <c r="P191" s="2"/>
-      <c r="Q191" s="2"/>
-    </row>
-    <row r="192" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A192" s="2"/>
       <c r="B192" s="2"/>
       <c r="C192" s="2"/>
@@ -14187,9 +13990,8 @@
       <c r="N192" s="2"/>
       <c r="O192" s="2"/>
       <c r="P192" s="2"/>
-      <c r="Q192" s="2"/>
-    </row>
-    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
       <c r="C193" s="2"/>
@@ -14206,9 +14008,8 @@
       <c r="N193" s="2"/>
       <c r="O193" s="2"/>
       <c r="P193" s="2"/>
-      <c r="Q193" s="2"/>
-    </row>
-    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A194" s="2"/>
       <c r="B194" s="2"/>
       <c r="C194" s="2"/>
@@ -14225,9 +14026,8 @@
       <c r="N194" s="2"/>
       <c r="O194" s="2"/>
       <c r="P194" s="2"/>
-      <c r="Q194" s="2"/>
-    </row>
-    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A195" s="2"/>
       <c r="B195" s="2"/>
       <c r="C195" s="2"/>
@@ -14244,9 +14044,8 @@
       <c r="N195" s="2"/>
       <c r="O195" s="2"/>
       <c r="P195" s="2"/>
-      <c r="Q195" s="2"/>
-    </row>
-    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A196" s="2"/>
       <c r="B196" s="2"/>
       <c r="C196" s="2"/>
@@ -14263,9 +14062,8 @@
       <c r="N196" s="2"/>
       <c r="O196" s="2"/>
       <c r="P196" s="2"/>
-      <c r="Q196" s="2"/>
-    </row>
-    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A197" s="2"/>
       <c r="B197" s="2"/>
       <c r="C197" s="2"/>
@@ -14282,9 +14080,8 @@
       <c r="N197" s="2"/>
       <c r="O197" s="2"/>
       <c r="P197" s="2"/>
-      <c r="Q197" s="2"/>
-    </row>
-    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="198" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A198" s="2"/>
       <c r="B198" s="2"/>
       <c r="C198" s="2"/>
@@ -14301,9 +14098,8 @@
       <c r="N198" s="2"/>
       <c r="O198" s="2"/>
       <c r="P198" s="2"/>
-      <c r="Q198" s="2"/>
-    </row>
-    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A199" s="2"/>
       <c r="B199" s="2"/>
       <c r="C199" s="2"/>
@@ -14320,9 +14116,8 @@
       <c r="N199" s="2"/>
       <c r="O199" s="2"/>
       <c r="P199" s="2"/>
-      <c r="Q199" s="2"/>
-    </row>
-    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A200" s="2"/>
       <c r="B200" s="2"/>
       <c r="C200" s="2"/>
@@ -14339,9 +14134,8 @@
       <c r="N200" s="2"/>
       <c r="O200" s="2"/>
       <c r="P200" s="2"/>
-      <c r="Q200" s="2"/>
-    </row>
-    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="201" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A201" s="2"/>
       <c r="B201" s="2"/>
       <c r="C201" s="2"/>
@@ -14358,9 +14152,8 @@
       <c r="N201" s="2"/>
       <c r="O201" s="2"/>
       <c r="P201" s="2"/>
-      <c r="Q201" s="2"/>
-    </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="202" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A202" s="2"/>
       <c r="B202" s="2"/>
       <c r="C202" s="2"/>
@@ -14377,9 +14170,8 @@
       <c r="N202" s="2"/>
       <c r="O202" s="2"/>
       <c r="P202" s="2"/>
-      <c r="Q202" s="2"/>
-    </row>
-    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="203" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A203" s="2"/>
       <c r="B203" s="2"/>
       <c r="C203" s="2"/>
@@ -14396,9 +14188,8 @@
       <c r="N203" s="2"/>
       <c r="O203" s="2"/>
       <c r="P203" s="2"/>
-      <c r="Q203" s="2"/>
-    </row>
-    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="204" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A204" s="2"/>
       <c r="B204" s="2"/>
       <c r="C204" s="2"/>
@@ -14415,33 +14206,31 @@
       <c r="N204" s="2"/>
       <c r="O204" s="2"/>
       <c r="P204" s="2"/>
-      <c r="Q204" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="6+yDI0OgPd4WYm3G6Z5geZ6OVSItsmzuI6pvXBhnqIBLkRwqZYhw/9myNYQcHogXrON+p0Vn9Al4arNGxWcvhQ==" saltValue="yoKDrVsoZTsh8FbYtsclwg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
-  <mergeCells count="14">
+  <sheetProtection algorithmName="SHA-512" hashValue="PoLs1kxIM/xJUmr7urrblsJ/5hObRoOum4QkrLl5n6UkTskAAW1rlDkj4UAOAaNPAxaZOLfva1Eeyyy3ErcvXg==" saltValue="hHLCZEhHQHH5LRknKlGm2A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <mergeCells count="13">
+    <mergeCell ref="P2:P4"/>
+    <mergeCell ref="O2:O4"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I2:I4"/>
+    <mergeCell ref="J2:M3"/>
+    <mergeCell ref="N2:N4"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="C2:E2"/>
-    <mergeCell ref="Q2:Q4"/>
-    <mergeCell ref="O2:O4"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="P2:P4"/>
-    <mergeCell ref="I2:I4"/>
-    <mergeCell ref="J2:M3"/>
-    <mergeCell ref="N2:N4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I4 M4 J4 K4 L4 Q2:Q4" xr:uid="{2FBCC481-6114-481E-B036-95624C9F7883}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I4 M4 J4 K4 L4 P2:P4" xr:uid="{2FBCC481-6114-481E-B036-95624C9F7883}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="Q2:Q4" r:id="rId1" location="samplingProtocols" display="SAMPLING_PROTOCOL_CODE" xr:uid="{C0C4727C-9767-4664-8796-43CDF0860627}"/>
+    <hyperlink ref="P2:P4" r:id="rId1" location="samplingProtocols" display="SAMPLING_PROTOCOL_CODE" xr:uid="{C0C4727C-9767-4664-8796-43CDF0860627}"/>
     <hyperlink ref="I2:I4" r:id="rId2" location="offalManagementTypes" display="OFFAL_MANAGEMENT" xr:uid="{408DFBD1-078D-43D4-8B22-538A09E39B98}"/>
     <hyperlink ref="J4" r:id="rId3" location="vesselSections" xr:uid="{140540DF-7251-4F70-BF34-280C13EE47A9}"/>
     <hyperlink ref="K4" r:id="rId4" location="vesselSections" xr:uid="{C6B0B34F-D5B5-4396-BD53-32117C4E0387}"/>
@@ -15763,7 +15552,7 @@
         <v>203</v>
       </c>
       <c r="H2" s="88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I2" s="115" t="s">
         <v>59</v>
@@ -15804,7 +15593,7 @@
         <v>60</v>
       </c>
       <c r="K4" s="50" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:11" s="55" customFormat="1" x14ac:dyDescent="0.25">
@@ -18514,10 +18303,10 @@
       <c r="D2" s="140" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="96" t="s">
+      <c r="E2" s="100" t="s">
         <v>202</v>
       </c>
-      <c r="F2" s="96" t="s">
+      <c r="F2" s="100" t="s">
         <v>203</v>
       </c>
       <c r="G2" s="88" t="s">
@@ -18526,18 +18315,18 @@
       <c r="H2" s="88"/>
       <c r="I2" s="88"/>
       <c r="J2" s="88"/>
-      <c r="K2" s="105" t="s">
+      <c r="K2" s="99" t="s">
         <v>208</v>
       </c>
-      <c r="L2" s="105"/>
-      <c r="M2" s="105"/>
-      <c r="N2" s="105"/>
-      <c r="O2" s="105" t="s">
+      <c r="L2" s="99"/>
+      <c r="M2" s="99"/>
+      <c r="N2" s="99"/>
+      <c r="O2" s="99" t="s">
         <v>59</v>
       </c>
-      <c r="P2" s="105"/>
-      <c r="Q2" s="105"/>
-      <c r="R2" s="111" t="s">
+      <c r="P2" s="99"/>
+      <c r="Q2" s="99"/>
+      <c r="R2" s="96" t="s">
         <v>62</v>
       </c>
       <c r="S2" s="90" t="s">
@@ -18549,18 +18338,18 @@
       </c>
       <c r="V2" s="91"/>
       <c r="W2" s="94"/>
-      <c r="X2" s="105" t="s">
+      <c r="X2" s="99" t="s">
         <v>210</v>
       </c>
-      <c r="Y2" s="105"/>
+      <c r="Y2" s="99"/>
     </row>
     <row r="3" spans="1:25" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="141"/>
       <c r="B3" s="141"/>
       <c r="C3" s="141"/>
       <c r="D3" s="141"/>
-      <c r="E3" s="97"/>
-      <c r="F3" s="97"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
       <c r="G3" s="56" t="s">
         <v>23</v>
       </c>
@@ -18592,9 +18381,9 @@
         <v>60</v>
       </c>
       <c r="Q3" s="50" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
-      <c r="R3" s="113"/>
+      <c r="R3" s="98"/>
       <c r="S3" s="43" t="s">
         <v>102</v>
       </c>
@@ -24121,16 +23910,16 @@
       <c r="D2" s="140" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="96" t="s">
+      <c r="E2" s="100" t="s">
         <v>193</v>
       </c>
-      <c r="F2" s="96" t="s">
+      <c r="F2" s="100" t="s">
         <v>194</v>
       </c>
-      <c r="G2" s="96" t="s">
+      <c r="G2" s="100" t="s">
         <v>195</v>
       </c>
-      <c r="H2" s="112" t="s">
+      <c r="H2" s="97" t="s">
         <v>196</v>
       </c>
       <c r="I2" s="86" t="s">
@@ -24141,7 +23930,7 @@
         <v>73</v>
       </c>
       <c r="L2" s="85"/>
-      <c r="M2" s="112" t="s">
+      <c r="M2" s="97" t="s">
         <v>201</v>
       </c>
       <c r="N2" s="142" t="s">
@@ -24150,7 +23939,7 @@
       <c r="O2" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="P2" s="112" t="s">
+      <c r="P2" s="97" t="s">
         <v>200</v>
       </c>
       <c r="Q2" s="142" t="s">
@@ -24169,10 +23958,10 @@
       <c r="B3" s="141"/>
       <c r="C3" s="141"/>
       <c r="D3" s="141"/>
-      <c r="E3" s="97"/>
-      <c r="F3" s="97"/>
-      <c r="G3" s="97"/>
-      <c r="H3" s="113"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="98"/>
       <c r="I3" s="50" t="s">
         <v>197</v>
       </c>
@@ -24185,10 +23974,10 @@
       <c r="L3" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="M3" s="113"/>
+      <c r="M3" s="98"/>
       <c r="N3" s="89"/>
       <c r="O3" s="89"/>
-      <c r="P3" s="113"/>
+      <c r="P3" s="98"/>
       <c r="Q3" s="89"/>
       <c r="R3" s="89"/>
       <c r="S3" s="50" t="s">
@@ -28601,6 +28390,16 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="owrGYnA0RoV/U9MjDeglShzyfAHibWrOJ91U+dfsJvx7FpXhtP7KXYqD/XawmrJ8WUgOAZj9nC2wQr9dD2KQZw==" saltValue="h+hFQsEVq78bir+WDv8nRA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="S2:T2"/>
     <mergeCell ref="H2:H3"/>
@@ -28608,16 +28407,6 @@
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="K2:L2"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F3 H2:H3 P2:P3 S3 J3 E2:E3 G2:G3 I3 M2:M3 T3" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -31359,7 +31148,7 @@
   <sheetData>
     <row r="1" spans="1:25" s="7" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="61" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B1" s="62"/>
       <c r="C1" s="62"/>
@@ -31406,7 +31195,7 @@
       <c r="L2" s="89"/>
       <c r="M2" s="89"/>
       <c r="N2" s="80" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="O2" s="81"/>
       <c r="P2" s="81"/>
@@ -31478,18 +31267,18 @@
         <v>98</v>
       </c>
       <c r="N4" s="78" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="O4" s="78"/>
       <c r="P4" s="79" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="Q4" s="79"/>
       <c r="R4" s="79"/>
       <c r="S4" s="79"/>
       <c r="T4" s="79"/>
       <c r="U4" s="79" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="V4" s="79"/>
       <c r="W4" s="79"/>
@@ -36826,80 +36615,80 @@
       <c r="A2" s="88" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="102" t="s">
-        <v>241</v>
+      <c r="B2" s="106" t="s">
+        <v>240</v>
       </c>
-      <c r="C2" s="103"/>
-      <c r="D2" s="103"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="103"/>
-      <c r="H2" s="103"/>
-      <c r="I2" s="103"/>
-      <c r="J2" s="103"/>
-      <c r="K2" s="103"/>
-      <c r="L2" s="103"/>
-      <c r="M2" s="103"/>
-      <c r="N2" s="103"/>
-      <c r="O2" s="103"/>
-      <c r="P2" s="104"/>
+      <c r="C2" s="107"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
+      <c r="H2" s="107"/>
+      <c r="I2" s="107"/>
+      <c r="J2" s="107"/>
+      <c r="K2" s="107"/>
+      <c r="L2" s="107"/>
+      <c r="M2" s="107"/>
+      <c r="N2" s="107"/>
+      <c r="O2" s="107"/>
+      <c r="P2" s="108"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="88"/>
-      <c r="B3" s="102" t="s">
+      <c r="B3" s="106" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="103"/>
-      <c r="D3" s="103"/>
-      <c r="E3" s="103"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="98" t="s">
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="102" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="99"/>
-      <c r="I3" s="100"/>
-      <c r="J3" s="111" t="s">
+      <c r="H3" s="103"/>
+      <c r="I3" s="104"/>
+      <c r="J3" s="96" t="s">
         <v>17</v>
       </c>
       <c r="K3" s="52" t="s">
         <v>108</v>
       </c>
-      <c r="L3" s="102" t="s">
+      <c r="L3" s="106" t="s">
         <v>128</v>
       </c>
-      <c r="M3" s="103"/>
-      <c r="N3" s="103"/>
-      <c r="O3" s="103"/>
-      <c r="P3" s="104"/>
+      <c r="M3" s="107"/>
+      <c r="N3" s="107"/>
+      <c r="O3" s="107"/>
+      <c r="P3" s="108"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="88"/>
       <c r="B4" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="109" t="s">
+      <c r="C4" s="112" t="s">
         <v>139</v>
       </c>
-      <c r="D4" s="110" t="s">
+      <c r="D4" s="113" t="s">
         <v>2</v>
       </c>
       <c r="E4" s="95" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="105" t="s">
+      <c r="F4" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="106" t="s">
+      <c r="G4" s="109" t="s">
         <v>134</v>
       </c>
-      <c r="H4" s="107" t="s">
+      <c r="H4" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="101" t="s">
+      <c r="I4" s="105" t="s">
         <v>177</v>
       </c>
-      <c r="J4" s="112"/>
-      <c r="K4" s="96" t="s">
+      <c r="J4" s="97"/>
+      <c r="K4" s="100" t="s">
         <v>141</v>
       </c>
       <c r="L4" s="78" t="s">
@@ -36910,35 +36699,35 @@
         <v>19</v>
       </c>
       <c r="O4" s="78"/>
-      <c r="P4" s="105" t="s">
+      <c r="P4" s="99" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="88"/>
-      <c r="C5" s="109"/>
-      <c r="D5" s="110"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="113"/>
       <c r="E5" s="89"/>
-      <c r="F5" s="105"/>
-      <c r="G5" s="106"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="101"/>
-      <c r="J5" s="113"/>
-      <c r="K5" s="97"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="109"/>
+      <c r="H5" s="111"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="98"/>
+      <c r="K5" s="101"/>
       <c r="L5" s="39" t="s">
         <v>3</v>
       </c>
       <c r="M5" s="56" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="N5" s="39" t="s">
         <v>3</v>
       </c>
       <c r="O5" s="56" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
-      <c r="P5" s="105"/>
+      <c r="P5" s="99"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -40543,11 +40332,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="9TADddINtH3/s8+B+YSEyrbqN3sXm6gNvmsaihCGVKf7Pla3vF7K/W63Z2DPtXhM7gpZzMQTmkRfISjjfsW2DA==" saltValue="PE4zbTBOxopTV3TBfcOFrw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="18">
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="I4:I5"/>
     <mergeCell ref="L3:P3"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="N4:O4"/>
@@ -40561,6 +40345,11 @@
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="B2:P2"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="I4:I5"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M5 J6 K4:K5 G4:I5 O5" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40621,20 +40410,20 @@
       <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="B2" s="99" t="s">
+        <v>232</v>
+      </c>
+      <c r="C2" s="99"/>
+      <c r="D2" s="99"/>
+      <c r="E2" s="99"/>
+      <c r="F2" s="99"/>
+      <c r="G2" s="99" t="s">
         <v>233</v>
       </c>
-      <c r="C2" s="105"/>
-      <c r="D2" s="105"/>
-      <c r="E2" s="105"/>
-      <c r="F2" s="105"/>
-      <c r="G2" s="105" t="s">
-        <v>234</v>
-      </c>
-      <c r="H2" s="105"/>
-      <c r="I2" s="105"/>
-      <c r="J2" s="105"/>
-      <c r="K2" s="105"/>
+      <c r="H2" s="99"/>
+      <c r="I2" s="99"/>
+      <c r="J2" s="99"/>
+      <c r="K2" s="99"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
@@ -43408,29 +43197,29 @@
       <c r="A2" s="88" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="B2" s="99" t="s">
         <v>190</v>
       </c>
-      <c r="C2" s="105"/>
-      <c r="D2" s="105"/>
-      <c r="E2" s="105"/>
-      <c r="F2" s="105"/>
-      <c r="G2" s="105"/>
-      <c r="H2" s="105"/>
-      <c r="I2" s="105"/>
-      <c r="J2" s="105"/>
-      <c r="K2" s="105"/>
-      <c r="L2" s="105"/>
-      <c r="M2" s="105"/>
-      <c r="N2" s="105"/>
-      <c r="O2" s="105"/>
-      <c r="P2" s="105"/>
-      <c r="Q2" s="105"/>
-      <c r="R2" s="105"/>
-      <c r="S2" s="105"/>
-      <c r="T2" s="105"/>
+      <c r="C2" s="99"/>
+      <c r="D2" s="99"/>
+      <c r="E2" s="99"/>
+      <c r="F2" s="99"/>
+      <c r="G2" s="99"/>
+      <c r="H2" s="99"/>
+      <c r="I2" s="99"/>
+      <c r="J2" s="99"/>
+      <c r="K2" s="99"/>
+      <c r="L2" s="99"/>
+      <c r="M2" s="99"/>
+      <c r="N2" s="99"/>
+      <c r="O2" s="99"/>
+      <c r="P2" s="99"/>
+      <c r="Q2" s="99"/>
+      <c r="R2" s="99"/>
+      <c r="S2" s="99"/>
+      <c r="T2" s="99"/>
       <c r="U2" s="115" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="V2" s="116"/>
       <c r="W2" s="116"/>
@@ -43445,7 +43234,7 @@
       <c r="AF2" s="116"/>
       <c r="AG2" s="117"/>
       <c r="AH2" s="115" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AI2" s="116"/>
       <c r="AJ2" s="116"/>
@@ -43457,25 +43246,25 @@
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A3" s="88"/>
-      <c r="B3" s="105"/>
-      <c r="C3" s="105"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="105"/>
-      <c r="F3" s="105"/>
-      <c r="G3" s="105"/>
-      <c r="H3" s="105"/>
-      <c r="I3" s="105"/>
-      <c r="J3" s="105"/>
-      <c r="K3" s="105"/>
-      <c r="L3" s="105"/>
-      <c r="M3" s="105"/>
-      <c r="N3" s="105"/>
-      <c r="O3" s="105"/>
-      <c r="P3" s="105"/>
-      <c r="Q3" s="105"/>
-      <c r="R3" s="105"/>
-      <c r="S3" s="105"/>
-      <c r="T3" s="105"/>
+      <c r="B3" s="99"/>
+      <c r="C3" s="99"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="99"/>
+      <c r="F3" s="99"/>
+      <c r="G3" s="99"/>
+      <c r="H3" s="99"/>
+      <c r="I3" s="99"/>
+      <c r="J3" s="99"/>
+      <c r="K3" s="99"/>
+      <c r="L3" s="99"/>
+      <c r="M3" s="99"/>
+      <c r="N3" s="99"/>
+      <c r="O3" s="99"/>
+      <c r="P3" s="99"/>
+      <c r="Q3" s="99"/>
+      <c r="R3" s="99"/>
+      <c r="S3" s="99"/>
+      <c r="T3" s="99"/>
       <c r="U3" s="86"/>
       <c r="V3" s="118"/>
       <c r="W3" s="118"/>
@@ -43506,7 +43295,7 @@
       <c r="C4" s="95" t="s">
         <v>144</v>
       </c>
-      <c r="D4" s="111" t="s">
+      <c r="D4" s="96" t="s">
         <v>145</v>
       </c>
       <c r="E4" s="79" t="s">
@@ -43537,59 +43326,59 @@
         <v>28</v>
       </c>
       <c r="T4" s="79"/>
-      <c r="U4" s="105" t="s">
+      <c r="U4" s="99" t="s">
         <v>155</v>
       </c>
-      <c r="V4" s="105" t="s">
+      <c r="V4" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="W4" s="105" t="s">
+      <c r="W4" s="99" t="s">
         <v>40</v>
       </c>
-      <c r="X4" s="105" t="s">
+      <c r="X4" s="99" t="s">
         <v>31</v>
       </c>
-      <c r="Y4" s="105" t="s">
+      <c r="Y4" s="99" t="s">
         <v>32</v>
       </c>
-      <c r="Z4" s="105" t="s">
+      <c r="Z4" s="99" t="s">
         <v>33</v>
       </c>
-      <c r="AA4" s="105" t="s">
+      <c r="AA4" s="99" t="s">
         <v>34</v>
       </c>
-      <c r="AB4" s="105" t="s">
+      <c r="AB4" s="99" t="s">
         <v>35</v>
       </c>
-      <c r="AC4" s="105" t="s">
+      <c r="AC4" s="99" t="s">
         <v>36</v>
       </c>
-      <c r="AD4" s="105" t="s">
+      <c r="AD4" s="99" t="s">
         <v>37</v>
       </c>
-      <c r="AE4" s="105" t="s">
+      <c r="AE4" s="99" t="s">
         <v>38</v>
       </c>
-      <c r="AF4" s="105" t="s">
+      <c r="AF4" s="99" t="s">
         <v>147</v>
       </c>
-      <c r="AG4" s="105" t="s">
+      <c r="AG4" s="99" t="s">
         <v>39</v>
       </c>
-      <c r="AH4" s="98" t="s">
+      <c r="AH4" s="102" t="s">
+        <v>236</v>
+      </c>
+      <c r="AI4" s="104"/>
+      <c r="AJ4" s="79" t="s">
         <v>237</v>
-      </c>
-      <c r="AI4" s="100"/>
-      <c r="AJ4" s="79" t="s">
-        <v>238</v>
       </c>
       <c r="AK4" s="79"/>
       <c r="AL4" s="79" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AM4" s="79"/>
       <c r="AN4" s="79" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AO4" s="79"/>
     </row>
@@ -43597,7 +43386,7 @@
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
-      <c r="D5" s="113"/>
+      <c r="D5" s="98"/>
       <c r="E5" s="41" t="s">
         <v>25</v>
       </c>
@@ -43644,19 +43433,19 @@
       <c r="T5" s="44" t="s">
         <v>148</v>
       </c>
-      <c r="U5" s="105"/>
-      <c r="V5" s="105"/>
-      <c r="W5" s="105"/>
-      <c r="X5" s="105"/>
-      <c r="Y5" s="105"/>
-      <c r="Z5" s="105"/>
-      <c r="AA5" s="105"/>
-      <c r="AB5" s="105"/>
-      <c r="AC5" s="105"/>
-      <c r="AD5" s="105"/>
-      <c r="AE5" s="105"/>
-      <c r="AF5" s="105"/>
-      <c r="AG5" s="105"/>
+      <c r="U5" s="99"/>
+      <c r="V5" s="99"/>
+      <c r="W5" s="99"/>
+      <c r="X5" s="99"/>
+      <c r="Y5" s="99"/>
+      <c r="Z5" s="99"/>
+      <c r="AA5" s="99"/>
+      <c r="AB5" s="99"/>
+      <c r="AC5" s="99"/>
+      <c r="AD5" s="99"/>
+      <c r="AE5" s="99"/>
+      <c r="AF5" s="99"/>
+      <c r="AG5" s="99"/>
       <c r="AH5" s="38" t="s">
         <v>156</v>
       </c>
@@ -52285,20 +52074,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="NiKKXtjpQMePcsqc5jjUDaSQ7PwYr9+sjfqfZD87x0KbSUAFE8Baue/7fXFs4bMxVWpKhzgpmVEg8+jmkTDZbw==" saltValue="/cWUcVxNNlNaEWVwXWfzkw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="U2:AG3"/>
-    <mergeCell ref="AB4:AB5"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="P4:R4"/>
-    <mergeCell ref="B2:T3"/>
-    <mergeCell ref="U4:U5"/>
-    <mergeCell ref="V4:V5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AH2:AO3"/>
     <mergeCell ref="D4:D5"/>
@@ -52315,6 +52090,20 @@
     <mergeCell ref="AG4:AG5"/>
     <mergeCell ref="L4:O4"/>
     <mergeCell ref="AL4:AM4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="U2:AG3"/>
+    <mergeCell ref="AB4:AB5"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="B2:T3"/>
+    <mergeCell ref="U4:U5"/>
+    <mergeCell ref="V4:V5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:D5 R5 AI5 AK5 AM5 L5 M5 N5 O5 P5 Q5 AO5 AJ5 AL5 AN5 AH5" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -53650,15 +53439,15 @@
       <c r="A2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="B2" s="99" t="s">
+        <v>224</v>
+      </c>
+      <c r="C2" s="99"/>
+      <c r="D2" s="99"/>
+      <c r="E2" s="99"/>
+      <c r="F2" s="99"/>
+      <c r="G2" s="90" t="s">
         <v>225</v>
-      </c>
-      <c r="C2" s="105"/>
-      <c r="D2" s="105"/>
-      <c r="E2" s="105"/>
-      <c r="F2" s="105"/>
-      <c r="G2" s="90" t="s">
-        <v>226</v>
       </c>
       <c r="H2" s="91"/>
       <c r="I2" s="91"/>
@@ -53672,22 +53461,22 @@
       <c r="C3" s="95" t="s">
         <v>165</v>
       </c>
-      <c r="D3" s="106" t="s">
+      <c r="D3" s="109" t="s">
         <v>166</v>
       </c>
-      <c r="E3" s="105" t="s">
+      <c r="E3" s="99" t="s">
         <v>171</v>
       </c>
       <c r="F3" s="117" t="s">
         <v>172</v>
       </c>
-      <c r="G3" s="111" t="s">
+      <c r="G3" s="96" t="s">
         <v>167</v>
       </c>
-      <c r="H3" s="111" t="s">
+      <c r="H3" s="96" t="s">
         <v>168</v>
       </c>
-      <c r="I3" s="111" t="s">
+      <c r="I3" s="96" t="s">
         <v>169</v>
       </c>
       <c r="J3" s="121" t="s">
@@ -53698,12 +53487,12 @@
       <c r="A4" s="77"/>
       <c r="B4" s="89"/>
       <c r="C4" s="89"/>
-      <c r="D4" s="106"/>
-      <c r="E4" s="105"/>
+      <c r="D4" s="109"/>
+      <c r="E4" s="99"/>
       <c r="F4" s="87"/>
-      <c r="G4" s="113"/>
-      <c r="H4" s="113"/>
-      <c r="I4" s="113"/>
+      <c r="G4" s="98"/>
+      <c r="H4" s="98"/>
+      <c r="I4" s="98"/>
       <c r="J4" s="122"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -56109,11 +55898,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="rbaELUtMLiFIUzK2Lo99z9d9U/+7pUd8ywEap5Et9u8xKeEcXwzK/YHzlDzNf0b31XcPQzpRtM0zLEm0RaQL/w==" saltValue="qBVdEFs3JSBOU1K55aehjA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="12">
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="G2:J2"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
@@ -56121,6 +55905,11 @@
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="G2:J2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D4 G3 H3 I3 J3" xr:uid="{17D462F2-8B43-4EF8-AF0E-D9F26228FDD4}">
@@ -56195,7 +55984,7 @@
       <c r="J2" s="125"/>
       <c r="K2" s="120"/>
       <c r="L2" s="115" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="M2" s="116"/>
       <c r="N2" s="116"/>
@@ -56221,7 +56010,7 @@
         <v>182</v>
       </c>
       <c r="J3" s="123" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="K3" s="124"/>
       <c r="L3" s="86"/>
@@ -59990,10 +59779,10 @@
       <c r="G2" s="125"/>
       <c r="H2" s="120"/>
       <c r="I2" s="114" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J2" s="114" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="K2" s="115" t="s">
         <v>43</v>
@@ -60005,32 +59794,32 @@
       </c>
       <c r="O2" s="117"/>
       <c r="P2" s="88" t="s">
+        <v>261</v>
+      </c>
+      <c r="Q2" s="99" t="s">
         <v>262</v>
       </c>
-      <c r="Q2" s="105" t="s">
+      <c r="R2" s="88" t="s">
         <v>263</v>
       </c>
-      <c r="R2" s="88" t="s">
-        <v>264</v>
-      </c>
       <c r="S2" s="88" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="T2" s="88"/>
       <c r="U2" s="133" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="V2" s="134"/>
       <c r="W2" s="133" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="X2" s="134"/>
       <c r="Y2" s="133" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="Z2" s="134"/>
       <c r="AA2" s="88" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="AB2" s="88"/>
       <c r="AC2" s="88"/>
@@ -60061,7 +59850,7 @@
       <c r="N3" s="86"/>
       <c r="O3" s="87"/>
       <c r="P3" s="88"/>
-      <c r="Q3" s="105"/>
+      <c r="Q3" s="99"/>
       <c r="R3" s="88"/>
       <c r="S3" s="88"/>
       <c r="T3" s="88"/>
@@ -60099,10 +59888,10 @@
         <v>212</v>
       </c>
       <c r="L4" s="42" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="M4" s="59" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="N4" s="42" t="s">
         <v>48</v>
@@ -60111,13 +59900,13 @@
         <v>49</v>
       </c>
       <c r="P4" s="88"/>
-      <c r="Q4" s="105"/>
+      <c r="Q4" s="99"/>
       <c r="R4" s="88"/>
       <c r="S4" s="39" t="s">
         <v>51</v>
       </c>
       <c r="T4" s="42" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="U4" s="39" t="s">
         <v>23</v>
@@ -60138,16 +59927,16 @@
         <v>148</v>
       </c>
       <c r="AA4" s="56" t="s">
+        <v>265</v>
+      </c>
+      <c r="AB4" s="50" t="s">
         <v>266</v>
       </c>
-      <c r="AB4" s="50" t="s">
+      <c r="AC4" s="50" t="s">
         <v>267</v>
       </c>
-      <c r="AC4" s="50" t="s">
+      <c r="AD4" s="50" t="s">
         <v>268</v>
-      </c>
-      <c r="AD4" s="50" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.25">
@@ -66525,6 +66314,10 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="Npdc6hR1jWNwlUd78HFJSJlOVnyVZEkwE3li2w9MaNYbr3qpWORdGSkVHRoIs6ZmqiHg7fNUc25lo9m1DLSPvg==" saltValue="CpsBwfeTpFYKyUOX8eB08w==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="C2:E2"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="Y2:Z3"/>
@@ -66541,10 +66334,6 @@
     <mergeCell ref="N2:O3"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="C2:E2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 AA4:AD4" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">

</xml_diff>

<commit_message>
Further improvements to longline form and description. This will never end
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE237DD-1B0B-44E3-951A-85282E8A3179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F68486-8307-4B9B-8B70-28C6DC801163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="272">
   <si>
     <t>LATITUDE</t>
   </si>
@@ -127,9 +127,6 @@
   </si>
   <si>
     <t>TYPE</t>
-  </si>
-  <si>
-    <t>TYPE_CODE</t>
   </si>
   <si>
     <t>MAKE</t>
@@ -253,12 +250,6 @@
   </si>
   <si>
     <t>RECOVERY</t>
-  </si>
-  <si>
-    <t>TAG_NUMBER_1</t>
-  </si>
-  <si>
-    <t>TAG_NUMBER_2</t>
   </si>
   <si>
     <t>DIAMETER_MM</t>
@@ -813,9 +804,6 @@
     <t>MINIMUM_DECK_LIGHTING_USED</t>
   </si>
   <si>
-    <t>AVERAGE_BRANCHLINE_WEIGHT_G</t>
-  </si>
-  <si>
     <t>NATIONALITY</t>
   </si>
   <si>
@@ -849,9 +837,6 @@
     <t>NUMBER_HOOKS_BETWEEN_FLOATS</t>
   </si>
   <si>
-    <t>NUMBER_LINES</t>
-  </si>
-  <si>
     <t>SPECIES_1</t>
   </si>
   <si>
@@ -877,6 +862,15 @@
   </si>
   <si>
     <t>BRANCHLINE LENGTH MAXIMUM</t>
+  </si>
+  <si>
+    <t>AVERAGE_SINKER_WEIGHT_G</t>
+  </si>
+  <si>
+    <t>TAG_ID_1</t>
+  </si>
+  <si>
+    <t>TAG_ID_2</t>
   </si>
 </sst>
 </file>
@@ -1450,7 +1444,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1545,29 +1539,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1590,6 +1561,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1608,6 +1582,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2037,7 +2031,7 @@
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="66" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C2" s="67"/>
       <c r="D2" s="67"/>
@@ -2058,14 +2052,14 @@
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="12"/>
       <c r="C4" s="13" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G4" s="16">
         <v>1</v>
@@ -2084,7 +2078,7 @@
     <row r="6" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B6" s="18"/>
       <c r="C6" s="21" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="19"/>
@@ -2104,12 +2098,12 @@
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="18"/>
       <c r="C8" s="72" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D8" s="72"/>
       <c r="E8" s="19"/>
       <c r="F8" s="72" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G8" s="72"/>
       <c r="H8" s="20"/>
@@ -2117,12 +2111,12 @@
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="18"/>
       <c r="C9" s="22" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D9" s="23"/>
       <c r="E9" s="19"/>
       <c r="F9" s="22" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G9" s="23"/>
       <c r="H9" s="20"/>
@@ -2130,12 +2124,12 @@
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="18"/>
       <c r="C10" s="24" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D10" s="23"/>
       <c r="E10" s="19"/>
       <c r="F10" s="19" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G10" s="23"/>
       <c r="H10" s="20"/>
@@ -2152,7 +2146,7 @@
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="18"/>
       <c r="C12" s="24" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D12" s="26"/>
       <c r="E12" s="19"/>
@@ -2163,7 +2157,7 @@
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="18"/>
       <c r="C13" s="24" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D13" s="26"/>
       <c r="E13" s="19"/>
@@ -2192,7 +2186,7 @@
     <row r="16" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B16" s="18"/>
       <c r="C16" s="21" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D16" s="19"/>
       <c r="E16" s="19"/>
@@ -2212,7 +2206,7 @@
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="18"/>
       <c r="C18" s="24" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="19"/>
@@ -2223,7 +2217,7 @@
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="18"/>
       <c r="C19" s="29" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D19" s="28"/>
       <c r="E19" s="19"/>
@@ -2234,7 +2228,7 @@
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="18"/>
       <c r="C20" s="36" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D20" s="28"/>
       <c r="E20" s="19"/>
@@ -2245,7 +2239,7 @@
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="18"/>
       <c r="C21" s="24" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D21" s="28"/>
       <c r="E21" s="19"/>
@@ -2274,7 +2268,7 @@
     <row r="24" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B24" s="18"/>
       <c r="C24" s="21" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D24" s="25"/>
       <c r="E24" s="19"/>
@@ -2352,7 +2346,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -2361,19 +2355,19 @@
     </row>
     <row r="2" spans="1:5" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C2" s="56" t="s">
         <v>23</v>
       </c>
       <c r="D2" s="56" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E2" s="60" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="55" customFormat="1" x14ac:dyDescent="0.25">
@@ -3814,7 +3808,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -3833,38 +3827,38 @@
     </row>
     <row r="2" spans="1:15" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="114" t="s">
-        <v>110</v>
-      </c>
       <c r="C2" s="114" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D2" s="114" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E2" s="95" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="114" t="s">
+        <v>269</v>
+      </c>
+      <c r="G2" s="114" t="s">
+        <v>246</v>
+      </c>
+      <c r="H2" s="114" t="s">
         <v>55</v>
       </c>
-      <c r="F2" s="114" t="s">
-        <v>252</v>
-      </c>
-      <c r="G2" s="114" t="s">
-        <v>249</v>
-      </c>
-      <c r="H2" s="114" t="s">
-        <v>56</v>
-      </c>
       <c r="I2" s="114" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="J2" s="90" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="K2" s="94"/>
       <c r="L2" s="119" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="M2" s="125"/>
       <c r="N2" s="125"/>
@@ -3881,22 +3875,22 @@
       <c r="H3" s="77"/>
       <c r="I3" s="77"/>
       <c r="J3" s="42" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L3" s="56" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="M3" s="56" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="N3" s="56" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="O3" s="56" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -7299,7 +7293,7 @@
       <c r="O203" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="ZHZ61xEMWo2GozKFDfIGwtbJZnm3eVYJpvIE2b76e/O5EaOFEu4qUPnEZ+3+QLMo4fMOZjuAZJWBGppNj6h0fg==" saltValue="p7UsgbvwfBAQ3S2mqNofIA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="i54u068XThYDfxhseUVm7j5UOX6o6sLA/paOyFGBfnG2ueK1l9vp0KVJDHX+jDagofUZDK+i4w0EkGdmr+cm5A==" saltValue="YMFvCB9MnqWRAENMsMJcZw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
@@ -7345,7 +7339,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -7354,13 +7348,13 @@
     </row>
     <row r="2" spans="1:5" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="114" t="s">
-        <v>110</v>
-      </c>
       <c r="C2" s="119" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D2" s="125"/>
       <c r="E2" s="120"/>
@@ -7372,10 +7366,10 @@
         <v>23</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E3" s="42" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -8810,7 +8804,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -8820,13 +8814,13 @@
     </row>
     <row r="2" spans="1:6" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="114" t="s">
-        <v>110</v>
-      </c>
       <c r="C2" s="119" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D2" s="125"/>
       <c r="E2" s="125"/>
@@ -8836,16 +8830,16 @@
       <c r="A3" s="77"/>
       <c r="B3" s="77"/>
       <c r="C3" s="56" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E3" s="39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F3" s="42" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -10493,7 +10487,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -10513,62 +10507,62 @@
     </row>
     <row r="2" spans="1:16" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="114" t="s">
-        <v>110</v>
-      </c>
       <c r="C2" s="119" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D2" s="125"/>
       <c r="E2" s="120"/>
       <c r="F2" s="119" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G2" s="125"/>
       <c r="H2" s="120"/>
-      <c r="I2" s="109" t="s">
+      <c r="I2" s="104" t="s">
+        <v>56</v>
+      </c>
+      <c r="J2" s="103" t="s">
+        <v>211</v>
+      </c>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="88" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="99" t="s">
-        <v>214</v>
-      </c>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="88" t="s">
-        <v>58</v>
-      </c>
       <c r="O2" s="88" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="P2" s="135" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:16" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
       <c r="B3" s="76"/>
       <c r="C3" s="114" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D3" s="119" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E3" s="120"/>
       <c r="F3" s="114" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="G3" s="119" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H3" s="120"/>
-      <c r="I3" s="109"/>
-      <c r="J3" s="99"/>
-      <c r="K3" s="99"/>
-      <c r="L3" s="99"/>
-      <c r="M3" s="99"/>
+      <c r="I3" s="104"/>
+      <c r="J3" s="103"/>
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
       <c r="N3" s="88"/>
       <c r="O3" s="88"/>
       <c r="P3" s="135"/>
@@ -10590,18 +10584,18 @@
       <c r="H4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="109"/>
+      <c r="I4" s="104"/>
       <c r="J4" s="50" t="s">
+        <v>210</v>
+      </c>
+      <c r="K4" s="50" t="s">
+        <v>212</v>
+      </c>
+      <c r="L4" s="50" t="s">
         <v>213</v>
       </c>
-      <c r="K4" s="50" t="s">
-        <v>215</v>
-      </c>
-      <c r="L4" s="50" t="s">
-        <v>216</v>
-      </c>
       <c r="M4" s="50" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="N4" s="88"/>
       <c r="O4" s="88"/>
@@ -14257,7 +14251,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -14265,13 +14259,13 @@
     </row>
     <row r="2" spans="1:4" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="114" t="s">
-        <v>110</v>
-      </c>
       <c r="C2" s="90" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D2" s="94"/>
     </row>
@@ -14279,10 +14273,10 @@
       <c r="A3" s="77"/>
       <c r="B3" s="77"/>
       <c r="C3" s="42" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -15518,7 +15512,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -15533,29 +15527,29 @@
     </row>
     <row r="2" spans="1:11" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="114" t="s">
-        <v>110</v>
-      </c>
       <c r="C2" s="114" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D2" s="135" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E2" s="136" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F2" s="137"/>
       <c r="G2" s="135" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H2" s="88" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I2" s="115" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J2" s="116"/>
       <c r="K2" s="117"/>
@@ -15582,18 +15576,18 @@
         <v>23</v>
       </c>
       <c r="F4" s="56" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G4" s="135"/>
       <c r="H4" s="88"/>
       <c r="I4" s="50" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="J4" s="42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K4" s="50" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:11" s="55" customFormat="1" x14ac:dyDescent="0.25">
@@ -18263,7 +18257,7 @@
   <sheetData>
     <row r="1" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -18292,118 +18286,118 @@
     </row>
     <row r="2" spans="1:25" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="140" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="140" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="140" t="s">
+      <c r="C2" s="140" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="140" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="140" t="s">
-        <v>112</v>
+      <c r="E2" s="112" t="s">
+        <v>199</v>
       </c>
-      <c r="D2" s="140" t="s">
-        <v>113</v>
-      </c>
-      <c r="E2" s="100" t="s">
-        <v>202</v>
-      </c>
-      <c r="F2" s="100" t="s">
-        <v>203</v>
+      <c r="F2" s="112" t="s">
+        <v>200</v>
       </c>
       <c r="G2" s="88" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="H2" s="88"/>
       <c r="I2" s="88"/>
       <c r="J2" s="88"/>
-      <c r="K2" s="99" t="s">
-        <v>208</v>
+      <c r="K2" s="103" t="s">
+        <v>205</v>
       </c>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="99"/>
-      <c r="O2" s="99" t="s">
-        <v>59</v>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="103" t="s">
+        <v>58</v>
       </c>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="99"/>
-      <c r="R2" s="96" t="s">
-        <v>62</v>
+      <c r="P2" s="103"/>
+      <c r="Q2" s="103"/>
+      <c r="R2" s="109" t="s">
+        <v>61</v>
       </c>
       <c r="S2" s="90" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="T2" s="94"/>
       <c r="U2" s="90" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="V2" s="91"/>
       <c r="W2" s="94"/>
-      <c r="X2" s="99" t="s">
-        <v>210</v>
+      <c r="X2" s="103" t="s">
+        <v>207</v>
       </c>
-      <c r="Y2" s="99"/>
+      <c r="Y2" s="103"/>
     </row>
     <row r="3" spans="1:25" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="141"/>
       <c r="B3" s="141"/>
       <c r="C3" s="141"/>
       <c r="D3" s="141"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
+      <c r="E3" s="113"/>
+      <c r="F3" s="113"/>
       <c r="G3" s="56" t="s">
         <v>23</v>
       </c>
       <c r="H3" s="39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I3" s="56" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="J3" s="39" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="K3" s="50" t="s">
         <v>23</v>
       </c>
       <c r="L3" s="42" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M3" s="50" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="N3" s="42" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="O3" s="50" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="P3" s="42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="Q3" s="50" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
-      <c r="R3" s="98"/>
+      <c r="R3" s="111"/>
       <c r="S3" s="43" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="T3" s="43" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="U3" s="59" t="s">
         <v>23</v>
       </c>
       <c r="V3" s="42" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="W3" s="42" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="X3" s="50" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="Y3" s="50" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:25" s="55" customFormat="1" x14ac:dyDescent="0.25">
@@ -23807,7 +23801,7 @@
       <c r="Y203" s="9"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="e/mZipJ4AXPmTDIqBREzT6xE/UbCF4PciHFB1N4ngnHGkbhMYq2UP1EcRbtVoIsbMk/soeRGswyOaMGay/157g==" saltValue="feKRClgbT3qIjWu79ykSJg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="i+NWJhJ/dANY4y8V6yR0b2FD2rG8VYPEOJeWH5E9k/YJLZu+zWXk6/2fi7RZql3z8q9ENi+0H/lJGiOCaKLA2g==" saltValue="hNILL3j2lqXU8lRHPxsxbw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="13">
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
@@ -23875,7 +23869,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -23899,57 +23893,57 @@
     </row>
     <row r="2" spans="1:20" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="140" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="140" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="140" t="s">
+      <c r="C2" s="140" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="140" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="140" t="s">
-        <v>112</v>
+      <c r="E2" s="112" t="s">
+        <v>190</v>
       </c>
-      <c r="D2" s="140" t="s">
-        <v>113</v>
+      <c r="F2" s="112" t="s">
+        <v>191</v>
       </c>
-      <c r="E2" s="100" t="s">
+      <c r="G2" s="112" t="s">
+        <v>192</v>
+      </c>
+      <c r="H2" s="110" t="s">
         <v>193</v>
       </c>
-      <c r="F2" s="100" t="s">
-        <v>194</v>
-      </c>
-      <c r="G2" s="100" t="s">
-        <v>195</v>
-      </c>
-      <c r="H2" s="97" t="s">
-        <v>196</v>
-      </c>
       <c r="I2" s="86" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="J2" s="87"/>
       <c r="K2" s="83" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="L2" s="85"/>
-      <c r="M2" s="97" t="s">
-        <v>201</v>
+      <c r="M2" s="110" t="s">
+        <v>198</v>
       </c>
       <c r="N2" s="142" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="O2" s="142" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
-      <c r="P2" s="97" t="s">
-        <v>200</v>
+      <c r="P2" s="110" t="s">
+        <v>197</v>
       </c>
       <c r="Q2" s="142" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="R2" s="142" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="S2" s="89" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="T2" s="89"/>
     </row>
@@ -23958,33 +23952,33 @@
       <c r="B3" s="141"/>
       <c r="C3" s="141"/>
       <c r="D3" s="141"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="98"/>
+      <c r="E3" s="113"/>
+      <c r="F3" s="113"/>
+      <c r="G3" s="113"/>
+      <c r="H3" s="111"/>
       <c r="I3" s="50" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="J3" s="50" t="s">
         <v>23</v>
       </c>
       <c r="K3" s="56" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="L3" s="42" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
-      <c r="M3" s="98"/>
+      <c r="M3" s="111"/>
       <c r="N3" s="89"/>
       <c r="O3" s="89"/>
-      <c r="P3" s="98"/>
+      <c r="P3" s="111"/>
       <c r="Q3" s="89"/>
       <c r="R3" s="89"/>
       <c r="S3" s="50" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="T3" s="50" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="55" customFormat="1" x14ac:dyDescent="0.25">
@@ -28450,7 +28444,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -28465,37 +28459,37 @@
     </row>
     <row r="2" spans="1:11" s="53" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="65" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="65" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="65" t="s">
+      <c r="C2" s="65" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="65" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="65" t="s">
-        <v>112</v>
+      <c r="E2" s="42" t="s">
+        <v>63</v>
       </c>
-      <c r="D2" s="65" t="s">
-        <v>113</v>
-      </c>
-      <c r="E2" s="42" t="s">
+      <c r="F2" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="F2" s="42" t="s">
-        <v>65</v>
-      </c>
       <c r="G2" s="50" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H2" s="42" t="s">
-        <v>66</v>
+        <v>270</v>
       </c>
       <c r="I2" s="42" t="s">
-        <v>67</v>
+        <v>271</v>
       </c>
       <c r="J2" s="42" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K2" s="42" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:11" s="53" customFormat="1" x14ac:dyDescent="0.25">
@@ -31099,14 +31093,14 @@
       <c r="K202" s="9"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="qOApQt+f2TsOI5aABva9oFhDaMC8tY6SmLrXY5zZMla4EE44P/H2PtJCJ3eAXXCegs0uTPk+51WoRp//Mv+vlg==" saltValue="LQGXhg9x1P3A7pPeXXmcRw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="PSeRJ1qUwmkn/r+zZDXNQ6Dr0J7lATaoNihkurJ9p93KMKe4NwkwW4CfN9Klss8IHE2M6laOf+tSvLGiZISszQ==" saltValue="L+SeJSUOmI8CoOgPWC3lYQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{4FDCD393-A02F-41DC-AAE5-5D41DD47867C}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" location="tagTypes" xr:uid="{ECAFC5F2-6FEB-4806-8763-D5FABB0EB5EB}"/>
+    <hyperlink ref="G2" r:id="rId1" location="tagTypes" display="TYPE_CODE" xr:uid="{ECAFC5F2-6FEB-4806-8763-D5FABB0EB5EB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -31148,7 +31142,7 @@
   <sheetData>
     <row r="1" spans="1:25" s="7" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="61" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B1" s="62"/>
       <c r="C1" s="62"/>
@@ -31176,14 +31170,14 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="76" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B2" s="77" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C2" s="77"/>
       <c r="D2" s="89" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="E2" s="89"/>
       <c r="F2" s="89"/>
@@ -31195,7 +31189,7 @@
       <c r="L2" s="89"/>
       <c r="M2" s="89"/>
       <c r="N2" s="80" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="O2" s="81"/>
       <c r="P2" s="81"/>
@@ -31214,14 +31208,14 @@
       <c r="B3" s="88"/>
       <c r="C3" s="88"/>
       <c r="D3" s="90" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E3" s="91"/>
       <c r="F3" s="91"/>
       <c r="G3" s="91"/>
       <c r="H3" s="94"/>
       <c r="I3" s="90" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="J3" s="91"/>
       <c r="K3" s="91"/>
@@ -31245,40 +31239,40 @@
       <c r="B4" s="88"/>
       <c r="C4" s="88"/>
       <c r="D4" s="86" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E4" s="87"/>
       <c r="F4" s="86" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G4" s="87"/>
       <c r="H4" s="95" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="I4" s="86" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="J4" s="87"/>
       <c r="K4" s="86" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L4" s="87"/>
       <c r="M4" s="92" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="N4" s="78" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="O4" s="78"/>
       <c r="P4" s="79" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="Q4" s="79"/>
       <c r="R4" s="79"/>
       <c r="S4" s="79"/>
       <c r="T4" s="79"/>
       <c r="U4" s="79" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="V4" s="79"/>
       <c r="W4" s="79"/>
@@ -31287,13 +31281,13 @@
     <row r="5" spans="1:25" s="54" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="77"/>
       <c r="B5" s="39" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>3</v>
       </c>
       <c r="D5" s="50" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E5" s="50" t="s">
         <v>4</v>
@@ -31306,7 +31300,7 @@
       </c>
       <c r="H5" s="89"/>
       <c r="I5" s="50" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="J5" s="50" t="s">
         <v>4</v>
@@ -31340,16 +31334,16 @@
         <v>10</v>
       </c>
       <c r="U5" s="38" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="V5" s="38" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="W5" s="38" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="X5" s="38" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -36593,7 +36587,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -36613,83 +36607,83 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="88" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
-      <c r="B2" s="106" t="s">
-        <v>240</v>
+      <c r="B2" s="100" t="s">
+        <v>237</v>
       </c>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
-      <c r="M2" s="107"/>
-      <c r="N2" s="107"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="108"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="101"/>
+      <c r="H2" s="101"/>
+      <c r="I2" s="101"/>
+      <c r="J2" s="101"/>
+      <c r="K2" s="101"/>
+      <c r="L2" s="101"/>
+      <c r="M2" s="101"/>
+      <c r="N2" s="101"/>
+      <c r="O2" s="101"/>
+      <c r="P2" s="102"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="88"/>
-      <c r="B3" s="106" t="s">
+      <c r="B3" s="100" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="107"/>
-      <c r="D3" s="107"/>
-      <c r="E3" s="107"/>
-      <c r="F3" s="108"/>
-      <c r="G3" s="102" t="s">
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="103"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="96" t="s">
+      <c r="H3" s="97"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="109" t="s">
         <v>17</v>
       </c>
       <c r="K3" s="52" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
-      <c r="L3" s="106" t="s">
-        <v>128</v>
+      <c r="L3" s="100" t="s">
+        <v>125</v>
       </c>
-      <c r="M3" s="107"/>
-      <c r="N3" s="107"/>
-      <c r="O3" s="107"/>
-      <c r="P3" s="108"/>
+      <c r="M3" s="101"/>
+      <c r="N3" s="101"/>
+      <c r="O3" s="101"/>
+      <c r="P3" s="102"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="88"/>
       <c r="B4" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="112" t="s">
-        <v>139</v>
+      <c r="C4" s="107" t="s">
+        <v>136</v>
       </c>
-      <c r="D4" s="113" t="s">
+      <c r="D4" s="108" t="s">
         <v>2</v>
       </c>
       <c r="E4" s="95" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="99" t="s">
+      <c r="F4" s="103" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="109" t="s">
-        <v>134</v>
+      <c r="G4" s="104" t="s">
+        <v>131</v>
       </c>
-      <c r="H4" s="110" t="s">
+      <c r="H4" s="105" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="105" t="s">
-        <v>177</v>
+      <c r="I4" s="99" t="s">
+        <v>174</v>
       </c>
-      <c r="J4" s="97"/>
-      <c r="K4" s="100" t="s">
-        <v>141</v>
+      <c r="J4" s="110"/>
+      <c r="K4" s="112" t="s">
+        <v>138</v>
       </c>
       <c r="L4" s="78" t="s">
         <v>18</v>
@@ -36699,35 +36693,35 @@
         <v>19</v>
       </c>
       <c r="O4" s="78"/>
-      <c r="P4" s="99" t="s">
+      <c r="P4" s="103" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="88"/>
-      <c r="C5" s="112"/>
-      <c r="D5" s="113"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
       <c r="E5" s="89"/>
-      <c r="F5" s="99"/>
-      <c r="G5" s="109"/>
-      <c r="H5" s="111"/>
-      <c r="I5" s="105"/>
-      <c r="J5" s="98"/>
-      <c r="K5" s="101"/>
+      <c r="F5" s="103"/>
+      <c r="G5" s="104"/>
+      <c r="H5" s="106"/>
+      <c r="I5" s="99"/>
+      <c r="J5" s="111"/>
+      <c r="K5" s="113"/>
       <c r="L5" s="39" t="s">
         <v>3</v>
       </c>
       <c r="M5" s="56" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="N5" s="39" t="s">
         <v>3</v>
       </c>
       <c r="O5" s="56" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
-      <c r="P5" s="99"/>
+      <c r="P5" s="103"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -40332,6 +40326,10 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="9TADddINtH3/s8+B+YSEyrbqN3sXm6gNvmsaihCGVKf7Pla3vF7K/W63Z2DPtXhM7gpZzMQTmkRfISjjfsW2DA==" saltValue="PE4zbTBOxopTV3TBfcOFrw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="18">
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="I4:I5"/>
     <mergeCell ref="L3:P3"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="N4:O4"/>
@@ -40346,10 +40344,6 @@
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="B2:P2"/>
     <mergeCell ref="J3:J5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="I4:I5"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M5 J6 K4:K5 G4:I5 O5" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40393,7 +40387,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -40408,22 +40402,22 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
-      <c r="B2" s="99" t="s">
-        <v>232</v>
+      <c r="B2" s="103" t="s">
+        <v>229</v>
       </c>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99" t="s">
-        <v>233</v>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103" t="s">
+        <v>230</v>
       </c>
-      <c r="H2" s="99"/>
-      <c r="I2" s="99"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
@@ -40434,7 +40428,7 @@
       <c r="D3" s="91"/>
       <c r="E3" s="91"/>
       <c r="F3" s="95" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="G3" s="90" t="s">
         <v>4</v>
@@ -40443,13 +40437,13 @@
       <c r="I3" s="91"/>
       <c r="J3" s="94"/>
       <c r="K3" s="95" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="77"/>
       <c r="B4" s="50" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C4" s="50" t="s">
         <v>4</v>
@@ -40462,7 +40456,7 @@
       </c>
       <c r="F4" s="89"/>
       <c r="G4" s="50" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H4" s="50" t="s">
         <v>4</v>
@@ -43150,7 +43144,7 @@
   <sheetData>
     <row r="1" spans="1:41" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -43195,31 +43189,31 @@
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A2" s="88" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
-      <c r="B2" s="99" t="s">
-        <v>190</v>
+      <c r="B2" s="103" t="s">
+        <v>187</v>
       </c>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99"/>
-      <c r="H2" s="99"/>
-      <c r="I2" s="99"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="99"/>
-      <c r="O2" s="99"/>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="99"/>
-      <c r="R2" s="99"/>
-      <c r="S2" s="99"/>
-      <c r="T2" s="99"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="103"/>
+      <c r="P2" s="103"/>
+      <c r="Q2" s="103"/>
+      <c r="R2" s="103"/>
+      <c r="S2" s="103"/>
+      <c r="T2" s="103"/>
       <c r="U2" s="115" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="V2" s="116"/>
       <c r="W2" s="116"/>
@@ -43234,7 +43228,7 @@
       <c r="AF2" s="116"/>
       <c r="AG2" s="117"/>
       <c r="AH2" s="115" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="AI2" s="116"/>
       <c r="AJ2" s="116"/>
@@ -43246,25 +43240,25 @@
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A3" s="88"/>
-      <c r="B3" s="99"/>
-      <c r="C3" s="99"/>
-      <c r="D3" s="99"/>
-      <c r="E3" s="99"/>
-      <c r="F3" s="99"/>
-      <c r="G3" s="99"/>
-      <c r="H3" s="99"/>
-      <c r="I3" s="99"/>
-      <c r="J3" s="99"/>
-      <c r="K3" s="99"/>
-      <c r="L3" s="99"/>
-      <c r="M3" s="99"/>
-      <c r="N3" s="99"/>
-      <c r="O3" s="99"/>
-      <c r="P3" s="99"/>
-      <c r="Q3" s="99"/>
-      <c r="R3" s="99"/>
-      <c r="S3" s="99"/>
-      <c r="T3" s="99"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="I3" s="103"/>
+      <c r="J3" s="103"/>
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
+      <c r="N3" s="103"/>
+      <c r="O3" s="103"/>
+      <c r="P3" s="103"/>
+      <c r="Q3" s="103"/>
+      <c r="R3" s="103"/>
+      <c r="S3" s="103"/>
+      <c r="T3" s="103"/>
       <c r="U3" s="86"/>
       <c r="V3" s="118"/>
       <c r="W3" s="118"/>
@@ -43290,95 +43284,95 @@
     <row r="4" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A4" s="88"/>
       <c r="B4" s="95" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C4" s="95" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
-      <c r="D4" s="96" t="s">
-        <v>145</v>
+      <c r="D4" s="109" t="s">
+        <v>142</v>
       </c>
       <c r="E4" s="79" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F4" s="79"/>
       <c r="G4" s="79"/>
       <c r="H4" s="79" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="I4" s="79"/>
       <c r="J4" s="79"/>
       <c r="K4" s="95" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="L4" s="79" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M4" s="79"/>
       <c r="N4" s="79"/>
       <c r="O4" s="79"/>
       <c r="P4" s="79" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q4" s="79"/>
       <c r="R4" s="79"/>
       <c r="S4" s="79" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T4" s="79"/>
-      <c r="U4" s="99" t="s">
-        <v>155</v>
+      <c r="U4" s="103" t="s">
+        <v>152</v>
       </c>
-      <c r="V4" s="99" t="s">
+      <c r="V4" s="103" t="s">
+        <v>29</v>
+      </c>
+      <c r="W4" s="103" t="s">
+        <v>39</v>
+      </c>
+      <c r="X4" s="103" t="s">
         <v>30</v>
       </c>
-      <c r="W4" s="99" t="s">
-        <v>40</v>
-      </c>
-      <c r="X4" s="99" t="s">
+      <c r="Y4" s="103" t="s">
         <v>31</v>
       </c>
-      <c r="Y4" s="99" t="s">
+      <c r="Z4" s="103" t="s">
         <v>32</v>
       </c>
-      <c r="Z4" s="99" t="s">
+      <c r="AA4" s="103" t="s">
         <v>33</v>
       </c>
-      <c r="AA4" s="99" t="s">
+      <c r="AB4" s="103" t="s">
         <v>34</v>
       </c>
-      <c r="AB4" s="99" t="s">
+      <c r="AC4" s="103" t="s">
         <v>35</v>
       </c>
-      <c r="AC4" s="99" t="s">
+      <c r="AD4" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="AD4" s="99" t="s">
+      <c r="AE4" s="103" t="s">
         <v>37</v>
       </c>
-      <c r="AE4" s="99" t="s">
+      <c r="AF4" s="103" t="s">
+        <v>144</v>
+      </c>
+      <c r="AG4" s="103" t="s">
         <v>38</v>
       </c>
-      <c r="AF4" s="99" t="s">
-        <v>147</v>
+      <c r="AH4" s="96" t="s">
+        <v>233</v>
       </c>
-      <c r="AG4" s="99" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH4" s="102" t="s">
-        <v>236</v>
-      </c>
-      <c r="AI4" s="104"/>
+      <c r="AI4" s="98"/>
       <c r="AJ4" s="79" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="AK4" s="79"/>
       <c r="AL4" s="79" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="AM4" s="79"/>
       <c r="AN4" s="79" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="AO4" s="79"/>
     </row>
@@ -43386,89 +43380,89 @@
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
-      <c r="D5" s="98"/>
+      <c r="D5" s="111"/>
       <c r="E5" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="41" t="s">
-        <v>26</v>
-      </c>
       <c r="G5" s="44" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H5" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="41" t="s">
-        <v>26</v>
-      </c>
       <c r="J5" s="44" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="K5" s="89"/>
       <c r="L5" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="M5" s="38" t="s">
         <v>146</v>
       </c>
-      <c r="M5" s="38" t="s">
+      <c r="N5" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="O5" s="38" t="s">
+        <v>148</v>
+      </c>
+      <c r="P5" s="38" t="s">
         <v>149</v>
       </c>
-      <c r="N5" s="38" t="s">
+      <c r="Q5" s="38" t="s">
         <v>150</v>
       </c>
-      <c r="O5" s="38" t="s">
+      <c r="R5" s="38" t="s">
         <v>151</v>
-      </c>
-      <c r="P5" s="38" t="s">
-        <v>152</v>
-      </c>
-      <c r="Q5" s="38" t="s">
-        <v>153</v>
-      </c>
-      <c r="R5" s="38" t="s">
-        <v>154</v>
       </c>
       <c r="S5" s="41" t="s">
         <v>22</v>
       </c>
       <c r="T5" s="44" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
-      <c r="U5" s="99"/>
-      <c r="V5" s="99"/>
-      <c r="W5" s="99"/>
-      <c r="X5" s="99"/>
-      <c r="Y5" s="99"/>
-      <c r="Z5" s="99"/>
-      <c r="AA5" s="99"/>
-      <c r="AB5" s="99"/>
-      <c r="AC5" s="99"/>
-      <c r="AD5" s="99"/>
-      <c r="AE5" s="99"/>
-      <c r="AF5" s="99"/>
-      <c r="AG5" s="99"/>
+      <c r="U5" s="103"/>
+      <c r="V5" s="103"/>
+      <c r="W5" s="103"/>
+      <c r="X5" s="103"/>
+      <c r="Y5" s="103"/>
+      <c r="Z5" s="103"/>
+      <c r="AA5" s="103"/>
+      <c r="AB5" s="103"/>
+      <c r="AC5" s="103"/>
+      <c r="AD5" s="103"/>
+      <c r="AE5" s="103"/>
+      <c r="AF5" s="103"/>
+      <c r="AG5" s="103"/>
       <c r="AH5" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="AI5" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="AJ5" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="AK5" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="AI5" s="38" t="s">
+      <c r="AL5" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="AJ5" s="38" t="s">
+      <c r="AM5" s="38" t="s">
         <v>158</v>
       </c>
-      <c r="AK5" s="38" t="s">
+      <c r="AN5" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="AL5" s="38" t="s">
+      <c r="AO5" s="38" t="s">
         <v>160</v>
-      </c>
-      <c r="AM5" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="AN5" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="AO5" s="38" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.25">
@@ -52148,7 +52142,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="5"/>
@@ -52156,10 +52150,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="88" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B2" s="88" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C2" s="88"/>
       <c r="D2" s="88"/>
@@ -52167,13 +52161,13 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="119"/>
       <c r="B3" s="88" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C3" s="120" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D3" s="88" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -53423,7 +53417,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -53437,17 +53431,17 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
-      <c r="B2" s="99" t="s">
-        <v>224</v>
+      <c r="B2" s="103" t="s">
+        <v>221</v>
       </c>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
       <c r="G2" s="90" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="H2" s="91"/>
       <c r="I2" s="91"/>
@@ -53456,43 +53450,43 @@
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
       <c r="B3" s="95" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" s="95" t="s">
+        <v>162</v>
+      </c>
+      <c r="D3" s="104" t="s">
+        <v>163</v>
+      </c>
+      <c r="E3" s="103" t="s">
+        <v>168</v>
+      </c>
+      <c r="F3" s="117" t="s">
+        <v>169</v>
+      </c>
+      <c r="G3" s="109" t="s">
         <v>164</v>
       </c>
-      <c r="C3" s="95" t="s">
+      <c r="H3" s="109" t="s">
         <v>165</v>
       </c>
-      <c r="D3" s="109" t="s">
+      <c r="I3" s="109" t="s">
         <v>166</v>
       </c>
-      <c r="E3" s="99" t="s">
-        <v>171</v>
-      </c>
-      <c r="F3" s="117" t="s">
-        <v>172</v>
-      </c>
-      <c r="G3" s="96" t="s">
+      <c r="J3" s="121" t="s">
         <v>167</v>
-      </c>
-      <c r="H3" s="96" t="s">
-        <v>168</v>
-      </c>
-      <c r="I3" s="96" t="s">
-        <v>169</v>
-      </c>
-      <c r="J3" s="121" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="77"/>
       <c r="B4" s="89"/>
       <c r="C4" s="89"/>
-      <c r="D4" s="109"/>
-      <c r="E4" s="99"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="103"/>
       <c r="F4" s="87"/>
-      <c r="G4" s="98"/>
-      <c r="H4" s="98"/>
-      <c r="I4" s="98"/>
+      <c r="G4" s="111"/>
+      <c r="H4" s="111"/>
+      <c r="I4" s="111"/>
       <c r="J4" s="122"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -55949,7 +55943,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="11"/>
@@ -55969,10 +55963,10 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B2" s="119" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C2" s="125"/>
       <c r="D2" s="125"/>
@@ -55984,7 +55978,7 @@
       <c r="J2" s="125"/>
       <c r="K2" s="120"/>
       <c r="L2" s="115" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M2" s="116"/>
       <c r="N2" s="116"/>
@@ -55994,23 +55988,23 @@
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
       <c r="B3" s="126" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C3" s="130" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D3" s="131"/>
       <c r="E3" s="131"/>
       <c r="F3" s="131"/>
       <c r="G3" s="132"/>
       <c r="H3" s="128" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I3" s="126" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="J3" s="123" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="K3" s="124"/>
       <c r="L3" s="86"/>
@@ -56026,16 +56020,16 @@
         <v>23</v>
       </c>
       <c r="D4" s="46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E4" s="45" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F4" s="46" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G4" s="45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H4" s="129"/>
       <c r="I4" s="127"/>
@@ -56046,19 +56040,19 @@
         <v>15</v>
       </c>
       <c r="L4" s="49" t="s">
+        <v>180</v>
+      </c>
+      <c r="M4" s="40" t="s">
+        <v>182</v>
+      </c>
+      <c r="N4" s="40" t="s">
         <v>183</v>
       </c>
-      <c r="M4" s="40" t="s">
-        <v>185</v>
-      </c>
-      <c r="N4" s="40" t="s">
-        <v>186</v>
-      </c>
       <c r="O4" s="40" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="P4" s="40" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -59729,7 +59723,7 @@
   <sheetData>
     <row r="1" spans="1:30" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -59763,63 +59757,63 @@
     </row>
     <row r="2" spans="1:30" s="55" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="114" t="s">
-        <v>110</v>
-      </c>
       <c r="C2" s="88" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D2" s="88"/>
       <c r="E2" s="88"/>
       <c r="F2" s="119" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G2" s="125"/>
       <c r="H2" s="120"/>
       <c r="I2" s="114" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="J2" s="114" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="K2" s="115" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L2" s="116"/>
       <c r="M2" s="117"/>
       <c r="N2" s="115" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O2" s="117"/>
       <c r="P2" s="88" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
-      <c r="Q2" s="99" t="s">
-        <v>262</v>
+      <c r="Q2" s="103" t="s">
+        <v>258</v>
       </c>
       <c r="R2" s="88" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="S2" s="88" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="T2" s="88"/>
       <c r="U2" s="133" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="V2" s="134"/>
       <c r="W2" s="133" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="X2" s="134"/>
       <c r="Y2" s="133" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="Z2" s="134"/>
       <c r="AA2" s="88" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="AB2" s="88"/>
       <c r="AC2" s="88"/>
@@ -59829,17 +59823,17 @@
       <c r="A3" s="76"/>
       <c r="B3" s="76"/>
       <c r="C3" s="80" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D3" s="119" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E3" s="120"/>
       <c r="F3" s="114" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="G3" s="119" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H3" s="120"/>
       <c r="I3" s="76"/>
@@ -59850,7 +59844,7 @@
       <c r="N3" s="86"/>
       <c r="O3" s="87"/>
       <c r="P3" s="88"/>
-      <c r="Q3" s="99"/>
+      <c r="Q3" s="103"/>
       <c r="R3" s="88"/>
       <c r="S3" s="88"/>
       <c r="T3" s="88"/>
@@ -59885,58 +59879,58 @@
       <c r="I4" s="77"/>
       <c r="J4" s="77"/>
       <c r="K4" s="50" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="L4" s="42" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="M4" s="59" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="N4" s="42" t="s">
+        <v>47</v>
+      </c>
+      <c r="O4" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="O4" s="42" t="s">
-        <v>49</v>
-      </c>
       <c r="P4" s="88"/>
-      <c r="Q4" s="99"/>
+      <c r="Q4" s="103"/>
       <c r="R4" s="88"/>
       <c r="S4" s="39" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="T4" s="42" t="s">
-        <v>264</v>
+        <v>15</v>
       </c>
       <c r="U4" s="39" t="s">
         <v>23</v>
       </c>
       <c r="V4" s="39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="W4" s="39" t="s">
         <v>22</v>
       </c>
       <c r="X4" s="39" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="Y4" s="39" t="s">
         <v>22</v>
       </c>
       <c r="Z4" s="39" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="AA4" s="56" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="AB4" s="50" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="AC4" s="50" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="AD4" s="50" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.25">
@@ -66312,12 +66306,8 @@
       <c r="B204" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="Npdc6hR1jWNwlUd78HFJSJlOVnyVZEkwE3li2w9MaNYbr3qpWORdGSkVHRoIs6ZmqiHg7fNUc25lo9m1DLSPvg==" saltValue="CpsBwfeTpFYKyUOX8eB08w==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="d21qlgp65jSu5W9pa5yJ5h6FXV3pmxRSPPtHFMi6kL/5Q045jK8F1FxQGWC8ChuBu/i/+ceDsCkP7hrPZBzfYg==" saltValue="OgP3geBPxDkKLe5cj3oUgQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="C2:E2"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="Y2:Z3"/>
@@ -66334,6 +66324,10 @@
     <mergeCell ref="N2:O3"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="C2:E2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 AA4:AD4" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">

</xml_diff>

<commit_message>
Some improvements to the forms and descriptions
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schirico\Repositories\iotc-reference-forms\form_reporting_templates\ros\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D85421-055F-455D-89D0-5E24FF03DF46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106F0932-A472-443F-9273-9E731CAEED6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="30030" yWindow="1245" windowWidth="26505" windowHeight="14100" tabRatio="879" firstSheet="11" activeTab="18" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" firstSheet="1" activeTab="1" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -1199,7 +1199,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="150">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
@@ -1342,6 +1342,17 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1435,6 +1446,24 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1465,9 +1494,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1487,19 +1513,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1512,15 +1532,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1542,93 +1553,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1639,6 +1563,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1978,24 +1911,24 @@
   <sheetData>
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="59" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="58"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="61"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="59"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="61"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="64"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="5"/>
@@ -2045,15 +1978,15 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="11"/>
-      <c r="C8" s="62" t="s">
+      <c r="C8" s="65" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="62"/>
+      <c r="D8" s="65"/>
       <c r="E8" s="12"/>
-      <c r="F8" s="62" t="s">
+      <c r="F8" s="65" t="s">
         <v>113</v>
       </c>
-      <c r="G8" s="62"/>
+      <c r="G8" s="65"/>
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2235,11 +2168,11 @@
     </row>
     <row r="26" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="11"/>
-      <c r="C26" s="63"/>
-      <c r="D26" s="64"/>
-      <c r="E26" s="64"/>
-      <c r="F26" s="64"/>
-      <c r="G26" s="65"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="67"/>
+      <c r="F26" s="67"/>
+      <c r="G26" s="68"/>
       <c r="H26" s="13"/>
     </row>
     <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3746,54 +3679,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="93" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="104" t="s">
+      <c r="C1" s="93" t="s">
         <v>228</v>
       </c>
-      <c r="D1" s="104" t="s">
+      <c r="D1" s="93" t="s">
         <v>229</v>
       </c>
-      <c r="E1" s="85" t="s">
+      <c r="E1" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="104" t="s">
+      <c r="F1" s="93" t="s">
         <v>250</v>
       </c>
-      <c r="G1" s="104" t="s">
+      <c r="G1" s="93" t="s">
         <v>227</v>
       </c>
-      <c r="H1" s="104" t="s">
+      <c r="H1" s="93" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="104" t="s">
+      <c r="I1" s="93" t="s">
         <v>93</v>
       </c>
-      <c r="J1" s="80" t="s">
+      <c r="J1" s="83" t="s">
         <v>221</v>
       </c>
-      <c r="K1" s="84"/>
-      <c r="L1" s="109" t="s">
+      <c r="K1" s="87"/>
+      <c r="L1" s="108" t="s">
         <v>222</v>
       </c>
-      <c r="M1" s="111"/>
-      <c r="N1" s="111"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
       <c r="O1" s="110"/>
     </row>
     <row r="2" spans="1:15" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
+      <c r="A2" s="70"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
       <c r="J2" s="35" t="s">
         <v>46</v>
       </c>
@@ -7215,17 +7148,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="i4Y2GDra9B4e5ZK9IT/yAgpGu83ed66ZNnyRoFvCqT5wVfLy2Lgs30SlszSGdCdYRpnULwm3Kg2BGFX0NXPahA==" saltValue="poZcuJUx5RFD549VWAk8zg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
+    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="E1:E2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="I1:I2"/>
-    <mergeCell ref="L1:O1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 M2 N2 O2" xr:uid="{35387E2C-FBDF-4B0A-A0B5-EF76A6744ABB}">
@@ -7258,21 +7191,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="93" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="109" t="s">
+      <c r="C1" s="108" t="s">
         <v>201</v>
       </c>
-      <c r="D1" s="111"/>
+      <c r="D1" s="109"/>
       <c r="E1" s="110"/>
     </row>
     <row r="2" spans="1:5" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67"/>
+      <c r="A2" s="70"/>
+      <c r="B2" s="70"/>
       <c r="C2" s="44" t="s">
         <v>23</v>
       </c>
@@ -8714,22 +8647,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="93" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="109" t="s">
+      <c r="C1" s="108" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
+      <c r="D1" s="109"/>
+      <c r="E1" s="109"/>
       <c r="F1" s="110"/>
     </row>
     <row r="2" spans="1:6" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67"/>
+      <c r="A2" s="70"/>
+      <c r="B2" s="70"/>
       <c r="C2" s="44" t="s">
         <v>178</v>
       </c>
@@ -10388,89 +10321,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="93" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="109" t="s">
+      <c r="C1" s="108" t="s">
         <v>207</v>
       </c>
-      <c r="D1" s="111"/>
+      <c r="D1" s="109"/>
       <c r="E1" s="110"/>
-      <c r="F1" s="109" t="s">
+      <c r="F1" s="108" t="s">
         <v>208</v>
       </c>
-      <c r="G1" s="111"/>
+      <c r="G1" s="109"/>
       <c r="H1" s="110"/>
-      <c r="I1" s="96" t="s">
+      <c r="I1" s="103" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="95" t="s">
+      <c r="J1" s="92" t="s">
         <v>195</v>
       </c>
-      <c r="K1" s="95"/>
-      <c r="L1" s="95"/>
-      <c r="M1" s="95"/>
-      <c r="N1" s="78" t="s">
+      <c r="K1" s="92"/>
+      <c r="L1" s="92"/>
+      <c r="M1" s="92"/>
+      <c r="N1" s="81" t="s">
         <v>57</v>
       </c>
-      <c r="O1" s="78" t="s">
+      <c r="O1" s="81" t="s">
         <v>200</v>
       </c>
-      <c r="P1" s="115" t="s">
+      <c r="P1" s="118" t="s">
         <v>253</v>
       </c>
-      <c r="Q1" s="114" t="s">
+      <c r="Q1" s="117" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="104" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="93" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="109" t="s">
+      <c r="D2" s="108" t="s">
         <v>79</v>
       </c>
       <c r="E2" s="110"/>
-      <c r="F2" s="104" t="s">
+      <c r="F2" s="93" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="109" t="s">
+      <c r="G2" s="108" t="s">
         <v>79</v>
       </c>
       <c r="H2" s="110"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="78"/>
-      <c r="O2" s="78"/>
-      <c r="P2" s="116"/>
-      <c r="Q2" s="114"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="92"/>
+      <c r="K2" s="92"/>
+      <c r="L2" s="92"/>
+      <c r="M2" s="92"/>
+      <c r="N2" s="81"/>
+      <c r="O2" s="81"/>
+      <c r="P2" s="119"/>
+      <c r="Q2" s="117"/>
     </row>
     <row r="3" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="67"/>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
+      <c r="A3" s="70"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
       <c r="D3" s="32" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="67"/>
+      <c r="F3" s="70"/>
       <c r="G3" s="32" t="s">
         <v>0</v>
       </c>
       <c r="H3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="96"/>
+      <c r="I3" s="103"/>
       <c r="J3" s="38" t="s">
         <v>194</v>
       </c>
@@ -10483,10 +10416,10 @@
       <c r="M3" s="38" t="s">
         <v>198</v>
       </c>
-      <c r="N3" s="78"/>
-      <c r="O3" s="78"/>
-      <c r="P3" s="117"/>
-      <c r="Q3" s="114"/>
+      <c r="N3" s="81"/>
+      <c r="O3" s="81"/>
+      <c r="P3" s="120"/>
+      <c r="Q3" s="117"/>
     </row>
     <row r="4" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -14291,6 +14224,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="j7MUMGPBrETWcazR2JxyYWg7EsALd6nWBPrG0+KpBwzqgUF6TIdENL/ZaQBEBI6zU+Z6UHRHz3zwzs6KvZx01A==" saltValue="H5P+A2rusa74O5dl1z34ZQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C1:E1"/>
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="O1:O3"/>
     <mergeCell ref="F1:H1"/>
@@ -14300,11 +14238,6 @@
     <mergeCell ref="J1:M2"/>
     <mergeCell ref="N1:N3"/>
     <mergeCell ref="P1:P3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C1:E1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I3 M3 J3 K3 L3 Q1:Q3" xr:uid="{2FBCC481-6114-481E-B036-95624C9F7883}">
@@ -14338,20 +14271,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="93" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="80" t="s">
+      <c r="C1" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="84"/>
+      <c r="D1" s="87"/>
     </row>
     <row r="2" spans="1:4" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67"/>
+      <c r="A2" s="70"/>
+      <c r="B2" s="70"/>
       <c r="C2" s="35" t="s">
         <v>145</v>
       </c>
@@ -15591,47 +15524,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="93" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="104" t="s">
+      <c r="C1" s="93" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="146" t="s">
+      <c r="D1" s="121" t="s">
         <v>121</v>
       </c>
-      <c r="E1" s="148" t="s">
+      <c r="E1" s="123" t="s">
         <v>89</v>
       </c>
-      <c r="F1" s="149"/>
-      <c r="G1" s="86" t="s">
+      <c r="F1" s="124"/>
+      <c r="G1" s="94" t="s">
         <v>184</v>
       </c>
-      <c r="H1" s="104" t="s">
+      <c r="H1" s="93" t="s">
         <v>209</v>
       </c>
-      <c r="I1" s="80" t="s">
+      <c r="I1" s="83" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="81"/>
-      <c r="K1" s="84"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="87"/>
     </row>
     <row r="2" spans="1:11" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="147"/>
+      <c r="A2" s="70"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="122"/>
       <c r="E2" s="44" t="s">
         <v>23</v>
       </c>
       <c r="F2" s="44" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="87"/>
-      <c r="H2" s="67"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="70"/>
       <c r="I2" s="38" t="s">
         <v>186</v>
       </c>
@@ -18245,14 +18178,14 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="JA+gDfx9HL2mV0Tdxs3H6w2uRT4wHZDQJ8yXQoLv5fxFnTThYZmX+TLadTXq48/15VXPdFGIRAdSIbF5KO1tGQ==" saltValue="Z6n+HwaoylFKFjVBtH70GA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="8">
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:K1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:F1"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:K1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2 E2:F2 K2 G1" xr:uid="{4E0B6771-5993-41A9-BE9D-F553134C1037}">
@@ -18307,65 +18240,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="118" t="s">
+      <c r="A1" s="125" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="118" t="s">
+      <c r="B1" s="125" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="118" t="s">
+      <c r="C1" s="125" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="118" t="s">
+      <c r="D1" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="86" t="s">
+      <c r="E1" s="94" t="s">
         <v>183</v>
       </c>
-      <c r="F1" s="86" t="s">
+      <c r="F1" s="94" t="s">
         <v>184</v>
       </c>
-      <c r="G1" s="78" t="s">
+      <c r="G1" s="81" t="s">
         <v>187</v>
       </c>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="95" t="s">
+      <c r="H1" s="81"/>
+      <c r="I1" s="81"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="92" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="95"/>
-      <c r="M1" s="95"/>
-      <c r="N1" s="95"/>
-      <c r="O1" s="95" t="s">
+      <c r="L1" s="92"/>
+      <c r="M1" s="92"/>
+      <c r="N1" s="92"/>
+      <c r="O1" s="92" t="s">
         <v>58</v>
       </c>
-      <c r="P1" s="95"/>
-      <c r="Q1" s="95"/>
-      <c r="R1" s="101" t="s">
+      <c r="P1" s="92"/>
+      <c r="Q1" s="92"/>
+      <c r="R1" s="89" t="s">
         <v>61</v>
       </c>
-      <c r="S1" s="80" t="s">
+      <c r="S1" s="83" t="s">
         <v>87</v>
       </c>
-      <c r="T1" s="84"/>
-      <c r="U1" s="80" t="s">
+      <c r="T1" s="87"/>
+      <c r="U1" s="83" t="s">
         <v>192</v>
       </c>
-      <c r="V1" s="81"/>
-      <c r="W1" s="84"/>
-      <c r="X1" s="95" t="s">
+      <c r="V1" s="84"/>
+      <c r="W1" s="87"/>
+      <c r="X1" s="92" t="s">
         <v>191</v>
       </c>
-      <c r="Y1" s="95"/>
+      <c r="Y1" s="92"/>
     </row>
     <row r="2" spans="1:25" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="119"/>
-      <c r="B2" s="119"/>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
+      <c r="A2" s="126"/>
+      <c r="B2" s="126"/>
+      <c r="C2" s="126"/>
+      <c r="D2" s="126"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
       <c r="G2" s="44" t="s">
         <v>23</v>
       </c>
@@ -18399,7 +18332,7 @@
       <c r="Q2" s="38" t="s">
         <v>204</v>
       </c>
-      <c r="R2" s="103"/>
+      <c r="R2" s="91"/>
       <c r="S2" s="36" t="s">
         <v>85</v>
       </c>
@@ -23892,70 +23825,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="118" t="s">
+      <c r="A1" s="125" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="118" t="s">
+      <c r="B1" s="125" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="118" t="s">
+      <c r="C1" s="125" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="118" t="s">
+      <c r="D1" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="86" t="s">
+      <c r="E1" s="94" t="s">
         <v>174</v>
       </c>
-      <c r="F1" s="86" t="s">
+      <c r="F1" s="94" t="s">
         <v>175</v>
       </c>
-      <c r="G1" s="86" t="s">
+      <c r="G1" s="94" t="s">
         <v>176</v>
       </c>
-      <c r="H1" s="102" t="s">
+      <c r="H1" s="90" t="s">
         <v>177</v>
       </c>
-      <c r="I1" s="76" t="s">
+      <c r="I1" s="79" t="s">
         <v>69</v>
       </c>
-      <c r="J1" s="77"/>
-      <c r="K1" s="73" t="s">
+      <c r="J1" s="80"/>
+      <c r="K1" s="76" t="s">
         <v>70</v>
       </c>
-      <c r="L1" s="75"/>
-      <c r="M1" s="102" t="s">
+      <c r="L1" s="78"/>
+      <c r="M1" s="90" t="s">
         <v>182</v>
       </c>
-      <c r="N1" s="120" t="s">
+      <c r="N1" s="127" t="s">
         <v>72</v>
       </c>
-      <c r="O1" s="120" t="s">
+      <c r="O1" s="127" t="s">
         <v>66</v>
       </c>
-      <c r="P1" s="102" t="s">
+      <c r="P1" s="90" t="s">
         <v>181</v>
       </c>
-      <c r="Q1" s="120" t="s">
+      <c r="Q1" s="127" t="s">
         <v>67</v>
       </c>
-      <c r="R1" s="120" t="s">
+      <c r="R1" s="127" t="s">
         <v>68</v>
       </c>
-      <c r="S1" s="79" t="s">
+      <c r="S1" s="82" t="s">
         <v>191</v>
       </c>
-      <c r="T1" s="79"/>
+      <c r="T1" s="82"/>
     </row>
     <row r="2" spans="1:20" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="119"/>
-      <c r="B2" s="119"/>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="103"/>
+      <c r="A2" s="126"/>
+      <c r="B2" s="126"/>
+      <c r="C2" s="126"/>
+      <c r="D2" s="126"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="91"/>
       <c r="I2" s="38" t="s">
         <v>178</v>
       </c>
@@ -23968,12 +23901,12 @@
       <c r="L2" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="M2" s="103"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="79"/>
-      <c r="P2" s="103"/>
-      <c r="Q2" s="79"/>
-      <c r="R2" s="79"/>
+      <c r="M2" s="91"/>
+      <c r="N2" s="82"/>
+      <c r="O2" s="82"/>
+      <c r="P2" s="91"/>
+      <c r="Q2" s="82"/>
+      <c r="R2" s="82"/>
       <c r="S2" s="38" t="s">
         <v>180</v>
       </c>
@@ -28384,16 +28317,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="l8KVIJiIcXBtA5Rxt+oHSTZCQcSscxoVEx71fajOPkkDzIq7y1m1u1pHAE+AUnT93CwTnM5PkUuxYj42pmVV9g==" saltValue="dsO/0LEKtl67ZZqtPejb6A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="N1:N2"/>
-    <mergeCell ref="O1:O2"/>
     <mergeCell ref="P1:P2"/>
     <mergeCell ref="S1:T1"/>
     <mergeCell ref="H1:H2"/>
@@ -28401,6 +28324,16 @@
     <mergeCell ref="R1:R2"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="K1:L1"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F2 H1:H2 P1:P2 S2 J2 E1:E2 G1:G2 I2 M1:M2 T2" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -31126,117 +31059,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="69" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="67" t="s">
+      <c r="B1" s="70" t="s">
         <v>156</v>
       </c>
-      <c r="C1" s="67"/>
-      <c r="D1" s="79" t="s">
+      <c r="C1" s="70"/>
+      <c r="D1" s="82" t="s">
         <v>157</v>
       </c>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="70" t="s">
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="82"/>
+      <c r="H1" s="82"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="73" t="s">
         <v>210</v>
       </c>
-      <c r="O1" s="71"/>
-      <c r="P1" s="71"/>
-      <c r="Q1" s="71"/>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="71"/>
-      <c r="U1" s="71"/>
-      <c r="V1" s="71"/>
-      <c r="W1" s="71"/>
-      <c r="X1" s="72"/>
+      <c r="O1" s="74"/>
+      <c r="P1" s="74"/>
+      <c r="Q1" s="74"/>
+      <c r="R1" s="74"/>
+      <c r="S1" s="74"/>
+      <c r="T1" s="74"/>
+      <c r="U1" s="74"/>
+      <c r="V1" s="74"/>
+      <c r="W1" s="74"/>
+      <c r="X1" s="75"/>
       <c r="Y1" s="41"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" s="66"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="80" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="83" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="80" t="s">
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="83" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="81"/>
-      <c r="K2" s="81"/>
-      <c r="L2" s="81"/>
-      <c r="M2" s="81"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="74"/>
-      <c r="P2" s="74"/>
-      <c r="Q2" s="74"/>
-      <c r="R2" s="74"/>
-      <c r="S2" s="74"/>
-      <c r="T2" s="74"/>
-      <c r="U2" s="74"/>
-      <c r="V2" s="74"/>
-      <c r="W2" s="74"/>
-      <c r="X2" s="75"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="84"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="84"/>
+      <c r="N2" s="76"/>
+      <c r="O2" s="77"/>
+      <c r="P2" s="77"/>
+      <c r="Q2" s="77"/>
+      <c r="R2" s="77"/>
+      <c r="S2" s="77"/>
+      <c r="T2" s="77"/>
+      <c r="U2" s="77"/>
+      <c r="V2" s="77"/>
+      <c r="W2" s="77"/>
+      <c r="X2" s="78"/>
       <c r="Y2" s="41"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="66"/>
-      <c r="B3" s="78"/>
-      <c r="C3" s="78"/>
-      <c r="D3" s="76" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="81"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="79" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="77"/>
-      <c r="F3" s="76" t="s">
+      <c r="E3" s="80"/>
+      <c r="F3" s="79" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="77"/>
-      <c r="H3" s="85" t="s">
+      <c r="G3" s="80"/>
+      <c r="H3" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="I3" s="76" t="s">
+      <c r="I3" s="79" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="77"/>
-      <c r="K3" s="76" t="s">
+      <c r="J3" s="80"/>
+      <c r="K3" s="79" t="s">
         <v>74</v>
       </c>
-      <c r="L3" s="77"/>
-      <c r="M3" s="82" t="s">
+      <c r="L3" s="80"/>
+      <c r="M3" s="85" t="s">
         <v>81</v>
       </c>
-      <c r="N3" s="68" t="s">
+      <c r="N3" s="71" t="s">
         <v>233</v>
       </c>
-      <c r="O3" s="68"/>
-      <c r="P3" s="69" t="s">
+      <c r="O3" s="71"/>
+      <c r="P3" s="72" t="s">
         <v>231</v>
       </c>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="69"/>
-      <c r="S3" s="69"/>
-      <c r="T3" s="69"/>
-      <c r="U3" s="69" t="s">
+      <c r="Q3" s="72"/>
+      <c r="R3" s="72"/>
+      <c r="S3" s="72"/>
+      <c r="T3" s="72"/>
+      <c r="U3" s="72" t="s">
         <v>232</v>
       </c>
-      <c r="V3" s="69"/>
-      <c r="W3" s="69"/>
-      <c r="X3" s="69"/>
+      <c r="V3" s="72"/>
+      <c r="W3" s="72"/>
+      <c r="X3" s="72"/>
     </row>
     <row r="4" spans="1:25" s="42" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="67"/>
+      <c r="A4" s="70"/>
       <c r="B4" s="32" t="s">
         <v>108</v>
       </c>
@@ -31255,7 +31188,7 @@
       <c r="G4" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="79"/>
+      <c r="H4" s="82"/>
       <c r="I4" s="38" t="s">
         <v>115</v>
       </c>
@@ -31268,7 +31201,7 @@
       <c r="L4" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="M4" s="83"/>
+      <c r="M4" s="86"/>
       <c r="N4" s="32" t="s">
         <v>5</v>
       </c>
@@ -36543,89 +36476,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="100" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="88" t="s">
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="89"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="101" t="s">
+      <c r="H1" s="97"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="89" t="s">
         <v>17</v>
       </c>
       <c r="K1" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="L1" s="92" t="s">
+      <c r="L1" s="100" t="s">
         <v>109</v>
       </c>
-      <c r="M1" s="93"/>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="94"/>
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="102"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="66"/>
-      <c r="B2" s="78" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="99" t="s">
+      <c r="C2" s="106" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="100" t="s">
+      <c r="D2" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="85" t="s">
+      <c r="E2" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="95" t="s">
+      <c r="F2" s="92" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="96" t="s">
+      <c r="G2" s="103" t="s">
         <v>115</v>
       </c>
-      <c r="H2" s="97" t="s">
+      <c r="H2" s="104" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="91" t="s">
+      <c r="I2" s="99" t="s">
         <v>158</v>
       </c>
-      <c r="J2" s="102"/>
-      <c r="K2" s="86" t="s">
+      <c r="J2" s="90"/>
+      <c r="K2" s="94" t="s">
         <v>122</v>
       </c>
-      <c r="L2" s="68" t="s">
+      <c r="L2" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68" t="s">
+      <c r="M2" s="71"/>
+      <c r="N2" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="68"/>
-      <c r="P2" s="95" t="s">
+      <c r="O2" s="71"/>
+      <c r="P2" s="92" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="67"/>
-      <c r="B3" s="78"/>
-      <c r="C3" s="99"/>
-      <c r="D3" s="100"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="98"/>
-      <c r="I3" s="91"/>
-      <c r="J3" s="103"/>
-      <c r="K3" s="87"/>
+      <c r="A3" s="70"/>
+      <c r="B3" s="81"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="92"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="105"/>
+      <c r="I3" s="99"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="95"/>
       <c r="L3" s="32" t="s">
         <v>3</v>
       </c>
@@ -36638,7 +36571,7 @@
       <c r="O3" s="44" t="s">
         <v>230</v>
       </c>
-      <c r="P3" s="95"/>
+      <c r="P3" s="92"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -40243,12 +40176,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="yP1GbBCgAdm0CH/gr8AK4RsVM1gtv82RP3HgfmHP3L5tX6iCxw/IjCz2X6Q4KidklCbEORnuuGS+Q9kp+KNj3w==" saltValue="R0+mSYCgXyR4udjvNYppsg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="I2:I3"/>
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P2:P3"/>
@@ -40260,6 +40187,12 @@
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="I2:I3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 J4 K2:K3 G2:I3 O3" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40302,47 +40235,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="95" t="s">
+      <c r="B1" s="92" t="s">
         <v>211</v>
       </c>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95" t="s">
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92" t="s">
         <v>212</v>
       </c>
-      <c r="H1" s="95"/>
-      <c r="I1" s="95"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
+      <c r="H1" s="92"/>
+      <c r="I1" s="92"/>
+      <c r="J1" s="92"/>
+      <c r="K1" s="92"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="66"/>
-      <c r="B2" s="80" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="83" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="85" t="s">
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="80" t="s">
+      <c r="G2" s="83" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="81"/>
-      <c r="I2" s="81"/>
-      <c r="J2" s="84"/>
-      <c r="K2" s="85" t="s">
+      <c r="H2" s="84"/>
+      <c r="I2" s="84"/>
+      <c r="J2" s="87"/>
+      <c r="K2" s="88" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="67"/>
+      <c r="A3" s="70"/>
       <c r="B3" s="38" t="s">
         <v>115</v>
       </c>
@@ -40355,7 +40288,7 @@
       <c r="E3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="79"/>
+      <c r="F3" s="82"/>
       <c r="G3" s="38" t="s">
         <v>115</v>
       </c>
@@ -40368,7 +40301,7 @@
       <c r="J3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="79"/>
+      <c r="K3" s="82"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -43044,156 +42977,156 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="80" t="s">
+      <c r="B1" s="83" t="s">
         <v>171</v>
       </c>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="81"/>
-      <c r="M1" s="81"/>
-      <c r="N1" s="81"/>
-      <c r="O1" s="81"/>
-      <c r="P1" s="81"/>
-      <c r="Q1" s="81"/>
-      <c r="R1" s="81"/>
-      <c r="S1" s="81"/>
-      <c r="T1" s="84"/>
-      <c r="U1" s="80" t="s">
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="84"/>
+      <c r="H1" s="84"/>
+      <c r="I1" s="84"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="87"/>
+      <c r="U1" s="83" t="s">
         <v>213</v>
       </c>
-      <c r="V1" s="81"/>
-      <c r="W1" s="81"/>
-      <c r="X1" s="81"/>
-      <c r="Y1" s="81"/>
-      <c r="Z1" s="81"/>
-      <c r="AA1" s="81"/>
-      <c r="AB1" s="81"/>
-      <c r="AC1" s="81"/>
-      <c r="AD1" s="81"/>
-      <c r="AE1" s="81"/>
-      <c r="AF1" s="81"/>
-      <c r="AG1" s="84"/>
-      <c r="AH1" s="80" t="s">
+      <c r="V1" s="84"/>
+      <c r="W1" s="84"/>
+      <c r="X1" s="84"/>
+      <c r="Y1" s="84"/>
+      <c r="Z1" s="84"/>
+      <c r="AA1" s="84"/>
+      <c r="AB1" s="84"/>
+      <c r="AC1" s="84"/>
+      <c r="AD1" s="84"/>
+      <c r="AE1" s="84"/>
+      <c r="AF1" s="84"/>
+      <c r="AG1" s="87"/>
+      <c r="AH1" s="83" t="s">
         <v>214</v>
       </c>
-      <c r="AI1" s="81"/>
-      <c r="AJ1" s="81"/>
-      <c r="AK1" s="81"/>
-      <c r="AL1" s="81"/>
-      <c r="AM1" s="81"/>
-      <c r="AN1" s="81"/>
-      <c r="AO1" s="84"/>
+      <c r="AI1" s="84"/>
+      <c r="AJ1" s="84"/>
+      <c r="AK1" s="84"/>
+      <c r="AL1" s="84"/>
+      <c r="AM1" s="84"/>
+      <c r="AN1" s="84"/>
+      <c r="AO1" s="87"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A2" s="66"/>
-      <c r="B2" s="85" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="88" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="85" t="s">
+      <c r="C2" s="88" t="s">
         <v>125</v>
       </c>
-      <c r="D2" s="101" t="s">
+      <c r="D2" s="89" t="s">
         <v>126</v>
       </c>
-      <c r="E2" s="69" t="s">
+      <c r="E2" s="72" t="s">
         <v>172</v>
       </c>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69" t="s">
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72" t="s">
         <v>173</v>
       </c>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="85" t="s">
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="88" t="s">
         <v>155</v>
       </c>
-      <c r="L2" s="69" t="s">
+      <c r="L2" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69" t="s">
+      <c r="M2" s="72"/>
+      <c r="N2" s="72"/>
+      <c r="O2" s="72"/>
+      <c r="P2" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="69"/>
-      <c r="S2" s="69" t="s">
+      <c r="Q2" s="72"/>
+      <c r="R2" s="72"/>
+      <c r="S2" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="T2" s="69"/>
-      <c r="U2" s="95" t="s">
+      <c r="T2" s="72"/>
+      <c r="U2" s="92" t="s">
         <v>136</v>
       </c>
-      <c r="V2" s="95" t="s">
+      <c r="V2" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="W2" s="95" t="s">
+      <c r="W2" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="X2" s="95" t="s">
+      <c r="X2" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="Y2" s="95" t="s">
+      <c r="Y2" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="95" t="s">
+      <c r="Z2" s="92" t="s">
         <v>32</v>
       </c>
-      <c r="AA2" s="95" t="s">
+      <c r="AA2" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AB2" s="95" t="s">
+      <c r="AB2" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AC2" s="95" t="s">
+      <c r="AC2" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="AD2" s="95" t="s">
+      <c r="AD2" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="AE2" s="95" t="s">
+      <c r="AE2" s="92" t="s">
         <v>37</v>
       </c>
-      <c r="AF2" s="95" t="s">
+      <c r="AF2" s="92" t="s">
         <v>128</v>
       </c>
-      <c r="AG2" s="95" t="s">
+      <c r="AG2" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="AH2" s="88" t="s">
+      <c r="AH2" s="96" t="s">
         <v>215</v>
       </c>
-      <c r="AI2" s="90"/>
-      <c r="AJ2" s="69" t="s">
+      <c r="AI2" s="98"/>
+      <c r="AJ2" s="72" t="s">
         <v>216</v>
       </c>
-      <c r="AK2" s="69"/>
-      <c r="AL2" s="69" t="s">
+      <c r="AK2" s="72"/>
+      <c r="AL2" s="72" t="s">
         <v>217</v>
       </c>
-      <c r="AM2" s="69"/>
-      <c r="AN2" s="69" t="s">
+      <c r="AM2" s="72"/>
+      <c r="AN2" s="72" t="s">
         <v>218</v>
       </c>
-      <c r="AO2" s="69"/>
+      <c r="AO2" s="72"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A3" s="67"/>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="103"/>
+      <c r="A3" s="70"/>
+      <c r="B3" s="82"/>
+      <c r="C3" s="82"/>
+      <c r="D3" s="91"/>
       <c r="E3" s="34" t="s">
         <v>24</v>
       </c>
@@ -43212,7 +43145,7 @@
       <c r="J3" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="K3" s="79"/>
+      <c r="K3" s="82"/>
       <c r="L3" s="31" t="s">
         <v>127</v>
       </c>
@@ -43240,19 +43173,19 @@
       <c r="T3" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="U3" s="95"/>
-      <c r="V3" s="95"/>
-      <c r="W3" s="95"/>
-      <c r="X3" s="95"/>
-      <c r="Y3" s="95"/>
-      <c r="Z3" s="95"/>
-      <c r="AA3" s="95"/>
-      <c r="AB3" s="95"/>
-      <c r="AC3" s="95"/>
-      <c r="AD3" s="95"/>
-      <c r="AE3" s="95"/>
-      <c r="AF3" s="95"/>
-      <c r="AG3" s="95"/>
+      <c r="U3" s="92"/>
+      <c r="V3" s="92"/>
+      <c r="W3" s="92"/>
+      <c r="X3" s="92"/>
+      <c r="Y3" s="92"/>
+      <c r="Z3" s="92"/>
+      <c r="AA3" s="92"/>
+      <c r="AB3" s="92"/>
+      <c r="AC3" s="92"/>
+      <c r="AD3" s="92"/>
+      <c r="AE3" s="92"/>
+      <c r="AF3" s="92"/>
+      <c r="AG3" s="92"/>
       <c r="AH3" s="31" t="s">
         <v>137</v>
       </c>
@@ -51881,6 +51814,20 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="wxJYPTS1M8YrpE+F5HXpzPvhVkWn+uzvbhQbX4zWGt7tgJJAc6rvipv1/0hraJgXbUY0X5vYRquC66cBDOGcbg==" saltValue="RWTcEymG3DdteXmtyGeu4A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="K2:K3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="U1:AG1"/>
@@ -51897,20 +51844,6 @@
     <mergeCell ref="AE2:AE3"/>
     <mergeCell ref="AD2:AD3"/>
     <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3 R3 AI3 AK3 AM3 L3 M3 N3 O3 P3 Q3 AO3 AJ3 AL3 AN3 AH3" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -51954,17 +51887,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="78" t="s">
+      <c r="B1" s="81" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="67"/>
+      <c r="A2" s="70"/>
       <c r="B2" s="32" t="s">
         <v>165</v>
       </c>
@@ -53206,25 +53139,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="95" t="s">
+      <c r="B1" s="92" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="80" t="s">
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="83" t="s">
         <v>206</v>
       </c>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="84"/>
+      <c r="H1" s="84"/>
+      <c r="I1" s="84"/>
+      <c r="J1" s="87"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="67"/>
+      <c r="A2" s="70"/>
       <c r="B2" s="50" t="s">
         <v>145</v>
       </c>
@@ -55697,96 +55630,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="122" t="s">
+      <c r="B1" s="108" t="s">
         <v>159</v>
       </c>
-      <c r="C1" s="123"/>
-      <c r="D1" s="123"/>
-      <c r="E1" s="123"/>
-      <c r="F1" s="123"/>
-      <c r="G1" s="123"/>
-      <c r="H1" s="123"/>
-      <c r="I1" s="123"/>
-      <c r="J1" s="123"/>
-      <c r="K1" s="124"/>
-      <c r="L1" s="125" t="s">
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
+      <c r="G1" s="109"/>
+      <c r="H1" s="109"/>
+      <c r="I1" s="109"/>
+      <c r="J1" s="109"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="111" t="s">
         <v>219</v>
       </c>
-      <c r="M1" s="126"/>
-      <c r="N1" s="126"/>
-      <c r="O1" s="126"/>
-      <c r="P1" s="127"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="112"/>
+      <c r="O1" s="112"/>
+      <c r="P1" s="113"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="128"/>
-      <c r="B2" s="121" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="93" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="129" t="s">
+      <c r="C2" s="100" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="131"/>
-      <c r="H2" s="132" t="s">
+      <c r="D2" s="101"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="88" t="s">
         <v>162</v>
       </c>
-      <c r="I2" s="121" t="s">
+      <c r="I2" s="93" t="s">
         <v>163</v>
       </c>
-      <c r="J2" s="133" t="s">
+      <c r="J2" s="83" t="s">
         <v>220</v>
       </c>
-      <c r="K2" s="134"/>
-      <c r="L2" s="135"/>
-      <c r="M2" s="136"/>
-      <c r="N2" s="136"/>
-      <c r="O2" s="136"/>
-      <c r="P2" s="137"/>
+      <c r="K2" s="87"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="114"/>
+      <c r="N2" s="114"/>
+      <c r="O2" s="114"/>
+      <c r="P2" s="80"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="138"/>
-      <c r="B3" s="138"/>
-      <c r="C3" s="139" t="s">
+      <c r="A3" s="70"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="140" t="s">
+      <c r="D3" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="141" t="s">
+      <c r="E3" s="51" t="s">
         <v>160</v>
       </c>
-      <c r="F3" s="140" t="s">
+      <c r="F3" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="G3" s="141" t="s">
+      <c r="G3" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="142"/>
-      <c r="I3" s="138"/>
-      <c r="J3" s="143" t="s">
+      <c r="H3" s="82"/>
+      <c r="I3" s="70"/>
+      <c r="J3" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="143" t="s">
+      <c r="K3" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="144" t="s">
+      <c r="L3" s="58" t="s">
         <v>164</v>
       </c>
-      <c r="M3" s="145" t="s">
+      <c r="M3" s="33" t="s">
         <v>166</v>
       </c>
-      <c r="N3" s="145" t="s">
+      <c r="N3" s="33" t="s">
         <v>167</v>
       </c>
-      <c r="O3" s="145" t="s">
+      <c r="O3" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="P3" s="145" t="s">
+      <c r="P3" s="33" t="s">
         <v>169</v>
       </c>
     </row>
@@ -59457,128 +59390,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="93" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="78" t="s">
+      <c r="C1" s="81" t="s">
         <v>77</v>
       </c>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="109" t="s">
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="108" t="s">
         <v>78</v>
       </c>
-      <c r="G1" s="111"/>
+      <c r="G1" s="109"/>
       <c r="H1" s="110"/>
-      <c r="I1" s="104" t="s">
+      <c r="I1" s="93" t="s">
         <v>236</v>
       </c>
-      <c r="J1" s="104" t="s">
+      <c r="J1" s="93" t="s">
         <v>237</v>
       </c>
-      <c r="K1" s="105" t="s">
+      <c r="K1" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="L1" s="106"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="105" t="s">
+      <c r="L1" s="112"/>
+      <c r="M1" s="113"/>
+      <c r="N1" s="111" t="s">
         <v>49</v>
       </c>
-      <c r="O1" s="107"/>
-      <c r="P1" s="78" t="s">
+      <c r="O1" s="113"/>
+      <c r="P1" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="Q1" s="95" t="s">
+      <c r="Q1" s="92" t="s">
         <v>239</v>
       </c>
-      <c r="R1" s="78" t="s">
+      <c r="R1" s="81" t="s">
         <v>240</v>
       </c>
-      <c r="S1" s="78" t="s">
+      <c r="S1" s="81" t="s">
         <v>246</v>
       </c>
-      <c r="T1" s="78"/>
-      <c r="U1" s="112" t="s">
+      <c r="T1" s="81"/>
+      <c r="U1" s="115" t="s">
         <v>247</v>
       </c>
-      <c r="V1" s="113"/>
-      <c r="W1" s="112" t="s">
+      <c r="V1" s="116"/>
+      <c r="W1" s="115" t="s">
         <v>248</v>
       </c>
-      <c r="X1" s="113"/>
-      <c r="Y1" s="112" t="s">
+      <c r="X1" s="116"/>
+      <c r="Y1" s="115" t="s">
         <v>249</v>
       </c>
-      <c r="Z1" s="113"/>
-      <c r="AA1" s="78" t="s">
+      <c r="Z1" s="116"/>
+      <c r="AA1" s="81" t="s">
         <v>245</v>
       </c>
-      <c r="AB1" s="78"/>
-      <c r="AC1" s="78"/>
-      <c r="AD1" s="78"/>
+      <c r="AB1" s="81"/>
+      <c r="AC1" s="81"/>
+      <c r="AD1" s="81"/>
     </row>
     <row r="2" spans="1:30" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="70" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="109" t="s">
+      <c r="D2" s="108" t="s">
         <v>79</v>
       </c>
       <c r="E2" s="110"/>
-      <c r="F2" s="104" t="s">
+      <c r="F2" s="93" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="109" t="s">
+      <c r="G2" s="108" t="s">
         <v>79</v>
       </c>
       <c r="H2" s="110"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="108"/>
-      <c r="M2" s="77"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="77"/>
-      <c r="P2" s="78"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="78"/>
-      <c r="S2" s="78"/>
-      <c r="T2" s="78"/>
-      <c r="U2" s="73"/>
-      <c r="V2" s="75"/>
-      <c r="W2" s="73"/>
-      <c r="X2" s="75"/>
-      <c r="Y2" s="73"/>
-      <c r="Z2" s="75"/>
-      <c r="AA2" s="78"/>
-      <c r="AB2" s="78"/>
-      <c r="AC2" s="78"/>
-      <c r="AD2" s="78"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="114"/>
+      <c r="M2" s="80"/>
+      <c r="N2" s="79"/>
+      <c r="O2" s="80"/>
+      <c r="P2" s="81"/>
+      <c r="Q2" s="92"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="76"/>
+      <c r="V2" s="78"/>
+      <c r="W2" s="76"/>
+      <c r="X2" s="78"/>
+      <c r="Y2" s="76"/>
+      <c r="Z2" s="78"/>
+      <c r="AA2" s="81"/>
+      <c r="AB2" s="81"/>
+      <c r="AC2" s="81"/>
+      <c r="AD2" s="81"/>
     </row>
     <row r="3" spans="1:30" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="67"/>
-      <c r="B3" s="67"/>
-      <c r="C3" s="73"/>
+      <c r="A3" s="70"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="76"/>
       <c r="D3" s="32" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="67"/>
+      <c r="F3" s="70"/>
       <c r="G3" s="32" t="s">
         <v>0</v>
       </c>
       <c r="H3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
+      <c r="I3" s="70"/>
+      <c r="J3" s="70"/>
       <c r="K3" s="38" t="s">
         <v>193</v>
       </c>
@@ -59594,9 +59527,9 @@
       <c r="O3" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="P3" s="78"/>
-      <c r="Q3" s="95"/>
-      <c r="R3" s="78"/>
+      <c r="P3" s="81"/>
+      <c r="Q3" s="92"/>
+      <c r="R3" s="81"/>
       <c r="S3" s="32" t="s">
         <v>50</v>
       </c>
@@ -66009,12 +65942,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="9xCUSnOba9+kjRTP4aA+IhYIhPNTdofqr3mLiTZOPQAzcWWZifDmPOI/0ItUaLA4hSjA/rC4jIft53nJzygclQ==" saltValue="aTfUQq44C7asIKTaLqEvww==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="N1:O2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E2"/>
     <mergeCell ref="Y1:Z2"/>
     <mergeCell ref="AA1:AD2"/>
     <mergeCell ref="U1:V2"/>
@@ -66024,11 +65956,12 @@
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="R1:R3"/>
     <mergeCell ref="S1:T2"/>
-    <mergeCell ref="I1:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="N1:O2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3 AA3:AD3" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">

</xml_diff>

<commit_message>
Revision of some urls
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106F0932-A472-443F-9273-9E731CAEED6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF4050EE-B9A4-4B1D-B2EE-22A34FC302D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" firstSheet="1" activeTab="1" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -1254,9 +1254,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -1446,21 +1443,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1494,6 +1476,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1512,6 +1497,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1574,6 +1571,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1911,24 +1909,24 @@
   <sheetData>
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="58" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="61"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="60"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="62"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="64"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="63"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="5"/>
@@ -1978,15 +1976,15 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="11"/>
-      <c r="C8" s="65" t="s">
+      <c r="C8" s="64" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="65"/>
+      <c r="D8" s="64"/>
       <c r="E8" s="12"/>
-      <c r="F8" s="65" t="s">
+      <c r="F8" s="64" t="s">
         <v>113</v>
       </c>
-      <c r="G8" s="65"/>
+      <c r="G8" s="64"/>
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2108,7 +2106,7 @@
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="11"/>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="22" t="s">
         <v>82</v>
       </c>
       <c r="D20" s="21"/>
@@ -2119,7 +2117,7 @@
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="11"/>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="127" t="s">
         <v>107</v>
       </c>
       <c r="D21" s="21"/>
@@ -2168,11 +2166,11 @@
     </row>
     <row r="26" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="11"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="67"/>
-      <c r="F26" s="67"/>
-      <c r="G26" s="68"/>
+      <c r="C26" s="65"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
+      <c r="F26" s="66"/>
+      <c r="G26" s="67"/>
       <c r="H26" s="13"/>
     </row>
     <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2189,7 +2187,7 @@
       <c r="D28" s="28"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="fECAul9Xub1IkDhYUJjwJS9OzYzo0I9Z1C6jwPBr+eEjzIjgSDIhJ1EXiZzgp9q6fPNfWYq+aXIj8dGPnToVoA==" saltValue="U4C95otBxdOcIHYcesbhsA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="4">
     <mergeCell ref="B2:H3"/>
     <mergeCell ref="C8:D8"/>
@@ -2204,9 +2202,10 @@
   <hyperlinks>
     <hyperlink ref="C19" r:id="rId1" location="entities" xr:uid="{384D1750-687F-4E8E-BDBD-927F2E2E470C}"/>
     <hyperlink ref="C20" r:id="rId2" location="fleets" xr:uid="{07140C16-0A83-41FD-984B-2B188EE4EBA5}"/>
+    <hyperlink ref="C21" r:id="rId3" location="sourcesRO" xr:uid="{14D27D57-85D2-43E5-9AF0-D8C32445BC32}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
@@ -2225,24 +2224,24 @@
     <col min="5" max="5" width="19.42578125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="51" t="s">
+    <row r="1" spans="1:5" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="50" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="43" t="s">
         <v>203</v>
       </c>
-      <c r="E1" s="48" t="s">
+      <c r="E1" s="47" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="43" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" s="42" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3678,71 +3677,71 @@
     <col min="12" max="15" width="17.5703125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+    <row r="1" spans="1:15" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="93" t="s">
+      <c r="C1" s="88" t="s">
         <v>228</v>
       </c>
-      <c r="D1" s="93" t="s">
+      <c r="D1" s="88" t="s">
         <v>229</v>
       </c>
-      <c r="E1" s="88" t="s">
+      <c r="E1" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="93" t="s">
+      <c r="F1" s="88" t="s">
         <v>250</v>
       </c>
-      <c r="G1" s="93" t="s">
+      <c r="G1" s="88" t="s">
         <v>227</v>
       </c>
-      <c r="H1" s="93" t="s">
+      <c r="H1" s="88" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="93" t="s">
+      <c r="I1" s="88" t="s">
         <v>93</v>
       </c>
-      <c r="J1" s="83" t="s">
+      <c r="J1" s="82" t="s">
         <v>221</v>
       </c>
-      <c r="K1" s="87"/>
-      <c r="L1" s="108" t="s">
+      <c r="K1" s="86"/>
+      <c r="L1" s="107" t="s">
         <v>222</v>
       </c>
-      <c r="M1" s="109"/>
-      <c r="N1" s="109"/>
-      <c r="O1" s="110"/>
-    </row>
-    <row r="2" spans="1:15" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="70"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="35" t="s">
+      <c r="M1" s="108"/>
+      <c r="N1" s="108"/>
+      <c r="O1" s="109"/>
+    </row>
+    <row r="2" spans="1:15" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="K2" s="35" t="s">
+      <c r="K2" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="L2" s="44" t="s">
+      <c r="L2" s="43" t="s">
         <v>223</v>
       </c>
-      <c r="M2" s="44" t="s">
+      <c r="M2" s="43" t="s">
         <v>224</v>
       </c>
-      <c r="N2" s="44" t="s">
+      <c r="N2" s="43" t="s">
         <v>225</v>
       </c>
-      <c r="O2" s="44" t="s">
+      <c r="O2" s="43" t="s">
         <v>226</v>
       </c>
     </row>
@@ -7190,29 +7189,29 @@
     <col min="5" max="5" width="14.42578125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+    <row r="1" spans="1:5" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="108" t="s">
+      <c r="C1" s="107" t="s">
         <v>201</v>
       </c>
-      <c r="D1" s="109"/>
-      <c r="E1" s="110"/>
-    </row>
-    <row r="2" spans="1:5" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="70"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="44" t="s">
+      <c r="D1" s="108"/>
+      <c r="E1" s="109"/>
+    </row>
+    <row r="2" spans="1:5" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="D2" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="34" t="s">
         <v>52</v>
       </c>
     </row>
@@ -8646,33 +8645,33 @@
     <col min="6" max="6" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+    <row r="1" spans="1:6" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="108" t="s">
+      <c r="C1" s="107" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="109"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="110"/>
-    </row>
-    <row r="2" spans="1:6" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="70"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="44" t="s">
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="109"/>
+    </row>
+    <row r="2" spans="1:6" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="43" t="s">
         <v>178</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="E2" s="32" t="s">
+      <c r="E2" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="35" t="s">
+      <c r="F2" s="34" t="s">
         <v>53</v>
       </c>
     </row>
@@ -10320,108 +10319,108 @@
     <col min="17" max="17" width="27.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+    <row r="1" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="108" t="s">
+      <c r="C1" s="107" t="s">
         <v>207</v>
       </c>
-      <c r="D1" s="109"/>
-      <c r="E1" s="110"/>
-      <c r="F1" s="108" t="s">
+      <c r="D1" s="108"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="107" t="s">
         <v>208</v>
       </c>
-      <c r="G1" s="109"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="103" t="s">
+      <c r="G1" s="108"/>
+      <c r="H1" s="109"/>
+      <c r="I1" s="99" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="92" t="s">
+      <c r="J1" s="98" t="s">
         <v>195</v>
       </c>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="81" t="s">
+      <c r="K1" s="98"/>
+      <c r="L1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="80" t="s">
         <v>57</v>
       </c>
-      <c r="O1" s="81" t="s">
+      <c r="O1" s="80" t="s">
         <v>200</v>
       </c>
-      <c r="P1" s="118" t="s">
+      <c r="P1" s="117" t="s">
         <v>253</v>
       </c>
-      <c r="Q1" s="117" t="s">
+      <c r="Q1" s="116" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="69"/>
-      <c r="B2" s="69"/>
-      <c r="C2" s="93" t="s">
+    <row r="2" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="68"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="108" t="s">
+      <c r="D2" s="107" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="110"/>
-      <c r="F2" s="93" t="s">
+      <c r="E2" s="109"/>
+      <c r="F2" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="108" t="s">
+      <c r="G2" s="107" t="s">
         <v>79</v>
       </c>
-      <c r="H2" s="110"/>
-      <c r="I2" s="103"/>
-      <c r="J2" s="92"/>
-      <c r="K2" s="92"/>
-      <c r="L2" s="92"/>
-      <c r="M2" s="92"/>
-      <c r="N2" s="81"/>
-      <c r="O2" s="81"/>
-      <c r="P2" s="119"/>
-      <c r="Q2" s="117"/>
-    </row>
-    <row r="3" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="70"/>
-      <c r="C3" s="70"/>
-      <c r="D3" s="32" t="s">
+      <c r="H2" s="109"/>
+      <c r="I2" s="99"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="98"/>
+      <c r="N2" s="80"/>
+      <c r="O2" s="80"/>
+      <c r="P2" s="118"/>
+      <c r="Q2" s="116"/>
+    </row>
+    <row r="3" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="69"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="32" t="s">
+      <c r="E3" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="70"/>
-      <c r="G3" s="32" t="s">
+      <c r="F3" s="69"/>
+      <c r="G3" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="32" t="s">
+      <c r="H3" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="103"/>
-      <c r="J3" s="38" t="s">
+      <c r="I3" s="99"/>
+      <c r="J3" s="37" t="s">
         <v>194</v>
       </c>
-      <c r="K3" s="38" t="s">
+      <c r="K3" s="37" t="s">
         <v>196</v>
       </c>
-      <c r="L3" s="38" t="s">
+      <c r="L3" s="37" t="s">
         <v>197</v>
       </c>
-      <c r="M3" s="38" t="s">
+      <c r="M3" s="37" t="s">
         <v>198</v>
       </c>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="120"/>
-      <c r="Q3" s="117"/>
-    </row>
-    <row r="4" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="119"/>
+      <c r="Q3" s="116"/>
+    </row>
+    <row r="4" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -14270,25 +14269,25 @@
     <col min="4" max="4" width="21.7109375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+    <row r="1" spans="1:4" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="83" t="s">
+      <c r="C1" s="82" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="87"/>
-    </row>
-    <row r="2" spans="1:4" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="70"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="35" t="s">
+      <c r="D1" s="86"/>
+    </row>
+    <row r="2" spans="1:4" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="D2" s="34" t="s">
         <v>185</v>
       </c>
     </row>
@@ -15523,59 +15522,59 @@
     <col min="11" max="11" width="27.42578125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+    <row r="1" spans="1:11" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="93" t="s">
+      <c r="C1" s="88" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="121" t="s">
+      <c r="D1" s="120" t="s">
         <v>121</v>
       </c>
-      <c r="E1" s="123" t="s">
+      <c r="E1" s="122" t="s">
         <v>89</v>
       </c>
-      <c r="F1" s="124"/>
-      <c r="G1" s="94" t="s">
+      <c r="F1" s="123"/>
+      <c r="G1" s="89" t="s">
         <v>184</v>
       </c>
-      <c r="H1" s="93" t="s">
+      <c r="H1" s="88" t="s">
         <v>209</v>
       </c>
-      <c r="I1" s="83" t="s">
+      <c r="I1" s="82" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="84"/>
-      <c r="K1" s="87"/>
-    </row>
-    <row r="2" spans="1:11" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="70"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="122"/>
-      <c r="E2" s="44" t="s">
+      <c r="J1" s="83"/>
+      <c r="K1" s="86"/>
+    </row>
+    <row r="2" spans="1:11" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="121"/>
+      <c r="E2" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="44" t="s">
+      <c r="F2" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="95"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="38" t="s">
+      <c r="G2" s="90"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="J2" s="35" t="s">
+      <c r="J2" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="K2" s="38" t="s">
+      <c r="K2" s="37" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="3" spans="1:11" s="43" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" s="42" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -18239,123 +18238,123 @@
     <col min="25" max="25" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="125" t="s">
+    <row r="1" spans="1:25" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="124" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="125" t="s">
+      <c r="B1" s="124" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="125" t="s">
+      <c r="C1" s="124" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="125" t="s">
+      <c r="D1" s="124" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="94" t="s">
+      <c r="E1" s="89" t="s">
         <v>183</v>
       </c>
-      <c r="F1" s="94" t="s">
+      <c r="F1" s="89" t="s">
         <v>184</v>
       </c>
-      <c r="G1" s="81" t="s">
+      <c r="G1" s="80" t="s">
         <v>187</v>
       </c>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="92" t="s">
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="80"/>
+      <c r="K1" s="98" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92" t="s">
+      <c r="L1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="98"/>
+      <c r="O1" s="98" t="s">
         <v>58</v>
       </c>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="89" t="s">
+      <c r="P1" s="98"/>
+      <c r="Q1" s="98"/>
+      <c r="R1" s="104" t="s">
         <v>61</v>
       </c>
-      <c r="S1" s="83" t="s">
+      <c r="S1" s="82" t="s">
         <v>87</v>
       </c>
-      <c r="T1" s="87"/>
-      <c r="U1" s="83" t="s">
+      <c r="T1" s="86"/>
+      <c r="U1" s="82" t="s">
         <v>192</v>
       </c>
-      <c r="V1" s="84"/>
-      <c r="W1" s="87"/>
-      <c r="X1" s="92" t="s">
+      <c r="V1" s="83"/>
+      <c r="W1" s="86"/>
+      <c r="X1" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="Y1" s="92"/>
-    </row>
-    <row r="2" spans="1:25" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="126"/>
-      <c r="B2" s="126"/>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="44" t="s">
+      <c r="Y1" s="98"/>
+    </row>
+    <row r="2" spans="1:25" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="125"/>
+      <c r="B2" s="125"/>
+      <c r="C2" s="125"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="32" t="s">
+      <c r="H2" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="44" t="s">
+      <c r="I2" s="43" t="s">
         <v>188</v>
       </c>
-      <c r="J2" s="32" t="s">
+      <c r="J2" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="K2" s="38" t="s">
+      <c r="K2" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="35" t="s">
+      <c r="L2" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="M2" s="38" t="s">
+      <c r="M2" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="N2" s="35" t="s">
+      <c r="N2" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="O2" s="38" t="s">
+      <c r="O2" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="P2" s="35" t="s">
+      <c r="P2" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="Q2" s="38" t="s">
+      <c r="Q2" s="37" t="s">
         <v>204</v>
       </c>
-      <c r="R2" s="91"/>
-      <c r="S2" s="36" t="s">
+      <c r="R2" s="106"/>
+      <c r="S2" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="T2" s="36" t="s">
+      <c r="T2" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="U2" s="55" t="s">
+      <c r="U2" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="V2" s="55" t="s">
+      <c r="V2" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="W2" s="35" t="s">
+      <c r="W2" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="X2" s="38" t="s">
+      <c r="X2" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="Y2" s="38" t="s">
+      <c r="Y2" s="37" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:25" s="43" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" s="42" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -23824,97 +23823,97 @@
     <col min="19" max="20" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="125" t="s">
+    <row r="1" spans="1:20" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="124" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="125" t="s">
+      <c r="B1" s="124" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="125" t="s">
+      <c r="C1" s="124" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="125" t="s">
+      <c r="D1" s="124" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="94" t="s">
+      <c r="E1" s="89" t="s">
         <v>174</v>
       </c>
-      <c r="F1" s="94" t="s">
+      <c r="F1" s="89" t="s">
         <v>175</v>
       </c>
-      <c r="G1" s="94" t="s">
+      <c r="G1" s="89" t="s">
         <v>176</v>
       </c>
-      <c r="H1" s="90" t="s">
+      <c r="H1" s="105" t="s">
         <v>177</v>
       </c>
-      <c r="I1" s="79" t="s">
+      <c r="I1" s="78" t="s">
         <v>69</v>
       </c>
-      <c r="J1" s="80"/>
-      <c r="K1" s="76" t="s">
+      <c r="J1" s="79"/>
+      <c r="K1" s="75" t="s">
         <v>70</v>
       </c>
-      <c r="L1" s="78"/>
-      <c r="M1" s="90" t="s">
+      <c r="L1" s="77"/>
+      <c r="M1" s="105" t="s">
         <v>182</v>
       </c>
-      <c r="N1" s="127" t="s">
+      <c r="N1" s="126" t="s">
         <v>72</v>
       </c>
-      <c r="O1" s="127" t="s">
+      <c r="O1" s="126" t="s">
         <v>66</v>
       </c>
-      <c r="P1" s="90" t="s">
+      <c r="P1" s="105" t="s">
         <v>181</v>
       </c>
-      <c r="Q1" s="127" t="s">
+      <c r="Q1" s="126" t="s">
         <v>67</v>
       </c>
-      <c r="R1" s="127" t="s">
+      <c r="R1" s="126" t="s">
         <v>68</v>
       </c>
-      <c r="S1" s="82" t="s">
+      <c r="S1" s="81" t="s">
         <v>191</v>
       </c>
-      <c r="T1" s="82"/>
-    </row>
-    <row r="2" spans="1:20" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="126"/>
-      <c r="B2" s="126"/>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="91"/>
-      <c r="I2" s="38" t="s">
+      <c r="T1" s="81"/>
+    </row>
+    <row r="2" spans="1:20" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="125"/>
+      <c r="B2" s="125"/>
+      <c r="C2" s="125"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="106"/>
+      <c r="I2" s="37" t="s">
         <v>178</v>
       </c>
-      <c r="J2" s="38" t="s">
+      <c r="J2" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="44" t="s">
+      <c r="K2" s="43" t="s">
         <v>193</v>
       </c>
-      <c r="L2" s="35" t="s">
+      <c r="L2" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="M2" s="91"/>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
-      <c r="P2" s="91"/>
-      <c r="Q2" s="82"/>
-      <c r="R2" s="82"/>
-      <c r="S2" s="38" t="s">
+      <c r="M2" s="106"/>
+      <c r="N2" s="81"/>
+      <c r="O2" s="81"/>
+      <c r="P2" s="106"/>
+      <c r="Q2" s="81"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="T2" s="38" t="s">
+      <c r="T2" s="37" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:20" s="43" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" s="42" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -28375,55 +28374,55 @@
     <col min="11" max="11" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+    <row r="1" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="49" t="s">
+      <c r="B1" s="48" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="49" t="s">
+      <c r="C1" s="48" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="49" t="s">
+      <c r="D1" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="G1" s="38" t="s">
+      <c r="G1" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="35" t="s">
+      <c r="H1" s="34" t="s">
         <v>251</v>
       </c>
-      <c r="I1" s="35" t="s">
+      <c r="I1" s="34" t="s">
         <v>252</v>
       </c>
-      <c r="J1" s="35" t="s">
+      <c r="J1" s="34" t="s">
         <v>110</v>
       </c>
-      <c r="K1" s="35" t="s">
+      <c r="K1" s="34" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45"/>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-    </row>
-    <row r="3" spans="1:11" s="41" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="44"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+    </row>
+    <row r="3" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -31059,180 +31058,180 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="68" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="70" t="s">
+      <c r="B1" s="69" t="s">
         <v>156</v>
       </c>
-      <c r="C1" s="70"/>
-      <c r="D1" s="82" t="s">
+      <c r="C1" s="69"/>
+      <c r="D1" s="81" t="s">
         <v>157</v>
       </c>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="M1" s="82"/>
-      <c r="N1" s="73" t="s">
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="81"/>
+      <c r="I1" s="81"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="81"/>
+      <c r="L1" s="81"/>
+      <c r="M1" s="81"/>
+      <c r="N1" s="72" t="s">
         <v>210</v>
       </c>
-      <c r="O1" s="74"/>
-      <c r="P1" s="74"/>
-      <c r="Q1" s="74"/>
-      <c r="R1" s="74"/>
-      <c r="S1" s="74"/>
-      <c r="T1" s="74"/>
-      <c r="U1" s="74"/>
-      <c r="V1" s="74"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="75"/>
-      <c r="Y1" s="41"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
+      <c r="Q1" s="73"/>
+      <c r="R1" s="73"/>
+      <c r="S1" s="73"/>
+      <c r="T1" s="73"/>
+      <c r="U1" s="73"/>
+      <c r="V1" s="73"/>
+      <c r="W1" s="73"/>
+      <c r="X1" s="74"/>
+      <c r="Y1" s="40"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" s="69"/>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="83" t="s">
+      <c r="A2" s="68"/>
+      <c r="B2" s="80"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="82" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="84"/>
-      <c r="F2" s="84"/>
-      <c r="G2" s="84"/>
-      <c r="H2" s="87"/>
-      <c r="I2" s="83" t="s">
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="82" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="84"/>
-      <c r="K2" s="84"/>
-      <c r="L2" s="84"/>
-      <c r="M2" s="84"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="77"/>
-      <c r="P2" s="77"/>
-      <c r="Q2" s="77"/>
-      <c r="R2" s="77"/>
-      <c r="S2" s="77"/>
-      <c r="T2" s="77"/>
-      <c r="U2" s="77"/>
-      <c r="V2" s="77"/>
-      <c r="W2" s="77"/>
-      <c r="X2" s="78"/>
-      <c r="Y2" s="41"/>
+      <c r="J2" s="83"/>
+      <c r="K2" s="83"/>
+      <c r="L2" s="83"/>
+      <c r="M2" s="83"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="76"/>
+      <c r="P2" s="76"/>
+      <c r="Q2" s="76"/>
+      <c r="R2" s="76"/>
+      <c r="S2" s="76"/>
+      <c r="T2" s="76"/>
+      <c r="U2" s="76"/>
+      <c r="V2" s="76"/>
+      <c r="W2" s="76"/>
+      <c r="X2" s="77"/>
+      <c r="Y2" s="40"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="69"/>
-      <c r="B3" s="81"/>
-      <c r="C3" s="81"/>
-      <c r="D3" s="79" t="s">
+      <c r="A3" s="68"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="78" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="80"/>
-      <c r="F3" s="79" t="s">
+      <c r="E3" s="79"/>
+      <c r="F3" s="78" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="80"/>
-      <c r="H3" s="88" t="s">
+      <c r="G3" s="79"/>
+      <c r="H3" s="87" t="s">
         <v>81</v>
       </c>
-      <c r="I3" s="79" t="s">
+      <c r="I3" s="78" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="80"/>
-      <c r="K3" s="79" t="s">
+      <c r="J3" s="79"/>
+      <c r="K3" s="78" t="s">
         <v>74</v>
       </c>
-      <c r="L3" s="80"/>
-      <c r="M3" s="85" t="s">
+      <c r="L3" s="79"/>
+      <c r="M3" s="84" t="s">
         <v>81</v>
       </c>
-      <c r="N3" s="71" t="s">
+      <c r="N3" s="70" t="s">
         <v>233</v>
       </c>
-      <c r="O3" s="71"/>
-      <c r="P3" s="72" t="s">
+      <c r="O3" s="70"/>
+      <c r="P3" s="71" t="s">
         <v>231</v>
       </c>
-      <c r="Q3" s="72"/>
-      <c r="R3" s="72"/>
-      <c r="S3" s="72"/>
-      <c r="T3" s="72"/>
-      <c r="U3" s="72" t="s">
+      <c r="Q3" s="71"/>
+      <c r="R3" s="71"/>
+      <c r="S3" s="71"/>
+      <c r="T3" s="71"/>
+      <c r="U3" s="71" t="s">
         <v>232</v>
       </c>
-      <c r="V3" s="72"/>
-      <c r="W3" s="72"/>
-      <c r="X3" s="72"/>
-    </row>
-    <row r="4" spans="1:25" s="42" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="70"/>
-      <c r="B4" s="32" t="s">
+      <c r="V3" s="71"/>
+      <c r="W3" s="71"/>
+      <c r="X3" s="71"/>
+    </row>
+    <row r="4" spans="1:25" s="41" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="69"/>
+      <c r="B4" s="31" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="38" t="s">
+      <c r="E4" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="F4" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="35" t="s">
+      <c r="G4" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="82"/>
-      <c r="I4" s="38" t="s">
+      <c r="H4" s="81"/>
+      <c r="I4" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="J4" s="38" t="s">
+      <c r="J4" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="35" t="s">
+      <c r="K4" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="L4" s="35" t="s">
+      <c r="L4" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="M4" s="86"/>
-      <c r="N4" s="32" t="s">
+      <c r="M4" s="85"/>
+      <c r="N4" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="32" t="s">
+      <c r="O4" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="P4" s="35" t="s">
+      <c r="P4" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="Q4" s="35" t="s">
+      <c r="Q4" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="R4" s="35" t="s">
+      <c r="R4" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="S4" s="35" t="s">
+      <c r="S4" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="T4" s="35" t="s">
+      <c r="T4" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="U4" s="31" t="s">
+      <c r="U4" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="V4" s="31" t="s">
+      <c r="V4" s="30" t="s">
         <v>117</v>
       </c>
-      <c r="W4" s="31" t="s">
+      <c r="W4" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="X4" s="31" t="s">
+      <c r="X4" s="30" t="s">
         <v>119</v>
       </c>
     </row>
@@ -36476,102 +36475,102 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="100" t="s">
+      <c r="B1" s="95" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="102"/>
-      <c r="G1" s="96" t="s">
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="97"/>
-      <c r="I1" s="98"/>
-      <c r="J1" s="89" t="s">
+      <c r="H1" s="92"/>
+      <c r="I1" s="93"/>
+      <c r="J1" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="40" t="s">
+      <c r="K1" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="L1" s="100" t="s">
+      <c r="L1" s="95" t="s">
         <v>109</v>
       </c>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="102"/>
+      <c r="M1" s="96"/>
+      <c r="N1" s="96"/>
+      <c r="O1" s="96"/>
+      <c r="P1" s="97"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="69"/>
-      <c r="B2" s="81" t="s">
+      <c r="A2" s="68"/>
+      <c r="B2" s="80" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="106" t="s">
+      <c r="C2" s="102" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="107" t="s">
+      <c r="D2" s="103" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="88" t="s">
+      <c r="E2" s="87" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="92" t="s">
+      <c r="F2" s="98" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="103" t="s">
+      <c r="G2" s="99" t="s">
         <v>115</v>
       </c>
-      <c r="H2" s="104" t="s">
+      <c r="H2" s="100" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="99" t="s">
+      <c r="I2" s="94" t="s">
         <v>158</v>
       </c>
-      <c r="J2" s="90"/>
-      <c r="K2" s="94" t="s">
+      <c r="J2" s="105"/>
+      <c r="K2" s="89" t="s">
         <v>122</v>
       </c>
-      <c r="L2" s="71" t="s">
+      <c r="L2" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71" t="s">
+      <c r="M2" s="70"/>
+      <c r="N2" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="71"/>
-      <c r="P2" s="92" t="s">
+      <c r="O2" s="70"/>
+      <c r="P2" s="98" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="81"/>
-      <c r="C3" s="106"/>
-      <c r="D3" s="107"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="92"/>
-      <c r="G3" s="103"/>
-      <c r="H3" s="105"/>
-      <c r="I3" s="99"/>
-      <c r="J3" s="91"/>
-      <c r="K3" s="95"/>
-      <c r="L3" s="32" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="99"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="94"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="44" t="s">
+      <c r="M3" s="43" t="s">
         <v>230</v>
       </c>
-      <c r="N3" s="32" t="s">
+      <c r="N3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="44" t="s">
+      <c r="O3" s="43" t="s">
         <v>230</v>
       </c>
-      <c r="P3" s="92"/>
+      <c r="P3" s="98"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -40174,8 +40173,13 @@
       <c r="P203" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="yP1GbBCgAdm0CH/gr8AK4RsVM1gtv82RP3HgfmHP3L5tX6iCxw/IjCz2X6Q4KidklCbEORnuuGS+Q9kp+KNj3w==" saltValue="R0+mSYCgXyR4udjvNYppsg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="CVc9Y6zTViK+qNBvkHM6Vw9LbbIcQvJhEGHDobnK2WxxzdUIpXEi5D/0B5vCJa09eTPUkAUYi73wUk86TeXIgw==" saltValue="8ea3UICepsiuwTlX9cWVdA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="I2:I3"/>
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P2:P3"/>
@@ -40188,11 +40192,6 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="J1:J3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="I2:I3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 J4 K2:K3 G2:I3 O3" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40208,6 +40207,7 @@
     <hyperlink ref="H2" r:id="rId6" display="PORT_CODE" xr:uid="{C4D05E8A-B26C-4196-BF44-6883318591EB}"/>
     <hyperlink ref="K2:K3" r:id="rId7" location="gears" display="MAIN_FISHING_GEAR" xr:uid="{ADDD99C7-B692-4517-AF11-C5F4715C3781}"/>
     <hyperlink ref="H2:H3" r:id="rId8" location="Ports" display="PORT" xr:uid="{4BCE8909-E3DB-4961-B5C5-527D383D1926}"/>
+    <hyperlink ref="J1:J3" r:id="rId9" location="targetSpecies" display="LICENSED_TARGET_SPECIES" xr:uid="{8145BEA5-06D1-4F1F-890E-1ACE66463F94}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -40235,73 +40235,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="98" t="s">
         <v>211</v>
       </c>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92" t="s">
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98" t="s">
         <v>212</v>
       </c>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
+      <c r="H1" s="98"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="98"/>
+      <c r="K1" s="98"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="69"/>
-      <c r="B2" s="83" t="s">
+      <c r="A2" s="68"/>
+      <c r="B2" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="84"/>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="88" t="s">
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="87" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="83" t="s">
+      <c r="G2" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="84"/>
-      <c r="I2" s="84"/>
-      <c r="J2" s="87"/>
-      <c r="K2" s="88" t="s">
+      <c r="H2" s="83"/>
+      <c r="I2" s="83"/>
+      <c r="J2" s="86"/>
+      <c r="K2" s="87" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="38" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="38" t="s">
+      <c r="C3" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="39" t="s">
+      <c r="E3" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="82"/>
-      <c r="G3" s="38" t="s">
+      <c r="F3" s="81"/>
+      <c r="G3" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="H3" s="38" t="s">
+      <c r="H3" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="39" t="s">
+      <c r="I3" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="J3" s="39" t="s">
+      <c r="J3" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="82"/>
+      <c r="K3" s="81"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -42977,237 +42977,237 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="83" t="s">
+      <c r="B1" s="82" t="s">
         <v>171</v>
       </c>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="84"/>
-      <c r="M1" s="84"/>
-      <c r="N1" s="84"/>
-      <c r="O1" s="84"/>
-      <c r="P1" s="84"/>
-      <c r="Q1" s="84"/>
-      <c r="R1" s="84"/>
-      <c r="S1" s="84"/>
-      <c r="T1" s="87"/>
-      <c r="U1" s="83" t="s">
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
+      <c r="K1" s="83"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+      <c r="N1" s="83"/>
+      <c r="O1" s="83"/>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="83"/>
+      <c r="R1" s="83"/>
+      <c r="S1" s="83"/>
+      <c r="T1" s="86"/>
+      <c r="U1" s="82" t="s">
         <v>213</v>
       </c>
-      <c r="V1" s="84"/>
-      <c r="W1" s="84"/>
-      <c r="X1" s="84"/>
-      <c r="Y1" s="84"/>
-      <c r="Z1" s="84"/>
-      <c r="AA1" s="84"/>
-      <c r="AB1" s="84"/>
-      <c r="AC1" s="84"/>
-      <c r="AD1" s="84"/>
-      <c r="AE1" s="84"/>
-      <c r="AF1" s="84"/>
-      <c r="AG1" s="87"/>
-      <c r="AH1" s="83" t="s">
+      <c r="V1" s="83"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="83"/>
+      <c r="AF1" s="83"/>
+      <c r="AG1" s="86"/>
+      <c r="AH1" s="82" t="s">
         <v>214</v>
       </c>
-      <c r="AI1" s="84"/>
-      <c r="AJ1" s="84"/>
-      <c r="AK1" s="84"/>
-      <c r="AL1" s="84"/>
-      <c r="AM1" s="84"/>
-      <c r="AN1" s="84"/>
-      <c r="AO1" s="87"/>
+      <c r="AI1" s="83"/>
+      <c r="AJ1" s="83"/>
+      <c r="AK1" s="83"/>
+      <c r="AL1" s="83"/>
+      <c r="AM1" s="83"/>
+      <c r="AN1" s="83"/>
+      <c r="AO1" s="86"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A2" s="69"/>
-      <c r="B2" s="88" t="s">
+      <c r="A2" s="68"/>
+      <c r="B2" s="87" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="88" t="s">
+      <c r="C2" s="87" t="s">
         <v>125</v>
       </c>
-      <c r="D2" s="89" t="s">
+      <c r="D2" s="104" t="s">
         <v>126</v>
       </c>
-      <c r="E2" s="72" t="s">
+      <c r="E2" s="71" t="s">
         <v>172</v>
       </c>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72" t="s">
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71" t="s">
         <v>173</v>
       </c>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="88" t="s">
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="87" t="s">
         <v>155</v>
       </c>
-      <c r="L2" s="72" t="s">
+      <c r="L2" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="72"/>
-      <c r="N2" s="72"/>
-      <c r="O2" s="72"/>
-      <c r="P2" s="72" t="s">
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="71" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="72"/>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72" t="s">
+      <c r="Q2" s="71"/>
+      <c r="R2" s="71"/>
+      <c r="S2" s="71" t="s">
         <v>27</v>
       </c>
-      <c r="T2" s="72"/>
-      <c r="U2" s="92" t="s">
+      <c r="T2" s="71"/>
+      <c r="U2" s="98" t="s">
         <v>136</v>
       </c>
-      <c r="V2" s="92" t="s">
+      <c r="V2" s="98" t="s">
         <v>29</v>
       </c>
-      <c r="W2" s="92" t="s">
+      <c r="W2" s="98" t="s">
         <v>39</v>
       </c>
-      <c r="X2" s="92" t="s">
+      <c r="X2" s="98" t="s">
         <v>30</v>
       </c>
-      <c r="Y2" s="92" t="s">
+      <c r="Y2" s="98" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="92" t="s">
+      <c r="Z2" s="98" t="s">
         <v>32</v>
       </c>
-      <c r="AA2" s="92" t="s">
+      <c r="AA2" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="AB2" s="92" t="s">
+      <c r="AB2" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="AC2" s="92" t="s">
+      <c r="AC2" s="98" t="s">
         <v>35</v>
       </c>
-      <c r="AD2" s="92" t="s">
+      <c r="AD2" s="98" t="s">
         <v>36</v>
       </c>
-      <c r="AE2" s="92" t="s">
+      <c r="AE2" s="98" t="s">
         <v>37</v>
       </c>
-      <c r="AF2" s="92" t="s">
+      <c r="AF2" s="98" t="s">
         <v>128</v>
       </c>
-      <c r="AG2" s="92" t="s">
+      <c r="AG2" s="98" t="s">
         <v>38</v>
       </c>
-      <c r="AH2" s="96" t="s">
+      <c r="AH2" s="91" t="s">
         <v>215</v>
       </c>
-      <c r="AI2" s="98"/>
-      <c r="AJ2" s="72" t="s">
+      <c r="AI2" s="93"/>
+      <c r="AJ2" s="71" t="s">
         <v>216</v>
       </c>
-      <c r="AK2" s="72"/>
-      <c r="AL2" s="72" t="s">
+      <c r="AK2" s="71"/>
+      <c r="AL2" s="71" t="s">
         <v>217</v>
       </c>
-      <c r="AM2" s="72"/>
-      <c r="AN2" s="72" t="s">
+      <c r="AM2" s="71"/>
+      <c r="AN2" s="71" t="s">
         <v>218</v>
       </c>
-      <c r="AO2" s="72"/>
+      <c r="AO2" s="71"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="91"/>
-      <c r="E3" s="34" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="81"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="106"/>
+      <c r="E3" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="34" t="s">
+      <c r="F3" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="37" t="s">
+      <c r="G3" s="36" t="s">
         <v>123</v>
       </c>
-      <c r="H3" s="34" t="s">
+      <c r="H3" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="34" t="s">
+      <c r="I3" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="37" t="s">
+      <c r="J3" s="36" t="s">
         <v>123</v>
       </c>
-      <c r="K3" s="82"/>
-      <c r="L3" s="31" t="s">
+      <c r="K3" s="81"/>
+      <c r="L3" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="M3" s="31" t="s">
+      <c r="M3" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="N3" s="31" t="s">
+      <c r="N3" s="30" t="s">
         <v>131</v>
       </c>
-      <c r="O3" s="31" t="s">
+      <c r="O3" s="30" t="s">
         <v>132</v>
       </c>
-      <c r="P3" s="31" t="s">
+      <c r="P3" s="30" t="s">
         <v>133</v>
       </c>
-      <c r="Q3" s="31" t="s">
+      <c r="Q3" s="30" t="s">
         <v>134</v>
       </c>
-      <c r="R3" s="31" t="s">
+      <c r="R3" s="30" t="s">
         <v>135</v>
       </c>
-      <c r="S3" s="34" t="s">
+      <c r="S3" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="T3" s="37" t="s">
+      <c r="T3" s="36" t="s">
         <v>129</v>
       </c>
-      <c r="U3" s="92"/>
-      <c r="V3" s="92"/>
-      <c r="W3" s="92"/>
-      <c r="X3" s="92"/>
-      <c r="Y3" s="92"/>
-      <c r="Z3" s="92"/>
-      <c r="AA3" s="92"/>
-      <c r="AB3" s="92"/>
-      <c r="AC3" s="92"/>
-      <c r="AD3" s="92"/>
-      <c r="AE3" s="92"/>
-      <c r="AF3" s="92"/>
-      <c r="AG3" s="92"/>
-      <c r="AH3" s="31" t="s">
+      <c r="U3" s="98"/>
+      <c r="V3" s="98"/>
+      <c r="W3" s="98"/>
+      <c r="X3" s="98"/>
+      <c r="Y3" s="98"/>
+      <c r="Z3" s="98"/>
+      <c r="AA3" s="98"/>
+      <c r="AB3" s="98"/>
+      <c r="AC3" s="98"/>
+      <c r="AD3" s="98"/>
+      <c r="AE3" s="98"/>
+      <c r="AF3" s="98"/>
+      <c r="AG3" s="98"/>
+      <c r="AH3" s="30" t="s">
         <v>137</v>
       </c>
-      <c r="AI3" s="31" t="s">
+      <c r="AI3" s="30" t="s">
         <v>138</v>
       </c>
-      <c r="AJ3" s="31" t="s">
+      <c r="AJ3" s="30" t="s">
         <v>139</v>
       </c>
-      <c r="AK3" s="31" t="s">
+      <c r="AK3" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="AL3" s="31" t="s">
+      <c r="AL3" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="AM3" s="31" t="s">
+      <c r="AM3" s="30" t="s">
         <v>142</v>
       </c>
-      <c r="AN3" s="31" t="s">
+      <c r="AN3" s="30" t="s">
         <v>143</v>
       </c>
-      <c r="AO3" s="31" t="s">
+      <c r="AO3" s="30" t="s">
         <v>144</v>
       </c>
     </row>
@@ -51887,30 +51887,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="81" t="s">
+      <c r="B1" s="80" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="70"/>
-      <c r="B2" s="32" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="31" t="s">
         <v>165</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="31" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
-      <c r="B3" s="30"/>
+      <c r="B3" s="29"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
     </row>
@@ -53139,50 +53139,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="98" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="83" t="s">
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="82" t="s">
         <v>206</v>
       </c>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="87"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="86"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="70"/>
-      <c r="B2" s="50" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="49" t="s">
         <v>145</v>
       </c>
-      <c r="C2" s="50" t="s">
+      <c r="C2" s="49" t="s">
         <v>146</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="37" t="s">
         <v>147</v>
       </c>
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="34" t="s">
         <v>152</v>
       </c>
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="51" t="s">
         <v>153</v>
       </c>
-      <c r="G2" s="33" t="s">
+      <c r="G2" s="32" t="s">
         <v>148</v>
       </c>
-      <c r="H2" s="33" t="s">
+      <c r="H2" s="32" t="s">
         <v>149</v>
       </c>
-      <c r="I2" s="33" t="s">
+      <c r="I2" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="J2" s="54" t="s">
+      <c r="J2" s="53" t="s">
         <v>151</v>
       </c>
     </row>
@@ -55630,96 +55630,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="108" t="s">
+      <c r="B1" s="107" t="s">
         <v>159</v>
       </c>
-      <c r="C1" s="109"/>
-      <c r="D1" s="109"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="109"/>
-      <c r="G1" s="109"/>
-      <c r="H1" s="109"/>
-      <c r="I1" s="109"/>
-      <c r="J1" s="109"/>
-      <c r="K1" s="110"/>
-      <c r="L1" s="111" t="s">
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="109"/>
+      <c r="L1" s="110" t="s">
         <v>219</v>
       </c>
-      <c r="M1" s="112"/>
-      <c r="N1" s="112"/>
-      <c r="O1" s="112"/>
-      <c r="P1" s="113"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
+      <c r="P1" s="112"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="69"/>
-      <c r="B2" s="93" t="s">
+      <c r="A2" s="68"/>
+      <c r="B2" s="88" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="100" t="s">
+      <c r="C2" s="95" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="88" t="s">
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="87" t="s">
         <v>162</v>
       </c>
-      <c r="I2" s="93" t="s">
+      <c r="I2" s="88" t="s">
         <v>163</v>
       </c>
-      <c r="J2" s="83" t="s">
+      <c r="J2" s="82" t="s">
         <v>220</v>
       </c>
-      <c r="K2" s="87"/>
-      <c r="L2" s="79"/>
-      <c r="M2" s="114"/>
-      <c r="N2" s="114"/>
-      <c r="O2" s="114"/>
-      <c r="P2" s="80"/>
+      <c r="K2" s="86"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="113"/>
+      <c r="N2" s="113"/>
+      <c r="O2" s="113"/>
+      <c r="P2" s="79"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="70"/>
-      <c r="C3" s="56" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="51" t="s">
+      <c r="E3" s="50" t="s">
         <v>160</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="G3" s="51" t="s">
+      <c r="G3" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="82"/>
-      <c r="I3" s="70"/>
-      <c r="J3" s="57" t="s">
+      <c r="H3" s="81"/>
+      <c r="I3" s="69"/>
+      <c r="J3" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="57" t="s">
+      <c r="K3" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="58" t="s">
+      <c r="L3" s="57" t="s">
         <v>164</v>
       </c>
-      <c r="M3" s="33" t="s">
+      <c r="M3" s="32" t="s">
         <v>166</v>
       </c>
-      <c r="N3" s="33" t="s">
+      <c r="N3" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="O3" s="33" t="s">
+      <c r="O3" s="32" t="s">
         <v>168</v>
       </c>
-      <c r="P3" s="33" t="s">
+      <c r="P3" s="32" t="s">
         <v>169</v>
       </c>
     </row>
@@ -59389,181 +59389,181 @@
     <col min="27" max="30" width="15.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="93" t="s">
+    <row r="1" spans="1:30" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="81" t="s">
+      <c r="C1" s="80" t="s">
         <v>77</v>
       </c>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="108" t="s">
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="107" t="s">
         <v>78</v>
       </c>
-      <c r="G1" s="109"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="93" t="s">
+      <c r="G1" s="108"/>
+      <c r="H1" s="109"/>
+      <c r="I1" s="88" t="s">
         <v>236</v>
       </c>
-      <c r="J1" s="93" t="s">
+      <c r="J1" s="88" t="s">
         <v>237</v>
       </c>
-      <c r="K1" s="111" t="s">
+      <c r="K1" s="110" t="s">
         <v>42</v>
       </c>
-      <c r="L1" s="112"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="111" t="s">
+      <c r="L1" s="111"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="110" t="s">
         <v>49</v>
       </c>
-      <c r="O1" s="113"/>
-      <c r="P1" s="81" t="s">
+      <c r="O1" s="112"/>
+      <c r="P1" s="80" t="s">
         <v>238</v>
       </c>
-      <c r="Q1" s="92" t="s">
+      <c r="Q1" s="98" t="s">
         <v>239</v>
       </c>
-      <c r="R1" s="81" t="s">
+      <c r="R1" s="80" t="s">
         <v>240</v>
       </c>
-      <c r="S1" s="81" t="s">
+      <c r="S1" s="80" t="s">
         <v>246</v>
       </c>
-      <c r="T1" s="81"/>
-      <c r="U1" s="115" t="s">
+      <c r="T1" s="80"/>
+      <c r="U1" s="114" t="s">
         <v>247</v>
       </c>
-      <c r="V1" s="116"/>
-      <c r="W1" s="115" t="s">
+      <c r="V1" s="115"/>
+      <c r="W1" s="114" t="s">
         <v>248</v>
       </c>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="115" t="s">
+      <c r="X1" s="115"/>
+      <c r="Y1" s="114" t="s">
         <v>249</v>
       </c>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="81" t="s">
+      <c r="Z1" s="115"/>
+      <c r="AA1" s="80" t="s">
         <v>245</v>
       </c>
-      <c r="AB1" s="81"/>
-      <c r="AC1" s="81"/>
-      <c r="AD1" s="81"/>
-    </row>
-    <row r="2" spans="1:30" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="69"/>
-      <c r="B2" s="69"/>
-      <c r="C2" s="73" t="s">
+      <c r="AB1" s="80"/>
+      <c r="AC1" s="80"/>
+      <c r="AD1" s="80"/>
+    </row>
+    <row r="2" spans="1:30" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="68"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="72" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="108" t="s">
+      <c r="D2" s="107" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="110"/>
-      <c r="F2" s="93" t="s">
+      <c r="E2" s="109"/>
+      <c r="F2" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="108" t="s">
+      <c r="G2" s="107" t="s">
         <v>79</v>
       </c>
-      <c r="H2" s="110"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="114"/>
-      <c r="M2" s="80"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="80"/>
-      <c r="P2" s="81"/>
-      <c r="Q2" s="92"/>
-      <c r="R2" s="81"/>
-      <c r="S2" s="81"/>
-      <c r="T2" s="81"/>
-      <c r="U2" s="76"/>
-      <c r="V2" s="78"/>
-      <c r="W2" s="76"/>
-      <c r="X2" s="78"/>
-      <c r="Y2" s="76"/>
-      <c r="Z2" s="78"/>
-      <c r="AA2" s="81"/>
-      <c r="AB2" s="81"/>
-      <c r="AC2" s="81"/>
-      <c r="AD2" s="81"/>
-    </row>
-    <row r="3" spans="1:30" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="70"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="32" t="s">
+      <c r="H2" s="109"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="113"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="78"/>
+      <c r="O2" s="79"/>
+      <c r="P2" s="80"/>
+      <c r="Q2" s="98"/>
+      <c r="R2" s="80"/>
+      <c r="S2" s="80"/>
+      <c r="T2" s="80"/>
+      <c r="U2" s="75"/>
+      <c r="V2" s="77"/>
+      <c r="W2" s="75"/>
+      <c r="X2" s="77"/>
+      <c r="Y2" s="75"/>
+      <c r="Z2" s="77"/>
+      <c r="AA2" s="80"/>
+      <c r="AB2" s="80"/>
+      <c r="AC2" s="80"/>
+      <c r="AD2" s="80"/>
+    </row>
+    <row r="3" spans="1:30" s="42" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="69"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="32" t="s">
+      <c r="E3" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="70"/>
-      <c r="G3" s="32" t="s">
+      <c r="F3" s="69"/>
+      <c r="G3" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="32" t="s">
+      <c r="H3" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="70"/>
-      <c r="J3" s="70"/>
-      <c r="K3" s="38" t="s">
+      <c r="I3" s="69"/>
+      <c r="J3" s="69"/>
+      <c r="K3" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="L3" s="35" t="s">
+      <c r="L3" s="34" t="s">
         <v>234</v>
       </c>
-      <c r="M3" s="47" t="s">
+      <c r="M3" s="46" t="s">
         <v>235</v>
       </c>
-      <c r="N3" s="35" t="s">
+      <c r="N3" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="O3" s="35" t="s">
+      <c r="O3" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="92"/>
-      <c r="R3" s="81"/>
-      <c r="S3" s="32" t="s">
+      <c r="P3" s="80"/>
+      <c r="Q3" s="98"/>
+      <c r="R3" s="80"/>
+      <c r="S3" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="T3" s="35" t="s">
+      <c r="T3" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="U3" s="32" t="s">
+      <c r="U3" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="V3" s="32" t="s">
+      <c r="V3" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="W3" s="32" t="s">
+      <c r="W3" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="X3" s="32" t="s">
+      <c r="X3" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="Y3" s="32" t="s">
+      <c r="Y3" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="32" t="s">
+      <c r="Z3" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="AA3" s="44" t="s">
+      <c r="AA3" s="43" t="s">
         <v>241</v>
       </c>
-      <c r="AB3" s="38" t="s">
+      <c r="AB3" s="37" t="s">
         <v>242</v>
       </c>
-      <c r="AC3" s="38" t="s">
+      <c r="AC3" s="37" t="s">
         <v>243</v>
       </c>
-      <c r="AD3" s="38" t="s">
+      <c r="AD3" s="37" t="s">
         <v>244</v>
       </c>
     </row>
@@ -65942,11 +65942,12 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="9xCUSnOba9+kjRTP4aA+IhYIhPNTdofqr3mLiTZOPQAzcWWZifDmPOI/0ItUaLA4hSjA/rC4jIft53nJzygclQ==" saltValue="aTfUQq44C7asIKTaLqEvww==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="I1:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="N1:O2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
     <mergeCell ref="Y1:Z2"/>
     <mergeCell ref="AA1:AD2"/>
     <mergeCell ref="U1:V2"/>
@@ -65956,12 +65957,11 @@
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="R1:R3"/>
     <mergeCell ref="S1:T2"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="N1:O2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3 AA3:AD3" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">

</xml_diff>

<commit_message>
updating code lists E-SET - target species - code list changed to "all species" V-INFO - liscence target species - changed to "all species"
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_reporting_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30757A4F-25A2-024E-9738-058DEC4BF661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB19908E-E8C6-2F49-8A36-62E01249F779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="20600" windowHeight="16740" tabRatio="879" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="24680" windowHeight="16680" tabRatio="879" firstSheet="5" activeTab="8" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -1444,6 +1444,30 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1484,30 +1508,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -3678,31 +3678,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="89" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="101" t="s">
+      <c r="C1" s="89" t="s">
         <v>228</v>
       </c>
-      <c r="D1" s="101" t="s">
+      <c r="D1" s="89" t="s">
         <v>229</v>
       </c>
       <c r="E1" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="101" t="s">
+      <c r="F1" s="89" t="s">
         <v>250</v>
       </c>
-      <c r="G1" s="101" t="s">
+      <c r="G1" s="89" t="s">
         <v>227</v>
       </c>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="89" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="89" t="s">
         <v>93</v>
       </c>
       <c r="J1" s="83" t="s">
@@ -7147,17 +7147,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="i4Y2GDra9B4e5ZK9IT/yAgpGu83ed66ZNnyRoFvCqT5wVfLy2Lgs30SlszSGdCdYRpnULwm3Kg2BGFX0NXPahA==" saltValue="poZcuJUx5RFD549VWAk8zg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
-    <mergeCell ref="L1:O1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="E1:E2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="I1:I2"/>
+    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 M2 N2 O2" xr:uid="{35387E2C-FBDF-4B0A-A0B5-EF76A6744ABB}">
@@ -7190,10 +7190,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="89" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -8645,10 +8645,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="89" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -10319,10 +10319,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="89" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -10335,15 +10335,15 @@
       </c>
       <c r="G1" s="109"/>
       <c r="H1" s="110"/>
-      <c r="I1" s="93" t="s">
+      <c r="I1" s="100" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="92" t="s">
+      <c r="J1" s="99" t="s">
         <v>195</v>
       </c>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
+      <c r="K1" s="99"/>
+      <c r="L1" s="99"/>
+      <c r="M1" s="99"/>
       <c r="N1" s="81" t="s">
         <v>57</v>
       </c>
@@ -10360,25 +10360,25 @@
     <row r="2" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
       <c r="B2" s="69"/>
-      <c r="C2" s="101" t="s">
+      <c r="C2" s="89" t="s">
         <v>81</v>
       </c>
       <c r="D2" s="108" t="s">
         <v>79</v>
       </c>
       <c r="E2" s="110"/>
-      <c r="F2" s="101" t="s">
+      <c r="F2" s="89" t="s">
         <v>81</v>
       </c>
       <c r="G2" s="108" t="s">
         <v>79</v>
       </c>
       <c r="H2" s="110"/>
-      <c r="I2" s="93"/>
-      <c r="J2" s="92"/>
-      <c r="K2" s="92"/>
-      <c r="L2" s="92"/>
-      <c r="M2" s="92"/>
+      <c r="I2" s="100"/>
+      <c r="J2" s="99"/>
+      <c r="K2" s="99"/>
+      <c r="L2" s="99"/>
+      <c r="M2" s="99"/>
       <c r="N2" s="81"/>
       <c r="O2" s="81"/>
       <c r="P2" s="119"/>
@@ -10401,7 +10401,7 @@
       <c r="H3" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="93"/>
+      <c r="I3" s="100"/>
       <c r="J3" s="37" t="s">
         <v>194</v>
       </c>
@@ -14222,11 +14222,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="XFozxK9hJMWP6ySEAZQ3h3enG2BhQeHoAidLHumULHWCGWuk01gbtIGf+HTrIiPiIpU+5yeeijnd0s/LDXPnUw==" saltValue="w5vF1VniVgRmNU/Yweiy+Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C1:E1"/>
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="O1:O3"/>
     <mergeCell ref="F1:H1"/>
@@ -14236,6 +14231,11 @@
     <mergeCell ref="J1:M2"/>
     <mergeCell ref="N1:N3"/>
     <mergeCell ref="P1:P3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C1:E1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I3 M3 J3 K3 L3 Q1:Q3" xr:uid="{2FBCC481-6114-481E-B036-95624C9F7883}">
@@ -14269,10 +14269,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="89" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="83" t="s">
@@ -15522,13 +15522,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="89" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="101" t="s">
+      <c r="C1" s="89" t="s">
         <v>94</v>
       </c>
       <c r="D1" s="121" t="s">
@@ -15538,10 +15538,10 @@
         <v>89</v>
       </c>
       <c r="F1" s="124"/>
-      <c r="G1" s="102" t="s">
+      <c r="G1" s="90" t="s">
         <v>184</v>
       </c>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="89" t="s">
         <v>209</v>
       </c>
       <c r="I1" s="83" t="s">
@@ -15561,7 +15561,7 @@
       <c r="F2" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="103"/>
+      <c r="G2" s="91"/>
       <c r="H2" s="70"/>
       <c r="I2" s="37" t="s">
         <v>186</v>
@@ -18251,10 +18251,10 @@
       <c r="D1" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="102" t="s">
+      <c r="E1" s="90" t="s">
         <v>183</v>
       </c>
-      <c r="F1" s="102" t="s">
+      <c r="F1" s="90" t="s">
         <v>184</v>
       </c>
       <c r="G1" s="81" t="s">
@@ -18263,18 +18263,18 @@
       <c r="H1" s="81"/>
       <c r="I1" s="81"/>
       <c r="J1" s="81"/>
-      <c r="K1" s="92" t="s">
+      <c r="K1" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92" t="s">
+      <c r="L1" s="99"/>
+      <c r="M1" s="99"/>
+      <c r="N1" s="99"/>
+      <c r="O1" s="99" t="s">
         <v>58</v>
       </c>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="98" t="s">
+      <c r="P1" s="99"/>
+      <c r="Q1" s="99"/>
+      <c r="R1" s="105" t="s">
         <v>61</v>
       </c>
       <c r="S1" s="83" t="s">
@@ -18286,18 +18286,18 @@
       </c>
       <c r="V1" s="84"/>
       <c r="W1" s="87"/>
-      <c r="X1" s="92" t="s">
+      <c r="X1" s="99" t="s">
         <v>191</v>
       </c>
-      <c r="Y1" s="92"/>
+      <c r="Y1" s="99"/>
     </row>
     <row r="2" spans="1:25" s="42" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="126"/>
       <c r="B2" s="126"/>
       <c r="C2" s="126"/>
       <c r="D2" s="126"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
       <c r="G2" s="43" t="s">
         <v>23</v>
       </c>
@@ -18331,7 +18331,7 @@
       <c r="Q2" s="37" t="s">
         <v>204</v>
       </c>
-      <c r="R2" s="100"/>
+      <c r="R2" s="107"/>
       <c r="S2" s="35" t="s">
         <v>85</v>
       </c>
@@ -23835,16 +23835,16 @@
       <c r="D1" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="102" t="s">
+      <c r="E1" s="90" t="s">
         <v>174</v>
       </c>
-      <c r="F1" s="102" t="s">
+      <c r="F1" s="90" t="s">
         <v>175</v>
       </c>
-      <c r="G1" s="102" t="s">
+      <c r="G1" s="90" t="s">
         <v>176</v>
       </c>
-      <c r="H1" s="99" t="s">
+      <c r="H1" s="106" t="s">
         <v>177</v>
       </c>
       <c r="I1" s="79" t="s">
@@ -23855,7 +23855,7 @@
         <v>70</v>
       </c>
       <c r="L1" s="78"/>
-      <c r="M1" s="99" t="s">
+      <c r="M1" s="106" t="s">
         <v>182</v>
       </c>
       <c r="N1" s="127" t="s">
@@ -23864,7 +23864,7 @@
       <c r="O1" s="127" t="s">
         <v>66</v>
       </c>
-      <c r="P1" s="99" t="s">
+      <c r="P1" s="106" t="s">
         <v>181</v>
       </c>
       <c r="Q1" s="127" t="s">
@@ -23883,10 +23883,10 @@
       <c r="B2" s="126"/>
       <c r="C2" s="126"/>
       <c r="D2" s="126"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="103"/>
-      <c r="H2" s="100"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="107"/>
       <c r="I2" s="37" t="s">
         <v>178</v>
       </c>
@@ -23899,10 +23899,10 @@
       <c r="L2" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="M2" s="100"/>
+      <c r="M2" s="107"/>
       <c r="N2" s="82"/>
       <c r="O2" s="82"/>
-      <c r="P2" s="100"/>
+      <c r="P2" s="107"/>
       <c r="Q2" s="82"/>
       <c r="R2" s="82"/>
       <c r="S2" s="37" t="s">
@@ -28315,6 +28315,16 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="l8KVIJiIcXBtA5Rxt+oHSTZCQcSscxoVEx71fajOPkkDzIq7y1m1u1pHAE+AUnT93CwTnM5PkUuxYj42pmVV9g==" saltValue="dsO/0LEKtl67ZZqtPejb6A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="O1:O2"/>
     <mergeCell ref="P1:P2"/>
     <mergeCell ref="S1:T1"/>
     <mergeCell ref="H1:H2"/>
@@ -28322,16 +28332,6 @@
     <mergeCell ref="R1:R2"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="K1:L1"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="N1:N2"/>
-    <mergeCell ref="O1:O2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F2 H1:H2 P1:P2 S2 J2 E1:E2 G1:G2 I2 M1:M2 T2" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -36474,63 +36474,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="96" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="104" t="s">
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="92" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="105"/>
-      <c r="I1" s="106"/>
-      <c r="J1" s="98" t="s">
+      <c r="H1" s="93"/>
+      <c r="I1" s="94"/>
+      <c r="J1" s="105" t="s">
         <v>17</v>
       </c>
       <c r="K1" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="L1" s="89" t="s">
+      <c r="L1" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="91"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="98"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
       <c r="B2" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="96" t="s">
+      <c r="C2" s="103" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="97" t="s">
+      <c r="D2" s="104" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="92" t="s">
+      <c r="F2" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="93" t="s">
+      <c r="G2" s="100" t="s">
         <v>115</v>
       </c>
-      <c r="H2" s="94" t="s">
+      <c r="H2" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="107" t="s">
+      <c r="I2" s="95" t="s">
         <v>158</v>
       </c>
-      <c r="J2" s="99"/>
-      <c r="K2" s="102" t="s">
+      <c r="J2" s="106"/>
+      <c r="K2" s="90" t="s">
         <v>122</v>
       </c>
       <c r="L2" s="71" t="s">
@@ -36541,22 +36541,22 @@
         <v>19</v>
       </c>
       <c r="O2" s="71"/>
-      <c r="P2" s="92" t="s">
+      <c r="P2" s="99" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="70"/>
       <c r="B3" s="81"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="97"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="104"/>
       <c r="E3" s="82"/>
-      <c r="F3" s="92"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="95"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="103"/>
+      <c r="F3" s="99"/>
+      <c r="G3" s="100"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="95"/>
+      <c r="J3" s="107"/>
+      <c r="K3" s="91"/>
       <c r="L3" s="31" t="s">
         <v>3</v>
       </c>
@@ -36569,7 +36569,7 @@
       <c r="O3" s="43" t="s">
         <v>230</v>
       </c>
-      <c r="P3" s="92"/>
+      <c r="P3" s="99"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
@@ -40172,8 +40172,9 @@
       <c r="P203" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="CVc9Y6zTViK+qNBvkHM6Vw9LbbIcQvJhEGHDobnK2WxxzdUIpXEi5D/0B5vCJa09eTPUkAUYi73wUk86TeXIgw==" saltValue="8ea3UICepsiuwTlX9cWVdA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="CgzEmPt3Hk/Mhl0UL9A2LlPy9AK4yG5OneGJhJUq4FdJtqq7lG98GOjE3DOYWxyUk/x/OG6IB9bbOiXFzMXJrw==" saltValue="nv5eOc6x2cuQYecC/aOIFA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="F2:F3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="G1:I1"/>
@@ -40190,7 +40191,6 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="J1:J3"/>
-    <mergeCell ref="F2:F3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 J4 K2:K3 G2:I3 O3" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40206,7 +40206,7 @@
     <hyperlink ref="H2" r:id="rId6" display="PORT_CODE" xr:uid="{C4D05E8A-B26C-4196-BF44-6883318591EB}"/>
     <hyperlink ref="K2:K3" r:id="rId7" location="gears" display="MAIN_FISHING_GEAR" xr:uid="{ADDD99C7-B692-4517-AF11-C5F4715C3781}"/>
     <hyperlink ref="H2:H3" r:id="rId8" location="Ports" display="PORT" xr:uid="{4BCE8909-E3DB-4961-B5C5-527D383D1926}"/>
-    <hyperlink ref="J1:J3" r:id="rId9" location="targetSpecies" display="LICENSED_TARGET_SPECIES" xr:uid="{8145BEA5-06D1-4F1F-890E-1ACE66463F94}"/>
+    <hyperlink ref="J1:J3" r:id="rId9" location="allSpecies" display="LICENSED_TARGET_SPECIES" xr:uid="{8145BEA5-06D1-4F1F-890E-1ACE66463F94}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -40234,23 +40234,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="99" t="s">
         <v>211</v>
       </c>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92" t="s">
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99" t="s">
         <v>212</v>
       </c>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="99"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
@@ -42976,7 +42976,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="83" t="s">
@@ -43034,7 +43034,7 @@
       <c r="C2" s="88" t="s">
         <v>125</v>
       </c>
-      <c r="D2" s="98" t="s">
+      <c r="D2" s="105" t="s">
         <v>126</v>
       </c>
       <c r="E2" s="72" t="s">
@@ -43065,49 +43065,49 @@
         <v>27</v>
       </c>
       <c r="T2" s="72"/>
-      <c r="U2" s="92" t="s">
+      <c r="U2" s="99" t="s">
         <v>136</v>
       </c>
-      <c r="V2" s="92" t="s">
+      <c r="V2" s="99" t="s">
         <v>29</v>
       </c>
-      <c r="W2" s="92" t="s">
+      <c r="W2" s="99" t="s">
         <v>39</v>
       </c>
-      <c r="X2" s="92" t="s">
+      <c r="X2" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="Y2" s="92" t="s">
+      <c r="Y2" s="99" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="92" t="s">
+      <c r="Z2" s="99" t="s">
         <v>32</v>
       </c>
-      <c r="AA2" s="92" t="s">
+      <c r="AA2" s="99" t="s">
         <v>33</v>
       </c>
-      <c r="AB2" s="92" t="s">
+      <c r="AB2" s="99" t="s">
         <v>34</v>
       </c>
-      <c r="AC2" s="92" t="s">
+      <c r="AC2" s="99" t="s">
         <v>35</v>
       </c>
-      <c r="AD2" s="92" t="s">
+      <c r="AD2" s="99" t="s">
         <v>36</v>
       </c>
-      <c r="AE2" s="92" t="s">
+      <c r="AE2" s="99" t="s">
         <v>37</v>
       </c>
-      <c r="AF2" s="92" t="s">
+      <c r="AF2" s="99" t="s">
         <v>128</v>
       </c>
-      <c r="AG2" s="92" t="s">
+      <c r="AG2" s="99" t="s">
         <v>38</v>
       </c>
-      <c r="AH2" s="104" t="s">
+      <c r="AH2" s="92" t="s">
         <v>215</v>
       </c>
-      <c r="AI2" s="106"/>
+      <c r="AI2" s="94"/>
       <c r="AJ2" s="72" t="s">
         <v>216</v>
       </c>
@@ -43125,7 +43125,7 @@
       <c r="A3" s="70"/>
       <c r="B3" s="82"/>
       <c r="C3" s="82"/>
-      <c r="D3" s="100"/>
+      <c r="D3" s="107"/>
       <c r="E3" s="33" t="s">
         <v>24</v>
       </c>
@@ -43172,19 +43172,19 @@
       <c r="T3" s="36" t="s">
         <v>129</v>
       </c>
-      <c r="U3" s="92"/>
-      <c r="V3" s="92"/>
-      <c r="W3" s="92"/>
-      <c r="X3" s="92"/>
-      <c r="Y3" s="92"/>
-      <c r="Z3" s="92"/>
-      <c r="AA3" s="92"/>
-      <c r="AB3" s="92"/>
-      <c r="AC3" s="92"/>
-      <c r="AD3" s="92"/>
-      <c r="AE3" s="92"/>
-      <c r="AF3" s="92"/>
-      <c r="AG3" s="92"/>
+      <c r="U3" s="99"/>
+      <c r="V3" s="99"/>
+      <c r="W3" s="99"/>
+      <c r="X3" s="99"/>
+      <c r="Y3" s="99"/>
+      <c r="Z3" s="99"/>
+      <c r="AA3" s="99"/>
+      <c r="AB3" s="99"/>
+      <c r="AC3" s="99"/>
+      <c r="AD3" s="99"/>
+      <c r="AE3" s="99"/>
+      <c r="AF3" s="99"/>
+      <c r="AG3" s="99"/>
       <c r="AH3" s="30" t="s">
         <v>137</v>
       </c>
@@ -51813,20 +51813,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="wxJYPTS1M8YrpE+F5HXpzPvhVkWn+uzvbhQbX4zWGt7tgJJAc6rvipv1/0hraJgXbUY0X5vYRquC66cBDOGcbg==" saltValue="RWTcEymG3DdteXmtyGeu4A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="K2:K3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="U1:AG1"/>
@@ -51843,6 +51829,20 @@
     <mergeCell ref="AE2:AE3"/>
     <mergeCell ref="AD2:AD3"/>
     <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:V3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3 R3 AI3 AK3 AM3 L3 M3 N3 O3 P3 Q3 AO3 AJ3 AL3 AN3 AH3" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -51886,7 +51886,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="81" t="s">
@@ -53138,16 +53138,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="99" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
       <c r="G1" s="83" t="s">
         <v>206</v>
       </c>
@@ -55629,7 +55629,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="108" t="s">
@@ -55654,20 +55654,20 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
-      <c r="B2" s="101" t="s">
+      <c r="B2" s="89" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="89" t="s">
+      <c r="C2" s="96" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="91"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="98"/>
       <c r="H2" s="88" t="s">
         <v>162</v>
       </c>
-      <c r="I2" s="101" t="s">
+      <c r="I2" s="89" t="s">
         <v>163</v>
       </c>
       <c r="J2" s="83" t="s">
@@ -59389,10 +59389,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="89" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="81" t="s">
@@ -59405,10 +59405,10 @@
       </c>
       <c r="G1" s="109"/>
       <c r="H1" s="110"/>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="89" t="s">
         <v>236</v>
       </c>
-      <c r="J1" s="101" t="s">
+      <c r="J1" s="89" t="s">
         <v>237</v>
       </c>
       <c r="K1" s="111" t="s">
@@ -59423,7 +59423,7 @@
       <c r="P1" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="Q1" s="92" t="s">
+      <c r="Q1" s="99" t="s">
         <v>239</v>
       </c>
       <c r="R1" s="81" t="s">
@@ -59462,7 +59462,7 @@
         <v>79</v>
       </c>
       <c r="E2" s="110"/>
-      <c r="F2" s="101" t="s">
+      <c r="F2" s="89" t="s">
         <v>81</v>
       </c>
       <c r="G2" s="108" t="s">
@@ -59477,7 +59477,7 @@
       <c r="N2" s="79"/>
       <c r="O2" s="80"/>
       <c r="P2" s="81"/>
-      <c r="Q2" s="92"/>
+      <c r="Q2" s="99"/>
       <c r="R2" s="81"/>
       <c r="S2" s="81"/>
       <c r="T2" s="81"/>
@@ -59527,7 +59527,7 @@
         <v>48</v>
       </c>
       <c r="P3" s="81"/>
-      <c r="Q3" s="92"/>
+      <c r="Q3" s="99"/>
       <c r="R3" s="81"/>
       <c r="S3" s="31" t="s">
         <v>50</v>
@@ -65939,8 +65939,12 @@
       <c r="B203" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="9xCUSnOba9+kjRTP4aA+IhYIhPNTdofqr3mLiTZOPQAzcWWZifDmPOI/0ItUaLA4hSjA/rC4jIft53nJzygclQ==" saltValue="aTfUQq44C7asIKTaLqEvww==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="WuDPT1+slParW8lK5SfJrIiCuXUqugKfunXVVDY0YB00pOtHXcdvDQyUD/jzqYTc2x6TyFXXd8XFSXwF4cqxTw==" saltValue="kHXwsv450+CnM8/ussNlMw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="C1:E1"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:B3"/>
     <mergeCell ref="Y1:Z2"/>
@@ -65957,10 +65961,6 @@
     <mergeCell ref="N1:O2"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="C1:E1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3 AA3:AD3" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">
@@ -65968,10 +65968,10 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="AA3" r:id="rId1" location="targetSpecies" display="SPECIES_1_CODE" xr:uid="{2BC6450F-A7B4-4044-BEA6-59E54066E449}"/>
-    <hyperlink ref="AB3" r:id="rId2" location="targetSpecies" display="SPECIES_2_CODE" xr:uid="{9EEA8352-0631-4B4E-BB1B-FF880D8B8ED2}"/>
-    <hyperlink ref="AC3" r:id="rId3" location="targetSpecies" display="SPECIES_3_CODE" xr:uid="{B78A1E77-3003-40C6-9B0C-101A94179479}"/>
-    <hyperlink ref="AD3" r:id="rId4" location="targetSpecies" display="SPECIES_4_CODE" xr:uid="{22DD36F0-D891-4763-8CC9-508C73D63CC9}"/>
+    <hyperlink ref="AA3" r:id="rId1" location="allSpecies" xr:uid="{2BC6450F-A7B4-4044-BEA6-59E54066E449}"/>
+    <hyperlink ref="AB3" r:id="rId2" location="allSpecies" xr:uid="{9EEA8352-0631-4B4E-BB1B-FF880D8B8ED2}"/>
+    <hyperlink ref="AC3" r:id="rId3" location="allSpecies" xr:uid="{B78A1E77-3003-40C6-9B0C-101A94179479}"/>
+    <hyperlink ref="AD3" r:id="rId4" location="allSpecies" xr:uid="{22DD36F0-D891-4763-8CC9-508C73D63CC9}"/>
     <hyperlink ref="K3" r:id="rId5" location="lineMaterialTypes" display="MATERIAL_CODE" xr:uid="{53874CDA-60F7-44F3-A738-546AA82ACA2B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
E-SET-CATCH: Sampling method code list changed to methods --> total catch estimation
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_reporting_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB19908E-E8C6-2F49-8A36-62E01249F779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715C7FB4-8E0B-6B44-9CE8-C92F48F088E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="24680" windowHeight="16680" tabRatio="879" firstSheet="5" activeTab="8" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="8080" yWindow="740" windowWidth="20920" windowHeight="16680" tabRatio="879" firstSheet="11" activeTab="15" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -1444,6 +1444,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1476,9 +1479,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3678,31 +3678,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="89" t="s">
+      <c r="C1" s="90" t="s">
         <v>228</v>
       </c>
-      <c r="D1" s="89" t="s">
+      <c r="D1" s="90" t="s">
         <v>229</v>
       </c>
       <c r="E1" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="89" t="s">
+      <c r="F1" s="90" t="s">
         <v>250</v>
       </c>
-      <c r="G1" s="89" t="s">
+      <c r="G1" s="90" t="s">
         <v>227</v>
       </c>
-      <c r="H1" s="89" t="s">
+      <c r="H1" s="90" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="89" t="s">
+      <c r="I1" s="90" t="s">
         <v>93</v>
       </c>
       <c r="J1" s="83" t="s">
@@ -7147,17 +7147,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="i4Y2GDra9B4e5ZK9IT/yAgpGu83ed66ZNnyRoFvCqT5wVfLy2Lgs30SlszSGdCdYRpnULwm3Kg2BGFX0NXPahA==" saltValue="poZcuJUx5RFD549VWAk8zg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
+    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="E1:E2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="I1:I2"/>
-    <mergeCell ref="L1:O1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 M2 N2 O2" xr:uid="{35387E2C-FBDF-4B0A-A0B5-EF76A6744ABB}">
@@ -7190,10 +7190,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -8645,10 +8645,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -10319,10 +10319,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -10338,12 +10338,12 @@
       <c r="I1" s="100" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="99" t="s">
+      <c r="J1" s="89" t="s">
         <v>195</v>
       </c>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
       <c r="N1" s="81" t="s">
         <v>57</v>
       </c>
@@ -10360,14 +10360,14 @@
     <row r="2" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
       <c r="B2" s="69"/>
-      <c r="C2" s="89" t="s">
+      <c r="C2" s="90" t="s">
         <v>81</v>
       </c>
       <c r="D2" s="108" t="s">
         <v>79</v>
       </c>
       <c r="E2" s="110"/>
-      <c r="F2" s="89" t="s">
+      <c r="F2" s="90" t="s">
         <v>81</v>
       </c>
       <c r="G2" s="108" t="s">
@@ -10375,10 +10375,10 @@
       </c>
       <c r="H2" s="110"/>
       <c r="I2" s="100"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
+      <c r="J2" s="89"/>
+      <c r="K2" s="89"/>
+      <c r="L2" s="89"/>
+      <c r="M2" s="89"/>
       <c r="N2" s="81"/>
       <c r="O2" s="81"/>
       <c r="P2" s="119"/>
@@ -14222,6 +14222,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="XFozxK9hJMWP6ySEAZQ3h3enG2BhQeHoAidLHumULHWCGWuk01gbtIGf+HTrIiPiIpU+5yeeijnd0s/LDXPnUw==" saltValue="w5vF1VniVgRmNU/Yweiy+Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C1:E1"/>
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="O1:O3"/>
     <mergeCell ref="F1:H1"/>
@@ -14231,11 +14236,6 @@
     <mergeCell ref="J1:M2"/>
     <mergeCell ref="N1:N3"/>
     <mergeCell ref="P1:P3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C1:E1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I3 M3 J3 K3 L3 Q1:Q3" xr:uid="{2FBCC481-6114-481E-B036-95624C9F7883}">
@@ -14269,10 +14269,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="83" t="s">
@@ -15522,13 +15522,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="89" t="s">
+      <c r="C1" s="90" t="s">
         <v>94</v>
       </c>
       <c r="D1" s="121" t="s">
@@ -15538,10 +15538,10 @@
         <v>89</v>
       </c>
       <c r="F1" s="124"/>
-      <c r="G1" s="90" t="s">
+      <c r="G1" s="91" t="s">
         <v>184</v>
       </c>
-      <c r="H1" s="89" t="s">
+      <c r="H1" s="90" t="s">
         <v>209</v>
       </c>
       <c r="I1" s="83" t="s">
@@ -15561,7 +15561,7 @@
       <c r="F2" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="91"/>
+      <c r="G2" s="92"/>
       <c r="H2" s="70"/>
       <c r="I2" s="37" t="s">
         <v>186</v>
@@ -18174,7 +18174,7 @@
       <c r="K202" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="cIPMEB/7FdMJ59GLwUBjIJq7Z/ouJdnlvwNMkIwQQWO7k50m2ZyZ15EcA5FLZczYTiVocNtetk4wR+pQEJ425w==" saltValue="SnUtD4HRD9laqxb+y5V31A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="fTPkI9qmI0rPQTpef4UOHdSjNfD2cKgp41nTyI6DmyUhtwK/gK7x3ceTGV0x+9YGBk8Txgzr/CZn7PiM7+29PA==" saltValue="dNKoS5Q8OasFDXsltDFa1Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="8">
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="H1:H2"/>
@@ -18196,7 +18196,7 @@
     <hyperlink ref="E2" r:id="rId3" location="typesOfFate" xr:uid="{F8152E0B-B9D5-4E81-A374-4985E0AF2D58}"/>
     <hyperlink ref="F2" r:id="rId4" location="fates" xr:uid="{5DE917A8-1BC5-48A5-BE95-3206B5EEB7AC}"/>
     <hyperlink ref="D1" r:id="rId5" location="allSpecies" xr:uid="{7915C09B-5FFF-4B7E-84FB-D8B7D31EA643}"/>
-    <hyperlink ref="G1:G2" r:id="rId6" location="samplingProtocols" display="SAMPLING_METHOD" xr:uid="{C3154411-BFD2-3A41-99A0-2ECAAC5C9F3C}"/>
+    <hyperlink ref="G1:G2" r:id="rId6" location="samplingMethodsForCatchEstimation" display="SAMPLING_METHOD" xr:uid="{C3154411-BFD2-3A41-99A0-2ECAAC5C9F3C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
@@ -18251,10 +18251,10 @@
       <c r="D1" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="90" t="s">
+      <c r="E1" s="91" t="s">
         <v>183</v>
       </c>
-      <c r="F1" s="90" t="s">
+      <c r="F1" s="91" t="s">
         <v>184</v>
       </c>
       <c r="G1" s="81" t="s">
@@ -18263,17 +18263,17 @@
       <c r="H1" s="81"/>
       <c r="I1" s="81"/>
       <c r="J1" s="81"/>
-      <c r="K1" s="99" t="s">
+      <c r="K1" s="89" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99" t="s">
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="89" t="s">
         <v>58</v>
       </c>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
+      <c r="P1" s="89"/>
+      <c r="Q1" s="89"/>
       <c r="R1" s="105" t="s">
         <v>61</v>
       </c>
@@ -18286,18 +18286,18 @@
       </c>
       <c r="V1" s="84"/>
       <c r="W1" s="87"/>
-      <c r="X1" s="99" t="s">
+      <c r="X1" s="89" t="s">
         <v>191</v>
       </c>
-      <c r="Y1" s="99"/>
+      <c r="Y1" s="89"/>
     </row>
     <row r="2" spans="1:25" s="42" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="126"/>
       <c r="B2" s="126"/>
       <c r="C2" s="126"/>
       <c r="D2" s="126"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
       <c r="G2" s="43" t="s">
         <v>23</v>
       </c>
@@ -23835,13 +23835,13 @@
       <c r="D1" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="90" t="s">
+      <c r="E1" s="91" t="s">
         <v>174</v>
       </c>
-      <c r="F1" s="90" t="s">
+      <c r="F1" s="91" t="s">
         <v>175</v>
       </c>
-      <c r="G1" s="90" t="s">
+      <c r="G1" s="91" t="s">
         <v>176</v>
       </c>
       <c r="H1" s="106" t="s">
@@ -23883,9 +23883,9 @@
       <c r="B2" s="126"/>
       <c r="C2" s="126"/>
       <c r="D2" s="126"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
       <c r="H2" s="107"/>
       <c r="I2" s="37" t="s">
         <v>178</v>
@@ -28315,16 +28315,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="l8KVIJiIcXBtA5Rxt+oHSTZCQcSscxoVEx71fajOPkkDzIq7y1m1u1pHAE+AUnT93CwTnM5PkUuxYj42pmVV9g==" saltValue="dsO/0LEKtl67ZZqtPejb6A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="N1:N2"/>
-    <mergeCell ref="O1:O2"/>
     <mergeCell ref="P1:P2"/>
     <mergeCell ref="S1:T1"/>
     <mergeCell ref="H1:H2"/>
@@ -28332,6 +28322,16 @@
     <mergeCell ref="R1:R2"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="K1:L1"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F2 H1:H2 P1:P2 S2 J2 E1:E2 G1:G2 I2 M1:M2 T2" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -36474,34 +36474,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="97" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="92" t="s">
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="93"/>
-      <c r="I1" s="94"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="95"/>
       <c r="J1" s="105" t="s">
         <v>17</v>
       </c>
       <c r="K1" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="L1" s="96" t="s">
+      <c r="L1" s="97" t="s">
         <v>109</v>
       </c>
-      <c r="M1" s="97"/>
-      <c r="N1" s="97"/>
-      <c r="O1" s="97"/>
-      <c r="P1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="98"/>
+      <c r="O1" s="98"/>
+      <c r="P1" s="99"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
@@ -36517,7 +36517,7 @@
       <c r="E2" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="99" t="s">
+      <c r="F2" s="89" t="s">
         <v>14</v>
       </c>
       <c r="G2" s="100" t="s">
@@ -36526,11 +36526,11 @@
       <c r="H2" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="95" t="s">
+      <c r="I2" s="96" t="s">
         <v>158</v>
       </c>
       <c r="J2" s="106"/>
-      <c r="K2" s="90" t="s">
+      <c r="K2" s="91" t="s">
         <v>122</v>
       </c>
       <c r="L2" s="71" t="s">
@@ -36541,7 +36541,7 @@
         <v>19</v>
       </c>
       <c r="O2" s="71"/>
-      <c r="P2" s="99" t="s">
+      <c r="P2" s="89" t="s">
         <v>20</v>
       </c>
     </row>
@@ -36551,12 +36551,12 @@
       <c r="C3" s="103"/>
       <c r="D3" s="104"/>
       <c r="E3" s="82"/>
-      <c r="F3" s="99"/>
+      <c r="F3" s="89"/>
       <c r="G3" s="100"/>
       <c r="H3" s="102"/>
-      <c r="I3" s="95"/>
+      <c r="I3" s="96"/>
       <c r="J3" s="107"/>
-      <c r="K3" s="91"/>
+      <c r="K3" s="92"/>
       <c r="L3" s="31" t="s">
         <v>3</v>
       </c>
@@ -36569,7 +36569,7 @@
       <c r="O3" s="43" t="s">
         <v>230</v>
       </c>
-      <c r="P3" s="99"/>
+      <c r="P3" s="89"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
@@ -40174,11 +40174,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="CgzEmPt3Hk/Mhl0UL9A2LlPy9AK4yG5OneGJhJUq4FdJtqq7lG98GOjE3DOYWxyUk/x/OG6IB9bbOiXFzMXJrw==" saltValue="nv5eOc6x2cuQYecC/aOIFA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="I2:I3"/>
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P2:P3"/>
@@ -40191,6 +40186,11 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="J1:J3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="I2:I3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 J4 K2:K3 G2:I3 O3" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40234,23 +40234,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="B1" s="89" t="s">
         <v>211</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99" t="s">
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89" t="s">
         <v>212</v>
       </c>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
@@ -42976,7 +42976,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="83" t="s">
@@ -43065,49 +43065,49 @@
         <v>27</v>
       </c>
       <c r="T2" s="72"/>
-      <c r="U2" s="99" t="s">
+      <c r="U2" s="89" t="s">
         <v>136</v>
       </c>
-      <c r="V2" s="99" t="s">
+      <c r="V2" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="W2" s="99" t="s">
+      <c r="W2" s="89" t="s">
         <v>39</v>
       </c>
-      <c r="X2" s="99" t="s">
+      <c r="X2" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="Y2" s="99" t="s">
+      <c r="Y2" s="89" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="99" t="s">
+      <c r="Z2" s="89" t="s">
         <v>32</v>
       </c>
-      <c r="AA2" s="99" t="s">
+      <c r="AA2" s="89" t="s">
         <v>33</v>
       </c>
-      <c r="AB2" s="99" t="s">
+      <c r="AB2" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="AC2" s="99" t="s">
+      <c r="AC2" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="AD2" s="99" t="s">
+      <c r="AD2" s="89" t="s">
         <v>36</v>
       </c>
-      <c r="AE2" s="99" t="s">
+      <c r="AE2" s="89" t="s">
         <v>37</v>
       </c>
-      <c r="AF2" s="99" t="s">
+      <c r="AF2" s="89" t="s">
         <v>128</v>
       </c>
-      <c r="AG2" s="99" t="s">
+      <c r="AG2" s="89" t="s">
         <v>38</v>
       </c>
-      <c r="AH2" s="92" t="s">
+      <c r="AH2" s="93" t="s">
         <v>215</v>
       </c>
-      <c r="AI2" s="94"/>
+      <c r="AI2" s="95"/>
       <c r="AJ2" s="72" t="s">
         <v>216</v>
       </c>
@@ -43172,19 +43172,19 @@
       <c r="T3" s="36" t="s">
         <v>129</v>
       </c>
-      <c r="U3" s="99"/>
-      <c r="V3" s="99"/>
-      <c r="W3" s="99"/>
-      <c r="X3" s="99"/>
-      <c r="Y3" s="99"/>
-      <c r="Z3" s="99"/>
-      <c r="AA3" s="99"/>
-      <c r="AB3" s="99"/>
-      <c r="AC3" s="99"/>
-      <c r="AD3" s="99"/>
-      <c r="AE3" s="99"/>
-      <c r="AF3" s="99"/>
-      <c r="AG3" s="99"/>
+      <c r="U3" s="89"/>
+      <c r="V3" s="89"/>
+      <c r="W3" s="89"/>
+      <c r="X3" s="89"/>
+      <c r="Y3" s="89"/>
+      <c r="Z3" s="89"/>
+      <c r="AA3" s="89"/>
+      <c r="AB3" s="89"/>
+      <c r="AC3" s="89"/>
+      <c r="AD3" s="89"/>
+      <c r="AE3" s="89"/>
+      <c r="AF3" s="89"/>
+      <c r="AG3" s="89"/>
       <c r="AH3" s="30" t="s">
         <v>137</v>
       </c>
@@ -51813,6 +51813,20 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="wxJYPTS1M8YrpE+F5HXpzPvhVkWn+uzvbhQbX4zWGt7tgJJAc6rvipv1/0hraJgXbUY0X5vYRquC66cBDOGcbg==" saltValue="RWTcEymG3DdteXmtyGeu4A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="K2:K3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="U1:AG1"/>
@@ -51829,20 +51843,6 @@
     <mergeCell ref="AE2:AE3"/>
     <mergeCell ref="AD2:AD3"/>
     <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:V3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3 R3 AI3 AK3 AM3 L3 M3 N3 O3 P3 Q3 AO3 AJ3 AL3 AN3 AH3" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -51886,7 +51886,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="81" t="s">
@@ -53138,16 +53138,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="B1" s="89" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
       <c r="G1" s="83" t="s">
         <v>206</v>
       </c>
@@ -55629,7 +55629,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="108" t="s">
@@ -55654,20 +55654,20 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="90" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="96" t="s">
+      <c r="C2" s="97" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="99"/>
       <c r="H2" s="88" t="s">
         <v>162</v>
       </c>
-      <c r="I2" s="89" t="s">
+      <c r="I2" s="90" t="s">
         <v>163</v>
       </c>
       <c r="J2" s="83" t="s">
@@ -59389,10 +59389,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="81" t="s">
@@ -59405,10 +59405,10 @@
       </c>
       <c r="G1" s="109"/>
       <c r="H1" s="110"/>
-      <c r="I1" s="89" t="s">
+      <c r="I1" s="90" t="s">
         <v>236</v>
       </c>
-      <c r="J1" s="89" t="s">
+      <c r="J1" s="90" t="s">
         <v>237</v>
       </c>
       <c r="K1" s="111" t="s">
@@ -59423,7 +59423,7 @@
       <c r="P1" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="Q1" s="99" t="s">
+      <c r="Q1" s="89" t="s">
         <v>239</v>
       </c>
       <c r="R1" s="81" t="s">
@@ -59462,7 +59462,7 @@
         <v>79</v>
       </c>
       <c r="E2" s="110"/>
-      <c r="F2" s="89" t="s">
+      <c r="F2" s="90" t="s">
         <v>81</v>
       </c>
       <c r="G2" s="108" t="s">
@@ -59477,7 +59477,7 @@
       <c r="N2" s="79"/>
       <c r="O2" s="80"/>
       <c r="P2" s="81"/>
-      <c r="Q2" s="99"/>
+      <c r="Q2" s="89"/>
       <c r="R2" s="81"/>
       <c r="S2" s="81"/>
       <c r="T2" s="81"/>
@@ -59527,7 +59527,7 @@
         <v>48</v>
       </c>
       <c r="P3" s="81"/>
-      <c r="Q3" s="99"/>
+      <c r="Q3" s="89"/>
       <c r="R3" s="81"/>
       <c r="S3" s="31" t="s">
         <v>50</v>
@@ -65941,12 +65941,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="WuDPT1+slParW8lK5SfJrIiCuXUqugKfunXVVDY0YB00pOtHXcdvDQyUD/jzqYTc2x6TyFXXd8XFSXwF4cqxTw==" saltValue="kHXwsv450+CnM8/ussNlMw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="N1:O2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E2"/>
     <mergeCell ref="Y1:Z2"/>
     <mergeCell ref="AA1:AD2"/>
     <mergeCell ref="U1:V2"/>
@@ -65956,11 +65955,12 @@
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="R1:R3"/>
     <mergeCell ref="S1:T2"/>
-    <mergeCell ref="I1:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="N1:O2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3 AA3:AD3" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">

</xml_diff>

<commit_message>
Updates in form descriptions
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_reporting_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB19908E-E8C6-2F49-8A36-62E01249F779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715C7FB4-8E0B-6B44-9CE8-C92F48F088E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="24680" windowHeight="16680" tabRatio="879" firstSheet="5" activeTab="8" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="8080" yWindow="740" windowWidth="20920" windowHeight="16680" tabRatio="879" firstSheet="11" activeTab="15" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -1444,6 +1444,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1476,9 +1479,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3678,31 +3678,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="89" t="s">
+      <c r="C1" s="90" t="s">
         <v>228</v>
       </c>
-      <c r="D1" s="89" t="s">
+      <c r="D1" s="90" t="s">
         <v>229</v>
       </c>
       <c r="E1" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="89" t="s">
+      <c r="F1" s="90" t="s">
         <v>250</v>
       </c>
-      <c r="G1" s="89" t="s">
+      <c r="G1" s="90" t="s">
         <v>227</v>
       </c>
-      <c r="H1" s="89" t="s">
+      <c r="H1" s="90" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="89" t="s">
+      <c r="I1" s="90" t="s">
         <v>93</v>
       </c>
       <c r="J1" s="83" t="s">
@@ -7147,17 +7147,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="i4Y2GDra9B4e5ZK9IT/yAgpGu83ed66ZNnyRoFvCqT5wVfLy2Lgs30SlszSGdCdYRpnULwm3Kg2BGFX0NXPahA==" saltValue="poZcuJUx5RFD549VWAk8zg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
+    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="E1:E2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="I1:I2"/>
-    <mergeCell ref="L1:O1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 M2 N2 O2" xr:uid="{35387E2C-FBDF-4B0A-A0B5-EF76A6744ABB}">
@@ -7190,10 +7190,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -8645,10 +8645,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -10319,10 +10319,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="108" t="s">
@@ -10338,12 +10338,12 @@
       <c r="I1" s="100" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="99" t="s">
+      <c r="J1" s="89" t="s">
         <v>195</v>
       </c>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
       <c r="N1" s="81" t="s">
         <v>57</v>
       </c>
@@ -10360,14 +10360,14 @@
     <row r="2" spans="1:17" s="42" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
       <c r="B2" s="69"/>
-      <c r="C2" s="89" t="s">
+      <c r="C2" s="90" t="s">
         <v>81</v>
       </c>
       <c r="D2" s="108" t="s">
         <v>79</v>
       </c>
       <c r="E2" s="110"/>
-      <c r="F2" s="89" t="s">
+      <c r="F2" s="90" t="s">
         <v>81</v>
       </c>
       <c r="G2" s="108" t="s">
@@ -10375,10 +10375,10 @@
       </c>
       <c r="H2" s="110"/>
       <c r="I2" s="100"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
+      <c r="J2" s="89"/>
+      <c r="K2" s="89"/>
+      <c r="L2" s="89"/>
+      <c r="M2" s="89"/>
       <c r="N2" s="81"/>
       <c r="O2" s="81"/>
       <c r="P2" s="119"/>
@@ -14222,6 +14222,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="XFozxK9hJMWP6ySEAZQ3h3enG2BhQeHoAidLHumULHWCGWuk01gbtIGf+HTrIiPiIpU+5yeeijnd0s/LDXPnUw==" saltValue="w5vF1VniVgRmNU/Yweiy+Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C1:E1"/>
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="O1:O3"/>
     <mergeCell ref="F1:H1"/>
@@ -14231,11 +14236,6 @@
     <mergeCell ref="J1:M2"/>
     <mergeCell ref="N1:N3"/>
     <mergeCell ref="P1:P3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C1:E1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I3 M3 J3 K3 L3 Q1:Q3" xr:uid="{2FBCC481-6114-481E-B036-95624C9F7883}">
@@ -14269,10 +14269,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="83" t="s">
@@ -15522,13 +15522,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="89" t="s">
+      <c r="C1" s="90" t="s">
         <v>94</v>
       </c>
       <c r="D1" s="121" t="s">
@@ -15538,10 +15538,10 @@
         <v>89</v>
       </c>
       <c r="F1" s="124"/>
-      <c r="G1" s="90" t="s">
+      <c r="G1" s="91" t="s">
         <v>184</v>
       </c>
-      <c r="H1" s="89" t="s">
+      <c r="H1" s="90" t="s">
         <v>209</v>
       </c>
       <c r="I1" s="83" t="s">
@@ -15561,7 +15561,7 @@
       <c r="F2" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="91"/>
+      <c r="G2" s="92"/>
       <c r="H2" s="70"/>
       <c r="I2" s="37" t="s">
         <v>186</v>
@@ -18174,7 +18174,7 @@
       <c r="K202" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="cIPMEB/7FdMJ59GLwUBjIJq7Z/ouJdnlvwNMkIwQQWO7k50m2ZyZ15EcA5FLZczYTiVocNtetk4wR+pQEJ425w==" saltValue="SnUtD4HRD9laqxb+y5V31A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="fTPkI9qmI0rPQTpef4UOHdSjNfD2cKgp41nTyI6DmyUhtwK/gK7x3ceTGV0x+9YGBk8Txgzr/CZn7PiM7+29PA==" saltValue="dNKoS5Q8OasFDXsltDFa1Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="8">
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="H1:H2"/>
@@ -18196,7 +18196,7 @@
     <hyperlink ref="E2" r:id="rId3" location="typesOfFate" xr:uid="{F8152E0B-B9D5-4E81-A374-4985E0AF2D58}"/>
     <hyperlink ref="F2" r:id="rId4" location="fates" xr:uid="{5DE917A8-1BC5-48A5-BE95-3206B5EEB7AC}"/>
     <hyperlink ref="D1" r:id="rId5" location="allSpecies" xr:uid="{7915C09B-5FFF-4B7E-84FB-D8B7D31EA643}"/>
-    <hyperlink ref="G1:G2" r:id="rId6" location="samplingProtocols" display="SAMPLING_METHOD" xr:uid="{C3154411-BFD2-3A41-99A0-2ECAAC5C9F3C}"/>
+    <hyperlink ref="G1:G2" r:id="rId6" location="samplingMethodsForCatchEstimation" display="SAMPLING_METHOD" xr:uid="{C3154411-BFD2-3A41-99A0-2ECAAC5C9F3C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
@@ -18251,10 +18251,10 @@
       <c r="D1" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="90" t="s">
+      <c r="E1" s="91" t="s">
         <v>183</v>
       </c>
-      <c r="F1" s="90" t="s">
+      <c r="F1" s="91" t="s">
         <v>184</v>
       </c>
       <c r="G1" s="81" t="s">
@@ -18263,17 +18263,17 @@
       <c r="H1" s="81"/>
       <c r="I1" s="81"/>
       <c r="J1" s="81"/>
-      <c r="K1" s="99" t="s">
+      <c r="K1" s="89" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99" t="s">
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="89" t="s">
         <v>58</v>
       </c>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
+      <c r="P1" s="89"/>
+      <c r="Q1" s="89"/>
       <c r="R1" s="105" t="s">
         <v>61</v>
       </c>
@@ -18286,18 +18286,18 @@
       </c>
       <c r="V1" s="84"/>
       <c r="W1" s="87"/>
-      <c r="X1" s="99" t="s">
+      <c r="X1" s="89" t="s">
         <v>191</v>
       </c>
-      <c r="Y1" s="99"/>
+      <c r="Y1" s="89"/>
     </row>
     <row r="2" spans="1:25" s="42" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="126"/>
       <c r="B2" s="126"/>
       <c r="C2" s="126"/>
       <c r="D2" s="126"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
       <c r="G2" s="43" t="s">
         <v>23</v>
       </c>
@@ -23835,13 +23835,13 @@
       <c r="D1" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="90" t="s">
+      <c r="E1" s="91" t="s">
         <v>174</v>
       </c>
-      <c r="F1" s="90" t="s">
+      <c r="F1" s="91" t="s">
         <v>175</v>
       </c>
-      <c r="G1" s="90" t="s">
+      <c r="G1" s="91" t="s">
         <v>176</v>
       </c>
       <c r="H1" s="106" t="s">
@@ -23883,9 +23883,9 @@
       <c r="B2" s="126"/>
       <c r="C2" s="126"/>
       <c r="D2" s="126"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
       <c r="H2" s="107"/>
       <c r="I2" s="37" t="s">
         <v>178</v>
@@ -28315,16 +28315,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="l8KVIJiIcXBtA5Rxt+oHSTZCQcSscxoVEx71fajOPkkDzIq7y1m1u1pHAE+AUnT93CwTnM5PkUuxYj42pmVV9g==" saltValue="dsO/0LEKtl67ZZqtPejb6A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="N1:N2"/>
-    <mergeCell ref="O1:O2"/>
     <mergeCell ref="P1:P2"/>
     <mergeCell ref="S1:T1"/>
     <mergeCell ref="H1:H2"/>
@@ -28332,6 +28322,16 @@
     <mergeCell ref="R1:R2"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="K1:L1"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F2 H1:H2 P1:P2 S2 J2 E1:E2 G1:G2 I2 M1:M2 T2" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -36474,34 +36474,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="97" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="92" t="s">
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="93"/>
-      <c r="I1" s="94"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="95"/>
       <c r="J1" s="105" t="s">
         <v>17</v>
       </c>
       <c r="K1" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="L1" s="96" t="s">
+      <c r="L1" s="97" t="s">
         <v>109</v>
       </c>
-      <c r="M1" s="97"/>
-      <c r="N1" s="97"/>
-      <c r="O1" s="97"/>
-      <c r="P1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="98"/>
+      <c r="O1" s="98"/>
+      <c r="P1" s="99"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
@@ -36517,7 +36517,7 @@
       <c r="E2" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="99" t="s">
+      <c r="F2" s="89" t="s">
         <v>14</v>
       </c>
       <c r="G2" s="100" t="s">
@@ -36526,11 +36526,11 @@
       <c r="H2" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="95" t="s">
+      <c r="I2" s="96" t="s">
         <v>158</v>
       </c>
       <c r="J2" s="106"/>
-      <c r="K2" s="90" t="s">
+      <c r="K2" s="91" t="s">
         <v>122</v>
       </c>
       <c r="L2" s="71" t="s">
@@ -36541,7 +36541,7 @@
         <v>19</v>
       </c>
       <c r="O2" s="71"/>
-      <c r="P2" s="99" t="s">
+      <c r="P2" s="89" t="s">
         <v>20</v>
       </c>
     </row>
@@ -36551,12 +36551,12 @@
       <c r="C3" s="103"/>
       <c r="D3" s="104"/>
       <c r="E3" s="82"/>
-      <c r="F3" s="99"/>
+      <c r="F3" s="89"/>
       <c r="G3" s="100"/>
       <c r="H3" s="102"/>
-      <c r="I3" s="95"/>
+      <c r="I3" s="96"/>
       <c r="J3" s="107"/>
-      <c r="K3" s="91"/>
+      <c r="K3" s="92"/>
       <c r="L3" s="31" t="s">
         <v>3</v>
       </c>
@@ -36569,7 +36569,7 @@
       <c r="O3" s="43" t="s">
         <v>230</v>
       </c>
-      <c r="P3" s="99"/>
+      <c r="P3" s="89"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
@@ -40174,11 +40174,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="CgzEmPt3Hk/Mhl0UL9A2LlPy9AK4yG5OneGJhJUq4FdJtqq7lG98GOjE3DOYWxyUk/x/OG6IB9bbOiXFzMXJrw==" saltValue="nv5eOc6x2cuQYecC/aOIFA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="I2:I3"/>
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P2:P3"/>
@@ -40191,6 +40186,11 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="J1:J3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="I2:I3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 J4 K2:K3 G2:I3 O3" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40234,23 +40234,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="B1" s="89" t="s">
         <v>211</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99" t="s">
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89" t="s">
         <v>212</v>
       </c>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
@@ -42976,7 +42976,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="83" t="s">
@@ -43065,49 +43065,49 @@
         <v>27</v>
       </c>
       <c r="T2" s="72"/>
-      <c r="U2" s="99" t="s">
+      <c r="U2" s="89" t="s">
         <v>136</v>
       </c>
-      <c r="V2" s="99" t="s">
+      <c r="V2" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="W2" s="99" t="s">
+      <c r="W2" s="89" t="s">
         <v>39</v>
       </c>
-      <c r="X2" s="99" t="s">
+      <c r="X2" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="Y2" s="99" t="s">
+      <c r="Y2" s="89" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="99" t="s">
+      <c r="Z2" s="89" t="s">
         <v>32</v>
       </c>
-      <c r="AA2" s="99" t="s">
+      <c r="AA2" s="89" t="s">
         <v>33</v>
       </c>
-      <c r="AB2" s="99" t="s">
+      <c r="AB2" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="AC2" s="99" t="s">
+      <c r="AC2" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="AD2" s="99" t="s">
+      <c r="AD2" s="89" t="s">
         <v>36</v>
       </c>
-      <c r="AE2" s="99" t="s">
+      <c r="AE2" s="89" t="s">
         <v>37</v>
       </c>
-      <c r="AF2" s="99" t="s">
+      <c r="AF2" s="89" t="s">
         <v>128</v>
       </c>
-      <c r="AG2" s="99" t="s">
+      <c r="AG2" s="89" t="s">
         <v>38</v>
       </c>
-      <c r="AH2" s="92" t="s">
+      <c r="AH2" s="93" t="s">
         <v>215</v>
       </c>
-      <c r="AI2" s="94"/>
+      <c r="AI2" s="95"/>
       <c r="AJ2" s="72" t="s">
         <v>216</v>
       </c>
@@ -43172,19 +43172,19 @@
       <c r="T3" s="36" t="s">
         <v>129</v>
       </c>
-      <c r="U3" s="99"/>
-      <c r="V3" s="99"/>
-      <c r="W3" s="99"/>
-      <c r="X3" s="99"/>
-      <c r="Y3" s="99"/>
-      <c r="Z3" s="99"/>
-      <c r="AA3" s="99"/>
-      <c r="AB3" s="99"/>
-      <c r="AC3" s="99"/>
-      <c r="AD3" s="99"/>
-      <c r="AE3" s="99"/>
-      <c r="AF3" s="99"/>
-      <c r="AG3" s="99"/>
+      <c r="U3" s="89"/>
+      <c r="V3" s="89"/>
+      <c r="W3" s="89"/>
+      <c r="X3" s="89"/>
+      <c r="Y3" s="89"/>
+      <c r="Z3" s="89"/>
+      <c r="AA3" s="89"/>
+      <c r="AB3" s="89"/>
+      <c r="AC3" s="89"/>
+      <c r="AD3" s="89"/>
+      <c r="AE3" s="89"/>
+      <c r="AF3" s="89"/>
+      <c r="AG3" s="89"/>
       <c r="AH3" s="30" t="s">
         <v>137</v>
       </c>
@@ -51813,6 +51813,20 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="wxJYPTS1M8YrpE+F5HXpzPvhVkWn+uzvbhQbX4zWGt7tgJJAc6rvipv1/0hraJgXbUY0X5vYRquC66cBDOGcbg==" saltValue="RWTcEymG3DdteXmtyGeu4A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="K2:K3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="U1:AG1"/>
@@ -51829,20 +51843,6 @@
     <mergeCell ref="AE2:AE3"/>
     <mergeCell ref="AD2:AD3"/>
     <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:V3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3 R3 AI3 AK3 AM3 L3 M3 N3 O3 P3 Q3 AO3 AJ3 AL3 AN3 AH3" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -51886,7 +51886,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="81" t="s">
@@ -53138,16 +53138,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="B1" s="89" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
       <c r="G1" s="83" t="s">
         <v>206</v>
       </c>
@@ -55629,7 +55629,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="108" t="s">
@@ -55654,20 +55654,20 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="69"/>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="90" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="96" t="s">
+      <c r="C2" s="97" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="99"/>
       <c r="H2" s="88" t="s">
         <v>162</v>
       </c>
-      <c r="I2" s="89" t="s">
+      <c r="I2" s="90" t="s">
         <v>163</v>
       </c>
       <c r="J2" s="83" t="s">
@@ -59389,10 +59389,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="42" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="90" t="s">
         <v>92</v>
       </c>
       <c r="C1" s="81" t="s">
@@ -59405,10 +59405,10 @@
       </c>
       <c r="G1" s="109"/>
       <c r="H1" s="110"/>
-      <c r="I1" s="89" t="s">
+      <c r="I1" s="90" t="s">
         <v>236</v>
       </c>
-      <c r="J1" s="89" t="s">
+      <c r="J1" s="90" t="s">
         <v>237</v>
       </c>
       <c r="K1" s="111" t="s">
@@ -59423,7 +59423,7 @@
       <c r="P1" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="Q1" s="99" t="s">
+      <c r="Q1" s="89" t="s">
         <v>239</v>
       </c>
       <c r="R1" s="81" t="s">
@@ -59462,7 +59462,7 @@
         <v>79</v>
       </c>
       <c r="E2" s="110"/>
-      <c r="F2" s="89" t="s">
+      <c r="F2" s="90" t="s">
         <v>81</v>
       </c>
       <c r="G2" s="108" t="s">
@@ -59477,7 +59477,7 @@
       <c r="N2" s="79"/>
       <c r="O2" s="80"/>
       <c r="P2" s="81"/>
-      <c r="Q2" s="99"/>
+      <c r="Q2" s="89"/>
       <c r="R2" s="81"/>
       <c r="S2" s="81"/>
       <c r="T2" s="81"/>
@@ -59527,7 +59527,7 @@
         <v>48</v>
       </c>
       <c r="P3" s="81"/>
-      <c r="Q3" s="99"/>
+      <c r="Q3" s="89"/>
       <c r="R3" s="81"/>
       <c r="S3" s="31" t="s">
         <v>50</v>
@@ -65941,12 +65941,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="WuDPT1+slParW8lK5SfJrIiCuXUqugKfunXVVDY0YB00pOtHXcdvDQyUD/jzqYTc2x6TyFXXd8XFSXwF4cqxTw==" saltValue="kHXwsv450+CnM8/ussNlMw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="N1:O2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E2"/>
     <mergeCell ref="Y1:Z2"/>
     <mergeCell ref="AA1:AD2"/>
     <mergeCell ref="U1:V2"/>
@@ -65956,11 +65955,12 @@
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="R1:R3"/>
     <mergeCell ref="S1:T2"/>
-    <mergeCell ref="I1:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="N1:O2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3 AA3:AD3" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">

</xml_diff>

<commit_message>
Changed URL and title from "Hooks" to "Hooks and terminal devices" in E-SET-HOOKS for LL gear to include trap lines
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-LL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-LL.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D907510-87CC-44C4-8B53-6CD82AD9A939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3611A48B-6C62-4FFF-9CBD-E5F471BDC6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="ZfpSTEX8tJoLKKS/2QPKxpUICc4sIZ3kzl8g4yv5govFiOeUEO9yg+BUjdxWSjUCwnz/IYo7CkpdetcZ9hh01Q==" workbookSaltValue="1lt51vMgZ/EPbNjf80VAWA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" activeTab="1" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="25" r:id="rId1"/>
@@ -660,9 +660,6 @@
     <t>NUMBER_BRANCHLINE_HAULINGS_OBSERVED</t>
   </si>
   <si>
-    <t>HOOKS</t>
-  </si>
-  <si>
     <t>NUMBER_OF_LIGHTS</t>
   </si>
   <si>
@@ -817,6 +814,9 @@
   </si>
   <si>
     <t>NUMBER_OF_HOOKS_RETRIEVED_DURING_OBSERVATION</t>
+  </si>
+  <si>
+    <t>HOOKS AND TERMINAL DEVICES</t>
   </si>
 </sst>
 </file>
@@ -1347,75 +1347,10 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1454,29 +1389,55 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1487,6 +1448,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1516,6 +1480,30 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1558,6 +1546,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1905,24 +1905,24 @@
   <sheetData>
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="77" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="70"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="79"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="71"/>
-      <c r="C3" s="72"/>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="73"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="82"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
@@ -1972,15 +1972,15 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="10"/>
-      <c r="C8" s="74" t="s">
+      <c r="C8" s="83" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="74"/>
+      <c r="D8" s="83"/>
       <c r="E8" s="11"/>
-      <c r="F8" s="74" t="s">
+      <c r="F8" s="83" t="s">
         <v>113</v>
       </c>
-      <c r="G8" s="74"/>
+      <c r="G8" s="83"/>
       <c r="H8" s="12"/>
     </row>
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2162,11 +2162,11 @@
     </row>
     <row r="26" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="10"/>
-      <c r="C26" s="75"/>
-      <c r="D26" s="76"/>
-      <c r="E26" s="76"/>
-      <c r="F26" s="76"/>
-      <c r="G26" s="77"/>
+      <c r="C26" s="84"/>
+      <c r="D26" s="85"/>
+      <c r="E26" s="85"/>
+      <c r="F26" s="85"/>
+      <c r="G26" s="86"/>
       <c r="H26" s="12"/>
     </row>
     <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2237,10 +2237,10 @@
         <v>23</v>
       </c>
       <c r="D1" s="42" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E1" s="45" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="41" customFormat="1" x14ac:dyDescent="0.25">
@@ -3680,54 +3680,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="C1" s="99" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1" s="99" t="s">
         <v>228</v>
       </c>
-      <c r="D1" s="59" t="s">
-        <v>229</v>
-      </c>
-      <c r="E1" s="93" t="s">
+      <c r="E1" s="76" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="59" t="s">
-        <v>250</v>
+      <c r="F1" s="99" t="s">
+        <v>249</v>
       </c>
-      <c r="G1" s="59" t="s">
-        <v>227</v>
+      <c r="G1" s="99" t="s">
+        <v>226</v>
       </c>
-      <c r="H1" s="59" t="s">
+      <c r="H1" s="99" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="59" t="s">
+      <c r="I1" s="99" t="s">
         <v>93</v>
       </c>
-      <c r="J1" s="61" t="s">
+      <c r="J1" s="71" t="s">
+        <v>220</v>
+      </c>
+      <c r="K1" s="75"/>
+      <c r="L1" s="106" t="s">
         <v>221</v>
       </c>
-      <c r="K1" s="63"/>
-      <c r="L1" s="110" t="s">
-        <v>222</v>
-      </c>
-      <c r="M1" s="111"/>
-      <c r="N1" s="111"/>
-      <c r="O1" s="112"/>
+      <c r="M1" s="107"/>
+      <c r="N1" s="107"/>
+      <c r="O1" s="108"/>
     </row>
     <row r="2" spans="1:15" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60"/>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
       <c r="J2" s="33" t="s">
         <v>46</v>
       </c>
@@ -3735,16 +3735,16 @@
         <v>80</v>
       </c>
       <c r="L2" s="42" t="s">
+        <v>222</v>
+      </c>
+      <c r="M2" s="42" t="s">
         <v>223</v>
       </c>
-      <c r="M2" s="42" t="s">
+      <c r="N2" s="42" t="s">
         <v>224</v>
       </c>
-      <c r="N2" s="42" t="s">
+      <c r="O2" s="42" t="s">
         <v>225</v>
-      </c>
-      <c r="O2" s="42" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -7149,17 +7149,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="i4Y2GDra9B4e5ZK9IT/yAgpGu83ed66ZNnyRoFvCqT5wVfLy2Lgs30SlszSGdCdYRpnULwm3Kg2BGFX0NXPahA==" saltValue="poZcuJUx5RFD549VWAk8zg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
+    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="E1:E2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="I1:I2"/>
-    <mergeCell ref="L1:O1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 M2 N2 O2" xr:uid="{35387E2C-FBDF-4B0A-A0B5-EF76A6744ABB}">
@@ -7192,21 +7192,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="110" t="s">
-        <v>201</v>
+      <c r="C1" s="106" t="s">
+        <v>253</v>
       </c>
-      <c r="D1" s="111"/>
-      <c r="E1" s="112"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
     </row>
     <row r="2" spans="1:5" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60"/>
-      <c r="B2" s="60"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
       <c r="C2" s="42" t="s">
         <v>23</v>
       </c>
@@ -8618,14 +8618,14 @@
       <c r="E202" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="7L7ysxAlvpkBotAvp596sYOylpEuvb/Ta11TwryFzRR9JnFyu2qT+9lTo+vY+D8FgTspPzRmMhpOG+a3DGDtGA==" saltValue="tiHQmWEfnba1P++46Gyl1g==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="SQW7Q+33fdeDxG4TZIWTcU/SvXZv2fX44vfby4iEcWtzZJTELGljGngkulk/4h40hVG9bmnvmfePke5awPVcqg==" saltValue="YyrlZm1PvFilAGwS6CjaGw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" location="hookTypes" display="TYPE_CODE" xr:uid="{76A15B78-243E-4A2E-A5A4-5CE8931F7C0B}"/>
+    <hyperlink ref="C2" r:id="rId1" location="hookAndTerminalDevices" xr:uid="{76A15B78-243E-4A2E-A5A4-5CE8931F7C0B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8647,22 +8647,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="110" t="s">
+      <c r="C1" s="106" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="112"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="107"/>
+      <c r="F1" s="108"/>
     </row>
     <row r="2" spans="1:6" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60"/>
-      <c r="B2" s="60"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
       <c r="C2" s="42" t="s">
         <v>178</v>
       </c>
@@ -10321,89 +10321,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="110" t="s">
+      <c r="C1" s="106" t="s">
+        <v>206</v>
+      </c>
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="106" t="s">
         <v>207</v>
       </c>
-      <c r="D1" s="111"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="110" t="s">
-        <v>208</v>
-      </c>
-      <c r="G1" s="111"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="102" t="s">
+      <c r="G1" s="107"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="94" t="s">
+      <c r="J1" s="90" t="s">
         <v>195</v>
       </c>
-      <c r="K1" s="94"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="89" t="s">
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="69" t="s">
         <v>57</v>
       </c>
-      <c r="O1" s="89" t="s">
+      <c r="O1" s="69" t="s">
         <v>200</v>
       </c>
-      <c r="P1" s="120" t="s">
-        <v>253</v>
+      <c r="P1" s="116" t="s">
+        <v>252</v>
       </c>
-      <c r="Q1" s="119" t="s">
+      <c r="Q1" s="115" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="59" t="s">
+      <c r="A2" s="57"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="99" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="110" t="s">
+      <c r="D2" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="112"/>
-      <c r="F2" s="59" t="s">
+      <c r="E2" s="108"/>
+      <c r="F2" s="99" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="110" t="s">
+      <c r="G2" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="H2" s="112"/>
-      <c r="I2" s="102"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
-      <c r="M2" s="94"/>
-      <c r="N2" s="89"/>
-      <c r="O2" s="89"/>
-      <c r="P2" s="121"/>
-      <c r="Q2" s="119"/>
+      <c r="H2" s="108"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="90"/>
+      <c r="K2" s="90"/>
+      <c r="L2" s="90"/>
+      <c r="M2" s="90"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="117"/>
+      <c r="Q2" s="115"/>
     </row>
     <row r="3" spans="1:17" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="60"/>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
       <c r="D3" s="30" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="60"/>
+      <c r="F3" s="58"/>
       <c r="G3" s="30" t="s">
         <v>0</v>
       </c>
       <c r="H3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="102"/>
+      <c r="I3" s="91"/>
       <c r="J3" s="36" t="s">
         <v>194</v>
       </c>
@@ -10416,10 +10416,10 @@
       <c r="M3" s="36" t="s">
         <v>198</v>
       </c>
-      <c r="N3" s="89"/>
-      <c r="O3" s="89"/>
-      <c r="P3" s="122"/>
-      <c r="Q3" s="119"/>
+      <c r="N3" s="69"/>
+      <c r="O3" s="69"/>
+      <c r="P3" s="118"/>
+      <c r="Q3" s="115"/>
     </row>
     <row r="4" spans="1:17" s="41" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -14224,6 +14224,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="XFozxK9hJMWP6ySEAZQ3h3enG2BhQeHoAidLHumULHWCGWuk01gbtIGf+HTrIiPiIpU+5yeeijnd0s/LDXPnUw==" saltValue="w5vF1VniVgRmNU/Yweiy+Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C1:E1"/>
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="O1:O3"/>
     <mergeCell ref="F1:H1"/>
@@ -14233,11 +14238,6 @@
     <mergeCell ref="J1:M2"/>
     <mergeCell ref="N1:N3"/>
     <mergeCell ref="P1:P3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C1:E1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I3 M3 J3 K3 L3 Q1:Q3" xr:uid="{2FBCC481-6114-481E-B036-95624C9F7883}">
@@ -14271,20 +14271,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="61" t="s">
+      <c r="C1" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="63"/>
+      <c r="D1" s="75"/>
     </row>
     <row r="2" spans="1:4" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60"/>
-      <c r="B2" s="60"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
       <c r="C2" s="33" t="s">
         <v>145</v>
       </c>
@@ -15524,47 +15524,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="C1" s="99" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="64" t="s">
+      <c r="D1" s="119" t="s">
         <v>121</v>
       </c>
-      <c r="E1" s="66" t="s">
+      <c r="E1" s="121" t="s">
         <v>89</v>
       </c>
-      <c r="F1" s="67"/>
-      <c r="G1" s="57" t="s">
+      <c r="F1" s="122"/>
+      <c r="G1" s="100" t="s">
         <v>184</v>
       </c>
-      <c r="H1" s="59" t="s">
-        <v>209</v>
+      <c r="H1" s="99" t="s">
+        <v>208</v>
       </c>
-      <c r="I1" s="61" t="s">
+      <c r="I1" s="71" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="75"/>
     </row>
     <row r="2" spans="1:11" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60"/>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="65"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="120"/>
       <c r="E2" s="42" t="s">
         <v>23</v>
       </c>
       <c r="F2" s="42" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="58"/>
-      <c r="H2" s="60"/>
+      <c r="G2" s="101"/>
+      <c r="H2" s="58"/>
       <c r="I2" s="36" t="s">
         <v>186</v>
       </c>
@@ -15572,7 +15572,7 @@
         <v>59</v>
       </c>
       <c r="K2" s="36" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:11" s="41" customFormat="1" x14ac:dyDescent="0.25">
@@ -18253,53 +18253,53 @@
       <c r="D1" s="123" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="57" t="s">
+      <c r="E1" s="100" t="s">
         <v>183</v>
       </c>
-      <c r="F1" s="57" t="s">
+      <c r="F1" s="100" t="s">
         <v>184</v>
       </c>
-      <c r="G1" s="89" t="s">
+      <c r="G1" s="69" t="s">
         <v>187</v>
       </c>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="94" t="s">
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="90" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94" t="s">
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90" t="s">
         <v>58</v>
       </c>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="107" t="s">
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="96" t="s">
         <v>61</v>
       </c>
-      <c r="S1" s="61" t="s">
+      <c r="S1" s="71" t="s">
         <v>87</v>
       </c>
-      <c r="T1" s="63"/>
-      <c r="U1" s="61" t="s">
+      <c r="T1" s="75"/>
+      <c r="U1" s="71" t="s">
         <v>192</v>
       </c>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="X1" s="94" t="s">
+      <c r="V1" s="72"/>
+      <c r="W1" s="75"/>
+      <c r="X1" s="90" t="s">
         <v>191</v>
       </c>
-      <c r="Y1" s="94"/>
+      <c r="Y1" s="90"/>
     </row>
     <row r="2" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="124"/>
       <c r="B2" s="124"/>
       <c r="C2" s="124"/>
       <c r="D2" s="124"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
       <c r="G2" s="42" t="s">
         <v>23</v>
       </c>
@@ -18331,9 +18331,9 @@
         <v>59</v>
       </c>
       <c r="Q2" s="36" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
-      <c r="R2" s="109"/>
+      <c r="R2" s="98"/>
       <c r="S2" s="34" t="s">
         <v>85</v>
       </c>
@@ -23837,27 +23837,27 @@
       <c r="D1" s="123" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="57" t="s">
+      <c r="E1" s="100" t="s">
         <v>174</v>
       </c>
-      <c r="F1" s="57" t="s">
+      <c r="F1" s="100" t="s">
         <v>175</v>
       </c>
-      <c r="G1" s="57" t="s">
+      <c r="G1" s="100" t="s">
         <v>176</v>
       </c>
-      <c r="H1" s="108" t="s">
+      <c r="H1" s="97" t="s">
         <v>177</v>
       </c>
-      <c r="I1" s="87" t="s">
+      <c r="I1" s="67" t="s">
         <v>69</v>
       </c>
-      <c r="J1" s="88"/>
-      <c r="K1" s="84" t="s">
+      <c r="J1" s="68"/>
+      <c r="K1" s="64" t="s">
         <v>70</v>
       </c>
-      <c r="L1" s="86"/>
-      <c r="M1" s="108" t="s">
+      <c r="L1" s="66"/>
+      <c r="M1" s="97" t="s">
         <v>182</v>
       </c>
       <c r="N1" s="125" t="s">
@@ -23866,7 +23866,7 @@
       <c r="O1" s="125" t="s">
         <v>66</v>
       </c>
-      <c r="P1" s="108" t="s">
+      <c r="P1" s="97" t="s">
         <v>181</v>
       </c>
       <c r="Q1" s="125" t="s">
@@ -23875,20 +23875,20 @@
       <c r="R1" s="125" t="s">
         <v>68</v>
       </c>
-      <c r="S1" s="90" t="s">
+      <c r="S1" s="70" t="s">
         <v>191</v>
       </c>
-      <c r="T1" s="90"/>
+      <c r="T1" s="70"/>
     </row>
     <row r="2" spans="1:20" s="41" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="124"/>
       <c r="B2" s="124"/>
       <c r="C2" s="124"/>
       <c r="D2" s="124"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="109"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="101"/>
+      <c r="H2" s="98"/>
       <c r="I2" s="36" t="s">
         <v>178</v>
       </c>
@@ -23901,12 +23901,12 @@
       <c r="L2" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="M2" s="109"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
-      <c r="P2" s="109"/>
-      <c r="Q2" s="90"/>
-      <c r="R2" s="90"/>
+      <c r="M2" s="98"/>
+      <c r="N2" s="70"/>
+      <c r="O2" s="70"/>
+      <c r="P2" s="98"/>
+      <c r="Q2" s="70"/>
+      <c r="R2" s="70"/>
       <c r="S2" s="36" t="s">
         <v>180</v>
       </c>
@@ -28317,16 +28317,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="LYFU8JE4J8WBzpl/b4zqaQPLnLsCDSe2zWW+8dNgs/2PHOZq06/1QnNdJiP29gcTnH4LQIS1HvbDau5S5pjwdg==" saltValue="bo/QzTypvgnDcZydb/HXQw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="N1:N2"/>
-    <mergeCell ref="O1:O2"/>
     <mergeCell ref="P1:P2"/>
     <mergeCell ref="S1:T1"/>
     <mergeCell ref="H1:H2"/>
@@ -28334,6 +28324,16 @@
     <mergeCell ref="R1:R2"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="K1:L1"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F2 H1:H2 P1:P2 S2 J2 E1:E2 G1:G2 I2 M1:M2 T2" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -28398,10 +28398,10 @@
         <v>23</v>
       </c>
       <c r="H1" s="33" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I1" s="33" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="J1" s="33" t="s">
         <v>110</v>
@@ -31059,117 +31059,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="57" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="60" t="s">
+      <c r="B1" s="58" t="s">
         <v>156</v>
       </c>
-      <c r="C1" s="60"/>
-      <c r="D1" s="90" t="s">
+      <c r="C1" s="58"/>
+      <c r="D1" s="70" t="s">
         <v>157</v>
       </c>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="81" t="s">
-        <v>210</v>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="61" t="s">
+        <v>209</v>
       </c>
-      <c r="O1" s="82"/>
-      <c r="P1" s="82"/>
-      <c r="Q1" s="82"/>
-      <c r="R1" s="82"/>
-      <c r="S1" s="82"/>
-      <c r="T1" s="82"/>
-      <c r="U1" s="82"/>
-      <c r="V1" s="82"/>
-      <c r="W1" s="82"/>
-      <c r="X1" s="83"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="63"/>
       <c r="Y1" s="39"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="89"/>
-      <c r="C2" s="89"/>
-      <c r="D2" s="61" t="s">
+      <c r="A2" s="57"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="71" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="63"/>
-      <c r="I2" s="61" t="s">
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="71" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62"/>
-      <c r="N2" s="84"/>
-      <c r="O2" s="85"/>
-      <c r="P2" s="85"/>
-      <c r="Q2" s="85"/>
-      <c r="R2" s="85"/>
-      <c r="S2" s="85"/>
-      <c r="T2" s="85"/>
-      <c r="U2" s="85"/>
-      <c r="V2" s="85"/>
-      <c r="W2" s="85"/>
-      <c r="X2" s="86"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="72"/>
+      <c r="M2" s="72"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="65"/>
+      <c r="X2" s="66"/>
       <c r="Y2" s="39"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="78"/>
-      <c r="B3" s="89"/>
-      <c r="C3" s="89"/>
-      <c r="D3" s="87" t="s">
+      <c r="A3" s="57"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="88"/>
-      <c r="F3" s="87" t="s">
+      <c r="E3" s="68"/>
+      <c r="F3" s="67" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="88"/>
-      <c r="H3" s="93" t="s">
+      <c r="G3" s="68"/>
+      <c r="H3" s="76" t="s">
         <v>81</v>
       </c>
-      <c r="I3" s="87" t="s">
+      <c r="I3" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="88"/>
-      <c r="K3" s="87" t="s">
+      <c r="J3" s="68"/>
+      <c r="K3" s="67" t="s">
         <v>74</v>
       </c>
-      <c r="L3" s="88"/>
-      <c r="M3" s="91" t="s">
+      <c r="L3" s="68"/>
+      <c r="M3" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="N3" s="79" t="s">
-        <v>233</v>
+      <c r="N3" s="59" t="s">
+        <v>232</v>
       </c>
-      <c r="O3" s="79"/>
-      <c r="P3" s="80" t="s">
+      <c r="O3" s="59"/>
+      <c r="P3" s="60" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60" t="s">
         <v>231</v>
       </c>
-      <c r="Q3" s="80"/>
-      <c r="R3" s="80"/>
-      <c r="S3" s="80"/>
-      <c r="T3" s="80"/>
-      <c r="U3" s="80" t="s">
-        <v>232</v>
-      </c>
-      <c r="V3" s="80"/>
-      <c r="W3" s="80"/>
-      <c r="X3" s="80"/>
+      <c r="V3" s="60"/>
+      <c r="W3" s="60"/>
+      <c r="X3" s="60"/>
     </row>
     <row r="4" spans="1:25" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60"/>
+      <c r="A4" s="58"/>
       <c r="B4" s="30" t="s">
         <v>108</v>
       </c>
@@ -31188,7 +31188,7 @@
       <c r="G4" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="90"/>
+      <c r="H4" s="70"/>
       <c r="I4" s="36" t="s">
         <v>115</v>
       </c>
@@ -31201,7 +31201,7 @@
       <c r="L4" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="M4" s="92"/>
+      <c r="M4" s="74"/>
       <c r="N4" s="30" t="s">
         <v>5</v>
       </c>
@@ -36476,102 +36476,102 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="B1" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="95" t="s">
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="102" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="96"/>
-      <c r="I1" s="97"/>
-      <c r="J1" s="107" t="s">
+      <c r="H1" s="103"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="96" t="s">
         <v>17</v>
       </c>
       <c r="K1" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="L1" s="99" t="s">
+      <c r="L1" s="87" t="s">
         <v>109</v>
       </c>
-      <c r="M1" s="100"/>
-      <c r="N1" s="100"/>
-      <c r="O1" s="100"/>
-      <c r="P1" s="101"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="89"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="89" t="s">
+      <c r="A2" s="57"/>
+      <c r="B2" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="94" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="106" t="s">
+      <c r="D2" s="95" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="93" t="s">
+      <c r="E2" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="94" t="s">
+      <c r="F2" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="102" t="s">
+      <c r="G2" s="91" t="s">
         <v>115</v>
       </c>
-      <c r="H2" s="103" t="s">
+      <c r="H2" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="98" t="s">
+      <c r="I2" s="105" t="s">
         <v>158</v>
       </c>
-      <c r="J2" s="108"/>
-      <c r="K2" s="57" t="s">
+      <c r="J2" s="97"/>
+      <c r="K2" s="100" t="s">
         <v>122</v>
       </c>
-      <c r="L2" s="79" t="s">
+      <c r="L2" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79" t="s">
+      <c r="M2" s="59"/>
+      <c r="N2" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="79"/>
-      <c r="P2" s="94" t="s">
+      <c r="O2" s="59"/>
+      <c r="P2" s="90" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="60"/>
-      <c r="B3" s="89"/>
-      <c r="C3" s="105"/>
-      <c r="D3" s="106"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="104"/>
-      <c r="I3" s="98"/>
-      <c r="J3" s="109"/>
-      <c r="K3" s="58"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="94"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="101"/>
       <c r="L3" s="30" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="42" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="N3" s="30" t="s">
         <v>3</v>
       </c>
       <c r="O3" s="42" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
-      <c r="P3" s="94"/>
+      <c r="P3" s="90"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -40175,6 +40175,10 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="1cicS5Lfrk+5Ikf7QAPb58hz7eEpXXWrVfI0HjUb1ZSCRmF1spVwuukBA70xdhXph1ojRMo4vKzKONUJgs2EdA==" saltValue="VZjUWywuY51JVfym8Ql6fg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="I2:I3"/>
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P2:P3"/>
@@ -40188,10 +40192,6 @@
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="J1:J3"/>
     <mergeCell ref="F2:F3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="I2:I3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 O3 K2:K3 G2:I3" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -40235,47 +40235,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="94" t="s">
+      <c r="B1" s="90" t="s">
+        <v>210</v>
+      </c>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90" t="s">
         <v>211</v>
       </c>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94" t="s">
-        <v>212</v>
-      </c>
-      <c r="H1" s="94"/>
-      <c r="I1" s="94"/>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="61" t="s">
+      <c r="A2" s="57"/>
+      <c r="B2" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="93" t="s">
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="76" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="61" t="s">
+      <c r="G2" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="63"/>
-      <c r="K2" s="93" t="s">
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="76" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="60"/>
+      <c r="A3" s="58"/>
       <c r="B3" s="36" t="s">
         <v>115</v>
       </c>
@@ -40288,7 +40288,7 @@
       <c r="E3" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="90"/>
+      <c r="F3" s="70"/>
       <c r="G3" s="36" t="s">
         <v>115</v>
       </c>
@@ -40301,7 +40301,7 @@
       <c r="J3" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="90"/>
+      <c r="K3" s="70"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -42977,156 +42977,156 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="61" t="s">
+      <c r="B1" s="71" t="s">
         <v>171</v>
       </c>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="63"/>
-      <c r="U1" s="61" t="s">
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+      <c r="P1" s="72"/>
+      <c r="Q1" s="72"/>
+      <c r="R1" s="72"/>
+      <c r="S1" s="72"/>
+      <c r="T1" s="75"/>
+      <c r="U1" s="71" t="s">
+        <v>212</v>
+      </c>
+      <c r="V1" s="72"/>
+      <c r="W1" s="72"/>
+      <c r="X1" s="72"/>
+      <c r="Y1" s="72"/>
+      <c r="Z1" s="72"/>
+      <c r="AA1" s="72"/>
+      <c r="AB1" s="72"/>
+      <c r="AC1" s="72"/>
+      <c r="AD1" s="72"/>
+      <c r="AE1" s="72"/>
+      <c r="AF1" s="72"/>
+      <c r="AG1" s="75"/>
+      <c r="AH1" s="71" t="s">
         <v>213</v>
       </c>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="63"/>
-      <c r="AH1" s="61" t="s">
+      <c r="AI1" s="72"/>
+      <c r="AJ1" s="72"/>
+      <c r="AK1" s="72"/>
+      <c r="AL1" s="72"/>
+      <c r="AM1" s="72"/>
+      <c r="AN1" s="72"/>
+      <c r="AO1" s="75"/>
+    </row>
+    <row r="2" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A2" s="57"/>
+      <c r="B2" s="76" t="s">
+        <v>124</v>
+      </c>
+      <c r="C2" s="76" t="s">
+        <v>125</v>
+      </c>
+      <c r="D2" s="96" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2" s="60" t="s">
+        <v>172</v>
+      </c>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60" t="s">
+        <v>173</v>
+      </c>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="76" t="s">
+        <v>155</v>
+      </c>
+      <c r="L2" s="60" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" s="60"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="60"/>
+      <c r="P2" s="60" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q2" s="60"/>
+      <c r="R2" s="60"/>
+      <c r="S2" s="60" t="s">
+        <v>27</v>
+      </c>
+      <c r="T2" s="60"/>
+      <c r="U2" s="90" t="s">
+        <v>136</v>
+      </c>
+      <c r="V2" s="90" t="s">
+        <v>29</v>
+      </c>
+      <c r="W2" s="90" t="s">
+        <v>39</v>
+      </c>
+      <c r="X2" s="90" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y2" s="90" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z2" s="90" t="s">
+        <v>32</v>
+      </c>
+      <c r="AA2" s="90" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB2" s="90" t="s">
+        <v>34</v>
+      </c>
+      <c r="AC2" s="90" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD2" s="90" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE2" s="90" t="s">
+        <v>37</v>
+      </c>
+      <c r="AF2" s="90" t="s">
+        <v>128</v>
+      </c>
+      <c r="AG2" s="90" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH2" s="102" t="s">
         <v>214</v>
       </c>
-      <c r="AI1" s="62"/>
-      <c r="AJ1" s="62"/>
-      <c r="AK1" s="62"/>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="63"/>
-    </row>
-    <row r="2" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="93" t="s">
-        <v>124</v>
-      </c>
-      <c r="C2" s="93" t="s">
-        <v>125</v>
-      </c>
-      <c r="D2" s="107" t="s">
-        <v>126</v>
-      </c>
-      <c r="E2" s="80" t="s">
-        <v>172</v>
-      </c>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80" t="s">
-        <v>173</v>
-      </c>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
-      <c r="K2" s="93" t="s">
-        <v>155</v>
-      </c>
-      <c r="L2" s="80" t="s">
-        <v>26</v>
-      </c>
-      <c r="M2" s="80"/>
-      <c r="N2" s="80"/>
-      <c r="O2" s="80"/>
-      <c r="P2" s="80" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q2" s="80"/>
-      <c r="R2" s="80"/>
-      <c r="S2" s="80" t="s">
-        <v>27</v>
-      </c>
-      <c r="T2" s="80"/>
-      <c r="U2" s="94" t="s">
-        <v>136</v>
-      </c>
-      <c r="V2" s="94" t="s">
-        <v>29</v>
-      </c>
-      <c r="W2" s="94" t="s">
-        <v>39</v>
-      </c>
-      <c r="X2" s="94" t="s">
-        <v>30</v>
-      </c>
-      <c r="Y2" s="94" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z2" s="94" t="s">
-        <v>32</v>
-      </c>
-      <c r="AA2" s="94" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB2" s="94" t="s">
-        <v>34</v>
-      </c>
-      <c r="AC2" s="94" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD2" s="94" t="s">
-        <v>36</v>
-      </c>
-      <c r="AE2" s="94" t="s">
-        <v>37</v>
-      </c>
-      <c r="AF2" s="94" t="s">
-        <v>128</v>
-      </c>
-      <c r="AG2" s="94" t="s">
-        <v>38</v>
-      </c>
-      <c r="AH2" s="95" t="s">
+      <c r="AI2" s="104"/>
+      <c r="AJ2" s="60" t="s">
         <v>215</v>
       </c>
-      <c r="AI2" s="97"/>
-      <c r="AJ2" s="80" t="s">
+      <c r="AK2" s="60"/>
+      <c r="AL2" s="60" t="s">
         <v>216</v>
       </c>
-      <c r="AK2" s="80"/>
-      <c r="AL2" s="80" t="s">
+      <c r="AM2" s="60"/>
+      <c r="AN2" s="60" t="s">
         <v>217</v>
       </c>
-      <c r="AM2" s="80"/>
-      <c r="AN2" s="80" t="s">
-        <v>218</v>
-      </c>
-      <c r="AO2" s="80"/>
+      <c r="AO2" s="60"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A3" s="60"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="109"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="98"/>
       <c r="E3" s="32" t="s">
         <v>24</v>
       </c>
@@ -43145,7 +43145,7 @@
       <c r="J3" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="K3" s="90"/>
+      <c r="K3" s="70"/>
       <c r="L3" s="29" t="s">
         <v>127</v>
       </c>
@@ -43173,19 +43173,19 @@
       <c r="T3" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="U3" s="94"/>
-      <c r="V3" s="94"/>
-      <c r="W3" s="94"/>
-      <c r="X3" s="94"/>
-      <c r="Y3" s="94"/>
-      <c r="Z3" s="94"/>
-      <c r="AA3" s="94"/>
-      <c r="AB3" s="94"/>
-      <c r="AC3" s="94"/>
-      <c r="AD3" s="94"/>
-      <c r="AE3" s="94"/>
-      <c r="AF3" s="94"/>
-      <c r="AG3" s="94"/>
+      <c r="U3" s="90"/>
+      <c r="V3" s="90"/>
+      <c r="W3" s="90"/>
+      <c r="X3" s="90"/>
+      <c r="Y3" s="90"/>
+      <c r="Z3" s="90"/>
+      <c r="AA3" s="90"/>
+      <c r="AB3" s="90"/>
+      <c r="AC3" s="90"/>
+      <c r="AD3" s="90"/>
+      <c r="AE3" s="90"/>
+      <c r="AF3" s="90"/>
+      <c r="AG3" s="90"/>
       <c r="AH3" s="29" t="s">
         <v>137</v>
       </c>
@@ -51814,6 +51814,20 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="wxJYPTS1M8YrpE+F5HXpzPvhVkWn+uzvbhQbX4zWGt7tgJJAc6rvipv1/0hraJgXbUY0X5vYRquC66cBDOGcbg==" saltValue="RWTcEymG3DdteXmtyGeu4A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="K2:K3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="U1:AG1"/>
@@ -51830,20 +51844,6 @@
     <mergeCell ref="AE2:AE3"/>
     <mergeCell ref="AD2:AD3"/>
     <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:V3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3 R3 AI3 AK3 AM3 L3 M3 N3 O3 P3 Q3 AO3 AJ3 AL3 AN3 AH3" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -51887,17 +51887,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="69" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="60"/>
+      <c r="A2" s="58"/>
       <c r="B2" s="30" t="s">
         <v>165</v>
       </c>
@@ -53139,25 +53139,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="94" t="s">
+      <c r="B1" s="90" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="71" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="61" t="s">
-        <v>206</v>
-      </c>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="63"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="75"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="60"/>
+      <c r="A2" s="58"/>
       <c r="B2" s="47" t="s">
         <v>145</v>
       </c>
@@ -55630,60 +55630,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="110" t="s">
+      <c r="B1" s="106" t="s">
         <v>159</v>
       </c>
-      <c r="C1" s="111"/>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="111"/>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="112"/>
-      <c r="L1" s="113" t="s">
+      <c r="C1" s="107"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="107"/>
+      <c r="F1" s="107"/>
+      <c r="G1" s="107"/>
+      <c r="H1" s="107"/>
+      <c r="I1" s="107"/>
+      <c r="J1" s="107"/>
+      <c r="K1" s="108"/>
+      <c r="L1" s="109" t="s">
+        <v>218</v>
+      </c>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="111"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="57"/>
+      <c r="B2" s="99" t="s">
+        <v>154</v>
+      </c>
+      <c r="C2" s="87" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="88"/>
+      <c r="E2" s="88"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="76" t="s">
+        <v>162</v>
+      </c>
+      <c r="I2" s="99" t="s">
+        <v>163</v>
+      </c>
+      <c r="J2" s="71" t="s">
         <v>219</v>
       </c>
-      <c r="M1" s="114"/>
-      <c r="N1" s="114"/>
-      <c r="O1" s="114"/>
-      <c r="P1" s="115"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="59" t="s">
-        <v>154</v>
-      </c>
-      <c r="C2" s="99" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="100"/>
-      <c r="E2" s="100"/>
-      <c r="F2" s="100"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="93" t="s">
-        <v>162</v>
-      </c>
-      <c r="I2" s="59" t="s">
-        <v>163</v>
-      </c>
-      <c r="J2" s="61" t="s">
-        <v>220</v>
-      </c>
-      <c r="K2" s="63"/>
-      <c r="L2" s="87"/>
-      <c r="M2" s="116"/>
-      <c r="N2" s="116"/>
-      <c r="O2" s="116"/>
-      <c r="P2" s="88"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="112"/>
+      <c r="N2" s="112"/>
+      <c r="O2" s="112"/>
+      <c r="P2" s="68"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="60"/>
-      <c r="B3" s="60"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="58"/>
       <c r="C3" s="53" t="s">
         <v>23</v>
       </c>
@@ -55699,8 +55699,8 @@
       <c r="G3" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="90"/>
-      <c r="I3" s="60"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="58"/>
       <c r="J3" s="54" t="s">
         <v>23</v>
       </c>
@@ -59390,136 +59390,136 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="99" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="89" t="s">
+      <c r="C1" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="110" t="s">
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="106" t="s">
         <v>78</v>
       </c>
-      <c r="G1" s="111"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="59" t="s">
+      <c r="G1" s="107"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="99" t="s">
+        <v>235</v>
+      </c>
+      <c r="J1" s="99" t="s">
         <v>236</v>
       </c>
-      <c r="J1" s="59" t="s">
+      <c r="K1" s="109" t="s">
+        <v>42</v>
+      </c>
+      <c r="L1" s="110"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="109" t="s">
+        <v>49</v>
+      </c>
+      <c r="O1" s="111"/>
+      <c r="P1" s="69" t="s">
         <v>237</v>
       </c>
-      <c r="K1" s="113" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="114"/>
-      <c r="M1" s="115"/>
-      <c r="N1" s="113" t="s">
-        <v>49</v>
-      </c>
-      <c r="O1" s="115"/>
-      <c r="P1" s="89" t="s">
+      <c r="Q1" s="90" t="s">
         <v>238</v>
       </c>
-      <c r="Q1" s="94" t="s">
+      <c r="R1" s="69" t="s">
         <v>239</v>
       </c>
-      <c r="R1" s="89" t="s">
-        <v>240</v>
+      <c r="S1" s="69" t="s">
+        <v>245</v>
       </c>
-      <c r="S1" s="89" t="s">
+      <c r="T1" s="69"/>
+      <c r="U1" s="113" t="s">
         <v>246</v>
       </c>
-      <c r="T1" s="89"/>
-      <c r="U1" s="117" t="s">
+      <c r="V1" s="114"/>
+      <c r="W1" s="113" t="s">
         <v>247</v>
       </c>
-      <c r="V1" s="118"/>
-      <c r="W1" s="117" t="s">
+      <c r="X1" s="114"/>
+      <c r="Y1" s="113" t="s">
         <v>248</v>
       </c>
-      <c r="X1" s="118"/>
-      <c r="Y1" s="117" t="s">
-        <v>249</v>
+      <c r="Z1" s="114"/>
+      <c r="AA1" s="69" t="s">
+        <v>244</v>
       </c>
-      <c r="Z1" s="118"/>
-      <c r="AA1" s="89" t="s">
-        <v>245</v>
-      </c>
-      <c r="AB1" s="89"/>
-      <c r="AC1" s="89"/>
-      <c r="AD1" s="89"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
     </row>
     <row r="2" spans="1:30" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="81" t="s">
+      <c r="A2" s="57"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="110" t="s">
+      <c r="D2" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="112"/>
-      <c r="F2" s="59" t="s">
+      <c r="E2" s="108"/>
+      <c r="F2" s="99" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="110" t="s">
+      <c r="G2" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="H2" s="112"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="87"/>
-      <c r="L2" s="116"/>
-      <c r="M2" s="88"/>
-      <c r="N2" s="87"/>
-      <c r="O2" s="88"/>
-      <c r="P2" s="89"/>
-      <c r="Q2" s="94"/>
-      <c r="R2" s="89"/>
-      <c r="S2" s="89"/>
-      <c r="T2" s="89"/>
-      <c r="U2" s="84"/>
-      <c r="V2" s="86"/>
-      <c r="W2" s="84"/>
-      <c r="X2" s="86"/>
-      <c r="Y2" s="84"/>
-      <c r="Z2" s="86"/>
-      <c r="AA2" s="89"/>
-      <c r="AB2" s="89"/>
-      <c r="AC2" s="89"/>
-      <c r="AD2" s="89"/>
+      <c r="H2" s="108"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="112"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="67"/>
+      <c r="O2" s="68"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="90"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="69"/>
+      <c r="T2" s="69"/>
+      <c r="U2" s="64"/>
+      <c r="V2" s="66"/>
+      <c r="W2" s="64"/>
+      <c r="X2" s="66"/>
+      <c r="Y2" s="64"/>
+      <c r="Z2" s="66"/>
+      <c r="AA2" s="69"/>
+      <c r="AB2" s="69"/>
+      <c r="AC2" s="69"/>
+      <c r="AD2" s="69"/>
     </row>
     <row r="3" spans="1:30" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="60"/>
-      <c r="B3" s="60"/>
-      <c r="C3" s="84"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="64"/>
       <c r="D3" s="30" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="60"/>
+      <c r="F3" s="58"/>
       <c r="G3" s="30" t="s">
         <v>0</v>
       </c>
       <c r="H3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
       <c r="K3" s="36" t="s">
         <v>193</v>
       </c>
       <c r="L3" s="33" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="M3" s="44" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N3" s="33" t="s">
         <v>47</v>
@@ -59527,9 +59527,9 @@
       <c r="O3" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="P3" s="89"/>
-      <c r="Q3" s="94"/>
-      <c r="R3" s="89"/>
+      <c r="P3" s="69"/>
+      <c r="Q3" s="90"/>
+      <c r="R3" s="69"/>
       <c r="S3" s="30" t="s">
         <v>50</v>
       </c>
@@ -59555,16 +59555,16 @@
         <v>129</v>
       </c>
       <c r="AA3" s="42" t="s">
+        <v>240</v>
+      </c>
+      <c r="AB3" s="36" t="s">
         <v>241</v>
       </c>
-      <c r="AB3" s="36" t="s">
+      <c r="AC3" s="36" t="s">
         <v>242</v>
       </c>
-      <c r="AC3" s="36" t="s">
+      <c r="AD3" s="36" t="s">
         <v>243</v>
-      </c>
-      <c r="AD3" s="36" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.25">
@@ -65942,11 +65942,8 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="WuDPT1+slParW8lK5SfJrIiCuXUqugKfunXVVDY0YB00pOtHXcdvDQyUD/jzqYTc2x6TyFXXd8XFSXwF4cqxTw==" saltValue="kHXwsv450+CnM8/ussNlMw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="I1:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="N1:O2"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
     <mergeCell ref="Y1:Z2"/>
     <mergeCell ref="AA1:AD2"/>
     <mergeCell ref="U1:V2"/>
@@ -65956,12 +65953,15 @@
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="R1:R3"/>
     <mergeCell ref="S1:T2"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="N1:O2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="C1:E1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3 AA3:AD3" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">

</xml_diff>